<commit_message>
Add local context compaction
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,9 +98,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P4：上下文治理准备</t>
+          <t>P4：上下文治理进行中</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P3 长任务运行基础已完成；P4 将处理 context summary/compaction 和中断恢复。</t>
+          <t>最小版本地 context compaction 已完成；下一步增强中断恢复。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -264,15 +264,32 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
+          <t>Context compaction</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>本地确定性</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>超过约 60000 字符时折叠早期历史，保留最近消息，并注入未完成 todo。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B11" s="0" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C11" s="0" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -487,17 +504,17 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>进行中</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>下一步启动 summary/compaction。</t>
+          <t>已完成本地 compaction；下一步补更强中断恢复。</t>
         </is>
       </c>
     </row>
@@ -574,9 +591,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
@@ -1245,25 +1262,52 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
+          <t>本地 Context Compaction</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>`context_char_budget` / `context_recent_messages`</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>折叠早期历史，保留最近消息，注入未完成 todo</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 LLM summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B26" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C26" s="0" t="inlineStr">
-        <is>
-          <t>当前 55 个测试通过</t>
-        </is>
-      </c>
-      <c r="D26" s="0" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>当前 57 个测试通过</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E26" s="0" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>继续补 P4 边界</t>
         </is>
@@ -1747,7 +1791,7 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
@@ -1762,7 +1806,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>超过阈值时折叠早期消息/工具输出</t>
+          <t>已实现本地 deterministic compaction，并注入未完成 todo</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2078,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="41" customWidth="1"/>
+    <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2104,12 +2148,12 @@
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>P4 做简单 summary/工具输出折叠</t>
+          <t>已做本地 compaction；后续评估 token 级阈值和 LLM summary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Handle interrupted tool calls safely
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,9 +98,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P4：上下文治理进行中</t>
+          <t>P5：安全与恢复增强进行中</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>最小版本地 context compaction 已完成；下一步增强中断恢复。</t>
+          <t>最小版本地 context compaction 已完成；正在增强 synthetic tool result 和恢复能力。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -281,15 +281,32 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
+          <t>Synthetic tool result</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>部分完成</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>deadline 到期和用户中断工具执行时会补齐剩余 tool_call 的 tool result。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B12" s="0" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C12" s="0" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -504,17 +521,17 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>已完成本地 compaction；下一步补更强中断恢复。</t>
+          <t>后续可评估 LLM summary 和 token 级阈值。</t>
         </is>
       </c>
     </row>
@@ -536,17 +553,17 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>进行中</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>P4 后补 synthetic tool result 与 patch preview/rollback。</t>
+          <t>已覆盖 deadline 和用户中断；下一步评估 patch preview/rollback。</t>
         </is>
       </c>
     </row>
@@ -591,13 +608,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1289,27 +1306,54 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
+          <t>Synthetic tool result</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>部分完成</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>deadline 到期和用户中断工具执行时补齐 tool result</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>避免 session 留下未配对 tool_calls</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>后续处理 `finish_reason=length`</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B27" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C27" s="0" t="inlineStr">
-        <is>
-          <t>当前 57 个测试通过</t>
-        </is>
-      </c>
-      <c r="D27" s="0" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>当前 58 个测试通过</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E27" s="0" t="inlineStr">
-        <is>
-          <t>继续补 P4 边界</t>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>继续补 P5 边界</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1330,7 +1374,7 @@
     <col min="4" max="4" width="31" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="7" max="7" width="36" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1833,7 +1877,7 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>部分完成</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -1848,7 +1892,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>未执行工具也写入配对 tool result</t>
+          <t>deadline 到期和用户中断已补齐；模型输出截断待评估</t>
         </is>
       </c>
     </row>
@@ -1959,7 +2003,7 @@
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
@@ -1974,7 +2018,7 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>用户 review 后提交</t>
+          <t>提交 `304fbdf` 已创建</t>
         </is>
       </c>
     </row>
@@ -2059,6 +2103,90 @@
       <c r="H18" s="0" t="inlineStr">
         <is>
           <t>LLM/tool timeout 按剩余预算夹紧；未执行工具有 synthetic result</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>T-017</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>提交 P4 compaction 变更</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>把上下文治理节点固化为 commit</t>
+        </is>
+      </c>
+      <c r="H19" s="0" t="inlineStr">
+        <is>
+          <t>提交 `4beb487` 已创建</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>T-018</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>处理模型输出截断 synthetic result</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>`finish_reason=length` 可能产生不完整工具参数</t>
+        </is>
+      </c>
+      <c r="H20" s="0" t="inlineStr">
+        <is>
+          <t>LLM 层暴露 finish_reason 并补可恢复提示</t>
         </is>
       </c>
     </row>
@@ -2244,12 +2372,12 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>P5 补 synthetic tool result</t>
+          <t>deadline 和用户中断已补齐；输出截断场景后续处理</t>
         </is>
       </c>
     </row>
@@ -2367,17 +2495,17 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>P3 变更尚未提交</t>
+          <t>P3/P4 变更尚未提交</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>用户 review 后提交第二个 commit</t>
+          <t>P3 提交 `304fbdf`，P4 提交 `4beb487`</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add patch dry-run preview
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -161,7 +161,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>最小版本地 context compaction 已完成；正在增强 synthetic tool result 和恢复能力。</t>
+          <t>最小版本地 context compaction 已完成；正在增强 synthetic tool result、patch preview 和恢复能力。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -298,15 +298,32 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
+          <t>Patch preview</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>`apply_patch dry_run=true` 只校验并返回 diff，不写文件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B13" s="0" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C13" s="0" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -558,12 +575,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline 和用户中断；下一步评估 patch preview/rollback。</t>
+          <t>已覆盖 deadline、用户中断和 patch preview；下一步评估 rollback。</t>
         </is>
       </c>
     </row>
@@ -608,7 +625,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -938,17 +955,17 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>replace/insert_before/insert_after</t>
+          <t>replace/insert_before/insert_after/dry_run</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>hash + old_text 校验</t>
+          <t>hash + old_text 校验；dry_run 只预览不写入</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>后续加 rollback/preview</t>
+          <t>后续加 rollback</t>
         </is>
       </c>
     </row>
@@ -1333,25 +1350,52 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
+          <t>Patch preview</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>`apply_patch dry_run=true`</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 rollback</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B28" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C28" s="0" t="inlineStr">
-        <is>
-          <t>当前 58 个测试通过</t>
-        </is>
-      </c>
-      <c r="D28" s="0" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>当前 60 个测试通过</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E28" s="0" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>继续补 P5 边界</t>
         </is>
@@ -1366,7 +1410,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1919,7 +1963,7 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>部分完成</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -1934,7 +1978,7 @@
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>先做最小设计再实现</t>
+          <t>已完成 dry_run 预览；rollback 待评估</t>
         </is>
       </c>
     </row>
@@ -2187,6 +2231,48 @@
       <c r="H20" s="0" t="inlineStr">
         <is>
           <t>LLM 层暴露 finish_reason 并补可恢复提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>T-019</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>实现 patch dry-run preview</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>写入前先看 diff，减少误改风险</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t>`apply_patch dry_run=true` 不写文件并返回 diff</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add session patch rollback
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -161,7 +161,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>最小版本地 context compaction 已完成；正在增强 synthetic tool result、patch preview 和恢复能力。</t>
+          <t>最小版本地 context compaction、patch preview 和 rollback 已完成；正在继续增强 synthetic tool result 和恢复能力。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -315,15 +315,32 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
+          <t>Patch rollback</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>`rollback_patch` 只回滚本 session 的 patch 记录，且要求当前文件仍匹配 after tag。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B14" s="0" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C14" s="0" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -575,12 +592,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>65%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断和 patch preview；下一步评估 rollback。</t>
+          <t>已覆盖 deadline、用户中断、patch preview 和 rollback；下一步处理 length 截断。</t>
         </is>
       </c>
     </row>
@@ -625,7 +642,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -965,41 +982,41 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>后续加 rollback</t>
+          <t>保持</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>write_file</t>
+          <t>rollback_patch</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>只创建新文件，拒绝覆盖</t>
+          <t>session patch log + after tag 校验</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>安全保守</t>
+          <t>只回滚本 session 中 apply_patch 写过且未被后续修改的文件</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>保持</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory</t>
+          <t>write_file</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -1009,24 +1026,24 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>project/decisions/conventions 基础版</t>
+          <t>只创建新文件，拒绝覆盖</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>轻量封闭 VM 友好</t>
+          <t>安全保守</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>保持</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Session JSONL</t>
+          <t>Markdown memory</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -1036,24 +1053,24 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>session/continue 基础恢复</t>
+          <t>project/decisions/conventions 基础版</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>已修缺 role 和坏尾部问题</t>
+          <t>轻量封闭 VM 友好</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>加 synthetic result</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>时间预算</t>
+          <t>Session JSONL</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -1063,24 +1080,24 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>`--budget-seconds` / `AGENT_BUDGET_SECONDS`</t>
+          <t>session/continue 基础恢复</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>默认 600 秒，0 可关闭</t>
+          <t>已修缺 role 和坏尾部问题</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>保持</t>
+          <t>加 synthetic result</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>预算细粒度检查</t>
+          <t>时间预算</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -1090,24 +1107,24 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>LLM/tool 使用剩余预算</t>
+          <t>`--budget-seconds` / `AGENT_BUDGET_SECONDS`</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>LLM timeout、shell/run_tests timeout 会被夹紧</t>
+          <t>默认 600 秒，0 可关闭</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>保持测试</t>
+          <t>保持</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>不限步主循环</t>
+          <t>预算细粒度检查</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -1117,24 +1134,24 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>`max_steps=0`</t>
+          <t>LLM/tool 使用剩余预算</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>默认不限步，显式设置才作为保险丝</t>
+          <t>LLM timeout、shell/run_tests timeout 会被夹紧</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>保持</t>
+          <t>保持测试</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>Todo 工具</t>
+          <t>不限步主循环</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -1144,24 +1161,24 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>`todo_read` / `todo_add` / `todo_update`</t>
+          <t>`max_steps=0`</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>session 级状态追踪</t>
+          <t>默认不限步，显式设置才作为保险丝</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>P4 长任务中继续验证</t>
+          <t>保持</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>ask_user</t>
+          <t>Todo 工具</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -1171,24 +1188,24 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>交互式终端可中途提问</t>
+          <t>`todo_read` / `todo_add` / `todo_update`</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>避免需求歧义时硬猜</t>
+          <t>session 级状态追踪</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>保持非交互错误提示</t>
+          <t>P4 长任务中继续验证</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>Per-tool approval</t>
+          <t>ask_user</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -1198,24 +1215,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>`--auto-approve-tools` / `AGENT_AUTO_APPROVE_TOOLS`</t>
+          <t>交互式终端可中途提问</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>ask 模式工具白名单</t>
+          <t>避免需求歧义时硬猜</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>按使用反馈微调</t>
+          <t>保持非交互错误提示</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>一键启动</t>
+          <t>Per-tool approval</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -1225,24 +1242,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>`./agent`</t>
+          <t>`--auto-approve-tools` / `AGENT_AUTO_APPROVE_TOOLS`</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>自动设置 `PYTHONPATH` 并以当前目录为 workspace</t>
+          <t>ask 模式工具白名单</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>日常入口</t>
+          <t>按使用反馈微调</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>`.env` 加载</t>
+          <t>一键启动</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -1252,24 +1269,24 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>workspace `.env`</t>
+          <t>`./agent`</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>可放 `DASHSCOPE_API_KEY`，被 gitignore</t>
+          <t>自动设置 `PYTHONPATH` 并以当前目录为 workspace</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>避免重复 export</t>
+          <t>日常入口</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记</t>
+          <t>`.env` 加载</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -1279,24 +1296,24 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>`docs/omp-core-architecture-notes.md`</t>
+          <t>workspace `.env`</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>固化主循环、deadline、compaction 结论</t>
+          <t>可放 `DASHSCOPE_API_KEY`，被 gitignore</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>后续设计依据</t>
+          <t>避免重复 export</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>本地 Context Compaction</t>
+          <t>OMP 核心架构笔记</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -1306,96 +1323,150 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>`context_char_budget` / `context_recent_messages`</t>
+          <t>`docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息，注入未完成 todo</t>
+          <t>固化主循环、deadline、compaction 结论</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>后续评估 LLM summary</t>
+          <t>后续设计依据</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>本地 Context Compaction</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>部分完成</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期和用户中断工具执行时补齐 tool result</t>
+          <t>`context_char_budget` / `context_recent_messages`</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>折叠早期历史，保留最近消息，注入未完成 todo</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>后续处理 `finish_reason=length`</t>
+          <t>后续评估 LLM summary</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>部分完成</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>deadline 到期和用户中断工具执行时补齐 tool result</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>后续处理 `finish_reason=length`</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
+          <t>Patch preview</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>`apply_patch dry_run=true`</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 rollback</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>Patch rollback</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>`rollback_patch`</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B29" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C29" s="0" t="inlineStr">
-        <is>
-          <t>当前 60 个测试通过</t>
-        </is>
-      </c>
-      <c r="D29" s="0" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>当前 62 个测试通过</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E29" s="0" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>继续补 P5 边界</t>
         </is>
@@ -1410,7 +1481,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1963,7 +2034,7 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>部分完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -1978,7 +2049,7 @@
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>已完成 dry_run 预览；rollback 待评估</t>
+          <t>已完成 dry_run 预览和 session 级 hash 校验 rollback</t>
         </is>
       </c>
     </row>
@@ -2273,6 +2344,48 @@
       <c r="H21" s="0" t="inlineStr">
         <is>
           <t>`apply_patch dry_run=true` 不写文件并返回 diff</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>T-020</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>实现 session 级 patch rollback</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>写错后可以在安全条件下恢复</t>
+        </is>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
+        <is>
+          <t>`rollback_patch` 校验 after tag 后恢复 before_text</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2293,6 +2406,7 @@
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2306,6 +2420,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2338,6 +2453,11 @@
           <t>应对/后续</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>OMP 是怎么实现的（建议实现方式）</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -2370,6 +2490,11 @@
           <t>已做本地 compaction；后续评估 token 级阈值和 LLM summary</t>
         </is>
       </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>OMP 用 token 估算触发 compaction，保留 recent 和输出 reserve；我们短期用字符阈值，后续补 token 估算和 LLM summary。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -2402,6 +2527,11 @@
           <t>已增加 session 级 todo 工具</t>
         </is>
       </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>OMP 把 todo 作为会话状态在 UI、session 和 reminder 中同步；我们保留轻量 `todo_read/add/update`，先满足长任务追踪。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -2434,6 +2564,11 @@
           <t>已增加 per-tool approval 白名单</t>
         </is>
       </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留白名单，危险 shell 仍强制确认。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -2466,6 +2601,11 @@
           <t>deadline 和用户中断已补齐；输出截断场景后续处理</t>
         </is>
       </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>OMP 在 abort、error、skipped、截断时补 synthetic tool result；我们按 call_id 补齐未执行工具，`finish_reason=length` 单独处理。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -2498,6 +2638,11 @@
           <t>已创建初始 commit</t>
         </is>
       </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>OMP 依赖 session、diff 和工作区状态追踪修改，但不替代 VCS 基线；我们继续用 git commit 作为回滚锚点。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -2530,6 +2675,11 @@
           <t>P6 暂缓，先稳定日用闭环</t>
         </is>
       </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们 P6 后置，先稳定单 Agent 闭环。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -2562,6 +2712,11 @@
           <t>文档提示；不信任仓库禁用 yolo</t>
         </is>
       </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将仓库 context 视为 advisory，并靠 approval/yolo 策略限制工具权限；我们默认不信任仓库内容，危险工具需确认。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -2594,6 +2749,11 @@
           <t>P3 提交 `304fbdf`，P4 提交 `4beb487`</t>
         </is>
       </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>OMP 持久化 session 和 compaction 以支持恢复，但代码里程碑仍要靠 VCS；我们继续阶段性 commit 固化节点。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -2626,6 +2786,11 @@
           <t>长任务需求尽量写清；后续评估 ask_user 超时策略</t>
         </is>
       </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 approval/elicitation 可以被拒绝或取消并回灌结果；我们后续给 `ask_user` 加 timeout/default，支持无人值守。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -2658,6 +2823,11 @@
           <t>每个能力做简化版</t>
         </is>
       </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>OMP 是平台型 Agent，能力面很宽；我们只借主循环、deadline、compaction、approval、memory 等边界，逐个做简化版。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -2690,6 +2860,11 @@
           <t>默认值已改为 0，不限步</t>
         </is>
       </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -2722,6 +2897,11 @@
           <t>P3 已实现</t>
         </is>
       </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -2754,6 +2934,11 @@
           <t>后续看需求升级</t>
         </is>
       </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -2786,6 +2971,11 @@
           <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -2818,6 +3008,11 @@
           <t>README 已写推荐工作流</t>
         </is>
       </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -2850,6 +3045,11 @@
           <t>依赖提前准备</t>
         </is>
       </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -2882,6 +3082,11 @@
           <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的事实上下文来自 session、memory 和 Markdown 规则，UI 只是视图；我们以 Markdown 为事实源，Excel 只生成展示。</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -2914,10 +3119,15 @@
           <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Handle truncated tool-call responses
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -161,7 +161,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>最小版本地 context compaction、patch preview 和 rollback 已完成；正在继续增强 synthetic tool result 和恢复能力。</t>
+          <t>最小版本地 context compaction、synthetic tool result、patch preview 和 rollback 已完成；正在继续做真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -286,12 +286,12 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>部分完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期和用户中断工具执行时会补齐剩余 tool_call 的 tool result。</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时会补齐剩余 tool_call 的 tool result。</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、patch preview 和 rollback；下一步处理 length 截断。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview 和 rollback；下一步真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1372,12 +1372,12 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>部分完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期和用户中断工具执行时补齐 tool result</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>后续处理 `finish_reason=length`</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>当前 62 个测试通过</t>
+          <t>当前 64 个测试通过</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>部分完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期和用户中断已补齐；模型输出截断待评估</t>
+          <t>deadline 到期、用户中断和 length 截断已补齐</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>LLM 层暴露 finish_reason 并补可恢复提示</t>
+          <t>LLM 层已暴露 finish_reason，并补可恢复提示</t>
         </is>
       </c>
     </row>
@@ -2593,17 +2593,17 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>deadline 和用户中断已补齐；输出截断场景后续处理</t>
+          <t>deadline、用户中断和输出截断已补齐</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>OMP 在 abort、error、skipped、截断时补 synthetic tool result；我们按 call_id 补齐未执行工具，`finish_reason=length` 单独处理。</t>
+          <t>OMP 在 abort、error、skipped、截断时补 synthetic tool result；我们按 call_id 补齐未执行工具，并已处理 `finish_reason=length`。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bound ask_user waiting time
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -161,7 +161,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>最小版本地 context compaction、synthetic tool result、patch preview 和 rollback 已完成；正在继续做真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback 和 ask_user timeout 已完成；正在继续做真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -332,15 +332,32 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
+          <t>ask_user timeout</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>`ask_user` 支持 `timeout_seconds` / `default_answer`，并受当前 budget 剩余时间约束。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B15" s="0" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C15" s="0" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -582,7 +599,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>synthetic tool result、patch preview、rollback</t>
+          <t>synthetic tool result、patch preview、rollback、ask_user timeout</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -592,12 +609,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview 和 rollback；下一步真实任务压测。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback 和 ask_user timeout；下一步真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -642,7 +659,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1215,17 +1232,17 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>交互式终端可中途提问</t>
+          <t>交互式终端可中途提问，支持 timeout/default</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>避免需求歧义时硬猜</t>
+          <t>避免需求歧义时硬猜，也避免长任务无限等待</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>保持非交互错误提示</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
@@ -1448,25 +1465,52 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
+          <t>ask_user timeout</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>长任务无人响应时可以继续或明确失败</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B31" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C31" s="0" t="inlineStr">
-        <is>
-          <t>当前 64 个测试通过</t>
-        </is>
-      </c>
-      <c r="D31" s="0" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>当前 67 个测试通过</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E31" s="0" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>继续补 P5 边界</t>
         </is>
@@ -1481,7 +1525,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2386,6 +2430,48 @@
       <c r="H22" s="0" t="inlineStr">
         <is>
           <t>`rollback_patch` 校验 after tag 后恢复 before_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>T-021</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>实现 ask_user timeout/default</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>防止长任务等待用户输入时无限阻塞</t>
+        </is>
+      </c>
+      <c r="H23" s="0" t="inlineStr">
+        <is>
+          <t>`ask_user` 支持 timeout/default，并受 budget 剩余时间约束</t>
         </is>
       </c>
     </row>
@@ -2778,17 +2864,17 @@
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>长任务需求尽量写清；后续评估 ask_user 超时策略</t>
+          <t>已支持 timeout/default，并自动受剩余 budget 约束</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 approval/elicitation 可以被拒绝或取消并回灌结果；我们后续给 `ask_user` 加 timeout/default，支持无人值守。</t>
+          <t>OMP 的 approval/elicitation 可以被拒绝或取消并回灌结果；我们给 `ask_user` 加 timeout/default，支持无人值守场景。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-tool approval policies
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -161,7 +161,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback 和 ask_user timeout 已完成；正在继续做真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 per-tool approval 已完成；正在继续做真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -349,15 +349,32 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
+          <t>Per-tool approval</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>`tool_approval` 支持每个工具 `allow` / `prompt` / `deny`，旧 auto approve 白名单兼容映射为 allow。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
           <t>OMP 核心判断</t>
         </is>
       </c>
-      <c r="B16" s="0" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>已固化</t>
         </is>
       </c>
-      <c r="C16" s="0" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`。</t>
         </is>
@@ -599,7 +616,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>synthetic tool result、patch preview、rollback、ask_user timeout</t>
+          <t>synthetic tool result、patch preview、rollback、ask_user timeout、per-tool approval</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -609,12 +626,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback 和 ask_user timeout；下一步真实任务压测。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout 和 per-tool policy；下一步真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -659,7 +676,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1259,17 +1276,17 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>`--auto-approve-tools` / `AGENT_AUTO_APPROVE_TOOLS`</t>
+          <t>`--auto-approve-tools` + `--tool-approval`</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>ask 模式工具白名单</t>
+          <t>兼容旧白名单，并支持每个工具 allow / prompt / deny</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>按使用反馈微调</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
@@ -1492,25 +1509,52 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
+          <t>Tool approval policy</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>`tool_approval`</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>`deny` 最强，`allow` 直接放行，`prompt` 强制询问</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B32" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C32" s="0" t="inlineStr">
-        <is>
-          <t>当前 67 个测试通过</t>
-        </is>
-      </c>
-      <c r="D32" s="0" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>当前 73 个测试通过</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>unittest + compileall 通过</t>
         </is>
       </c>
-      <c r="E32" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>继续补 P5 边界</t>
         </is>
@@ -1525,12 +1569,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="31" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="36" customWidth="1"/>
@@ -2472,6 +2516,48 @@
       <c r="H23" s="0" t="inlineStr">
         <is>
           <t>`ask_user` 支持 timeout/default，并受 budget 剩余时间约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>T-022</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>实现 tool_approval allow/prompt/deny</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>白名单不够表达显式拒绝和强制询问</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>`--tool-approval` / `AGENT_TOOL_APPROVAL` 支持每工具策略</t>
         </is>
       </c>
     </row>
@@ -2647,12 +2733,12 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>已增加 per-tool approval 白名单</t>
+          <t>已增加 per-tool allow/prompt/deny 策略</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留白名单，危险 shell 仍强制确认。</t>
+          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留旧白名单并补 `tool_approval`，危险 shell 仍可显式 deny。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete approval permission model
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强进行中</t>
+          <t>P5：安全与恢复增强 MVP 完成</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 per-tool approval 已完成；正在继续做真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 OMP 风格 approval model 已完成；下一步做真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -359,7 +359,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` 支持每个工具 `allow` / `prompt` / `deny`，旧 auto approve 白名单兼容映射为 allow。</t>
+          <t>支持 `always-ask` / `write` / `yolo`、per-tool `allow` / `prompt` / `deny`、session always allow/reject 和 REPL `/approval`。</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>后续可评估 LLM summary 和 token 级阈值。</t>
+          <t>下一步按 OMP 风格升级 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
         </is>
       </c>
     </row>
@@ -621,17 +621,17 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout 和 per-tool policy；下一步真实任务压测。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision 和 REPL 命令。</t>
         </is>
       </c>
     </row>
@@ -681,8 +681,8 @@
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>`--auto-approve-tools` + `--tool-approval`</t>
+          <t>`--auto-approve-tools` + `--tool-approval` + `/approval`</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>兼容旧白名单，并支持每个工具 allow / prompt / deny</t>
+          <t>兼容旧白名单，并支持每个工具 allow / prompt / deny、session always allow/reject</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>后续评估 LLM summary</t>
+          <t>下一步补 token 预算、输出 reserve 和可选 LLM summary；字符阈值保留兜底</t>
         </is>
       </c>
     </row>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval`</t>
+          <t>`tool_approval` + `session_tool_approval`</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>`deny` 最强，`allow` 直接放行，`prompt` 强制询问</t>
+          <t>config deny 最强，session allow/reject 可记住当前会话，prompt 可强制询问</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>当前 73 个测试通过</t>
+          <t>当前 79 个测试通过</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>继续补 P5 边界</t>
+          <t>继续补真实任务压测</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1569,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="36" customWidth="1"/>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>已实现本地 deterministic compaction，并注入未完成 todo</t>
+          <t>已实现字符阈值 deterministic compaction；下一步升级 token budget / reserve / LLM summary</t>
         </is>
       </c>
     </row>
@@ -2558,6 +2558,48 @@
       <c r="H24" s="0" t="inlineStr">
         <is>
           <t>`--tool-approval` / `AGENT_TOOL_APPROVAL` 支持每工具策略</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>T-023</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>实现 approvalMode / session decision / REPL 命令</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>对齐 OMP 三层审批模型的本地 MVP</t>
+        </is>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
+        <is>
+          <t>支持 `always-ask` / `write` / `yolo`、`s/d` 会话记忆、`/approval` 命令</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2619,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2654,17 +2696,17 @@
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>继续增强</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做本地 compaction；后续评估 token 级阈值和 LLM summary</t>
+          <t>已做字符阈值 compaction；下一步按 OMP 风格升级 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>OMP 用 token 估算触发 compaction，保留 recent 和输出 reserve；我们短期用字符阈值，后续补 token 估算和 LLM summary。</t>
+          <t>OMP 按上下文 token 预算触发压缩，给下一轮 prompt/输出预留 reserve，并把早期历史压成 summary；建议我们把字符阈值升级为 token 估算 + reserve + 可选 LLM summary，字符阈值只保留为兜底。</t>
         </is>
       </c>
     </row>
@@ -2728,17 +2770,17 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>已增加 per-tool allow/prompt/deny 策略</t>
+          <t>已增加 approvalMode、per-tool allow/prompt/deny、session allow/reject</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留旧白名单并补 `tool_approval`，危险 shell 仍可显式 deny。</t>
+          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留旧白名单并补 `tool_approval` 和 session decision，危险 shell 仍可显式 deny。</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3355,7 @@
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="46" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3431,7 +3473,7 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>默认 ask；只读可 auto-read；可信重复工具可 auto-approve；信任仓库才 yolo</t>
+          <t>默认 always-ask；写操作可用 write；可信重复工具可 tool-approval allow；信任仓库才 yolo</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
@@ -3441,12 +3483,12 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>P3+</t>
+          <t>P5+</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>`--auto-approve-tools run_tests,git_diff` 可用</t>
+          <t>`--tool-approval run_tests=allow,shell=prompt,write_file=deny` 可用</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten approval policy precedence
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 完成</t>
+          <t>P5：安全与恢复增强 MVP 完成，继续补体验缺口</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 OMP 风格 approval model 已完成；下一步做真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 OMP 风格 approval model 已完成；下一步优先做 T-024 approval prompt deadline/abort，然后真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -394,7 +394,7 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
@@ -621,7 +621,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成 MVP 版，继续增强</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision 和 REPL 命令。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision 和 REPL 命令；下一步补 approval prompt deadline/abort。</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1524,12 +1524,12 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>config deny 最强，session allow/reject 可记住当前会话，prompt 可强制询问</t>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步补 approval prompt deadline/abort，避免同步 `input()` 等待耗尽预算</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>当前 79 个测试通过</t>
+          <t>当前 82 个测试通过</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1577,7 +1577,7 @@
     <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="36" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2600,6 +2600,90 @@
       <c r="H25" s="0" t="inlineStr">
         <is>
           <t>支持 `always-ask` / `write` / `yolo`、`s/d` 会话记忆、`/approval` 命令</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>T-024</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>approval prompt 支持 deadline/abort</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>人工确认等待也消耗 wall-clock budget，当前 `input()` 不能被 deadline 打断</t>
+        </is>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t>对齐 OMP：权限请求受 abort signal 控制；超时自动取消/拒绝，并补齐 tool result</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>T-025</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>修复 approval 优先级和工具名校验</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>避免新 `tools.*` 被旧顶层字段静默覆盖、config prompt 被 session allow 绕过、REPL 工具名输错后假成功</t>
+        </is>
+      </c>
+      <c r="H27" s="0" t="inlineStr">
+        <is>
+          <t>新配置优先于旧字段；config prompt/deny 是硬护栏；REPL 校验未知工具名</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2696,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -3009,37 +3093,37 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-010</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>不照搬 OMP，只借鉴能力类型和边界</t>
+          <t>approval prompt 等待耗尽预算</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>开放</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>每个能力做简化版</t>
+          <t>当前 `input()` 等待期间会消耗 `budget_seconds`，确认后可能立刻停止；后续补 deadline/abort 型 approval prompt</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>OMP 是平台型 Agent，能力面很宽；我们只借主循环、deadline、compaction、approval、memory 等边界，逐个做简化版。</t>
+          <t>OMP 的 deadline 是 wall-clock absolute timestamp；但 ACP permission gate 会把 `requestPermission` 和 abort signal 竞争，deadline 到期可取消等待。</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3135,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -3061,22 +3145,22 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>不照搬 OMP，只借鉴能力类型和边界</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>每个能力做简化版</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是平台型 Agent，能力面很宽；我们只借主循环、deadline、compaction、approval、memory 等边界，逐个做简化版。</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3172,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -3098,7 +3182,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -3108,12 +3192,12 @@
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3209,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -3135,22 +3219,22 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3246,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -3172,7 +3256,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -3182,12 +3266,12 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3283,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -3209,7 +3293,7 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -3219,12 +3303,12 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3320,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -3246,7 +3330,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -3256,12 +3340,12 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3357,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -3283,7 +3367,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -3293,12 +3377,12 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 的事实上下文来自 session、memory 和 Markdown 规则，UI 只是视图；我们以 Markdown 为事实源，Excel 只生成展示。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -3310,30 +3394,67 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
+          <t>ADR-008</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Excel 给人看，Markdown 给 Agent 读</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>持续同步本文件和 `project-status.md`</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的事实上下文来自 session、memory 和 Markdown 规则，UI 只是视图；我们以 Markdown 为事实源，Excel 只生成展示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
           <t>ADR-009</t>
         </is>
       </c>
-      <c r="C20" s="0" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="D20" s="0" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
-      <c r="E20" s="0" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F20" s="0" t="inlineStr">
+      <c r="F21" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
-      <c r="G20" s="0" t="inlineStr">
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>

</xml_diff>

<commit_message>
Cancel approval prompts at deadline
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 完成，继续补体验缺口</t>
+          <t>P5：安全与恢复增强 MVP 完成，进入真实任务压测</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout 和 OMP 风格 approval model 已完成；下一步优先做 T-024 approval prompt deadline/abort，然后真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout、approval prompt deadline cancel 和 OMP 风格 approval model 已完成；下一步做真实任务压测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -394,7 +394,7 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
@@ -599,7 +599,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>下一步按 OMP 风格升级 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
+          <t>真实任务压测后再评估 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版，继续增强</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision 和 REPL 命令；下一步补 approval prompt deadline/abort。</t>
+          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision、REPL 命令和 approval deadline cancel。</t>
         </is>
       </c>
     </row>
@@ -1524,12 +1524,12 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名</t>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>下一步补 approval prompt deadline/abort，避免同步 `input()` 等待耗尽预算</t>
+          <t>继续真实任务压测</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>当前 82 个测试通过</t>
+          <t>当前 87 个测试通过</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>待办</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
@@ -2636,12 +2636,12 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>人工确认等待也消耗 wall-clock budget，当前 `input()` 不能被 deadline 打断</t>
+          <t>人工确认等待也消耗 wall-clock budget，不能让确认等待绕过 `budget_seconds`</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t>对齐 OMP：权限请求受 abort signal 控制；超时自动取消/拒绝，并补齐 tool result</t>
+          <t>approval prompt 使用 deadline-aware timed stdin；deadline 到期自动取消/拒绝，保留 `y/s/n/d` 和 session allow/reject</t>
         </is>
       </c>
     </row>
@@ -3113,17 +3113,17 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>当前 `input()` 等待期间会消耗 `budget_seconds`，确认后可能立刻停止；后续补 deadline/abort 型 approval prompt</t>
+          <t>approval prompt 已使用 deadline-aware timed stdin；deadline 已过或等待超时会取消工具调用</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 deadline 是 wall-clock absolute timestamp；但 ACP permission gate 会把 `requestPermission` 和 abort signal 竞争，deadline 到期可取消等待。</t>
+          <t>OMP 的 deadline 是 wall-clock absolute timestamp；ACP permission gate 会把 `requestPermission` 和 abort signal 竞争。我们本地版用 `select.select` 按剩余 deadline 等 stdin，超时即取消。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt OMP design pragmatically
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已形成不照搬、做简化版的原则。</t>
+          <t>已形成“优先吸收成熟设计，按本地目标裁剪”的原则。</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>不照搬 OMP，只借鉴能力类型和边界</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -3155,12 +3155,12 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>每个能力做简化版</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>OMP 是平台型 Agent，能力面很宽；我们只借主循环、deadline、compaction、approval、memory 等边界，逐个做简化版。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clamp ask_user budget and truncate tool compaction
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -274,7 +274,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>超过约 60000 字符时折叠早期历史，保留最近消息，并注入未完成 todo。</t>
+          <t>超过约 60000 字符时折叠早期历史，保留最近消息，注入未完成 todo，并截断发送给模型的超大 tool 输出。</t>
         </is>
       </c>
     </row>
@@ -342,7 +342,7 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>`ask_user` 支持 `timeout_seconds` / `default_answer`，并受当前 budget 剩余时间约束。</t>
+          <t>`ask_user` 支持 `timeout_seconds` / `default_answer`，显式 timeout 也会被当前 budget 剩余时间夹紧。</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息，注入未完成 todo</t>
+          <t>折叠早期历史，保留最近消息，注入未完成 todo，并截断发送给模型的超大 tool 输出</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败</t>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>当前 87 个测试通过</t>
+          <t>当前 89 个测试通过</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2684,6 +2684,48 @@
       <c r="H27" s="0" t="inlineStr">
         <is>
           <t>新配置优先于旧字段；config prompt/deny 是硬护栏；REPL 校验未知工具名</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>T-026</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>夹紧 ask_user timeout 并截断 compaction tool 输出</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>消除 ask_user 文档与代码不一致，降低长任务 compaction 软预算超标风险</t>
+        </is>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
+        <is>
+          <t>显式 `timeout_seconds` 会被剩余 budget 夹紧；recent tool 输出只在发送模型副本中截断，session 原文保留</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2744,7 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
@@ -2780,12 +2822,12 @@
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>继续增强</t>
+          <t>已进一步缓解，继续增强</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction；下一步按 OMP 风格升级 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction，并截断发送给模型的超大 tool 输出；下一步真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
@@ -3081,7 +3123,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>已支持 timeout/default，并自动受剩余 budget 约束</t>
+          <t>已支持 timeout/default，并自动受剩余 budget 约束；显式 timeout 也会被剩余 budget 夹紧</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Clarify project management docs are for development
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>让 Agent 可读项目路线</t>
+          <t>让开发协作 Agent 可读项目路线</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给 Agent 读</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>OMP 的事实上下文来自 session、memory 和 Markdown 规则，UI 只是视图；我们以 Markdown 为事实源，Excel 只生成展示。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="4" max="4" width="31" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Excel 是产物，Markdown 是事实源</t>
+          <t>Excel 是开发展示产物，Markdown 是开发事实源</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Merge compaction summary into system prompt
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -274,7 +274,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>超过约 60000 字符时折叠早期历史，保留最近消息，注入未完成 todo，并截断发送给模型的超大 tool 输出。</t>
+          <t>超过约 60000 字符时折叠早期历史，保留最近消息，注入未完成 todo，截断发送给模型的超大 tool 输出，并把摘要合并进首个 system prompt 以提升 provider 兼容性。</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息，注入未完成 todo，并截断发送给模型的超大 tool 输出</t>
+          <t>折叠早期历史，保留最近消息，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2726,6 +2726,48 @@
       <c r="H28" s="0" t="inlineStr">
         <is>
           <t>显式 `timeout_seconds` 会被剩余 budget 夹紧；recent tool 输出只在发送模型副本中截断，session 原文保留</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>T-027</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>compaction 保持单 system 消息</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>降低 OpenAI-compatible provider 对多 system 消息的兼容风险</t>
+        </is>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
+        <is>
+          <t>压缩摘要合并进首个 system prompt；测试锁定发送给模型时只有一条 system</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2869,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction，并截断发送给模型的超大 tool 输出；下一步真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction、超大 tool 输出截断和单 system 摘要合并；下一步真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Preserve current request during compaction
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -274,7 +274,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>超过约 60000 字符时折叠早期历史，保留最近消息，注入未完成 todo，截断发送给模型的超大 tool 输出，并把摘要合并进首个 system prompt 以提升 provider 兼容性。</t>
+          <t>超过约 60000 字符时折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并把摘要合并进首个 system prompt 以提升 provider 兼容性。</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
+          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2768,6 +2768,48 @@
       <c r="H29" s="0" t="inlineStr">
         <is>
           <t>压缩摘要合并进首个 system prompt；测试锁定发送给模型时只有一条 system</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>T-028</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>百炼只读压测后的目标漂移修复</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>极小上下文预算下，模型会被续读提示和最近代码片段带偏</t>
+        </is>
+      </c>
+      <c r="H30" s="0" t="inlineStr">
+        <is>
+          <t>compaction 摘要强保留当前用户请求；read_file 截断提示改为“任务需要才继续”</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2911,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction、超大 tool 输出截断和单 system 摘要合并；下一步真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；下一步继续真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Record Bailian compaction smoke test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 完成，进入真实任务压测</t>
+          <t>P5：安全与恢复增强 MVP 完成，首轮真实百炼只读压测通过</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout、approval prompt deadline cancel 和 OMP 风格 approval model 已完成；下一步做真实任务压测。</t>
+          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout、approval prompt deadline cancel 和 OMP 风格 approval model 已完成；百炼只读 compaction 压测已验证模型能在压缩后停止探索并按要求总结。</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>真实任务压测后再评估 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
+          <t>首轮百炼只读 compaction 压测已通过；继续用真实小改任务压测后再评估 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务压测</t>
+          <t>继续真实小改任务压测</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2810,6 +2810,90 @@
       <c r="H30" s="0" t="inlineStr">
         <is>
           <t>compaction 摘要强保留当前用户请求；read_file 截断提示改为“任务需要才继续”</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>T-029</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>复测百炼只读 compaction 压测</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>验证 T-028 是否真正修复目标漂移</t>
+        </is>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t>会话 `20260707T093557800154Z` 严格完成 5 个指定工具调用后输出三句话总结，未继续额外读文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>T-030</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>真实小改任务压测</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>验证 compaction、approval、patch preview/rollback、run_tests、git_diff 在真实修改任务中的协同</t>
+        </is>
+      </c>
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t>用百炼执行一个小 README/测试改动，要求 dry_run、apply_patch、run_tests、git_diff</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2995,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；下一步继续真实压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；首轮百炼只读压测通过，下一步继续真实小改压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Align write_file schema with create-only behavior
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="39" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 完成，首轮真实百炼只读压测通过</t>
+          <t>P5：安全与恢复增强 MVP 完成，真实百炼小改压测发现并修复工具描述问题</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Context compaction、synthetic tool result、patch preview、rollback、ask_user timeout、approval prompt deadline cancel 和 OMP 风格 approval model 已完成；百炼只读 compaction 压测已验证模型能在压缩后停止探索并按要求总结。</t>
+          <t>百炼只读 compaction 压测已通过；首轮真实小改压测跑通 dry_run、apply_patch、run_tests、git_diff，但暴露 `write_file` schema 描述误导模型，已修正并待复测。</t>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>继续真实小改任务压测</t>
+          <t>复测真实小改任务</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>当前 89 个测试通过</t>
+          <t>当前 90 个测试通过</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>首轮发现问题，待复测</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
@@ -2893,7 +2893,49 @@
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t>用百炼执行一个小 README/测试改动，要求 dry_run、apply_patch、run_tests、git_diff</t>
+          <t>首轮会话 `20260707T093733679947Z` 跑通链路，但因 `write_file` schema 描述错误导致 README 被改成不符合实现的说法</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>T-031</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>修正 `write_file` schema 描述误导</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>工具描述会进入模型上下文，错误描述会直接导致错误修改</t>
+        </is>
+      </c>
+      <c r="H33" s="0" t="inlineStr">
+        <is>
+          <t>`write_file` 描述已改为 create-only，并加测试确保不再出现 `fully overwrite`</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2948,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2995,7 +3037,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；首轮百炼只读压测通过，下一步继续真实小改压测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；首轮百炼只读压测通过，继续真实小改复测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
@@ -3012,7 +3054,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>R-002</t>
+          <t>R-011</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -3022,22 +3064,22 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>没有 todo 工具</t>
+          <t>工具 schema 描述与实现不一致会误导模型</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已关闭首例，持续关注</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>已增加 session 级 todo 工具</t>
+          <t>首轮真实小改压测发现 `write_file` 描述宣称可覆盖文件，但实现拒绝覆盖，导致模型把 README 改错</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>OMP 把 todo 作为会话状态在 UI、session 和 reminder 中同步；我们保留轻量 `todo_read/add/update`，先满足长任务追踪。</t>
+          <t>工具 schema 是模型的操作说明，应与实现和测试保持一致；已修正 `write_file` 描述并新增测试。</t>
         </is>
       </c>
     </row>
@@ -3049,32 +3091,32 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>R-003</t>
+          <t>R-002</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>ask 模式确认过多</t>
+          <t>没有 todo 工具</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>已增加 approvalMode、per-tool allow/prompt/deny、session allow/reject</t>
+          <t>已增加 session 级 todo 工具</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留旧白名单并补 `tool_approval` 和 session decision，危险 shell 仍可显式 deny。</t>
+          <t>OMP 把 todo 作为会话状态在 UI、session 和 reminder 中同步；我们保留轻量 `todo_read/add/update`，先满足长任务追踪。</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3128,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>R-003</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -3096,7 +3138,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>中断时 tool_calls 配对仍可增强</t>
+          <t>ask 模式确认过多</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -3106,12 +3148,12 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>deadline、用户中断和输出截断已补齐</t>
+          <t>已增加 approvalMode、per-tool allow/prompt/deny、session allow/reject</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>OMP 在 abort、error、skipped、截断时补 synthetic tool result；我们按 call_id 补齐未执行工具，并已处理 `finish_reason=length`。</t>
+          <t>OMP 用 tool approval tier、approvalMode 和 per-tool policy 控制确认；我们保留旧白名单并补 `tool_approval` 和 session decision，危险 shell 仍可显式 deny。</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3165,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>R-005</t>
+          <t>R-004</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -3133,22 +3175,22 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>没有初始 git commit</t>
+          <t>中断时 tool_calls 配对仍可增强</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>已创建初始 commit</t>
+          <t>deadline、用户中断和输出截断已补齐</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>OMP 依赖 session、diff 和工作区状态追踪修改，但不替代 VCS 基线；我们继续用 git commit 作为回滚锚点。</t>
+          <t>OMP 在 abort、error、skipped、截断时补 synthetic tool result；我们按 call_id 补齐未执行工具，并已处理 `finish_reason=length`。</t>
         </is>
       </c>
     </row>
@@ -3160,32 +3202,32 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>R-006</t>
+          <t>R-005</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>高级能力过早引入</t>
+          <t>没有初始 git commit</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>受控</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>P6 暂缓，先稳定日用闭环</t>
+          <t>已创建初始 commit</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们 P6 后置，先稳定单 Agent 闭环。</t>
+          <t>OMP 依赖 session、diff 和工作区状态追踪修改，但不替代 VCS 基线；我们继续用 git commit 作为回滚锚点。</t>
         </is>
       </c>
     </row>
@@ -3197,32 +3239,32 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>R-007</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>Prompt injection</t>
+          <t>高级能力过早引入</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>开放</t>
+          <t>受控</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>文档提示；不信任仓库禁用 yolo</t>
+          <t>P6 暂缓，先稳定日用闭环</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>OMP 将仓库 context 视为 advisory，并靠 approval/yolo 策略限制工具权限；我们默认不信任仓库内容，危险工具需确认。</t>
+          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们 P6 后置，先稳定单 Agent 闭环。</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3276,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>R-008</t>
+          <t>R-007</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -3244,22 +3286,22 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>P3/P4 变更尚未提交</t>
+          <t>Prompt injection</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>开放</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>P3 提交 `304fbdf`，P4 提交 `4beb487`</t>
+          <t>文档提示；不信任仓库禁用 yolo</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>OMP 持久化 session 和 compaction 以支持恢复，但代码里程碑仍要靠 VCS；我们继续阶段性 commit 固化节点。</t>
+          <t>OMP 将仓库 context 视为 advisory，并靠 approval/yolo 策略限制工具权限；我们默认不信任仓库内容，危险工具需确认。</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3313,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>R-009</t>
+          <t>R-008</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -3281,22 +3323,22 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>ask_user 会阻塞等待用户</t>
+          <t>P3/P4 变更尚未提交</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>已支持 timeout/default，并自动受剩余 budget 约束；显式 timeout 也会被剩余 budget 夹紧</t>
+          <t>P3 提交 `304fbdf`，P4 提交 `4beb487`</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 approval/elicitation 可以被拒绝或取消并回灌结果；我们给 `ask_user` 加 timeout/default，支持无人值守场景。</t>
+          <t>OMP 持久化 session 和 compaction 以支持恢复，但代码里程碑仍要靠 VCS；我们继续阶段性 commit 固化节点。</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3350,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>R-010</t>
+          <t>R-009</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -3318,59 +3360,59 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>approval prompt 等待耗尽预算</t>
+          <t>ask_user 会阻塞等待用户</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>approval prompt 已使用 deadline-aware timed stdin；deadline 已过或等待超时会取消工具调用</t>
+          <t>已支持 timeout/default，并自动受剩余 budget 约束；显式 timeout 也会被剩余 budget 夹紧</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 deadline 是 wall-clock absolute timestamp；ACP permission gate 会把 `requestPermission` 和 abort signal 竞争。我们本地版用 `select.select` 按剩余 deadline 等 stdin，超时即取消。</t>
+          <t>OMP 的 approval/elicitation 可以被拒绝或取消并回灌结果；我们给 `ask_user` 加 timeout/default，支持无人值守场景。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-010</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>approval prompt 等待耗尽预算</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>approval prompt 已使用 deadline-aware timed stdin；deadline 已过或等待超时会取消工具调用</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 的 deadline 是 wall-clock absolute timestamp；ACP permission gate 会把 `requestPermission` 和 abort signal 竞争。我们本地版用 `select.select` 按剩余 deadline 等 stdin，超时即取消。</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3424,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -3392,22 +3434,22 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3461,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -3429,7 +3471,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -3439,12 +3481,12 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3498,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -3466,22 +3508,22 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3535,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -3503,7 +3545,7 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -3513,12 +3555,12 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3572,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -3540,7 +3582,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -3550,12 +3592,12 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3609,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -3577,7 +3619,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -3587,12 +3629,12 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3646,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -3614,7 +3656,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -3624,12 +3666,12 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -3641,30 +3683,67 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
+          <t>ADR-008</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>持续同步本文件和 `project-status.md`</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
           <t>ADR-009</t>
         </is>
       </c>
-      <c r="C21" s="0" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="D21" s="0" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
-      <c r="E21" s="0" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F21" s="0" t="inlineStr">
+      <c r="F22" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
-      <c r="G21" s="0" t="inlineStr">
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>

</xml_diff>

<commit_message>
Record successful small-change smoke test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="39" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +156,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 完成，真实百炼小改压测发现并修复工具描述问题</t>
+          <t>P5：安全与恢复增强 MVP 主链路复测通过，进入收口检查</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>百炼只读 compaction 压测已通过；首轮真实小改压测跑通 dry_run、apply_patch、run_tests、git_diff，但暴露 `write_file` schema 描述误导模型，已修正并待复测。</t>
+          <t>百炼只读 compaction 压测已通过；真实小改复测跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff，P5 主链路已具备日用基础。</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>已覆盖 deadline、用户中断、length 截断、patch preview、rollback、ask_user timeout、approval mode、session decision、REPL 命令和 approval deadline cancel。</t>
+          <t>真实小改复测已覆盖 dry_run、apply_patch、session allow、rollback、run_tests、git_diff；下一步做 P5 收口检查。</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>复测真实小改任务</t>
+          <t>P5 收口检查</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>首轮发现问题，待复测</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t>首轮会话 `20260707T093733679947Z` 跑通链路，但因 `write_file` schema 描述错误导致 README 被改成不符合实现的说法</t>
+          <t>复测会话 `20260707T094246132064Z` 跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff；最终仅新增一个测试 docstring</t>
         </is>
       </c>
     </row>
@@ -2936,6 +2936,48 @@
       <c r="H33" s="0" t="inlineStr">
         <is>
           <t>`write_file` 描述已改为 create-only，并加测试确保不再出现 `fully overwrite`</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>T-032</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>P5 收口检查</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>收口前确认文档、测试、工作树和已知风险一致</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>运行全量测试、检查项目状态、确认未引入新的 P0/P1 阻塞问题</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3079,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；首轮百炼只读压测通过，继续真实小改复测后再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；百炼只读和真实小改压测均已通过，后续再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Close P5 MVP milestone
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -7,7 +7,8 @@
     <sheet name="已完成功能" sheetId="3" r:id="rId3"/>
     <sheet name="下一步 Todo" sheetId="4" r:id="rId4"/>
     <sheet name="风险与决策" sheetId="5" r:id="rId5"/>
-    <sheet name="推荐工作流" sheetId="6" r:id="rId6"/>
+    <sheet name="P5 收口结论" sheetId="6" r:id="rId6"/>
+    <sheet name="推荐工作流" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -101,7 +102,7 @@
   <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -156,12 +157,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 主链路复测通过，进入收口检查</t>
+          <t>P5：安全与恢复增强 MVP 收口完成，进入日用试用 / P6 取舍</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>百炼只读 compaction 压测已通过；真实小改复测跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff，P5 主链路已具备日用基础。</t>
+          <t>百炼只读 compaction 压测已通过；真实小改复测跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff；README 已补日用命令模板。</t>
         </is>
       </c>
     </row>
@@ -621,7 +622,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成并收口</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -631,7 +632,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>真实小改复测已覆盖 dry_run、apply_patch、session allow、rollback、run_tests、git_diff；下一步做 P5 收口检查。</t>
+          <t>主链路已通过真实百炼复测；后续只修日用反馈中的 P0/P1 问题。</t>
         </is>
       </c>
     </row>
@@ -648,12 +649,12 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>LSP、TUI、subagents、reviewer、AST edit、DAP</t>
+          <t>LSP、TUI、subagents、reviewer、AST edit、DAP、token budget / LLM summary</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待取舍</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -663,7 +664,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>日用闭环稳定后再评估。</t>
+          <t>先日用试用；再决定是否引入 token budget / LLM summary，LSP/TUI 等继续后置。</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1530,7 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>P5 收口检查</t>
+          <t>日用反馈</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1557,7 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>继续补真实任务压测</t>
+          <t>日用反馈补测</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2962,22 +2963,64 @@
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>收口前确认文档、测试、工作树和已知风险一致</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>README 已补日用模板；项目状态和 Excel 已同步；90 个测试、compileall、xlsx、diff check 通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>T-033</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>P6 取舍评估</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="F34" s="0" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="G34" s="0" t="inlineStr">
-        <is>
-          <t>收口前确认文档、测试、工作树和已知风险一致</t>
-        </is>
-      </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t>运行全量测试、检查项目状态、确认未引入新的 P0/P1 阻塞问题</t>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>决定下一阶段是继续日用打磨，还是引入 token budget / LLM summary / LSP / TUI 等高级能力</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>基于日用反馈和复杂任务失败样例做取舍</t>
         </is>
       </c>
     </row>
@@ -3800,6 +3843,133 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C7"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>P5 收口结论</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>主链路</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>百炼真实小改复测已跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>测试</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>90 个 unittest、compileall、xlsx 检查、diff check 均通过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>日用入口</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>README 已补只读分析和小改任务命令模板。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>开放风险</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>可接受</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / LLM summary 留到 P6 评估。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>下一阶段</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>待用户取舍</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>推荐先日用试用，再基于真实失败样例决定是否进入 P6。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>

</xml_diff>

<commit_message>
Add auto summary and lightweight LSP
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -99,10 +99,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -157,12 +157,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P5：安全与恢复增强 MVP 收口完成，进入日用试用 / P6 取舍</t>
+          <t>P7：轻量高级能力与真实压测</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>百炼只读 compaction 压测已通过；真实小改复测跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff；README 已补日用命令模板。</t>
+          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary 和多语言轻量 LSP 风格工具。</t>
         </is>
       </c>
     </row>
@@ -207,11 +207,11 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>完整 unittest 通过；compileall 通过。</t>
+          <t>完整 unittest、compileall、diff check、xlsx 检查通过。</t>
         </is>
       </c>
     </row>
@@ -270,12 +270,12 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>本地确定性</t>
+          <t>OMP 风格 auto 默认</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>超过约 60000 字符时折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并把摘要合并进首个 system prompt 以提升 provider 兼容性。</t>
+          <t>`context_char_budget` 近似上下文窗口，runtime 至少预留 15%；超过 reserve 阈值后 `--summary-mode auto` 调用当前 provider 生成语义摘要，失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -377,7 +377,58 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`。</t>
+          <t>见 `docs/omp-core-architecture-notes.md`，已补 OMP 如何通过系统提示、工具描述和 runtime 纠偏让用户不用指定工具顺序。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>默认工作流落地</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>system prompt + tool descriptions + runtime workflow reminder 已落地，用户不需要每次手写工具顺序。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>轻量 LSP</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`，覆盖 Python、Java、JavaScript、TypeScript、Vue。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Memory / Skills 设计</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>见 `docs/memory-skills-implementation-plan.md`；先做 Markdown memory 注入和 `learn`，再做 skills discovery，managed skills/autolearn 后置。</t>
         </is>
       </c>
     </row>
@@ -390,10 +441,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -600,7 +651,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>首轮百炼只读 compaction 压测已通过；继续用真实小改任务压测后再评估 token 预算、输出 reserve、recent 保留和可选 LLM summary。</t>
+          <t>首轮百炼只读 compaction 压测已通过；当前已补可选 LLM summary，后续再评估 token 预算、输出 reserve 和 recent 保留。</t>
         </is>
       </c>
     </row>
@@ -644,27 +695,59 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>高级工程能力</t>
+          <t>日用体验与默认工作流固化</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>LSP、TUI、subagents、reviewer、AST edit、DAP、token budget / LLM summary</t>
+          <t>OMP 默认工作流本地化：system prompt、工具描述、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>待取舍</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>先日用试用；再决定是否引入 token budget / LLM summary，LSP/TUI 等继续后置。</t>
+          <t>进入真实任务压测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>高级工程能力轻量版</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>OMP 风格 auto summary、轻量 LSP、memory/skills 方案、multi-root 方案评估</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>先验证 auto summary 和多语言 LSP 工具；下一步做 Markdown memory 注入；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -677,13 +760,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E38"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="5" max="5" width="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1363,7 +1446,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>固化主循环、deadline、compaction 结论</t>
+          <t>固化主循环、deadline、compaction、tool approval、默认工作流分层结论</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -1375,34 +1458,34 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>本地 Context Compaction</t>
+          <t>OMP 默认工作流源码依据</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>`context_char_budget` / `context_recent_messages`</t>
+          <t>`docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
+          <t>已记录 system prompt、project prompt、tool registry、tool descriptions、todo reminders、ToolChoiceQueue、agent-loop 的具体文件依据</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>下一步补 token 预算、输出 reserve 和可选 LLM summary；字符阈值保留兜底</t>
+          <t>P6 实现依据</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>本地 Context Compaction</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -1412,51 +1495,51 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`context_char_budget` / `context_recent_messages`</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>OMP 风格 Auto Summary</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>`--summary-mode auto` / `AGENT_SUMMARY_MODE=auto`</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>小历史不摘要；超过 reserve 阈值后调用当前 provider 总结早期历史；失败回退 local summary</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>需要百炼长上下文实测</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>默认工作流</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -1466,96 +1549,231 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`SYSTEM_PROMPT` + runtime workflow reminder</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>自然语言代码任务默认探索、todo、patch preview、验证、diff</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>需要真实任务实测</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>轻量 LSP 工具</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>`lsp_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>后续看是否升级完整 LSP</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
+          <t>下一步先做 Markdown memory 注入</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
+          <t>Synthetic tool result</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>避免 session 留下未配对 tool_calls</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>Patch preview</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>`apply_patch dry_run=true`</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 rollback</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>Patch rollback</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>`rollback_patch`</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>ask_user timeout</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>Tool approval policy</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>`tool_approval` + `session_tool_approval`</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B33" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C33" s="0" t="inlineStr">
-        <is>
-          <t>当前 90 个测试通过</t>
-        </is>
-      </c>
-      <c r="D33" s="0" t="inlineStr">
-        <is>
-          <t>unittest + compileall 通过</t>
-        </is>
-      </c>
-      <c r="E33" s="0" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>当前 106 个测试通过</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -1570,7 +1788,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H47"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2054,7 +2272,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>已实现字符阈值 deterministic compaction；下一步升级 token budget / reserve / LLM summary</t>
+          <t>已实现字符阈值 deterministic compaction；LLM summary 已补，下一步升级 token budget / reserve</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2383,7 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>已部分完成</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -2180,7 +2398,7 @@
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>P4/P5 稳定后再取舍</t>
+          <t>轻量 LSP 已做；TUI/subagents/AST edit/DAP 继续后置</t>
         </is>
       </c>
     </row>
@@ -3005,22 +3223,526 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
+          <t>已完成首轮</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>决定下一阶段是继续日用打磨，还是引入 token budget / LLM summary / LSP / TUI 等高级能力</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>已决定优先做 OMP 默认工作流本地化；随后按用户要求补 LLM summary 和轻量 LSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>T-034</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>固化 OMP 默认工作流源码依据</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>避免后续只凭“大概”实现；让设计有源码依据</t>
+        </is>
+      </c>
+      <c r="H36" s="0" t="inlineStr">
+        <is>
+          <t>`docs/omp-core-architecture-notes.md` 已新增“OMP 如何让用户不用指定工具顺序”</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>T-035</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>固化 LCA 默认工作流 system prompt</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>让用户不用每次手写 `list_files/read_file/dry_run/run_tests/git_diff`</t>
+        </is>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t>默认 prompt 覆盖理解、修改、验证、todo、ask_user、patch preview、diff</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>T-036</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>增强工具描述与真实能力一致性</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>模型会相信 tool schema；描述不准会直接导致错误动作</t>
+        </is>
+      </c>
+      <c r="H38" s="0" t="inlineStr">
+        <is>
+          <t>既有 create-only/patch dry_run 描述保持测试；新增 LSP 工具描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>T-037</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>实现轻量 runtime workflow nudge</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>复杂任务中提醒 todo 和验证，降低模型跑偏</t>
+        </is>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t>非平凡代码任务会注入 reminder；短 prompt 不注入</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>T-038</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>评估 multi-root workspace allow-dir</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
           <t>未开始</t>
         </is>
       </c>
-      <c r="F35" s="0" t="inlineStr">
+      <c r="F40" s="0" t="inlineStr">
         <is>
           <t>User + Agent</t>
         </is>
       </c>
-      <c r="G35" s="0" t="inlineStr">
-        <is>
-          <t>决定下一阶段是继续日用打磨，还是引入 token budget / LLM summary / LSP / TUI 等高级能力</t>
-        </is>
-      </c>
-      <c r="H35" s="0" t="inlineStr">
-        <is>
-          <t>基于日用反馈和复杂任务失败样例做取舍</t>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>支持“需求文档目录 + 代码项目目录”的真实工作流</t>
+        </is>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
+        <is>
+          <t>设计 `--allow-dir` / `AGENT_ALLOWED_DIRS`，先覆盖 read/list/search/apply_patch</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>T-039</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>实现 OMP 风格 auto summary</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>长上下文需要语义摘要能力，但不应小历史也额外调用模型</t>
+        </is>
+      </c>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t>默认 `--summary-mode auto`；超过 reserve 阈值才调用 LLM summary，失败回退 local summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>T-040</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>实现轻量 LSP 工具</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>提升主流项目定位效率</t>
+        </is>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics 已可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>T-041</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>固化 Memory / Skills 实现方案</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>OMP memory/autolearn/skills 机制复杂，需先裁剪成 LCA 可执行方案</t>
+        </is>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t>已新增 `docs/memory-skills-implementation-plan.md`，并补充 `docs/omp-core-architecture-notes.md`</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>T-042</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Markdown memory 启动注入</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>当前 memory 只能手动读写，不能跨 session 自动影响 agent</t>
+        </is>
+      </c>
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t>读取 `.local-agent/memory/*.md`，以 advisory block 注入 system prompt，带 source path 和预算</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>T-043</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>实现 `learn` 工具</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>让 agent 用显式工具沉淀可复用 lesson，而不是混写 project memory</t>
+        </is>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t>写入 `.local-agent/memory/learned.md`，限制长度并清洗会进入 prompt 的字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>T-044</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Authored skills discovery</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="F46" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>支持项目内可复用工作流，降低重复提示成本</t>
+        </is>
+      </c>
+      <c r="H46" s="0" t="inlineStr">
+        <is>
+          <t>先扫 `.local-agent/skills/&lt;name&gt;/SKILL.md`，system prompt 只列 name/description，正文按需读取</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>T-045</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Managed skills / autolearn</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>暂缓</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t>自动生成 skills 有长期污染和 prompt injection 风险</t>
+        </is>
+      </c>
+      <c r="H47" s="0" t="inlineStr">
+        <is>
+          <t>默认关闭；后续按 OMP `manage_skill` 思路隔离 generated skills，authored skills 优先</t>
         </is>
       </c>
     </row>
@@ -3033,12 +3755,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G28"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
@@ -3122,12 +3844,12 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做字符阈值 compaction、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；百炼只读和真实小改压测均已通过，后续再评估 token 预算、输出 reserve、recent 保留和 LLM summary</t>
+          <t>已做 OMP 风格 reserve 阈值、auto LLM summary、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；后续再评估精确 token 预算、输出 reserve、recent 保留</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>OMP 按上下文 token 预算触发压缩，给下一轮 prompt/输出预留 reserve，并把早期历史压成 summary；建议我们把字符阈值升级为 token 估算 + reserve + 可选 LLM summary，字符阈值只保留为兜底。</t>
+          <t>OMP 按上下文 token 预算触发压缩，给下一轮 prompt/输出预留 reserve，并把早期历史压成 summary；我们当前用字符窗口近似，下一步可升级为 token 估算。</t>
         </is>
       </c>
     </row>
@@ -3344,12 +4066,12 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>P6 暂缓，先稳定日用闭环</t>
+          <t>已只引入多语言轻量 LSP 和 auto summary，完整 DAP/TUI/subagents 继续后置</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们 P6 后置，先稳定单 Agent 闭环。</t>
+          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们先做无外部依赖的本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -3504,74 +4226,74 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-012</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>日用命令仍依赖用户手写工具流程</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>已把默认工作流沉到 system prompt 和 runtime nudge；后续靠真实任务验证效果</t>
         </is>
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 把默认工作流拆到 system prompt、tool descriptions 和 runtime nudge；我们先做本地 MVP 版，不急着引入完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-013</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>Memory / skills 注入长期 prompt injection 或陈旧事实</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>设计中</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>memory 和 generated skills 会跨 session 影响模型，错误或恶意内容可能持续放大</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 将 memory 标成 heuristic/advisory，managed skills 隔离且 authored skills 优先；我们先做 advisory 注入、预算限制、字段清洗，managed skills 默认关闭。</t>
         </is>
       </c>
     </row>
@@ -3583,7 +4305,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -3593,22 +4315,22 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -3620,7 +4342,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -3630,22 +4352,22 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -3657,7 +4379,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -3667,22 +4389,22 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -3694,7 +4416,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -3704,7 +4426,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -3714,12 +4436,12 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -3731,7 +4453,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -3741,7 +4463,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -3751,12 +4473,12 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -3768,7 +4490,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -3778,7 +4500,7 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -3788,12 +4510,12 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -3805,32 +4527,254 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
+          <t>ADR-007</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>依赖提前准备</t>
+        </is>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>ADR-008</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>持续同步本文件和 `project-status.md`</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
           <t>ADR-009</t>
         </is>
       </c>
-      <c r="C22" s="0" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="D22" s="0" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
-      <c r="E22" s="0" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F22" s="0" t="inlineStr">
+      <c r="F24" s="0" t="inlineStr">
         <is>
           <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
-      <c r="G22" s="0" t="inlineStr">
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>ADR-010</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>ADR-011</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>默认采用 OMP 风格 auto summary</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>ADR-012</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>LSP 第一版做轻量多语言静态工具</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>不启动外部 language server</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>先做 Markdown memory 启动注入和显式 `learn`</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>后续再做 authored skills discovery，最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -3846,7 +4790,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3906,7 +4850,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>90 个 unittest、compileall、xlsx 检查、diff check 均通过。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 106 个 unittest、compileall、xlsx 检查和 diff check。</t>
         </is>
       </c>
     </row>
@@ -3940,7 +4884,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / LLM summary 留到 P6 评估。</t>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / multi-root 继续后置评估。</t>
         </is>
       </c>
     </row>
@@ -3952,12 +4896,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>待用户取舍</t>
+          <t>P7 真实压测与 multi-root 评估</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>推荐先日用试用，再基于真实失败样例决定是否进入 P6。</t>
+          <t>验证默认工作流、auto summary、多语言轻量 LSP 是否足够日用，再评估需求文档目录 + 代码目录的 multi-root。</t>
         </is>
       </c>
     </row>
@@ -4125,7 +5069,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>要求 Agent `read_file/list_files/search_code`</t>
+          <t>Agent 默认会按需 `list_files/read_file/search_code/lsp_*`</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -4135,12 +5079,12 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>P1+</t>
+          <t>P6+</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>已在 prompt 中约束</t>
+          <t>用户不必手写工具顺序</t>
         </is>
       </c>
     </row>
@@ -4155,7 +5099,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>必须 `apply_patch`，修改已有文件不使用 `write_file`</t>
+          <t>修改已有文件使用 `apply_patch`，写入前优先 `dry_run=true`</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
@@ -4170,7 +5114,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>已支持插入模式</t>
+          <t>已写入默认 prompt 和工具描述</t>
         </is>
       </c>
     </row>
@@ -4185,7 +5129,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>必须 `run_tests + git_diff`</t>
+          <t>默认应 `run_tests + git_diff`</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -4195,12 +5139,12 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>P1+</t>
+          <t>P6+</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>初始 commit 后 diff 更好用</t>
+          <t>自然语言任务默认走验证闭环</t>
         </is>
       </c>
     </row>
@@ -4215,22 +5159,22 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>先 todo，再做实现，再验证</t>
+          <t>默认维护 todo，再做实现，再验证；默认 `--summary-mode auto` 按阈值触发 LLM summary</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>防止漏任务</t>
+          <t>防止漏任务并治理长上下文</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>P3+</t>
+          <t>P7+</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>`todo_read/add/update` 已可用</t>
+          <t>Auto summary 需真实 provider 压测</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multi-root workspace and startup memory
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -99,7 +99,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C23"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -162,7 +162,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary 和多语言轻量 LSP 风格工具。</t>
+          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory 和 learn。</t>
         </is>
       </c>
     </row>
@@ -207,7 +207,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -418,17 +418,68 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
+          <t>Multi-root workspace</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；shell/git/session/memory 仍锚定 `--cwd`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Startup memory</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>新 session 自动注入 `.local-agent/memory/{project,decisions,conventions,learned}.md`，作为 advisory context。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Learn 工具</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B20" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C20" s="0" t="inlineStr">
-        <is>
-          <t>见 `docs/memory-skills-implementation-plan.md`；先做 Markdown memory 注入和 `learn`，再做 skills discovery，managed skills/autolearn 后置。</t>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入和 `learn` 已完成，下一步做 skills discovery，managed skills/autolearn 后置。</t>
         </is>
       </c>
     </row>
@@ -732,7 +783,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、memory/skills 方案、multi-root 方案评估</t>
+          <t>OMP 风格 auto summary、轻量 LSP、multi-root、startup memory、learn、skills discovery</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -742,12 +793,12 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>先验证 auto summary 和多语言 LSP 工具；下一步做 Markdown memory 注入；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>下一步做真实 multi-root 压测和 authored skills discovery；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -760,7 +811,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E41"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1593,34 +1644,34 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>Memory / Skills 方案</t>
+          <t>Multi-root workspace</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>已完成设计</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>`docs/memory-skills-implementation-plan.md`</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS`</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
+          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>下一步先做 Markdown memory 注入</t>
+          <t>真实需求压测</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>Startup memory</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -1630,93 +1681,93 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Learn 工具</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>`learn`</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>写入 `.local-agent/memory/learned.md`，默认走写工具审批</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步做 authored skills discovery</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -1728,52 +1779,133 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>Patch preview</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`apply_patch dry_run=true`</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
+          <t>后续评估 rollback</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
+          <t>Patch rollback</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>`rollback_patch`</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>ask_user timeout</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>Tool approval policy</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>`tool_approval` + `session_tool_approval`</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B38" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C38" s="0" t="inlineStr">
-        <is>
-          <t>当前 106 个测试通过</t>
-        </is>
-      </c>
-      <c r="D38" s="0" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>当前 116 个测试通过</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E38" s="0" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -3433,7 +3565,7 @@
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
@@ -3448,7 +3580,7 @@
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
-          <t>设计 `--allow-dir` / `AGENT_ALLOWED_DIRS`，先覆盖 read/list/search/apply_patch</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 已覆盖 read/list/search/LSP/apply_patch/write_file/rollback_patch</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3733,7 @@
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
@@ -3643,7 +3775,7 @@
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
@@ -3761,7 +3893,7 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
@@ -4066,7 +4198,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>已只引入多语言轻量 LSP 和 auto summary，完整 DAP/TUI/subagents 继续后置</t>
+          <t>已只引入多语言轻量 LSP、auto summary、multi-root、startup memory 和 learn，完整 DAP/TUI/subagents 继续后置</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
@@ -4283,7 +4415,7 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>设计中</t>
+          <t>已缓解，skills 仍设计中</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -4293,7 +4425,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 memory 标成 heuristic/advisory，managed skills 隔离且 authored skills 优先；我们先做 advisory 注入、预算限制、字段清洗，managed skills 默认关闭。</t>
+          <t>OMP 将 memory 标成 heuristic/advisory，managed skills 隔离且 authored skills 优先；我们已做 advisory 注入、预算限制、learned 字段清洗，managed skills 默认关闭。</t>
         </is>
       </c>
     </row>
@@ -4764,12 +4896,12 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>先做 Markdown memory 启动注入和显式 `learn`</t>
+          <t>Markdown memory 启动注入和显式 `learn` 已完成</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
@@ -4790,7 +4922,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4850,7 +4982,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 106 个 unittest、compileall、xlsx 检查和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 116 个 unittest 和 compileall。</t>
         </is>
       </c>
     </row>
@@ -4884,7 +5016,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / multi-root 继续后置评估。</t>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / authored skills discovery 继续后置评估。</t>
         </is>
       </c>
     </row>
@@ -4896,12 +5028,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>P7 真实压测与 multi-root 评估</t>
+          <t>P7 真实压测与 authored skills discovery</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>验证默认工作流、auto summary、多语言轻量 LSP 是否足够日用，再评估需求文档目录 + 代码目录的 multi-root。</t>
+          <t>验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory 和 learn 是否足够日用，再做 authored skills discovery。</t>
         </is>
       </c>
     </row>
@@ -4914,7 +5046,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5184,27 +5316,27 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>有歧义</t>
+          <t>多目录任务</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>使用 `ask_user` 中途问用户</t>
+          <t>`./agent --cwd /path/to/code --allow-dir /path/to/requirements "读取需求并修改代码"`</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>避免模型瞎猜</t>
+          <t>支持需求文档目录 + 代码项目目录</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>P3+</t>
+          <t>P7+</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>非交互会返回明确错误</t>
+          <t>allowed dir 只扩展文件/search/LSP/patch 工具</t>
         </is>
       </c>
     </row>
@@ -5214,25 +5346,85 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
+          <t>项目记忆</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>减少重复交代项目约定</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>memory 是 advisory，当前用户指令优先</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>10</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>有歧义</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>使用 `ask_user` 中途问用户</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>避免模型瞎猜</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>P3+</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>非交互会返回明确错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
           <t>同步 Excel</t>
         </is>
       </c>
-      <c r="C11" s="0" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>`python3 scripts/sync_project_excel.py`</t>
         </is>
       </c>
-      <c r="D11" s="0" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Excel 是开发展示产物，Markdown 是开发事实源</t>
         </is>
       </c>
-      <c r="E11" s="0" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>P2+</t>
         </is>
       </c>
-      <c r="F11" s="0" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>无第三方依赖</t>
         </is>

</xml_diff>

<commit_message>
Add authored skills discovery
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -99,9 +99,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
@@ -162,7 +162,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory 和 learn。</t>
+          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn 和 authored skills discovery。</t>
         </is>
       </c>
     </row>
@@ -207,7 +207,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -469,17 +469,34 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
+          <t>Authored skills discovery</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B23" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入和 `learn` 已完成，下一步做 skills discovery，managed skills/autolearn 后置。</t>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn` 和 authored skills discovery 已完成，managed skills/autolearn 后置。</t>
         </is>
       </c>
     </row>
@@ -783,7 +800,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、multi-root、startup memory、learn、skills discovery</t>
+          <t>OMP 风格 auto summary、轻量 LSP、multi-root、startup memory、learn、authored skills discovery</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -793,12 +810,12 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>下一步做真实 multi-root 压测和 authored skills discovery；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>下一步做真实综合压测和 token 预算评估；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -811,9 +828,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
@@ -1725,130 +1742,130 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>Memory / Skills 方案</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>已完成设计</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>`docs/memory-skills-implementation-plan.md`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
+          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>下一步做 authored skills discovery</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步真实压测</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>Patch preview</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`apply_patch dry_run=true`</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>后续评估 rollback</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>Patch rollback</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>`rollback_patch`</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -1860,52 +1877,79 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>ask_user timeout</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
+          <t>Tool approval policy</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>`tool_approval` + `session_tool_approval`</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B41" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C41" s="0" t="inlineStr">
-        <is>
-          <t>当前 116 个测试通过</t>
-        </is>
-      </c>
-      <c r="D41" s="0" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>当前 118 个测试通过</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E41" s="0" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -3817,7 +3861,7 @@
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
@@ -3832,7 +3876,7 @@
       </c>
       <c r="H46" s="0" t="inlineStr">
         <is>
-          <t>先扫 `.local-agent/skills/&lt;name&gt;/SKILL.md`，system prompt 只列 name/description，正文按需读取</t>
+          <t>先扫 `.local-agent/skills/&lt;name&gt;/SKILL.md`，system prompt 只列 name/description/source，正文按需读取</t>
         </is>
       </c>
     </row>
@@ -3893,7 +3937,7 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
@@ -4415,7 +4459,7 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>已缓解，skills 仍设计中</t>
+          <t>已缓解，managed skills 仍暂缓</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -4425,7 +4469,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 memory 标成 heuristic/advisory，managed skills 隔离且 authored skills 优先；我们已做 advisory 注入、预算限制、learned 字段清洗，managed skills 默认关闭。</t>
+          <t>OMP 将 memory 标成 heuristic/advisory，managed skills 隔离且 authored skills 优先；我们已做 advisory 注入、预算限制、learned 字段和 skill description 清洗，managed skills 默认关闭。</t>
         </is>
       </c>
     </row>
@@ -4901,12 +4945,12 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入和显式 `learn` 已完成</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>后续再做 authored skills discovery，最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4966,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4982,7 +5026,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 116 个 unittest 和 compileall。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 118 个 unittest 和 compileall。</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5060,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / authored skills discovery 继续后置评估。</t>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / managed skills 继续后置评估。</t>
         </is>
       </c>
     </row>
@@ -5028,12 +5072,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>P7 真实压测与 authored skills discovery</t>
+          <t>P7 综合真实压测与 token 预算评估</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory 和 learn 是否足够日用，再做 authored skills discovery。</t>
+          <t>验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn 和 authored skills 是否足够日用。</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5090,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5376,27 +5420,27 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>有歧义</t>
+          <t>本地 skills</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>使用 `ask_user` 中途问用户</t>
+          <t>将可复用工作流写到 `.local-agent/skills/&lt;name&gt;/SKILL.md`，带 `name` / `description` frontmatter</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>避免模型瞎猜</t>
+          <t>降低重复提示成本</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>P3+</t>
+          <t>P7+</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>非交互会返回明确错误</t>
+          <t>启动只注入 metadata，正文按需 read_file</t>
         </is>
       </c>
     </row>
@@ -5406,25 +5450,55 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
+          <t>有歧义</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>使用 `ask_user` 中途问用户</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>避免模型瞎猜</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>P3+</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>非交互会返回明确错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
           <t>同步 Excel</t>
         </is>
       </c>
-      <c r="C13" s="0" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>`python3 scripts/sync_project_excel.py`</t>
         </is>
       </c>
-      <c r="D13" s="0" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Excel 是开发展示产物，Markdown 是开发事实源</t>
         </is>
       </c>
-      <c r="E13" s="0" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>P2+</t>
         </is>
       </c>
-      <c r="F13" s="0" t="inlineStr">
+      <c r="F14" s="0" t="inlineStr">
         <is>
           <t>无第三方依赖</t>
         </is>

</xml_diff>

<commit_message>
Advance P7 agent runtime and project tracking
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -7,8 +7,9 @@
     <sheet name="已完成功能" sheetId="3" r:id="rId3"/>
     <sheet name="下一步 Todo" sheetId="4" r:id="rId4"/>
     <sheet name="风险与决策" sheetId="5" r:id="rId5"/>
-    <sheet name="P5 收口结论" sheetId="6" r:id="rId6"/>
-    <sheet name="推荐工作流" sheetId="7" r:id="rId7"/>
+    <sheet name="P7 综合压测问题" sheetId="6" r:id="rId6"/>
+    <sheet name="P5 收口结论" sheetId="7" r:id="rId7"/>
+    <sheet name="推荐工作流" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -102,7 +103,7 @@
   <dimension ref="A1:C24"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -162,7 +163,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；本轮已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn 和 authored skills discovery。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering。</t>
         </is>
       </c>
     </row>
@@ -191,12 +192,12 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>`.env` 或环境变量</t>
+          <t>环境变量 / `--env-file` / `.env`</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>`.env` 可写 `DASHSCOPE_API_KEY=...`，该文件已被 `.gitignore` 忽略。</t>
+          <t>`./agent` 会自动加载安装目录 `.env`，也可显式传 `--env-file`；真实环境变量优先。</t>
         </is>
       </c>
     </row>
@@ -207,7 +208,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -411,7 +412,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`，覆盖 Python、Java、JavaScript、TypeScript、Vue。</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`，覆盖 Python、Java、JavaScript、TypeScript、Vue。</t>
         </is>
       </c>
     </row>
@@ -800,7 +801,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、multi-root、startup memory、learn、authored skills discovery</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -810,12 +811,12 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>下一步做真实综合压测和 token 预算评估；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -828,13 +829,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="35" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1472,7 +1473,7 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>`.env` 加载</t>
+          <t>`.env` / `--env-file` 加载</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -1482,17 +1483,17 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>workspace `.env`</t>
+          <t>`src/local_agent/config.py` + `./agent`</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>可放 `DASHSCOPE_API_KEY`，被 gitignore</t>
+          <t>`./agent` 自动加载安装目录 `.env`；CLI 支持显式 `--env-file`；目标 workspace `.env` 仍可用</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>避免重复 export</t>
+          <t>跨项目 token 与 `--cwd` 解耦</t>
         </is>
       </c>
     </row>
@@ -1644,12 +1645,12 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -1931,25 +1932,106 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
+          <t>重复工具调用熔断</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>Tool result pruning</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>`ToolResult.useless` + provider-bound context pruning</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>继续真实长任务观察</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>Todo steering</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>provider-bound runtime todo reminder</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B42" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="C42" s="0" t="inlineStr">
-        <is>
-          <t>当前 118 个测试通过</t>
-        </is>
-      </c>
-      <c r="D42" s="0" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>当前 124 个测试通过</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E42" s="0" t="inlineStr">
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -1964,13 +2046,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H53"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
@@ -3919,6 +4001,258 @@
       <c r="H47" s="0" t="inlineStr">
         <is>
           <t>默认关闭；后续按 OMP `manage_skill` 思路隔离 generated skills，authored skills 优先</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>T-046</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>P7 综合压测记录</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>真实压测发现的问题必须沉淀成可追踪事实源</t>
+        </is>
+      </c>
+      <c r="H48" s="0" t="inlineStr">
+        <is>
+          <t>新增 `docs/pressure-test-2026-07-08.md`，记录压测证据、OMP 对应机制和 LCA 措施</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>T-047</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>重复工具调用熔断</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>防止模型在同一工具参数上循环到 budget 耗尽而无最终回答</t>
+        </is>
+      </c>
+      <c r="H49" s="0" t="inlineStr">
+        <is>
+          <t>最近 12 次工具调用内同名同参超过 3 次会跳过；连续命中 8 次停止；测试覆盖 JSON 参数顺序归一化</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>T-048</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>企业项目外发策略确认</t>
+        </is>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
+          <t>用户已确认，当前 Codex 环境阻断代跑</t>
+        </is>
+      </c>
+      <c r="F50" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
+        <is>
+          <t>企业源码和需求发给百炼属于三方 API 外发，需要明确边界</t>
+        </is>
+      </c>
+      <c r="H50" s="0" t="inlineStr">
+        <is>
+          <t>LCA 产品设计不内置禁止外发；按 OMP 思路由用户、provider、permission 和运行环境策略决定。本次 Codex 环境无法代跑，已改成本地只读扫描。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>T-049</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>跨项目 `--env-file` / launcher env 加载</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>让 token 配置与目标 `--cwd` 解耦，跨项目一键启动更顺手</t>
+        </is>
+      </c>
+      <c r="H51" s="0" t="inlineStr">
+        <is>
+          <t>CLI 支持显式 `--env-file`；`./agent` 自动把安装目录 `.env` 注入为 env-file；测试覆盖优先级和缺失文件报错</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>T-050</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>OMP 风格 tool result pruning / todo steering</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F52" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G52" s="0" t="inlineStr">
+        <is>
+          <t>compaction 只是装得下上下文，还需要降低无效工具结果和旧结果对模型的污染</t>
+        </is>
+      </c>
+      <c r="H52" s="0" t="inlineStr">
+        <is>
+          <t>已新增 `ToolResult.useless`；空搜索/LSP 结果会标记 useless；provider-bound context 会折叠 useless/superseded 工具输出并注入 open todo reminder；session 原文保留</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>T-051</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>LSP workspace/document symbols 兼容别名</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>减少模型和用户从 OMP/Codex 概念迁移时的工具名摩擦</t>
+        </is>
+      </c>
+      <c r="H53" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_workspace_symbols` / `lsp_document_symbols` 已注册为 `lsp_symbols` 只读别名；测试覆盖 registry 和执行结果</t>
         </is>
       </c>
     </row>
@@ -3931,7 +4265,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G32"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4476,111 +4810,111 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-014</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>重复工具调用循环导致 budget 耗尽且无最终回答</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已进一步缓解</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>已补最近窗口同名同参工具调用熔断、`ToolResult.useless`、空结果标记、provider-bound useless/superseded pruning 和 open todo runtime reminder；后续评估 OMP 风格 ToolChoiceQueue / soft tool requirement</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 不靠主步数限制日常任务，而靠 deadline/abort、synthetic tool result、soft tool escalation 小上限、todo/tool-choice steering 和 compaction pruning 共同收敛；我们已落地本地轻量 pruning/steering。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-015</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>企业项目源码和需求可能被发送到三方 AI API</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>用户已确认，当前 Codex 环境阻断代跑</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>用户已确认可外发给百炼；本次由 Codex 执行环境策略拒绝代跑联网压测，已改为本地只读扫描并记录结果</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 由用户配置 provider 和 permission，但进入模型上下文的内容会发送给 provider；这不是自动隐私隔离，也不是 LCA 内置禁令，需要由用户、provider、permission 和运行环境策略控制。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>R-016</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>跨项目运行时 token 配置绑定目标 workspace `.env`</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>已新增 `--env-file` 和 launcher 安装目录 `.env` 自动加载；凭据与目标 `--cwd` 解耦</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 provider/model/apiKey 是 runtime 配置，cwd 是项目上下文；我们采用同一分层。</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4926,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -4602,7 +4936,7 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -4612,12 +4946,12 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4963,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -4639,22 +4973,22 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -4666,7 +5000,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -4676,22 +5010,22 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -4703,7 +5037,7 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -4713,7 +5047,7 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -4723,12 +5057,12 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -4740,7 +5074,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -4750,7 +5084,7 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -4760,12 +5094,12 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -4777,7 +5111,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -4787,7 +5121,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -4797,12 +5131,12 @@
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -4814,7 +5148,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -4824,22 +5158,22 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -4851,7 +5185,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -4861,22 +5195,22 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -4888,7 +5222,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -4898,22 +5232,22 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -4925,32 +5259,180 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
+          <t>ADR-010</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>ADR-011</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>默认采用 OMP 风格 auto summary</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+        </is>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>ADR-012</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>LSP 第一版做轻量多语言静态工具</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>不启动外部 language server</t>
+        </is>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
           <t>ADR-013</t>
         </is>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
-      <c r="E28" s="0" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>已接受并部分落地</t>
         </is>
       </c>
-      <c r="F28" s="0" t="inlineStr">
+      <c r="F31" s="0" t="inlineStr">
         <is>
           <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
-      <c r="G28" s="0" t="inlineStr">
+      <c r="G31" s="0" t="inlineStr">
         <is>
           <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -4962,6 +5444,261 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F8"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>P7 综合压测问题</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>现象</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>OMP 对应方式</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>LCA 措施</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>PT-001</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>已进一步缓解并复测</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>LCA 自身只读压测中重复 `search_code` / `todo_read`，最终由 `budget_seconds=240` 截断；修复后 session `20260708T025519414693Z` 按要求收尾。</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>OMP 组合使用 deadline/abort、synthetic tool result、soft tool escalation 小上限、todo/tool-choice steering、useless/superseded pruning，而不是主循环步数。</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>已实现最近窗口重复工具调用熔断，并补 `ToolResult.useless`、空搜索/LSP 结果 useless 标记、provider-bound useless/superseded pruning、open todo runtime reminder。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>PT-002</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>当前 Codex 环境阻断代跑，已改本地扫描</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>用户已确认可外发给百炼；本次 Codex 执行环境策略拒绝代跑把企业私有代码/需求发送到三方 API。</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>OMP 由用户配置 provider 和 permission；进入模型上下文的内容会发送给 provider，不是自动隐私隔离，也不是默认禁止外发。</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>不绕过当前执行环境策略；改成本地只读扫描，记录结构、关键词和候选落点。用户在自己的允许环境中运行 LCA 时，可按 provider/permission 策略执行联网只读分析。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>PT-003</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>已关闭 MVP 版</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>`--cwd` 指向企业项目后，LCA 仓库 `.env` 不会自动加载，需要手动 source。</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 provider/model/apiKey 属于 runtime 配置，cwd 是项目上下文。</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>已新增 `--env-file`；`./agent` 自动加载安装目录 `.env`，再加载目标 workspace `.env`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>PT-004</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>已关闭 MVP 版</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>prompt 中出现 `lsp_workspace_symbols` / `lsp_document_symbols` 时，模型会搜索这些旧概念而非直接用 `lsp_symbols`。</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>OMP 通过准确工具 schema、tool discovery 和 tool-choice steering 降低工具名漂移。</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>已增加 `lsp_workspace_symbols` / `lsp_document_symbols` 只读兼容别名，均复用 `lsp_symbols` handler 和 schema；system prompt 已说明它们是 alias。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>PT-005</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>已进一步缓解</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>compaction 能让上下文装下，但不自动保证任务收敛。</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将 compaction 与 todo reminder、tool choice、queued steering、deadline/abort、pruning 组合。</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>已补重复工具熔断、provider-bound useless/superseded pruning 和 open todo runtime reminder；后续评估 ToolChoiceQueue / soft tool requirement。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>PT-006</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>本地只读扫描完成，联网 LCA 未由 Codex 代跑</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>`zqyl-user-center-service` 为 Maven 多模块项目，约 5309 个 Java/XML/YAML 文件；`crcl-open` 约 2584 个 Java/XML/YAML 文件。本地扫描确认需求关键词可定位到投资方案、Charge、TradeBg、结算单枚举等方向，但百炼联网 LCA 在当前 Codex 执行环境被阻断。</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>OMP 可组合更完整工程工具、subagents/reviewer 和 compaction/pruning。</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>用户可在自己的允许环境中用 LCA 跑真实联网只读分析；LCA 已补轻量 pruning / steering，后续再评估更完整工程工具。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C7"/>
   <cols>
@@ -5026,7 +5763,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 118 个 unittest 和 compileall。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 124 个 unittest 和 compileall。</t>
         </is>
       </c>
     </row>
@@ -5088,14 +5825,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="31" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
@@ -5185,12 +5922,12 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>`./agent "描述当前项目"`</t>
+          <t>`./agent "描述当前项目"`；跨项目用 `./agent --cwd /path/to/project ...`</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>一键启动，默认当前目录为 workspace</t>
+          <t>一键启动，默认当前目录为 workspace；跨项目时安装目录 `.env` 会自动作为 `--env-file` 加载</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
@@ -5200,7 +5937,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>token 可来自环境变量或 `.env`</t>
+          <t>token 可来自环境变量、显式 `--env-file` 或 `.env`</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record enterprise read-only pressure test findings
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -163,7 +163,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 企业项目代跑暴露“只读任务仍写目标 workspace session 状态”，下一步按 OMP 思路把 runtime state 与 cwd 分层。</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；新增发现：只读任务仍在目标仓库写 `.local-agent/sessions`。下一步先做 OMP 风格 `--state-dir`，再评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H54"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4256,6 +4256,48 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>T-052</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>OMP 风格 runtime state 与 workspace 解耦</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F54" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>只读跨项目分析不应在目标仓库写 `.local-agent/sessions`；企业项目压测需要更干净的零业务落盘体验</t>
+        </is>
+      </c>
+      <c r="H54" s="0" t="inlineStr">
+        <is>
+          <t>增加 `--state-dir` / `AGENT_STATE_DIR`，默认 sessions/todos/patch logs 使用用户级状态目录；保留项目 memory/skills 的明确策略；测试覆盖跨 `--cwd` 不写目标 `.local-agent/sessions`</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -4265,7 +4307,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4921,37 +4963,37 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-017</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>只读任务仍在目标 workspace 写 runtime 状态</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新发现，待处理</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>当前 `JsonlSessionStore`、todo、patch log 默认写入 `--cwd/.local-agent`；2026-07-08 企业项目只读代跑创建了 `.local-agent/sessions/*.jsonl`</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 默认把 sessions 放在 `~/.omp/agent/sessions/&lt;cwd-encoded&gt;/`，项目 `.omp` 更偏 context/config/rules/skills；我们应增加用户级 `--state-dir`，把 sessions/todos/patch logs 与源码目录解耦。</t>
         </is>
       </c>
     </row>
@@ -4963,7 +5005,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -4973,22 +5015,22 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5042,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -5010,7 +5052,7 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -5020,12 +5062,12 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5079,7 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -5047,22 +5089,22 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5116,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -5084,7 +5126,7 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -5094,12 +5136,12 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5153,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -5121,7 +5163,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -5131,12 +5173,12 @@
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5190,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -5158,7 +5200,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -5168,12 +5210,12 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5227,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -5195,7 +5237,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -5205,12 +5247,12 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5264,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -5232,7 +5274,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -5242,12 +5284,12 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5301,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -5269,22 +5311,22 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5338,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -5306,7 +5348,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -5316,12 +5358,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5375,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -5343,7 +5385,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -5353,12 +5395,12 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -5370,7 +5412,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -5380,22 +5422,22 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -5407,30 +5449,67 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>已接受并部分落地</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
           <t>ADR-014</t>
         </is>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D32" s="0" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
-      <c r="E32" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F32" s="0" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
         <is>
           <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
-      <c r="G32" s="0" t="inlineStr">
+      <c r="G33" s="0" t="inlineStr">
         <is>
           <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
@@ -5445,7 +5524,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5688,6 +5767,70 @@
       <c r="F8" s="0" t="inlineStr">
         <is>
           <t>用户可在自己的允许环境中用 LCA 跑真实联网只读分析；LCA 已补轻量 pruning / steering，后续再评估更完整工程工具。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>PT-007</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>新发现，待处理</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>企业项目只读代跑在目标仓库创建 `.local-agent/sessions/20260708T053955405637Z.jsonl`，导致 `git status` 新增 `?? .local-agent/`。</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>OMP 默认 session 目录在用户 agent dir 的 `sessions/&lt;cwd-encoded&gt;` 下，而不是直接写进目标 repo。</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>下一步实现 `--state-dir` / `AGENT_STATE_DIR`，默认把 sessions/todos/patch logs 放到用户级状态目录；项目 memory/skills 另行明确。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>PT-008</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>已记录</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>`crcl-open/crcl-open` 本身已有大量 modified 文件，压测前后需要快照才能证明 LCA 是否污染业务文件。</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的更完整 task/worktree 能力可隔离 WIP；普通 CLI 也需要清楚记录 cwd/worktree 状态。</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>后续企业压测前先记录 `git status --short` 到 LCA 压测记录，压测后对比，不在目标 repo 写快照。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add user-level runtime state directory
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -100,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -163,7 +163,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 企业项目代跑暴露“只读任务仍写目标 workspace session 状态”，下一步按 OMP 思路把 runtime state 与 cwd 分层。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
         </is>
       </c>
     </row>
@@ -208,7 +208,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -487,15 +487,32 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
+          <t>Runtime state dir</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B24" s="0" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C24" s="0" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn` 和 authored skills discovery 已完成，managed skills/autolearn 后置。</t>
         </is>
@@ -801,7 +818,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -811,12 +828,12 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；新增发现：只读任务仍在目标仓库写 `.local-agent/sessions`。下一步先做 OMP 风格 `--state-dir`，再评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir`。下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -829,7 +846,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1500,34 +1517,34 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记</t>
+          <t>Runtime state dir</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>`docs/omp-core-architecture-notes.md`</t>
+          <t>`src/local_agent/state.py` + `--state-dir`</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>固化主循环、deadline、compaction、tool approval、默认工作流分层结论</t>
+          <t>sessions/todos/patch logs 默认写入用户级 state root；项目 memory/skills 保留在 workspace</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>后续设计依据</t>
+          <t>真实企业项目只读复测</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>OMP 默认工作流源码依据</t>
+          <t>OMP 核心架构笔记</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -1542,46 +1559,46 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>已记录 system prompt、project prompt、tool registry、tool descriptions、todo reminders、ToolChoiceQueue、agent-loop 的具体文件依据</t>
+          <t>固化主循环、deadline、compaction、tool approval、默认工作流分层结论</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>P6 实现依据</t>
+          <t>后续设计依据</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>本地 Context Compaction</t>
+          <t>OMP 默认工作流源码依据</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>`context_char_budget` / `context_recent_messages`</t>
+          <t>`docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
+          <t>已记录 system prompt、project prompt、tool registry、tool descriptions、todo reminders、ToolChoiceQueue、agent-loop 的具体文件依据</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
+          <t>P6 实现依据</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 Auto Summary</t>
+          <t>本地 Context Compaction</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -1591,24 +1608,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>`--summary-mode auto` / `AGENT_SUMMARY_MODE=auto`</t>
+          <t>`context_char_budget` / `context_recent_messages`</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值后调用当前 provider 总结早期历史；失败回退 local summary</t>
+          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>需要百炼长上下文实测</t>
+          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>默认工作流</t>
+          <t>OMP 风格 Auto Summary</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -1618,24 +1635,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>`SYSTEM_PROMPT` + runtime workflow reminder</t>
+          <t>`--summary-mode auto` / `AGENT_SUMMARY_MODE=auto`</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>自然语言代码任务默认探索、todo、patch preview、验证、diff</t>
+          <t>小历史不摘要；超过 reserve 阈值后调用当前 provider 总结早期历史；失败回退 local summary</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>需要真实任务实测</t>
+          <t>需要百炼长上下文实测</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>轻量 LSP 工具</t>
+          <t>默认工作流</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -1645,24 +1662,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
+          <t>`SYSTEM_PROMPT` + runtime workflow reminder</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
+          <t>自然语言代码任务默认探索、todo、patch preview、验证、diff</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>后续看是否升级完整 LSP</t>
+          <t>需要真实任务实测</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>Multi-root workspace</t>
+          <t>轻量 LSP 工具</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -1672,24 +1689,24 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS`</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>真实需求压测</t>
+          <t>后续看是否升级完整 LSP</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>Startup memory</t>
+          <t>Multi-root workspace</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -1699,24 +1716,24 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime` system prompt 构造</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS`</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
+          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>真实 session 验证</t>
+          <t>真实需求压测</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>Learn 工具</t>
+          <t>Startup memory</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -1726,12 +1743,12 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>`learn`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>写入 `.local-agent/memory/learned.md`，默认走写工具审批</t>
+          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -1743,7 +1760,7 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Learn 工具</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -1753,12 +1770,12 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime` system prompt 构造</t>
+          <t>`learn`</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
+          <t>写入 `.local-agent/memory/learned.md`，默认走写工具审批</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -1770,130 +1787,130 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>Memory / Skills 方案</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>已完成设计</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>`docs/memory-skills-implementation-plan.md`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
+          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>下一步真实压测</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步真实压测</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>Patch preview</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`apply_patch dry_run=true`</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>后续评估 rollback</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>Patch rollback</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>`rollback_patch`</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -1905,34 +1922,34 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>ask_user timeout</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>重复工具调用熔断</t>
+          <t>Tool approval policy</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
@@ -1942,24 +1959,24 @@
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
+          <t>`tool_approval` + `session_tool_approval`</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
+          <t>日用反馈</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>Tool result pruning</t>
+          <t>重复工具调用熔断</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
@@ -1969,24 +1986,24 @@
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>`ToolResult.useless` + provider-bound context pruning</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>继续真实长任务观察</t>
+          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>Todo steering</t>
+          <t>Tool result pruning</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -1996,42 +2013,69 @@
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>provider-bound runtime todo reminder</t>
+          <t>`ToolResult.useless` + provider-bound context pruning</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+          <t>继续真实长任务观察</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
+          <t>Todo steering</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>provider-bound runtime todo reminder</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B45" s="0" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C45" s="0" t="inlineStr">
-        <is>
-          <t>当前 124 个测试通过</t>
-        </is>
-      </c>
-      <c r="D45" s="0" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>当前 128 个测试通过</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E45" s="0" t="inlineStr">
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -4279,7 +4323,7 @@
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
@@ -4294,7 +4338,7 @@
       </c>
       <c r="H54" s="0" t="inlineStr">
         <is>
-          <t>增加 `--state-dir` / `AGENT_STATE_DIR`，默认 sessions/todos/patch logs 使用用户级状态目录；保留项目 memory/skills 的明确策略；测试覆盖跨 `--cwd` 不写目标 `.local-agent/sessions`</t>
+          <t>`--state-dir` / `AGENT_STATE_DIR` 已落地；默认 sessions/todos/patch logs 使用用户级状态目录；项目 memory/skills 保留在 workspace；测试覆盖跨 `--cwd` 不写目标 `.local-agent/sessions`</t>
         </is>
       </c>
     </row>
@@ -4983,17 +5027,17 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>新发现，待处理</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>当前 `JsonlSessionStore`、todo、patch log 默认写入 `--cwd/.local-agent`；2026-07-08 企业项目只读代跑创建了 `.local-agent/sessions/*.jsonl`</t>
+          <t>当前 `JsonlSessionStore`、todo、patch log 曾默认写入 `--cwd/.local-agent`；2026-07-08 企业项目只读代跑创建了 `.local-agent/sessions/*.jsonl`</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>OMP 默认把 sessions 放在 `~/.omp/agent/sessions/&lt;cwd-encoded&gt;/`，项目 `.omp` 更偏 context/config/rules/skills；我们应增加用户级 `--state-dir`，把 sessions/todos/patch logs 与源码目录解耦。</t>
+          <t>已参考 OMP 默认 session 目录在用户 agent dir 的设计，实现 `--state-dir`；sessions/todos/patch logs 与源码目录解耦，项目 memory/skills 仍保留在 workspace。</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5827,7 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>新发现，待处理</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -5798,7 +5842,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>下一步实现 `--state-dir` / `AGENT_STATE_DIR`，默认把 sessions/todos/patch logs 放到用户级状态目录；项目 memory/skills 另行明确。</t>
+          <t>已实现 `--state-dir` / `AGENT_STATE_DIR`，默认把 sessions/todos/patch logs 放到用户级状态目录；项目 memory/skills 仍保留在 workspace。</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5950,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 124 个 unittest 和 compileall。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 128 个 unittest 和 compileall。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record enterprise pressure test rerun status
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -100,9 +100,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
@@ -163,7 +163,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
         </is>
       </c>
     </row>
@@ -208,7 +208,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -436,7 +436,7 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>Startup memory</t>
+          <t>Startup context / sticky rules</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -446,14 +446,14 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>新 session 自动注入 `.local-agent/memory/{project,decisions,conventions,learned}.md`，作为 advisory context。</t>
+          <t>用户级和项目级 `AGENTS.md` 启动注入；用户级和项目级 `RULES.md` 每次 provider request 前注入。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>Learn 工具</t>
+          <t>Startup memory</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -463,14 +463,14 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
+          <t>新 session 自动注入 `.local-agent/memory/{project,decisions,conventions,learned}.md`，作为 advisory context。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Learn 工具</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -480,14 +480,14 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
+          <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>Runtime state dir</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -497,22 +497,39 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
+          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
+          <t>Runtime state dir</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B25" s="0" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C25" s="0" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn` 和 authored skills discovery 已完成，managed skills/autolearn 后置。</t>
         </is>
@@ -818,7 +835,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -833,7 +850,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir`。下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir` 和 AGENTS/RULES 分层。下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -846,9 +863,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
@@ -1544,34 +1561,34 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记</t>
+          <t>Startup context / sticky rules</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>`docs/omp-core-architecture-notes.md`</t>
+          <t>`AgentRuntime` system prompt / provider-bound context</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>固化主循环、deadline、compaction、tool approval、默认工作流分层结论</t>
+          <t>用户级和项目级 `AGENTS.md` 启动注入；用户级和项目级 `RULES.md` 每次 provider request 前注入</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>后续设计依据</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>OMP 默认工作流源码依据</t>
+          <t>OMP 核心架构笔记</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -1586,46 +1603,46 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>已记录 system prompt、project prompt、tool registry、tool descriptions、todo reminders、ToolChoiceQueue、agent-loop 的具体文件依据</t>
+          <t>固化主循环、deadline、compaction、tool approval、默认工作流分层结论</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>P6 实现依据</t>
+          <t>后续设计依据</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>本地 Context Compaction</t>
+          <t>OMP 默认工作流源码依据</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>`context_char_budget` / `context_recent_messages`</t>
+          <t>`docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
+          <t>已记录 system prompt、project prompt、tool registry、tool descriptions、todo reminders、ToolChoiceQueue、agent-loop 的具体文件依据</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
+          <t>P6 实现依据</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 Auto Summary</t>
+          <t>本地 Context Compaction</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -1635,24 +1652,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>`--summary-mode auto` / `AGENT_SUMMARY_MODE=auto`</t>
+          <t>`context_char_budget` / `context_recent_messages`</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值后调用当前 provider 总结早期历史；失败回退 local summary</t>
+          <t>折叠早期历史，保留最近消息和当前用户请求，注入未完成 todo，截断发送给模型的超大 tool 输出，并保持单 system 消息</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>需要百炼长上下文实测</t>
+          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>默认工作流</t>
+          <t>OMP 风格 Auto Summary</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -1662,24 +1679,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`SYSTEM_PROMPT` + runtime workflow reminder</t>
+          <t>`--summary-mode auto` / `AGENT_SUMMARY_MODE=auto`</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>自然语言代码任务默认探索、todo、patch preview、验证、diff</t>
+          <t>小历史不摘要；超过 reserve 阈值后调用当前 provider 总结早期历史；失败回退 local summary</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>需要真实任务实测</t>
+          <t>需要百炼长上下文实测</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>轻量 LSP 工具</t>
+          <t>默认工作流</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -1689,24 +1706,24 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
+          <t>`SYSTEM_PROMPT` + runtime workflow reminder</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
+          <t>自然语言代码任务默认探索、todo、patch preview、验证、diff</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>后续看是否升级完整 LSP</t>
+          <t>需要真实任务实测</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>Multi-root workspace</t>
+          <t>轻量 LSP 工具</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -1716,24 +1733,24 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS`</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>真实需求压测</t>
+          <t>后续看是否升级完整 LSP</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>Startup memory</t>
+          <t>Multi-root workspace</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -1743,24 +1760,24 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime` system prompt 构造</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS`</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
+          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>真实 session 验证</t>
+          <t>真实需求压测</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>Learn 工具</t>
+          <t>Startup memory</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -1770,12 +1787,12 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>`learn`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>写入 `.local-agent/memory/learned.md`，默认走写工具审批</t>
+          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -1787,7 +1804,7 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Learn 工具</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
@@ -1797,12 +1814,12 @@
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime` system prompt 构造</t>
+          <t>`learn`</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
+          <t>写入 `.local-agent/memory/learned.md`，默认走写工具审批</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -1814,130 +1831,130 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>Memory / Skills 方案</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>已完成设计</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>`docs/memory-skills-implementation-plan.md`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
+          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>下一步真实压测</t>
+          <t>真实 session 验证</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>下一步真实压测</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>Patch preview</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`apply_patch dry_run=true`</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
+          <t>后续评估 rollback</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>Patch rollback</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>`rollback_patch`</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -1949,34 +1966,34 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>ask_user timeout</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
+          <t>继续真实任务验证</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>重复工具调用熔断</t>
+          <t>Tool approval policy</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
@@ -1986,24 +2003,24 @@
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
+          <t>`tool_approval` + `session_tool_approval`</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
+          <t>日用反馈</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>Tool result pruning</t>
+          <t>重复工具调用熔断</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -2013,24 +2030,24 @@
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>`ToolResult.useless` + provider-bound context pruning</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>继续真实长任务观察</t>
+          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>Todo steering</t>
+          <t>Tool result pruning</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
@@ -2040,42 +2057,69 @@
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>provider-bound runtime todo reminder</t>
+          <t>`ToolResult.useless` + provider-bound context pruning</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+          <t>继续真实长任务观察</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
+          <t>Todo steering</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>provider-bound runtime todo reminder</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B46" s="0" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C46" s="0" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>当前 128 个测试通过</t>
         </is>
       </c>
-      <c r="D46" s="0" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E46" s="0" t="inlineStr">
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
@@ -2090,7 +2134,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H56"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4342,6 +4386,90 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>T-053</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>用户级/项目级 AGENTS 与 sticky RULES</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>对齐 Claude Code / OMP 的人工上下文层级，减少重复提示并让短规则跨长会话可见</t>
+        </is>
+      </c>
+      <c r="H55" s="0" t="inlineStr">
+        <is>
+          <t>`AGENT_CONFIG_DIR` 下的用户级 `AGENTS.md` / `RULES.md` 和 workspace `.local-agent/AGENTS.md` / `RULES.md` 已支持；测试覆盖启动注入和 provider-bound 注入</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>T-054</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>企业项目真实联网只读压测复跑</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>当前 Codex 环境阻断，用户本机待跑</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>验证 `--cwd` 企业项目 + `--allow-dir` 需求目录 + 百炼 provider + 用户级 state-dir 的真实链路</t>
+        </is>
+      </c>
+      <c r="H56" s="0" t="inlineStr">
+        <is>
+          <t>本次外部执行被 Codex 宿主策略拒绝；已记录可运行命令和本地 state-dir 验证结果。用户在允许环境中运行后，把 session 输出回贴即可继续分析。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -4351,7 +4479,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5044,37 +5172,37 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-018</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>AGENTS/RULES 长期注入可能与当前任务冲突</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，持续关注</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>注入区明确 advisory；system prompt 明确当前用户指令和源码证据优先；RULES 适合短规则，长背景放 AGENTS 或 memory</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>Claude Code 和 OMP 都把这类上下文作为指导而非硬约束；真正硬限制应靠 permission/hooks。我们先做 advisory 注入，危险动作仍靠 approval。</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5214,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -5096,22 +5224,22 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -5123,7 +5251,7 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -5133,7 +5261,7 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -5143,12 +5271,12 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5288,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -5170,22 +5298,22 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5325,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -5207,7 +5335,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -5217,12 +5345,12 @@
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5362,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -5244,7 +5372,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -5254,12 +5382,12 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5399,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -5281,7 +5409,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -5291,12 +5419,12 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5436,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -5318,7 +5446,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -5328,12 +5456,12 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -5345,7 +5473,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -5355,7 +5483,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -5365,12 +5493,12 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5510,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -5392,22 +5520,22 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5547,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -5429,7 +5557,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -5439,12 +5567,12 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5584,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -5466,7 +5594,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -5476,12 +5604,12 @@
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5621,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -5503,22 +5631,22 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -5530,32 +5658,106 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>已接受并部分落地</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+        </is>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
           <t>ADR-014</t>
         </is>
       </c>
-      <c r="C33" s="0" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D33" s="0" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
-      <c r="E33" s="0" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F33" s="0" t="inlineStr">
+      <c r="F34" s="0" t="inlineStr">
         <is>
           <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
-      <c r="G33" s="0" t="inlineStr">
+      <c r="G34" s="0" t="inlineStr">
         <is>
           <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>ADR-015</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -5827,12 +6029,12 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭并本地验证</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>企业项目只读代跑在目标仓库创建 `.local-agent/sessions/20260708T053955405637Z.jsonl`，导致 `git status` 新增 `?? .local-agent/`。</t>
+          <t>企业项目只读代跑曾在目标仓库创建 `.local-agent/sessions/20260708T053955405637Z.jsonl`，导致 `git status` 新增 `?? .local-agent/`。提交 `cb7400d` 后，本地配置解析确认 `crcl-open` 默认 state dir 为用户级 `/Users/chengming/.local/state/local-coding-agent/workspaces/mycode-project-crcl-open-crcl-open-966d4fe7a33b`，目标仓库未发现 `.local-agent`。</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -5864,7 +6066,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>`crcl-open/crcl-open` 本身已有大量 modified 文件，压测前后需要快照才能证明 LCA 是否污染业务文件。</t>
+          <t>`crcl-open/crcl-open` 本身已有大量 modified 文件，压测前后需要快照才能证明 LCA 是否污染业务文件。当前版本已把 runtime state 移出目标仓库，但真实联网压测仍要记录前后 `git status`。</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -5950,7 +6152,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 128 个 unittest 和 compileall。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 130 个 unittest 和 compileall。</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6216,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6314,17 +6516,17 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>项目记忆</t>
+          <t>常驻上下文</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`</t>
+          <t>用户级 `AGENTS.md` 放个人偏好，项目 `.local-agent/AGENTS.md` 放项目背景；短规则放对应 `RULES.md`</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>减少重复交代项目约定</t>
+          <t>减少重复提示，并让短规则跨长会话可见</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -6334,7 +6536,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>memory 是 advisory，当前用户指令优先</t>
+          <t>可用 `AGENT_CONFIG_DIR` 改用户级目录；都是 advisory</t>
         </is>
       </c>
     </row>
@@ -6344,17 +6546,17 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>本地 skills</t>
+          <t>项目记忆</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>将可复用工作流写到 `.local-agent/skills/&lt;name&gt;/SKILL.md`，带 `name` / `description` frontmatter</t>
+          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>降低重复提示成本</t>
+          <t>减少重复交代项目约定</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -6364,7 +6566,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>启动只注入 metadata，正文按需 read_file</t>
+          <t>memory 是 advisory，当前用户指令优先</t>
         </is>
       </c>
     </row>
@@ -6374,27 +6576,27 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>有歧义</t>
+          <t>本地 skills</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>使用 `ask_user` 中途问用户</t>
+          <t>将可复用工作流写到 `.local-agent/skills/&lt;name&gt;/SKILL.md`，带 `name` / `description` frontmatter</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>避免模型瞎猜</t>
+          <t>降低重复提示成本</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>P3+</t>
+          <t>P7+</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>非交互会返回明确错误</t>
+          <t>启动只注入 metadata，正文按需 read_file</t>
         </is>
       </c>
     </row>
@@ -6404,25 +6606,55 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
+          <t>有歧义</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>使用 `ask_user` 中途问用户</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>避免模型瞎猜</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>P3+</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>非交互会返回明确错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
           <t>同步 Excel</t>
         </is>
       </c>
-      <c r="C14" s="0" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>`python3 scripts/sync_project_excel.py`</t>
         </is>
       </c>
-      <c r="D14" s="0" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Excel 是开发展示产物，Markdown 是开发事实源</t>
         </is>
       </c>
-      <c r="E14" s="0" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>P2+</t>
         </is>
       </c>
-      <c r="F14" s="0" t="inlineStr">
+      <c r="F15" s="0" t="inlineStr">
         <is>
           <t>无第三方依赖</t>
         </is>

</xml_diff>

<commit_message>
Add optional session memory consolidation
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -100,11 +100,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:D27"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -115,6 +116,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -132,6 +134,7 @@
           <t>说明</t>
         </is>
       </c>
+      <c r="D2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -149,6 +152,7 @@
           <t>本地优先、封闭 VM 可用、只访问指定 AI API，能读代码、搜代码、改代码、跑测试、生成 diff、沉淀项目记忆。</t>
         </is>
       </c>
+      <c r="D3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -163,9 +167,10 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
-        </is>
-      </c>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
+        </is>
+      </c>
+      <c r="D4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -183,6 +188,7 @@
           <t>自动设置 `PYTHONPATH=src`，默认当前目录为 workspace。</t>
         </is>
       </c>
+      <c r="D5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -200,6 +206,7 @@
           <t>`./agent` 会自动加载安装目录 `.env`，也可显式传 `--env-file`；真实环境变量优先。</t>
         </is>
       </c>
+      <c r="D6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -208,13 +215,14 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
           <t>完整 unittest、compileall、diff check、xlsx 检查通过。</t>
         </is>
       </c>
+      <c r="D7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -230,6 +238,7 @@
           <t>单次任务默认 10 分钟墙钟预算；`--budget-seconds 0` 可关闭。</t>
         </is>
       </c>
+      <c r="D8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -245,6 +254,7 @@
           <t>表示不限步；仅在用户显式设置时作为防失控保险丝。</t>
         </is>
       </c>
+      <c r="D9" s="0"/>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -262,6 +272,7 @@
           <t>LLM 请求和 shell/run_tests timeout 会按剩余预算夹紧；deadline 到期会补齐未执行工具结果。</t>
         </is>
       </c>
+      <c r="D10" s="0"/>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -279,6 +290,7 @@
           <t>`context_char_budget` 近似上下文窗口，runtime 至少预留 15%；超过 reserve 阈值后 `--summary-mode auto` 调用当前 provider 生成语义摘要，失败回退 local summary。</t>
         </is>
       </c>
+      <c r="D11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -296,6 +308,7 @@
           <t>deadline 到期、用户中断和 `finish_reason=length` 时会补齐剩余 tool_call 的 tool result。</t>
         </is>
       </c>
+      <c r="D12" s="0"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -313,6 +326,7 @@
           <t>`apply_patch dry_run=true` 只校验并返回 diff，不写文件。</t>
         </is>
       </c>
+      <c r="D13" s="0"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -330,6 +344,7 @@
           <t>`rollback_patch` 只回滚本 session 的 patch 记录，且要求当前文件仍匹配 after tag。</t>
         </is>
       </c>
+      <c r="D14" s="0"/>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -347,6 +362,7 @@
           <t>`ask_user` 支持 `timeout_seconds` / `default_answer`，显式 timeout 也会被当前 budget 剩余时间夹紧。</t>
         </is>
       </c>
+      <c r="D15" s="0"/>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -364,6 +380,7 @@
           <t>支持 `always-ask` / `write` / `yolo`、per-tool `allow` / `prompt` / `deny`、session always allow/reject 和 REPL `/approval`。</t>
         </is>
       </c>
+      <c r="D16" s="0"/>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -381,6 +398,7 @@
           <t>见 `docs/omp-core-architecture-notes.md`，已补 OMP 如何通过系统提示、工具描述和 runtime 纠偏让用户不用指定工具顺序。</t>
         </is>
       </c>
+      <c r="D17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -398,6 +416,7 @@
           <t>system prompt + tool descriptions + runtime workflow reminder 已落地，用户不需要每次手写工具顺序。</t>
         </is>
       </c>
+      <c r="D18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -415,6 +434,7 @@
           <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`，覆盖 Python、Java、JavaScript、TypeScript、Vue。</t>
         </is>
       </c>
+      <c r="D19" s="0"/>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -432,6 +452,7 @@
           <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；shell/git/session/memory 仍锚定 `--cwd`。</t>
         </is>
       </c>
+      <c r="D20" s="0"/>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -449,6 +470,7 @@
           <t>用户级和项目级 `AGENTS.md` 启动注入；用户级和项目级 `RULES.md` 每次 provider request 前注入。</t>
         </is>
       </c>
+      <c r="D21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -466,6 +488,7 @@
           <t>新 session 自动注入 `.local-agent/memory/{project,decisions,conventions,learned}.md`，作为 advisory context。</t>
         </is>
       </c>
+      <c r="D22" s="0"/>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -483,11 +506,12 @@
           <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
         </is>
       </c>
+      <c r="D23" s="0"/>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Memory consolidation</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -497,14 +521,19 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
+          <t>默认 `off`；显式 `--memory-consolidation auto</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>llm` 后，从 session 抽取长期经验并写入 `.local-agent/memory/*.md`。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>Runtime state dir</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -514,30 +543,50 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
-        </is>
-      </c>
+          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
+        </is>
+      </c>
+      <c r="D25" s="0"/>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
+          <t>Runtime state dir</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
+        </is>
+      </c>
+      <c r="D26" s="0"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B26" s="0" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C26" s="0" t="inlineStr">
-        <is>
-          <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn` 和 authored skills discovery 已完成，managed skills/autolearn 后置。</t>
-        </is>
-      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
+        </is>
+      </c>
+      <c r="D27" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -835,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -850,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir` 和 AGENTS/RULES 分层。下一步评估 ToolChoiceQueue / soft tool requirement 和精确 token 预算；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir`、AGENTS/RULES 分层和可选 memory consolidation。下一步等待用户本机真实联网压测输出，再决定 path-scoped rules、ToolChoiceQueue / soft tool requirement 或精确 token 预算哪个优先；完整 DAP/TUI/subagents/managed skills 后置。</t>
         </is>
       </c>
     </row>
@@ -863,13 +912,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:G48"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -882,6 +933,8 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -909,6 +962,8 @@
           <t>下一步</t>
         </is>
       </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -936,6 +991,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -963,6 +1020,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -990,6 +1049,8 @@
           <t>保留 base_url/model 可配置</t>
         </is>
       </c>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -1017,6 +1078,8 @@
           <t>P4 做上下文治理</t>
         </is>
       </c>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -1044,6 +1107,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -1071,6 +1136,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -1098,6 +1165,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -1125,6 +1194,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F10" s="0"/>
+      <c r="G10" s="0"/>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -1152,6 +1223,8 @@
           <t>per-tool auto allow 可选</t>
         </is>
       </c>
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -1179,6 +1252,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -1206,6 +1281,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -1233,6 +1310,8 @@
           <t>继续真实任务验证</t>
         </is>
       </c>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -1260,6 +1339,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -1287,6 +1368,8 @@
           <t>后续看需求升级</t>
         </is>
       </c>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1314,6 +1397,8 @@
           <t>加 synthetic result</t>
         </is>
       </c>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1341,6 +1426,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1368,6 +1455,8 @@
           <t>保持测试</t>
         </is>
       </c>
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -1395,6 +1484,8 @@
           <t>保持</t>
         </is>
       </c>
+      <c r="F20" s="0"/>
+      <c r="G20" s="0"/>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -1422,6 +1513,8 @@
           <t>P4 长任务中继续验证</t>
         </is>
       </c>
+      <c r="F21" s="0"/>
+      <c r="G21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -1449,6 +1542,8 @@
           <t>继续真实任务验证</t>
         </is>
       </c>
+      <c r="F22" s="0"/>
+      <c r="G22" s="0"/>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -1476,6 +1571,8 @@
           <t>继续真实任务验证</t>
         </is>
       </c>
+      <c r="F23" s="0"/>
+      <c r="G23" s="0"/>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -1503,6 +1600,8 @@
           <t>日常入口</t>
         </is>
       </c>
+      <c r="F24" s="0"/>
+      <c r="G24" s="0"/>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
@@ -1530,6 +1629,8 @@
           <t>跨项目 token 与 `--cwd` 解耦</t>
         </is>
       </c>
+      <c r="F25" s="0"/>
+      <c r="G25" s="0"/>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
@@ -1557,6 +1658,8 @@
           <t>真实企业项目只读复测</t>
         </is>
       </c>
+      <c r="F26" s="0"/>
+      <c r="G26" s="0"/>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
@@ -1584,6 +1687,8 @@
           <t>真实 session 验证</t>
         </is>
       </c>
+      <c r="F27" s="0"/>
+      <c r="G27" s="0"/>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
@@ -1611,6 +1716,8 @@
           <t>后续设计依据</t>
         </is>
       </c>
+      <c r="F28" s="0"/>
+      <c r="G28" s="0"/>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
@@ -1638,6 +1745,8 @@
           <t>P6 实现依据</t>
         </is>
       </c>
+      <c r="F29" s="0"/>
+      <c r="G29" s="0"/>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
@@ -1665,6 +1774,8 @@
           <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
         </is>
       </c>
+      <c r="F30" s="0"/>
+      <c r="G30" s="0"/>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
@@ -1692,6 +1803,8 @@
           <t>需要百炼长上下文实测</t>
         </is>
       </c>
+      <c r="F31" s="0"/>
+      <c r="G31" s="0"/>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
@@ -1719,6 +1832,8 @@
           <t>需要真实任务实测</t>
         </is>
       </c>
+      <c r="F32" s="0"/>
+      <c r="G32" s="0"/>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
@@ -1746,6 +1861,8 @@
           <t>后续看是否升级完整 LSP</t>
         </is>
       </c>
+      <c r="F33" s="0"/>
+      <c r="G33" s="0"/>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
@@ -1773,6 +1890,8 @@
           <t>真实需求压测</t>
         </is>
       </c>
+      <c r="F34" s="0"/>
+      <c r="G34" s="0"/>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
@@ -1800,6 +1919,8 @@
           <t>真实 session 验证</t>
         </is>
       </c>
+      <c r="F35" s="0"/>
+      <c r="G35" s="0"/>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
@@ -1827,11 +1948,13 @@
           <t>真实 session 验证</t>
         </is>
       </c>
+      <c r="F36" s="0"/>
+      <c r="G36" s="0"/>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Memory consolidation</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
@@ -1841,15 +1964,25 @@
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime` system prompt 构造</t>
+          <t>`memory_consolidation=off</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
+          <t>auto</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>llm`</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>默认 off；显式开启后从 session 抽取长期 project/decisions/conventions/learned 并追加到 `.local-agent/memory/*.md`</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
         <is>
           <t>真实 session 验证</t>
         </is>
@@ -1858,130 +1991,138 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>Memory / Skills 方案</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>已完成设计</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>`docs/memory-skills-implementation-plan.md`</t>
+          <t>`AgentRuntime` system prompt 构造</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>分阶段对齐 OMP：memory 注入、`learn`、authored skills、managed skills/autolearn</t>
+          <t>`.local-agent/skills/&lt;name&gt;/SKILL.md` 只注入 name/description/source，正文按需读取</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>下一步真实压测</t>
-        </is>
-      </c>
+          <t>真实 session 验证</t>
+        </is>
+      </c>
+      <c r="F38" s="0"/>
+      <c r="G38" s="0"/>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>Synthetic tool result</t>
+          <t>Memory / Skills 方案</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成设计</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
+          <t>`docs/memory-skills-implementation-plan.md`</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>避免 session 留下未配对 tool_calls</t>
+          <t>分阶段对齐 OMP：memory 注入、`learn`、memory consolidation、authored skills、managed skills/autolearn</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
-        </is>
-      </c>
+          <t>下一步真实压测</t>
+        </is>
+      </c>
+      <c r="F39" s="0"/>
+      <c r="G39" s="0"/>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>Patch preview</t>
+          <t>Synthetic tool result</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>`apply_patch dry_run=true`</t>
+          <t>deadline 到期、用户中断和 `finish_reason=length` 时补齐 tool result</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>复用 anchored 校验并返回 diff，不写文件</t>
+          <t>避免 session 留下未配对 tool_calls</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>后续评估 rollback</t>
-        </is>
-      </c>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+      <c r="F40" s="0"/>
+      <c r="G40" s="0"/>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>Patch rollback</t>
+          <t>Patch preview</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>`rollback_patch`</t>
+          <t>`apply_patch dry_run=true`</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>校验当前文件 hash 后恢复 patch 前内容</t>
+          <t>复用 anchored 校验并返回 diff，不写文件</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>继续真实任务验证</t>
-        </is>
-      </c>
+          <t>后续评估 rollback</t>
+        </is>
+      </c>
+      <c r="F41" s="0"/>
+      <c r="G41" s="0"/>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>ask_user timeout</t>
+          <t>Patch rollback</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
+          <t>`rollback_patch`</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
+          <t>校验当前文件 hash 后恢复 patch 前内容</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -1989,38 +2130,42 @@
           <t>继续真实任务验证</t>
         </is>
       </c>
+      <c r="F42" s="0"/>
+      <c r="G42" s="0"/>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>Tool approval policy</t>
+          <t>ask_user timeout</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>`tool_approval` + `session_tool_approval`</t>
+          <t>`timeout_seconds` / `default_answer` / budget 剩余时间</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
+          <t>长任务无人响应时可以继续或明确失败；显式 timeout 也受 budget 夹紧</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>日用反馈</t>
-        </is>
-      </c>
+          <t>继续真实任务验证</t>
+        </is>
+      </c>
+      <c r="F43" s="0"/>
+      <c r="G43" s="0"/>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>重复工具调用熔断</t>
+          <t>Tool approval policy</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -2030,24 +2175,26 @@
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
+          <t>`tool_approval` + `session_tool_approval`</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
+          <t>config deny/prompt 是硬护栏，session allow/reject 可记住当前会话，REPL 会校验工具名，approval prompt 受 deadline 约束</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
-        </is>
-      </c>
+          <t>日用反馈</t>
+        </is>
+      </c>
+      <c r="F44" s="0"/>
+      <c r="G44" s="0"/>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>Tool result pruning</t>
+          <t>重复工具调用熔断</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
@@ -2057,24 +2204,26 @@
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>`ToolResult.useless` + provider-bound context pruning</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>继续真实长任务观察</t>
-        </is>
-      </c>
+          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
+        </is>
+      </c>
+      <c r="F45" s="0"/>
+      <c r="G45" s="0"/>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t>Todo steering</t>
+          <t>Tool result pruning</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
@@ -2084,57 +2233,90 @@
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>provider-bound runtime todo reminder</t>
+          <t>`ToolResult.useless` + provider-bound context pruning</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
-        </is>
-      </c>
+          <t>继续真实长任务观察</t>
+        </is>
+      </c>
+      <c r="F46" s="0"/>
+      <c r="G46" s="0"/>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
+          <t>Todo steering</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>provider-bound runtime todo reminder</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+        </is>
+      </c>
+      <c r="F47" s="0"/>
+      <c r="G47" s="0"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
           <t>测试覆盖</t>
         </is>
       </c>
-      <c r="B47" s="0" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C47" s="0" t="inlineStr">
-        <is>
-          <t>当前 128 个测试通过</t>
-        </is>
-      </c>
-      <c r="D47" s="0" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>当前 136 个测试通过</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>unittest、compileall、diff check、xlsx 检查通过</t>
         </is>
       </c>
-      <c r="E47" s="0" t="inlineStr">
+      <c r="E48" s="0" t="inlineStr">
         <is>
           <t>日用反馈补测</t>
         </is>
       </c>
+      <c r="F48" s="0"/>
+      <c r="G48" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:I57"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2144,6 +2326,7 @@
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
+    <col min="9" max="9" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2159,6 +2342,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2201,6 +2385,7 @@
           <t>完成标准</t>
         </is>
       </c>
+      <c r="I2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -2243,6 +2428,7 @@
           <t>Excel 已复核；Markdown 看板已建立</t>
         </is>
       </c>
+      <c r="I3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -2285,6 +2471,7 @@
           <t>文档已存在</t>
         </is>
       </c>
+      <c r="I4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -2327,6 +2514,7 @@
           <t>提交 `2c4348b` 已创建</t>
         </is>
       </c>
+      <c r="I5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -2369,6 +2557,7 @@
           <t>CLI/env/config 已支持；默认 600 秒</t>
         </is>
       </c>
+      <c r="I6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -2411,6 +2600,7 @@
           <t>默认值 0；显式设置才作为保险丝</t>
         </is>
       </c>
+      <c r="I7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -2453,6 +2643,7 @@
           <t>`todo_read/add/update` 可用</t>
         </is>
       </c>
+      <c r="I8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -2495,6 +2686,7 @@
           <t>交互式终端可提问</t>
         </is>
       </c>
+      <c r="I9" s="0"/>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -2537,6 +2729,7 @@
           <t>`--auto-approve-tools` 可用</t>
         </is>
       </c>
+      <c r="I10" s="0"/>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -2579,6 +2772,7 @@
           <t>README 已更新</t>
         </is>
       </c>
+      <c r="I11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -2621,6 +2815,7 @@
           <t>已实现字符阈值 deterministic compaction；LLM summary 已补，下一步升级 token budget / reserve</t>
         </is>
       </c>
+      <c r="I12" s="0"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -2663,6 +2858,7 @@
           <t>deadline 到期、用户中断和 length 截断已补齐</t>
         </is>
       </c>
+      <c r="I13" s="0"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -2705,6 +2901,7 @@
           <t>已完成 dry_run 预览和 session 级 hash 校验 rollback</t>
         </is>
       </c>
+      <c r="I14" s="0"/>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -2747,6 +2944,7 @@
           <t>轻量 LSP 已做；TUI/subagents/AST edit/DAP 继续后置</t>
         </is>
       </c>
+      <c r="I15" s="0"/>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -2789,6 +2987,7 @@
           <t>提交 `304fbdf` 已创建</t>
         </is>
       </c>
+      <c r="I16" s="0"/>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -2831,6 +3030,7 @@
           <t>`scripts/sync_project_excel.py` 可从本文件生成 Excel</t>
         </is>
       </c>
+      <c r="I17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -2873,6 +3073,7 @@
           <t>LLM/tool timeout 按剩余预算夹紧；未执行工具有 synthetic result</t>
         </is>
       </c>
+      <c r="I18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -2915,6 +3116,7 @@
           <t>提交 `4beb487` 已创建</t>
         </is>
       </c>
+      <c r="I19" s="0"/>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -2957,6 +3159,7 @@
           <t>LLM 层已暴露 finish_reason，并补可恢复提示</t>
         </is>
       </c>
+      <c r="I20" s="0"/>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -2999,6 +3202,7 @@
           <t>`apply_patch dry_run=true` 不写文件并返回 diff</t>
         </is>
       </c>
+      <c r="I21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -3041,6 +3245,7 @@
           <t>`rollback_patch` 校验 after tag 后恢复 before_text</t>
         </is>
       </c>
+      <c r="I22" s="0"/>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -3083,6 +3288,7 @@
           <t>`ask_user` 支持 timeout/default，并受 budget 剩余时间约束</t>
         </is>
       </c>
+      <c r="I23" s="0"/>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -3125,6 +3331,7 @@
           <t>`--tool-approval` / `AGENT_TOOL_APPROVAL` 支持每工具策略</t>
         </is>
       </c>
+      <c r="I24" s="0"/>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
@@ -3167,6 +3374,7 @@
           <t>支持 `always-ask` / `write` / `yolo`、`s/d` 会话记忆、`/approval` 命令</t>
         </is>
       </c>
+      <c r="I25" s="0"/>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
@@ -3209,6 +3417,7 @@
           <t>approval prompt 使用 deadline-aware timed stdin；deadline 到期自动取消/拒绝，保留 `y/s/n/d` 和 session allow/reject</t>
         </is>
       </c>
+      <c r="I26" s="0"/>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
@@ -3251,6 +3460,7 @@
           <t>新配置优先于旧字段；config prompt/deny 是硬护栏；REPL 校验未知工具名</t>
         </is>
       </c>
+      <c r="I27" s="0"/>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
@@ -3293,6 +3503,7 @@
           <t>显式 `timeout_seconds` 会被剩余 budget 夹紧；recent tool 输出只在发送模型副本中截断，session 原文保留</t>
         </is>
       </c>
+      <c r="I28" s="0"/>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
@@ -3335,6 +3546,7 @@
           <t>压缩摘要合并进首个 system prompt；测试锁定发送给模型时只有一条 system</t>
         </is>
       </c>
+      <c r="I29" s="0"/>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
@@ -3377,6 +3589,7 @@
           <t>compaction 摘要强保留当前用户请求；read_file 截断提示改为“任务需要才继续”</t>
         </is>
       </c>
+      <c r="I30" s="0"/>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
@@ -3419,6 +3632,7 @@
           <t>会话 `20260707T093557800154Z` 严格完成 5 个指定工具调用后输出三句话总结，未继续额外读文件</t>
         </is>
       </c>
+      <c r="I31" s="0"/>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
@@ -3461,6 +3675,7 @@
           <t>复测会话 `20260707T094246132064Z` 跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff；最终仅新增一个测试 docstring</t>
         </is>
       </c>
+      <c r="I32" s="0"/>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
@@ -3503,6 +3718,7 @@
           <t>`write_file` 描述已改为 create-only，并加测试确保不再出现 `fully overwrite`</t>
         </is>
       </c>
+      <c r="I33" s="0"/>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
@@ -3545,6 +3761,7 @@
           <t>README 已补日用模板；项目状态和 Excel 已同步；90 个测试、compileall、xlsx、diff check 通过</t>
         </is>
       </c>
+      <c r="I34" s="0"/>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
@@ -3587,6 +3804,7 @@
           <t>已决定优先做 OMP 默认工作流本地化；随后按用户要求补 LLM summary 和轻量 LSP</t>
         </is>
       </c>
+      <c r="I35" s="0"/>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
@@ -3629,6 +3847,7 @@
           <t>`docs/omp-core-architecture-notes.md` 已新增“OMP 如何让用户不用指定工具顺序”</t>
         </is>
       </c>
+      <c r="I36" s="0"/>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
@@ -3671,6 +3890,7 @@
           <t>默认 prompt 覆盖理解、修改、验证、todo、ask_user、patch preview、diff</t>
         </is>
       </c>
+      <c r="I37" s="0"/>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
@@ -3713,6 +3933,7 @@
           <t>既有 create-only/patch dry_run 描述保持测试；新增 LSP 工具描述</t>
         </is>
       </c>
+      <c r="I38" s="0"/>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
@@ -3755,6 +3976,7 @@
           <t>非平凡代码任务会注入 reminder；短 prompt 不注入</t>
         </is>
       </c>
+      <c r="I39" s="0"/>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
@@ -3797,6 +4019,7 @@
           <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 已覆盖 read/list/search/LSP/apply_patch/write_file/rollback_patch</t>
         </is>
       </c>
+      <c r="I40" s="0"/>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
@@ -3839,6 +4062,7 @@
           <t>默认 `--summary-mode auto`；超过 reserve 阈值才调用 LLM summary，失败回退 local summary</t>
         </is>
       </c>
+      <c r="I41" s="0"/>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
@@ -3881,6 +4105,7 @@
           <t>Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics 已可用</t>
         </is>
       </c>
+      <c r="I42" s="0"/>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
@@ -3923,6 +4148,7 @@
           <t>已新增 `docs/memory-skills-implementation-plan.md`，并补充 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
+      <c r="I43" s="0"/>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
@@ -3965,6 +4191,7 @@
           <t>读取 `.local-agent/memory/*.md`，以 advisory block 注入 system prompt，带 source path 和预算</t>
         </is>
       </c>
+      <c r="I44" s="0"/>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
@@ -4007,6 +4234,7 @@
           <t>写入 `.local-agent/memory/learned.md`，限制长度并清洗会进入 prompt 的字段</t>
         </is>
       </c>
+      <c r="I45" s="0"/>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
@@ -4049,6 +4277,7 @@
           <t>先扫 `.local-agent/skills/&lt;name&gt;/SKILL.md`，system prompt 只列 name/description/source，正文按需读取</t>
         </is>
       </c>
+      <c r="I46" s="0"/>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
@@ -4091,6 +4320,7 @@
           <t>默认关闭；后续按 OMP `manage_skill` 思路隔离 generated skills，authored skills 优先</t>
         </is>
       </c>
+      <c r="I47" s="0"/>
     </row>
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
@@ -4133,6 +4363,7 @@
           <t>新增 `docs/pressure-test-2026-07-08.md`，记录压测证据、OMP 对应机制和 LCA 措施</t>
         </is>
       </c>
+      <c r="I48" s="0"/>
     </row>
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
@@ -4175,6 +4406,7 @@
           <t>最近 12 次工具调用内同名同参超过 3 次会跳过；连续命中 8 次停止；测试覆盖 JSON 参数顺序归一化</t>
         </is>
       </c>
+      <c r="I49" s="0"/>
     </row>
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
@@ -4217,6 +4449,7 @@
           <t>LCA 产品设计不内置禁止外发；按 OMP 思路由用户、provider、permission 和运行环境策略决定。本次 Codex 环境无法代跑，已改成本地只读扫描。</t>
         </is>
       </c>
+      <c r="I50" s="0"/>
     </row>
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
@@ -4259,6 +4492,7 @@
           <t>CLI 支持显式 `--env-file`；`./agent` 自动把安装目录 `.env` 注入为 env-file；测试覆盖优先级和缺失文件报错</t>
         </is>
       </c>
+      <c r="I51" s="0"/>
     </row>
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
@@ -4301,6 +4535,7 @@
           <t>已新增 `ToolResult.useless`；空搜索/LSP 结果会标记 useless；provider-bound context 会折叠 useless/superseded 工具输出并注入 open todo reminder；session 原文保留</t>
         </is>
       </c>
+      <c r="I52" s="0"/>
     </row>
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
@@ -4343,6 +4578,7 @@
           <t>`lsp_workspace_symbols` / `lsp_document_symbols` 已注册为 `lsp_symbols` 只读别名；测试覆盖 registry 和执行结果</t>
         </is>
       </c>
+      <c r="I53" s="0"/>
     </row>
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
@@ -4385,6 +4621,7 @@
           <t>`--state-dir` / `AGENT_STATE_DIR` 已落地；默认 sessions/todos/patch logs 使用用户级状态目录；项目 memory/skills 保留在 workspace；测试覆盖跨 `--cwd` 不写目标 `.local-agent/sessions`</t>
         </is>
       </c>
+      <c r="I54" s="0"/>
     </row>
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
@@ -4427,6 +4664,7 @@
           <t>`AGENT_CONFIG_DIR` 下的用户级 `AGENTS.md` / `RULES.md` 和 workspace `.local-agent/AGENTS.md` / `RULES.md` 已支持；测试覆盖启动注入和 provider-bound 注入</t>
         </is>
       </c>
+      <c r="I55" s="0"/>
     </row>
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
@@ -4466,20 +4704,68 @@
       </c>
       <c r="H56" s="0" t="inlineStr">
         <is>
-          <t>本次外部执行被 Codex 宿主策略拒绝；已记录可运行命令和本地 state-dir 验证结果。用户在允许环境中运行后，把 session 输出回贴即可继续分析。</t>
+          <t>memory consolidation 完成后已用 `--memory-consolidation off` 再次尝试；sandbox 因 DNS/网络失败，外部执行仍被 Codex 宿主策略拒绝。目标仓库未发现 `.local-agent`。用户在允许环境中运行后，把 session 输出回贴即可继续分析。</t>
+        </is>
+      </c>
+      <c r="I56" s="0"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>T-055</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>已完成并 review</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>把 session 中的可复用经验定期整理进 `.local-agent/memory`，减少后续重复交代</t>
+        </is>
+      </c>
+      <c r="H57" s="0" t="inlineStr">
+        <is>
+          <t>`--memory-consolidation auto</t>
+        </is>
+      </c>
+      <c r="I57" s="0" t="inlineStr">
+        <is>
+          <t>llm` 已支持；默认 off，坏 JSON/空结果/deadline 耗尽/本轮已显式写 memory 时不写；测试覆盖成功写入、坏 JSON 不写、默认 off 不额外调用 LLM/不写 memory</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5049,7 +5335,7 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>已补最近窗口同名同参工具调用熔断、`ToolResult.useless`、空结果标记、provider-bound useless/superseded pruning 和 open todo runtime reminder；后续评估 OMP 风格 ToolChoiceQueue / soft tool requirement</t>
+          <t>已补最近窗口同名同参工具调用熔断、`ToolResult.useless`、空结果标记、provider-bound useless/superseded pruning 和 open todo runtime reminder；等待用户本机真实联网压测输出后再决定是否引入 OMP 风格 ToolChoiceQueue / soft tool requirement</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
@@ -5209,37 +5495,37 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-019</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>memory consolidation 可能隐式写入陈旧或敏感内容</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，持续关注</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>默认 off；显式开启才写；只接受严格 JSON 的短条目；坏 JSON、空结果、deadline 耗尽、本轮已显式写 memory 时不写</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP/Claude Code 的自动记忆也是启发式上下文，不是事实源硬约束。我们先做显式开启的本地 Markdown MVP，后续再评估 path-scoped rules 和 managed skills。</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5537,7 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -5261,22 +5547,22 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5574,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -5298,7 +5584,7 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -5308,12 +5594,12 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -5325,7 +5611,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -5335,22 +5621,22 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -5362,7 +5648,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -5372,7 +5658,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -5382,12 +5668,12 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5685,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -5409,7 +5695,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -5419,12 +5705,12 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5722,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -5446,7 +5732,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -5456,12 +5742,12 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -5473,7 +5759,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -5483,7 +5769,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -5493,12 +5779,12 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5796,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -5520,7 +5806,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -5530,12 +5816,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5833,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -5557,22 +5843,22 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5870,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -5594,7 +5880,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -5604,12 +5890,12 @@
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5907,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -5631,7 +5917,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -5641,12 +5927,12 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5944,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -5668,22 +5954,22 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -5695,32 +5981,32 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -5732,32 +6018,106 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
           <t>ADR-015</t>
         </is>
       </c>
-      <c r="C35" s="0" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D35" s="0" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
-      <c r="E35" s="0" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F35" s="0" t="inlineStr">
+      <c r="F36" s="0" t="inlineStr">
         <is>
           <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
-      <c r="G35" s="0" t="inlineStr">
+      <c r="G36" s="0" t="inlineStr">
         <is>
           <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation 默认关闭</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>这一步会写项目 `.local-agent/memory`，不同于只发给模型的 context compaction；默认 off 可以保护只读分析和企业项目零业务落盘</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -5770,7 +6130,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5980,7 +6340,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>已补重复工具熔断、provider-bound useless/superseded pruning 和 open todo runtime reminder；后续评估 ToolChoiceQueue / soft tool requirement。</t>
+          <t>已补重复工具熔断、provider-bound useless/superseded pruning 和 open todo runtime reminder；当前不因宿主外发阻断引入 ToolChoiceQueue，等待用户本机真实联网压测结果。</t>
         </is>
       </c>
     </row>
@@ -6077,6 +6437,38 @@
       <c r="F10" s="0" t="inlineStr">
         <is>
           <t>后续企业压测前先记录 `git status --short` 到 LCA 压测记录，压测后对比，不在目标 repo 写快照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>PT-009</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>已关闭并补测试</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>memory consolidation 可能让只读压测产生隐式项目 memory 写入。</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>OMP/Claude Code 的自动记忆是启发式长期上下文，必须与普通 context compaction 区分；默认策略要避免只读任务隐式写项目文件。</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>默认 `off`；只读压测命令显式 `--memory-consolidation off`；新增 runtime 默认 off 回归测试，确认不会额外调用 LLM 或写 `.local-agent/memory`。</t>
         </is>
       </c>
     </row>
@@ -6152,7 +6544,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 130 个 unittest 和 compileall。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 136 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6943,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`</t>
+          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`；需要自动整理时开启 `--memory-consolidation auto`</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -6566,7 +6958,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>memory 是 advisory，当前用户指令优先</t>
+          <t>memory 是 advisory，当前用户指令优先；默认不隐式写</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Steer duplicate tool loops to final answers
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -449,7 +449,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；shell/git/session/memory 仍锚定 `--cwd`。</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
         </is>
       </c>
       <c r="D20" s="0"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>新 session 自动注入 `.local-agent/memory/{project,decisions,conventions,learned}.md`，作为 advisory context。</t>
+          <t>新 session 自动注入项目 `.local-agent/memory/{project,decisions,conventions,learned}.md` 和 state dir `memory/*.md`，作为 advisory context。</t>
         </is>
       </c>
       <c r="D22" s="0"/>
@@ -526,7 +526,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>llm` 后，从 session 抽取长期经验并写入 `.local-agent/memory/*.md`。</t>
+          <t>llm` 后从 session 抽取长期经验；默认写 state dir，`--memory-scope project` 才写 `.local-agent/memory/*.md`。</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，但本次 Codex 执行环境策略阻断代跑，已改为本地只读扫描；已完成 OMP 风格 `--state-dir`、AGENTS/RULES 分层和可选 memory consolidation。下一步等待用户本机真实联网压测输出，再决定 path-scoped rules、ToolChoiceQueue / soft tool requirement 或精确 token 预算哪个优先；完整 DAP/TUI/subagents/managed skills 后置。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停。已补 OMP 风格轻量 forced-final steering；下一步用户复跑同一命令验证是否能产出最终分析，再决定是否引入完整 ToolChoiceQueue / soft tool requirement、path-scoped rules 或精确 token 预算。</t>
         </is>
       </c>
     </row>
@@ -912,15 +912,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:H48"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="48" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -935,6 +936,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -964,6 +966,7 @@
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -993,6 +996,7 @@
       </c>
       <c r="F3" s="0"/>
       <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -1022,6 +1026,7 @@
       </c>
       <c r="F4" s="0"/>
       <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -1051,6 +1056,7 @@
       </c>
       <c r="F5" s="0"/>
       <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -1080,6 +1086,7 @@
       </c>
       <c r="F6" s="0"/>
       <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -1109,6 +1116,7 @@
       </c>
       <c r="F7" s="0"/>
       <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -1138,6 +1146,7 @@
       </c>
       <c r="F8" s="0"/>
       <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -1167,6 +1176,7 @@
       </c>
       <c r="F9" s="0"/>
       <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -1196,6 +1206,7 @@
       </c>
       <c r="F10" s="0"/>
       <c r="G10" s="0"/>
+      <c r="H10" s="0"/>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -1225,6 +1236,7 @@
       </c>
       <c r="F11" s="0"/>
       <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -1254,6 +1266,7 @@
       </c>
       <c r="F12" s="0"/>
       <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -1283,6 +1296,7 @@
       </c>
       <c r="F13" s="0"/>
       <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -1312,6 +1326,7 @@
       </c>
       <c r="F14" s="0"/>
       <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -1341,6 +1356,7 @@
       </c>
       <c r="F15" s="0"/>
       <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -1370,6 +1386,7 @@
       </c>
       <c r="F16" s="0"/>
       <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1399,6 +1416,7 @@
       </c>
       <c r="F17" s="0"/>
       <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1428,6 +1446,7 @@
       </c>
       <c r="F18" s="0"/>
       <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1457,6 +1476,7 @@
       </c>
       <c r="F19" s="0"/>
       <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -1486,6 +1506,7 @@
       </c>
       <c r="F20" s="0"/>
       <c r="G20" s="0"/>
+      <c r="H20" s="0"/>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -1515,6 +1536,7 @@
       </c>
       <c r="F21" s="0"/>
       <c r="G21" s="0"/>
+      <c r="H21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -1544,6 +1566,7 @@
       </c>
       <c r="F22" s="0"/>
       <c r="G22" s="0"/>
+      <c r="H22" s="0"/>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -1573,6 +1596,7 @@
       </c>
       <c r="F23" s="0"/>
       <c r="G23" s="0"/>
+      <c r="H23" s="0"/>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -1602,6 +1626,7 @@
       </c>
       <c r="F24" s="0"/>
       <c r="G24" s="0"/>
+      <c r="H24" s="0"/>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
@@ -1631,6 +1656,7 @@
       </c>
       <c r="F25" s="0"/>
       <c r="G25" s="0"/>
+      <c r="H25" s="0"/>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
@@ -1650,7 +1676,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>sessions/todos/patch logs 默认写入用户级 state root；项目 memory/skills 保留在 workspace</t>
+          <t>sessions/todos/patch logs 默认写入用户级 state root；显式项目 memory/skills 保留在 workspace，自动 consolidation 默认写 state memory</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -1660,6 +1686,7 @@
       </c>
       <c r="F26" s="0"/>
       <c r="G26" s="0"/>
+      <c r="H26" s="0"/>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
@@ -1689,6 +1716,7 @@
       </c>
       <c r="F27" s="0"/>
       <c r="G27" s="0"/>
+      <c r="H27" s="0"/>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
@@ -1718,6 +1746,7 @@
       </c>
       <c r="F28" s="0"/>
       <c r="G28" s="0"/>
+      <c r="H28" s="0"/>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
@@ -1747,6 +1776,7 @@
       </c>
       <c r="F29" s="0"/>
       <c r="G29" s="0"/>
+      <c r="H29" s="0"/>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
@@ -1776,6 +1806,7 @@
       </c>
       <c r="F30" s="0"/>
       <c r="G30" s="0"/>
+      <c r="H30" s="0"/>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
@@ -1805,6 +1836,7 @@
       </c>
       <c r="F31" s="0"/>
       <c r="G31" s="0"/>
+      <c r="H31" s="0"/>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
@@ -1834,6 +1866,7 @@
       </c>
       <c r="F32" s="0"/>
       <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
@@ -1863,6 +1896,7 @@
       </c>
       <c r="F33" s="0"/>
       <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
@@ -1882,7 +1916,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/session/memory 仍锚定 `--cwd`</t>
+          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -1892,6 +1926,7 @@
       </c>
       <c r="F34" s="0"/>
       <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
@@ -1911,7 +1946,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/memory/{project,decisions,conventions,learned}.md` 作为 advisory context 注入</t>
+          <t>项目 `.local-agent/memory/{project,decisions,conventions,learned}.md` 和 state dir `memory/*.md` 作为 advisory context 注入</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -1921,6 +1956,7 @@
       </c>
       <c r="F35" s="0"/>
       <c r="G35" s="0"/>
+      <c r="H35" s="0"/>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
@@ -1950,6 +1986,7 @@
       </c>
       <c r="F36" s="0"/>
       <c r="G36" s="0"/>
+      <c r="H36" s="0"/>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
@@ -1974,15 +2011,20 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>llm`</t>
+          <t>llm` + `memory_scope=state</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>默认 off；显式开启后从 session 抽取长期 project/decisions/conventions/learned 并追加到 `.local-agent/memory/*.md`</t>
+          <t>project`</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>默认 off；显式开启后从 session 抽取长期 project/decisions/conventions/learned；默认追加到 state dir `memory/*.md`，显式 project 才写 `.local-agent/memory/*.md`</t>
+        </is>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
         <is>
           <t>真实 session 验证</t>
         </is>
@@ -2016,6 +2058,7 @@
       </c>
       <c r="F38" s="0"/>
       <c r="G38" s="0"/>
+      <c r="H38" s="0"/>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
@@ -2045,6 +2088,7 @@
       </c>
       <c r="F39" s="0"/>
       <c r="G39" s="0"/>
+      <c r="H39" s="0"/>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
@@ -2074,6 +2118,7 @@
       </c>
       <c r="F40" s="0"/>
       <c r="G40" s="0"/>
+      <c r="H40" s="0"/>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
@@ -2103,6 +2148,7 @@
       </c>
       <c r="F41" s="0"/>
       <c r="G41" s="0"/>
+      <c r="H41" s="0"/>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
@@ -2132,6 +2178,7 @@
       </c>
       <c r="F42" s="0"/>
       <c r="G42" s="0"/>
+      <c r="H42" s="0"/>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
@@ -2161,6 +2208,7 @@
       </c>
       <c r="F43" s="0"/>
       <c r="G43" s="0"/>
+      <c r="H43" s="0"/>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
@@ -2190,11 +2238,12 @@
       </c>
       <c r="F44" s="0"/>
       <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>重复工具调用熔断</t>
+          <t>重复工具调用熔断 / forced-final steering</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
@@ -2204,21 +2253,22 @@
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()`</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `_steer_after_duplicate_tool_call()`</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error，连续命中后停止本轮，避免只靠 budget 截断坏循环</t>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error；重复命中后注入 runtime steering，下一轮不给工具 schema，强制模型从已有证据输出最终回答；连续命中仍有硬停兜底</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>后续评估是否替换为更完整 ToolChoiceQueue / soft tool requirement</t>
+          <t>用户本机复跑企业需求压测；后续视结果评估完整 ToolChoiceQueue / soft tool requirement</t>
         </is>
       </c>
       <c r="F45" s="0"/>
       <c r="G45" s="0"/>
+      <c r="H45" s="0"/>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
@@ -2248,6 +2298,7 @@
       </c>
       <c r="F46" s="0"/>
       <c r="G46" s="0"/>
+      <c r="H46" s="0"/>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
@@ -2277,6 +2328,7 @@
       </c>
       <c r="F47" s="0"/>
       <c r="G47" s="0"/>
+      <c r="H47" s="0"/>
     </row>
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
@@ -2291,7 +2343,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>当前 136 个测试通过</t>
+          <t>当前 140 个测试通过</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -2306,17 +2358,18 @@
       </c>
       <c r="F48" s="0"/>
       <c r="G48" s="0"/>
+      <c r="H48" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:J58"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2326,7 +2379,8 @@
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
-    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2343,6 +2397,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2386,6 +2441,7 @@
         </is>
       </c>
       <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -2429,6 +2485,7 @@
         </is>
       </c>
       <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -2472,6 +2529,7 @@
         </is>
       </c>
       <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -2515,6 +2573,7 @@
         </is>
       </c>
       <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -2558,6 +2617,7 @@
         </is>
       </c>
       <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -2601,6 +2661,7 @@
         </is>
       </c>
       <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -2644,6 +2705,7 @@
         </is>
       </c>
       <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -2687,6 +2749,7 @@
         </is>
       </c>
       <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -2730,6 +2793,7 @@
         </is>
       </c>
       <c r="I10" s="0"/>
+      <c r="J10" s="0"/>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -2773,6 +2837,7 @@
         </is>
       </c>
       <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -2816,6 +2881,7 @@
         </is>
       </c>
       <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -2859,6 +2925,7 @@
         </is>
       </c>
       <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -2902,6 +2969,7 @@
         </is>
       </c>
       <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -2945,6 +3013,7 @@
         </is>
       </c>
       <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -2988,6 +3057,7 @@
         </is>
       </c>
       <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -3031,6 +3101,7 @@
         </is>
       </c>
       <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -3074,6 +3145,7 @@
         </is>
       </c>
       <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -3117,6 +3189,7 @@
         </is>
       </c>
       <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -3160,6 +3233,7 @@
         </is>
       </c>
       <c r="I20" s="0"/>
+      <c r="J20" s="0"/>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -3203,6 +3277,7 @@
         </is>
       </c>
       <c r="I21" s="0"/>
+      <c r="J21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -3246,6 +3321,7 @@
         </is>
       </c>
       <c r="I22" s="0"/>
+      <c r="J22" s="0"/>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -3289,6 +3365,7 @@
         </is>
       </c>
       <c r="I23" s="0"/>
+      <c r="J23" s="0"/>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -3332,6 +3409,7 @@
         </is>
       </c>
       <c r="I24" s="0"/>
+      <c r="J24" s="0"/>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
@@ -3375,6 +3453,7 @@
         </is>
       </c>
       <c r="I25" s="0"/>
+      <c r="J25" s="0"/>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
@@ -3418,6 +3497,7 @@
         </is>
       </c>
       <c r="I26" s="0"/>
+      <c r="J26" s="0"/>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
@@ -3461,6 +3541,7 @@
         </is>
       </c>
       <c r="I27" s="0"/>
+      <c r="J27" s="0"/>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
@@ -3504,6 +3585,7 @@
         </is>
       </c>
       <c r="I28" s="0"/>
+      <c r="J28" s="0"/>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
@@ -3547,6 +3629,7 @@
         </is>
       </c>
       <c r="I29" s="0"/>
+      <c r="J29" s="0"/>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
@@ -3590,6 +3673,7 @@
         </is>
       </c>
       <c r="I30" s="0"/>
+      <c r="J30" s="0"/>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
@@ -3633,6 +3717,7 @@
         </is>
       </c>
       <c r="I31" s="0"/>
+      <c r="J31" s="0"/>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
@@ -3676,6 +3761,7 @@
         </is>
       </c>
       <c r="I32" s="0"/>
+      <c r="J32" s="0"/>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
@@ -3719,6 +3805,7 @@
         </is>
       </c>
       <c r="I33" s="0"/>
+      <c r="J33" s="0"/>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
@@ -3762,6 +3849,7 @@
         </is>
       </c>
       <c r="I34" s="0"/>
+      <c r="J34" s="0"/>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
@@ -3805,6 +3893,7 @@
         </is>
       </c>
       <c r="I35" s="0"/>
+      <c r="J35" s="0"/>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
@@ -3848,6 +3937,7 @@
         </is>
       </c>
       <c r="I36" s="0"/>
+      <c r="J36" s="0"/>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
@@ -3891,6 +3981,7 @@
         </is>
       </c>
       <c r="I37" s="0"/>
+      <c r="J37" s="0"/>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
@@ -3934,6 +4025,7 @@
         </is>
       </c>
       <c r="I38" s="0"/>
+      <c r="J38" s="0"/>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
@@ -3977,6 +4069,7 @@
         </is>
       </c>
       <c r="I39" s="0"/>
+      <c r="J39" s="0"/>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
@@ -4020,6 +4113,7 @@
         </is>
       </c>
       <c r="I40" s="0"/>
+      <c r="J40" s="0"/>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
@@ -4063,6 +4157,7 @@
         </is>
       </c>
       <c r="I41" s="0"/>
+      <c r="J41" s="0"/>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
@@ -4106,6 +4201,7 @@
         </is>
       </c>
       <c r="I42" s="0"/>
+      <c r="J42" s="0"/>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
@@ -4149,6 +4245,7 @@
         </is>
       </c>
       <c r="I43" s="0"/>
+      <c r="J43" s="0"/>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
@@ -4188,10 +4285,11 @@
       </c>
       <c r="H44" s="0" t="inlineStr">
         <is>
-          <t>读取 `.local-agent/memory/*.md`，以 advisory block 注入 system prompt，带 source path 和预算</t>
+          <t>读取项目 `.local-agent/memory/*.md` 和 state dir `memory/*.md`，以 advisory block 注入 system prompt，带 source path 和预算</t>
         </is>
       </c>
       <c r="I44" s="0"/>
+      <c r="J44" s="0"/>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
@@ -4235,6 +4333,7 @@
         </is>
       </c>
       <c r="I45" s="0"/>
+      <c r="J45" s="0"/>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
@@ -4278,6 +4377,7 @@
         </is>
       </c>
       <c r="I46" s="0"/>
+      <c r="J46" s="0"/>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
@@ -4321,6 +4421,7 @@
         </is>
       </c>
       <c r="I47" s="0"/>
+      <c r="J47" s="0"/>
     </row>
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
@@ -4364,6 +4465,7 @@
         </is>
       </c>
       <c r="I48" s="0"/>
+      <c r="J48" s="0"/>
     </row>
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
@@ -4407,6 +4509,7 @@
         </is>
       </c>
       <c r="I49" s="0"/>
+      <c r="J49" s="0"/>
     </row>
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
@@ -4450,6 +4553,7 @@
         </is>
       </c>
       <c r="I50" s="0"/>
+      <c r="J50" s="0"/>
     </row>
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
@@ -4493,6 +4597,7 @@
         </is>
       </c>
       <c r="I51" s="0"/>
+      <c r="J51" s="0"/>
     </row>
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
@@ -4536,6 +4641,7 @@
         </is>
       </c>
       <c r="I52" s="0"/>
+      <c r="J52" s="0"/>
     </row>
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
@@ -4579,6 +4685,7 @@
         </is>
       </c>
       <c r="I53" s="0"/>
+      <c r="J53" s="0"/>
     </row>
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
@@ -4622,6 +4729,7 @@
         </is>
       </c>
       <c r="I54" s="0"/>
+      <c r="J54" s="0"/>
     </row>
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
@@ -4665,6 +4773,7 @@
         </is>
       </c>
       <c r="I55" s="0"/>
+      <c r="J55" s="0"/>
     </row>
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
@@ -4708,6 +4817,7 @@
         </is>
       </c>
       <c r="I56" s="0"/>
+      <c r="J56" s="0"/>
     </row>
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
@@ -4742,7 +4852,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>把 session 中的可复用经验定期整理进 `.local-agent/memory`，减少后续重复交代</t>
+          <t>把 session 中的可复用经验定期整理进长期 memory，减少后续重复交代，同时避免默认写项目文件</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -4752,13 +4862,62 @@
       </c>
       <c r="I57" s="0" t="inlineStr">
         <is>
-          <t>llm` 已支持；默认 off，坏 JSON/空结果/deadline 耗尽/本轮已显式写 memory 时不写；测试覆盖成功写入、坏 JSON 不写、默认 off 不额外调用 LLM/不写 memory</t>
-        </is>
-      </c>
+          <t>llm` 和 `--memory-scope state</t>
+        </is>
+      </c>
+      <c r="J57" s="0" t="inlineStr">
+        <is>
+          <t>project` 已支持；默认 off，开启后默认写 state dir，显式 project 才写 `.local-agent/memory`；测试覆盖默认 state、显式 project、坏 JSON 不写、默认 off 不额外调用 LLM/不写 memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>T-056</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>重复工具后强制最终回答 steering</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F58" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G58" s="0" t="inlineStr">
+        <is>
+          <t>用户本机企业压测已证明“重复工具硬停”仍会让真实需求分析没有最终答案</t>
+        </is>
+      </c>
+      <c r="H58" s="0" t="inlineStr">
+        <is>
+          <t>重复同参工具超过阈值后，runtime 追加 steering 并让下一次 LLM 请求 `tools=[]`；回归测试确认模型会返回 `final answer from collected evidence`</t>
+        </is>
+      </c>
+      <c r="I58" s="0"/>
+      <c r="J58" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -4770,7 +4929,7 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="45" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
@@ -5335,12 +5494,12 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>已补最近窗口同名同参工具调用熔断、`ToolResult.useless`、空结果标记、provider-bound useless/superseded pruning 和 open todo runtime reminder；等待用户本机真实联网压测输出后再决定是否引入 OMP 风格 ToolChoiceQueue / soft tool requirement</t>
+          <t>已补最近窗口同名同参工具调用熔断、`ToolResult.useless`、空结果标记、provider-bound useless/superseded pruning、open todo runtime reminder，以及 duplicate-tool forced-final steering；下一步用户本机复跑企业压测验证</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>OMP 不靠主步数限制日常任务，而靠 deadline/abort、synthetic tool result、soft tool escalation 小上限、todo/tool-choice steering 和 compaction pruning 共同收敛；我们已落地本地轻量 pruning/steering。</t>
+          <t>OMP 不靠主步数限制日常任务，而靠 deadline/abort、synthetic tool result、soft tool escalation 小上限、todo/tool-choice steering 和 compaction pruning 共同收敛；我们已落地本地轻量 pruning/steering，并在重复工具后强制下一轮无工具最终回答。</t>
         </is>
       </c>
     </row>
@@ -5515,17 +5674,17 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>已缓解，持续关注</t>
+          <t>已进一步缓解，持续关注</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>默认 off；显式开启才写；只接受严格 JSON 的短条目；坏 JSON、空结果、deadline 耗尽、本轮已显式写 memory 时不写</t>
+          <t>默认 off；显式开启后默认写用户级 state dir 的 memory，只有 `memory_scope=project` 才写项目 `.local-agent/memory`；只接受严格 JSON 的短条目；坏 JSON、空结果、deadline 耗尽、本轮已显式写 memory 时不写</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>OMP/Claude Code 的自动记忆也是启发式上下文，不是事实源硬约束。我们先做显式开启的本地 Markdown MVP，后续再评估 path-scoped rules 和 managed skills。</t>
+          <t>OMP local memory 位于用户 agent dir，项目 `.omp/` 主要承载人工 context/rules/skills；我们按同一边界把自动 consolidation 默认放入 state dir，项目 memory 仍需显式写入。</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6261,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -6112,7 +6271,7 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>这一步会写项目 `.local-agent/memory`，不同于只发给模型的 context compaction；默认 off 可以保护只读分析和企业项目零业务落盘</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
@@ -6130,7 +6289,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6202,7 +6361,7 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>LCA 自身只读压测中重复 `search_code` / `todo_read`，最终由 `budget_seconds=240` 截断；修复后 session `20260708T025519414693Z` 按要求收尾。</t>
+          <t>LCA 自身只读压测中重复 `search_code` / `todo_read`，最终由 `budget_seconds=240` 截断；修复后 session `20260708T025519414693Z` 按要求收尾。用户本机企业压测 session `20260708T062614211387Z` 又在 `feePlan` 搜索上重复，触发重复工具硬停且没有最终分析。</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
@@ -6212,7 +6371,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已实现最近窗口重复工具调用熔断，并补 `ToolResult.useless`、空搜索/LSP 结果 useless 标记、provider-bound useless/superseded pruning、open todo runtime reminder。</t>
+          <t>已实现最近窗口重复工具调用熔断、`ToolResult.useless`、空搜索/LSP useless 标记、provider-bound pruning、open todo reminder；并新增 duplicate-tool forced-final steering，重复工具后下一轮不给工具 schema，强制模型基于已有证据回答。</t>
         </is>
       </c>
     </row>
@@ -6340,7 +6499,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>已补重复工具熔断、provider-bound useless/superseded pruning 和 open todo runtime reminder；当前不因宿主外发阻断引入 ToolChoiceQueue，等待用户本机真实联网压测结果。</t>
+          <t>已补重复工具熔断、provider-bound useless/superseded pruning、open todo runtime reminder 和 duplicate-tool forced-final steering；当前先不上完整 ToolChoiceQueue，等同一企业命令复跑后再判断。</t>
         </is>
       </c>
     </row>
@@ -6463,12 +6622,44 @@
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>OMP/Claude Code 的自动记忆是启发式长期上下文，必须与普通 context compaction 区分；默认策略要避免只读任务隐式写项目文件。</t>
+          <t>OMP/Claude Code 的自动记忆是启发式长期上下文，必须与普通 context compaction 区分；OMP local memory 位于用户 agent dir，默认策略要避免只读任务隐式写项目文件。</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>默认 `off`；只读压测命令显式 `--memory-consolidation off`；新增 runtime 默认 off 回归测试，确认不会额外调用 LLM 或写 `.local-agent/memory`。</t>
+          <t>默认 `off`；开启后默认 `--memory-scope state` 写 state dir；只有显式 `project` 才写 `.local-agent/memory`；新增 runtime 回归测试覆盖默认 off、默认 state 写入、显式 project 写入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>PT-010</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 修复，待用户复跑</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>企业需求只读压测中，模型围绕 `feePlan` 在相近目录重复 `search_code`，最终硬停且无最终需求落点分析。</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>OMP 把重复/软强制工具看作 runtime steering 问题：小上限后切回回答或换策略，而不是无限工具探索。</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>已新增 duplicate-tool forced-final steering；下一步用户用 session `20260708T062614211387Z` 的同一命令复跑，验证是否能输出结构化分析。</t>
         </is>
       </c>
     </row>
@@ -6544,7 +6735,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 136 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 140 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -6943,7 +7134,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`；需要自动整理时开启 `--memory-consolidation auto`</t>
+          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`；需要自动整理时开启 `--memory-consolidation auto`，默认写 state memory，团队共享才加 `--memory-scope project`</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -6958,7 +7149,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>memory 是 advisory，当前用户指令优先；默认不隐式写</t>
+          <t>memory 是 advisory，当前用户指令优先；默认不隐式写项目文件</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expose allowed roots to the model
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` 证明硬停改善，但暴露 allowed-dir 具体路径未告知模型，已补 workspace roots 注入。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -449,7 +449,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；system prompt 会列出 primary workspace 和 allowed dirs；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
         </is>
       </c>
       <c r="D20" s="0"/>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停。已补 OMP 风格轻量 forced-final steering；下一步用户复跑同一命令验证是否能产出最终分析，再决定是否引入完整 ToolChoiceQueue / soft tool requirement、path-scoped rules 或精确 token 预算。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir workspace roots 注入；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
+          <t>支持需求文档目录 + 代码项目目录；system prompt 会列出 allowed dirs，文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -2369,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J60"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4915,6 +4915,94 @@
       <c r="I58" s="0"/>
       <c r="J58" s="0"/>
     </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>T-057</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>allowed-dir workspace roots 注入</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T065705459243Z` 暴露模型不知道 `--allow-dir` 具体路径，误猜 `requirements` 目录</t>
+        </is>
+      </c>
+      <c r="H59" s="0" t="inlineStr">
+        <is>
+          <t>system prompt/provider-bound context 增加 `[Workspace roots]`，列出 primary `--cwd` 和 allowed dirs；file tool descriptions 同步说明 allowed directory；测试覆盖不重复注入</t>
+        </is>
+      </c>
+      <c r="I59" s="0"/>
+      <c r="J59" s="0"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t>T-058</t>
+        </is>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>跨项目需求覆盖边界记录</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>已完成记录</t>
+        </is>
+      </c>
+      <c r="F60" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G60" s="0" t="inlineStr">
+        <is>
+          <t>用户确认当前测试项目可能无法完全覆盖需求，尤其结算需求可能需要其他项目协同</t>
+        </is>
+      </c>
+      <c r="H60" s="0" t="inlineStr">
+        <is>
+          <t>压测记录已说明单仓库只能输出候选前置能力和缺口；后续把相关项目也作为 `--allow-dir`，或让 Agent 先列“需要补充的项目清单”</t>
+        </is>
+      </c>
+      <c r="I60" s="0"/>
+      <c r="J60" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -4924,7 +5012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G40"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5691,74 +5779,74 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-020</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>multi-root allowed dir 没有显式进入模型上下文</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>session `20260708T065705459243Z` 中模型不知道需求目录绝对路径，尝试 `requirements` 并失败，导致未读需求文档就反推代码</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 会显式提供 cwd/project context/rules；我们新增 `[Workspace roots]`，把 primary `--cwd` 和 allowed dirs 写入启动 system prompt 与 provider-bound context。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-021</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>单仓库无法覆盖跨服务需求</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已记录，持续关注</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>用户确认当前测试项目可能不覆盖完整需求；`拓展服务费结算` 可能在 incentive/settlement 等其他项目</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 依赖用户提供完整 workspace/context；我们记录为压测边界，后续用多个 `--allow-dir` 接入相关项目，或者要求 Agent 明确输出“还需要哪个项目”。</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5858,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -5780,22 +5868,22 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5895,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -5817,22 +5905,22 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5932,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -5854,22 +5942,22 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -5881,7 +5969,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -5891,7 +5979,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -5901,12 +5989,12 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -5918,7 +6006,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -5928,7 +6016,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -5938,12 +6026,12 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -5955,7 +6043,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -5965,7 +6053,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -5975,12 +6063,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -5992,7 +6080,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -6002,7 +6090,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -6012,12 +6100,12 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6117,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -6039,22 +6127,22 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6154,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6076,22 +6164,22 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6191,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6113,7 +6201,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
@@ -6123,12 +6211,12 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6228,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6150,22 +6238,22 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -6177,32 +6265,32 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -6214,32 +6302,32 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -6251,32 +6339,143 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>ADR-015</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+        </is>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
           <t>ADR-016</t>
         </is>
       </c>
-      <c r="C37" s="0" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D37" s="0" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
-      <c r="E37" s="0" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F37" s="0" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
         <is>
           <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
-      <c r="G37" s="0" t="inlineStr">
+      <c r="G39" s="0" t="inlineStr">
         <is>
           <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>ADR-017</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+        </is>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -6289,7 +6488,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6660,6 +6859,70 @@
       <c r="F12" s="0" t="inlineStr">
         <is>
           <t>已新增 duplicate-tool forced-final steering；下一步用户用 session `20260708T062614211387Z` 的同一命令复跑，验证是否能输出结构化分析。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>PT-011</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>已关闭 MVP 版，待用户复跑验证</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>`--allow-dir` 具体路径没有进入模型上下文，模型猜 `requirements` 目录失败后没有读取真实需求文档。</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会把 cwd/project context 和工具可用范围显式放进运行上下文。</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>已补 `[Workspace roots]` 注入和 file tool 描述；下一次同命令应先 list/read allowed-dir 绝对路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>PT-012</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>已记录</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>用户确认当前测试项目可能无法完全覆盖需求，结算需求可能需要其他项目配合。</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>OMP 需要完整 workspace/context 才能做跨项目判断；证据缺失时应输出不确定点和需要补充的项目。</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>后续压测把相关项目也作为 `--allow-dir`，或让 Agent 先列出需要补充的项目/服务。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Surface allowed roots in tool observations
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` 证明硬停改善，但暴露 allowed-dir 具体路径未告知模型，已补 workspace roots 注入。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` / `20260708T070722601499Z` 证明硬停改善，但仍未读取 allowed-dir 需求文档，已补 workspace roots 工具观察提示。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -449,7 +449,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；system prompt 会列出 primary workspace 和 allowed dirs；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；system prompt 和 `list_files`/path-not-found 等工具观察会列出 primary workspace 和 allowed dirs；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
         </is>
       </c>
       <c r="D20" s="0"/>
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir workspace roots 注入；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` / `20260708T070722601499Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir roots 的 system prompt 与工具观察双层提示；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；system prompt 会列出 allowed dirs，文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
+          <t>支持需求文档目录 + 代码项目目录；system prompt 和工具观察会列出 allowed dirs，文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成第二版，待复跑</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
@@ -4948,12 +4948,12 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T065705459243Z` 暴露模型不知道 `--allow-dir` 具体路径，误猜 `requirements` 目录</t>
+          <t>session `20260708T065705459243Z` / `20260708T070722601499Z` 暴露模型仍会误猜 `requirements`，仅 system prompt 注入 roots 不够</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
         <is>
-          <t>system prompt/provider-bound context 增加 `[Workspace roots]`，列出 primary `--cwd` 和 allowed dirs；file tool descriptions 同步说明 allowed directory；测试覆盖不重复注入</t>
+          <t>system prompt/provider-bound context 增加 `[Workspace roots]`；`list_files {}` 根目录输出、path-not-found 和带 allowed-dir 的空搜索会提示 exact allowed dirs；file tool descriptions 同步说明 allowed directory；测试覆盖不重复注入和工具观察提示</t>
         </is>
       </c>
       <c r="I59" s="0"/>
@@ -5794,22 +5794,22 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>multi-root allowed dir 没有显式进入模型上下文</t>
+          <t>multi-root allowed dir 没有稳定进入模型操作路径</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已补第二版，待复跑</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T065705459243Z` 中模型不知道需求目录绝对路径，尝试 `requirements` 并失败，导致未读需求文档就反推代码</t>
+          <t>session `20260708T065705459243Z` 和 `20260708T070722601499Z` 中模型都尝试 `requirements` 并失败，导致未读需求文档就反推代码</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 会显式提供 cwd/project context/rules；我们新增 `[Workspace roots]`，把 primary `--cwd` 和 allowed dirs 写入启动 system prompt 与 provider-bound context。</t>
+          <t>OMP 会显式提供 cwd/project context/rules，并通过运行时上下文/工具观察持续影响模型；我们新增 `[Workspace roots]`，并让 `list_files` 根目录输出、path-not-found 和带 allowed-dir 的空搜索都提示 exact allowed dirs。</t>
         </is>
       </c>
     </row>
@@ -6875,22 +6875,22 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版，待用户复跑验证</t>
+          <t>已补第二版，待用户复跑验证</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` 具体路径没有进入模型上下文，模型猜 `requirements` 目录失败后没有读取真实需求文档。</t>
+          <t>`--allow-dir` 具体路径没有稳定进入模型操作路径，模型猜 `requirements` 目录失败后没有读取真实需求文档。</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>OMP 会把 cwd/project context 和工具可用范围显式放进运行上下文。</t>
+          <t>OMP 会把 cwd/project context 和工具可用范围显式放进运行上下文，并通过工具观察持续纠偏。</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已补 `[Workspace roots]` 注入和 file tool 描述；下一次同命令应先 list/read allowed-dir 绝对路径。</t>
+          <t>已补 `[Workspace roots]` 注入、file tool 描述、`list_files` 根目录 roots 输出、path-not-found roots 提示和带 allowed-dir 的空搜索提示；下一次同命令应先 list/read allowed-dir 绝对路径。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Require allowed-dir docs before code search
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` / `20260708T070722601499Z` 证明硬停改善，但仍未读取 allowed-dir 需求文档，已补 workspace roots 工具观察提示。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` / `20260708T070722601499Z` / `20260708T072404789287Z` 证明硬停改善，但仍未读取 allowed-dir 需求文档，已补 OMP 风格 allowed-dir soft tool requirement。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -449,7 +449,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；system prompt 和 `list_files`/path-not-found 等工具观察会列出 primary workspace 和 allowed dirs；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
+          <t>`--allow-dir` / `AGENT_ALLOWED_DIRS` 支持显式授权额外目录给文件、搜索、LSP、patch 工具；system prompt 和 `list_files`/path-not-found 等工具观察会列出 primary workspace 和 allowed dirs；需求/文档类任务会先用 soft tool requirement 要求读取 allowed-dir 文档；shell/git/显式项目 memory/skills 仍锚定 `--cwd`，session/todo/patch logs 和默认 consolidation memory 走 state dir。</t>
         </is>
       </c>
       <c r="D20" s="0"/>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` / `20260708T070722601499Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir roots 的 system prompt 与工具观察双层提示；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` / `20260708T070722601499Z` / `20260708T072404789287Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir soft tool requirement；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>支持需求文档目录 + 代码项目目录；system prompt 和工具观察会列出 allowed dirs，文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
+          <t>支持需求文档目录 + 代码项目目录；system prompt 和工具观察会列出 allowed dirs；需求/文档类任务先 soft-require `read_file` allowed-dir 文档；文件/search/LSP/patch 可访问 allowed dirs，shell/git/显式项目 memory/skills 仍锚定 `--cwd`，默认 consolidation memory 走 state dir</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已完成第二版，待复跑</t>
+          <t>已完成第三版，待复跑</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
@@ -4948,12 +4948,12 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T065705459243Z` / `20260708T070722601499Z` 暴露模型仍会误猜 `requirements`，仅 system prompt 注入 roots 不够</t>
+          <t>session `20260708T065705459243Z` / `20260708T070722601499Z` / `20260708T072404789287Z` 暴露模型仍不稳定读取 allowed-dir 需求文档，仅提示和工具观察不够</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
         <is>
-          <t>system prompt/provider-bound context 增加 `[Workspace roots]`；`list_files {}` 根目录输出、path-not-found 和带 allowed-dir 的空搜索会提示 exact allowed dirs；file tool descriptions 同步说明 allowed directory；测试覆盖不重复注入和工具观察提示</t>
+          <t>system prompt/provider-bound context 增加 `[Workspace roots]`；`list_files {}` 根目录输出、path-not-found 和带 allowed-dir 的空搜索会提示 exact allowed dirs；需求/文档类任务创建 soft tool requirement，满足前只暴露 `list_files` / `read_file` 并要求读 allowed-dir 文档；测试覆盖不重复注入、工具观察提示和 soft requirement</t>
         </is>
       </c>
       <c r="I59" s="0"/>
@@ -5799,17 +5799,17 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已补第二版，待复跑</t>
+          <t>已补第三版，待复跑</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T065705459243Z` 和 `20260708T070722601499Z` 中模型都尝试 `requirements` 并失败，导致未读需求文档就反推代码</t>
+          <t>session `20260708T065705459243Z` 和 `20260708T070722601499Z` 中模型尝试 `requirements` 并失败；session `20260708T072404789287Z` 已看到 roots 提示但仍未读需求文档，导致代码侧反推</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 会显式提供 cwd/project context/rules，并通过运行时上下文/工具观察持续影响模型；我们新增 `[Workspace roots]`，并让 `list_files` 根目录输出、path-not-found 和带 allowed-dir 的空搜索都提示 exact allowed dirs。</t>
+          <t>OMP 会显式提供 cwd/project context/rules，并通过 ToolChoiceQueue / soft tool requirement 做小上限纠偏；我们新增 `[Workspace roots]`、工具观察 roots 提示，并对需求/文档类任务前置 soft tool requirement。</t>
         </is>
       </c>
     </row>
@@ -6875,22 +6875,22 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>已补第二版，待用户复跑验证</t>
+          <t>已补第三版，待用户复跑验证</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>`--allow-dir` 具体路径没有稳定进入模型操作路径，模型猜 `requirements` 目录失败后没有读取真实需求文档。</t>
+          <t>`--allow-dir` 具体路径进入了提示和工具观察，但模型仍未稳定 `read_file` 真实需求文档。</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>OMP 会把 cwd/project context 和工具可用范围显式放进运行上下文，并通过工具观察持续纠偏。</t>
+          <t>OMP 会把 cwd/project context 放进运行上下文，并用 ToolChoiceQueue / soft tool requirement 在模型偏航时限制工具和持续纠偏。</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已补 `[Workspace roots]` 注入、file tool 描述、`list_files` 根目录 roots 输出、path-not-found roots 提示和带 allowed-dir 的空搜索提示；下一次同命令应先 list/read allowed-dir 绝对路径。</t>
+          <t>已补 allowed-dir soft tool requirement：任务明确提到需求/文档且有 allowed dirs 时，满足前只暴露 `list_files` / `read_file`，要求先 `read_file` allowed-dir 下候选需求文档；下一次同命令应先读需求文档再搜索主代码库。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Steer repeated file reads to final answer
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T062614211387Z` 暴露 `feePlan` 重复搜索无最终回答，已补 duplicate-tool forced-final steering；session `20260708T065705459243Z` / `20260708T070722601499Z` / `20260708T072404789287Z` 证明硬停改善，但仍未读取 allowed-dir 需求文档，已补 OMP 风格 allowed-dir soft tool requirement。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T073252231781Z` 已验证 allowed-dir 需求文档前置读取成功，但暴露同文件连续切片读取漂移，已补 repeated read_file final-answer steering。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T062614211387Z` 证明真实百炼链路可读企业项目，但在 `feePlan` 重复搜索后硬停；session `20260708T065705459243Z` / `20260708T070722601499Z` / `20260708T072404789287Z` 已能最终回答，但没读真实需求目录。已补 allowed-dir soft tool requirement；下一步用户复跑同一命令，验证是否先读取需求文档，并按需把其他相关项目加入 `--allow-dir`。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T073252231781Z` 已先读真实需求 md，但后半段连续读取同一个大文件并偏离最终 5 点输出。已补 repeated read_file final-answer steering；下一步用户复跑同一命令，验证是否能先读需求、再搜索代码、最后按 5 点输出收束。</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J61"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5003,6 +5003,50 @@
       <c r="I60" s="0"/>
       <c r="J60" s="0"/>
     </row>
+    <row r="61">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t>T-059</t>
+        </is>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>同文件连续切片读取漂移 guard</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>已完成，待复跑</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T073252231781Z` 已读需求文档，但后半段连续读取 `HandleCrclServiceApplication.java` 大量相邻范围，最终回答偏离用户要求</t>
+        </is>
+      </c>
+      <c r="H61" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP 病态子循环小上限：只读/分析类任务中，近期同一路径 `read_file` 超阈值后返回 tool error，并注入 final-answer steering；下一轮 `tools=[]`，要求回到原始输出结构；编辑类任务不触发</t>
+        </is>
+      </c>
+      <c r="I61" s="0"/>
+      <c r="J61" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5012,7 +5056,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5853,37 +5897,37 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-022</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>同文件连续切片读取导致任务漂移</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已补 MVP 版，待复跑</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间，最后只总结该文件导出逻辑，没有按原始企业需求分析结构输出</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline 收束；我们新增只读/分析任务的 repeated read_file guard，触发后强制下一轮无工具最终回答；编辑类任务不触发。</t>
         </is>
       </c>
     </row>
@@ -5895,7 +5939,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -5905,22 +5949,22 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5976,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -5942,7 +5986,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -5952,12 +5996,12 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -5969,7 +6013,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -5979,22 +6023,22 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6050,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -6016,7 +6060,7 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -6026,12 +6070,12 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6043,7 +6087,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -6053,7 +6097,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -6063,12 +6107,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6124,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -6090,7 +6134,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -6100,12 +6144,12 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6161,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -6127,7 +6171,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -6137,12 +6181,12 @@
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6154,7 +6198,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6164,7 +6208,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -6174,12 +6218,12 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6235,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6201,22 +6245,22 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -6228,7 +6272,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6238,7 +6282,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -6248,12 +6292,12 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -6265,7 +6309,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6275,7 +6319,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -6285,12 +6329,12 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6346,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6312,22 +6356,22 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -6339,32 +6383,32 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6420,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -6386,22 +6430,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6457,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -6423,7 +6467,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -6433,12 +6477,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -6450,30 +6494,67 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+        </is>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
           <t>ADR-017</t>
         </is>
       </c>
-      <c r="C40" s="0" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D40" s="0" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
-      <c r="E40" s="0" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F40" s="0" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
-      <c r="G40" s="0" t="inlineStr">
+      <c r="G41" s="0" t="inlineStr">
         <is>
           <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
@@ -6488,7 +6569,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6923,6 +7004,38 @@
       <c r="F14" s="0" t="inlineStr">
         <is>
           <t>后续压测把相关项目也作为 `--allow-dir`，或让 Agent 先列出需要补充的项目/服务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>PT-013</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>已补 MVP 版，待用户复跑验证</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>allowed-dir 需求文档已前置读取，但模型后续连续读取同一个大文件相邻区间，最终偏离原始 5 点输出。</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>OMP 对病态工具子循环用小上限和 runtime steering 收束，不靠主步数。</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>已补同文件切片读取漂移 guard；下一次同命令应在证据足够后按 5 点要求输出，而不是继续读同一文件。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten read-only drift steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T073252231781Z` 已验证 allowed-dir 需求文档前置读取成功，但暴露同文件连续切片读取漂移，已补 repeated read_file final-answer steering。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T074609696125Z` 已验证 allowed-dir 需求文档前置读取持续生效，但暴露“只读压测 + 下一步实现”误关同文件读取 guard 以及最终回答遗忘已读文档，已补显式只读优先和 forced-final 已读文件证据摘要。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T073252231781Z` 已先读真实需求 md，但后半段连续读取同一个大文件并偏离最终 5 点输出。已补 repeated read_file final-answer steering；下一步用户复跑同一命令，验证是否能先读需求、再搜索代码、最后按 5 点输出收束。</t>
+          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T074609696125Z` 已持续先读真实需求 md，但“只读压测 + 下一步实现”误关 read-file drift guard，最终回答还错误声称 V1.1 未读。已补显式只读优先和 forced-final 已读文件证据摘要；下一步用户复跑同一命令，验证是否能先读需求、再搜索代码、最后按 5 点输出收束。</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>当前 140 个测试通过</t>
+          <t>当前 147 个测试通过</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -2369,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已完成，待复跑</t>
+          <t>已完成第二版，待复跑</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
@@ -5036,16 +5036,60 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T073252231781Z` 已读需求文档，但后半段连续读取 `HandleCrclServiceApplication.java` 大量相邻范围，最终回答偏离用户要求</t>
+          <t>session `20260708T073252231781Z` 已读需求文档但连续读大文件漂移；session `20260708T074609696125Z` 又暴露“只读压测 + 下一步实现”误关 guard</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 病态子循环小上限：只读/分析类任务中，近期同一路径 `read_file` 超阈值后返回 tool error，并注入 final-answer steering；下一轮 `tools=[]`，要求回到原始输出结构；编辑类任务不触发</t>
+          <t>参考 OMP 病态子循环小上限：显式只读/不要修改文件/不要写文件优先于编辑词；只读/分析任务中近期同一路径 `read_file` 超阈值后返回 tool error，并注入 final-answer steering；下一轮 `tools=[]`</t>
         </is>
       </c>
       <c r="I61" s="0"/>
       <c r="J61" s="0"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="inlineStr">
+        <is>
+          <t>T-060</t>
+        </is>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="inlineStr">
+        <is>
+          <t>forced-final 已读文件证据摘要</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>已完成，待复跑</t>
+        </is>
+      </c>
+      <c r="F62" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T074609696125Z` 明明已读 V1.1 需求文档，最终回答却称未读</t>
+        </is>
+      </c>
+      <c r="H62" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime context/steering：重复工具 forced-final 消息会列出本轮已成功 `read_file` 的路径，要求模型不要声称这些文件未读，并回到用户原始输出结构</t>
+        </is>
+      </c>
+      <c r="I62" s="0"/>
+      <c r="J62" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5917,17 +5961,17 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已补 MVP 版，待复跑</t>
+          <t>已补第二版，待复跑</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间，最后只总结该文件导出逻辑，没有按原始企业需求分析结构输出</t>
+          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间；session `20260708T074609696125Z` 中显式只读任务因“下一步实现”措辞误关 guard，最终还遗忘已读需求文档</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline 收束；我们新增只读/分析任务的 repeated read_file guard，触发后强制下一轮无工具最终回答；编辑类任务不触发。</t>
+          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline/runtime context 收束；我们新增显式只读优先级、repeated read_file guard 和 forced-final 已读文件证据摘要，触发后强制下一轮无工具最终回答。</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6613,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7036,6 +7080,38 @@
       <c r="F15" s="0" t="inlineStr">
         <is>
           <t>已补同文件切片读取漂移 guard；下一次同命令应在证据足够后按 5 点要求输出，而不是继续读同一文件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>PT-014</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>已补第二版，待用户复跑验证</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T074609696125Z` 已先读两份需求 md，但 prompt 中“如果下一步要实现”误触编辑词排除，导致只读 drift guard 未开启；最终回答还错误声称 V1.1 未读。</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将当前用户硬约束和 runtime state 持续放入上下文，并用 steering/tool-choice 小上限让模型回到原始任务；显式 readonly/permission 语义不应被后续普通业务词覆盖。</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t>已改为显式只读/不要修改文件/不要写文件优先于编辑词；重复工具 forced-final steering 会列出本轮已读文件，要求模型不要声称这些文件未读；新增回归测试覆盖该 prompt 形态。</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7187,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 140 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 147 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record enterprise run and strengthen final steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；用户本机企业压测 session `20260708T074609696125Z` 已验证 allowed-dir 需求文档前置读取持续生效，但暴露“只读压测 + 下一步实现”误关同文件读取 guard 以及最终回答遗忘已读文档，已补显式只读优先和 forced-final 已读文件证据摘要。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 代跑企业压测 session `20260708T081827983347Z`，已验证 allowed-dir 需求文档前置读取和 repeated read-file guard 生效，但暴露 forced-final 后仍可能把已读文件说成未读，已补原始请求摘要和已读文件一致性规则。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>企业项目联网压测已获用户允许，Codex 宿主不能代跑；用户本机 session `20260708T074609696125Z` 已持续先读真实需求 md，但“只读压测 + 下一步实现”误关 read-file drift guard，最终回答还错误声称 V1.1 未读。已补显式只读优先和 forced-final 已读文件证据摘要；下一步用户复跑同一命令，验证是否能先读需求、再搜索代码、最后按 5 点输出收束。</t>
+          <t>full-access 后 Agent 已代跑企业项目联网压测 session `20260708T081827983347Z`：先读真实需求 md，读文件漂移 guard 成功触发并收束；但最终回答仍把已读 `QueryFeePlanInfoReq.java` 写成未读。已补 forced-final 原始请求摘要和已读文件一致性规则；下一步复跑同一命令，验证最终 5 点结构和证据一致性。</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J63"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>用户已确认，当前 Codex 环境阻断代跑</t>
+          <t>用户已确认，full-access 已代跑</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="H50" s="0" t="inlineStr">
         <is>
-          <t>LCA 产品设计不内置禁止外发；按 OMP 思路由用户、provider、permission 和运行环境策略决定。本次 Codex 环境无法代跑，已改成本地只读扫描。</t>
+          <t>LCA 产品设计不内置禁止外发；按 OMP 思路由用户、provider、permission 和运行环境策略决定。早期受限 Codex 环境曾阻断代跑；切换 full-access + network enabled 后已由 Agent 代跑 session `20260708T081827983347Z`。</t>
         </is>
       </c>
       <c r="I50" s="0"/>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>当前 Codex 环境阻断，用户本机待跑</t>
+          <t>已由 Agent 代跑，继续复测收尾质量</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="H56" s="0" t="inlineStr">
         <is>
-          <t>memory consolidation 完成后已用 `--memory-consolidation off` 再次尝试；sandbox 因 DNS/网络失败，外部执行仍被 Codex 宿主策略拒绝。目标仓库未发现 `.local-agent`。用户在允许环境中运行后，把 session 输出回贴即可继续分析。</t>
+          <t>session `20260708T081827983347Z` 已跑通真实百炼链路；需求文档前置读取和 repeated read-file guard 通过，forced-final 后证据一致性仍需复测。目标仓库 runtime state 不应写入 `.local-agent`。</t>
         </is>
       </c>
       <c r="I56" s="0"/>
@@ -5090,6 +5090,50 @@
       </c>
       <c r="I62" s="0"/>
       <c r="J62" s="0"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t>T-061</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t>forced-final 原始请求和已读一致性约束</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t>已完成，待复跑</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T081827983347Z` 中 `QueryFeePlanInfoReq.java` 已读，但最终回答仍写成 not yet read，且未完全按用户 5 点结构输出</t>
+        </is>
+      </c>
+      <c r="H63" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime context/steering：forced-final 消息注入原始用户请求摘要，并明确已读文件不得称未读；如还需实现级深读，只能说明已读但缺少哪些细节</t>
+        </is>
+      </c>
+      <c r="I63" s="0"/>
+      <c r="J63" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5702,12 +5746,12 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>用户已确认，当前 Codex 环境阻断代跑</t>
+          <t>用户已确认，full-access 已代跑</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>用户已确认可外发给百炼；本次由 Codex 执行环境策略拒绝代跑联网压测，已改为本地只读扫描并记录结果</t>
+          <t>用户已确认可外发给百炼；早期受限 Codex 环境拒绝代跑，full-access + network enabled 后已由 Agent 代跑 session `20260708T081827983347Z`</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
@@ -5961,17 +6005,17 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已补第二版，待复跑</t>
+          <t>已补第三版，待复跑</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间；session `20260708T074609696125Z` 中显式只读任务因“下一步实现”措辞误关 guard，最终还遗忘已读需求文档</t>
+          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间；session `20260708T074609696125Z` 中显式只读任务因“下一步实现”措辞误关 guard；session `20260708T081827983347Z` 中 guard 成功收束，但最终仍把已读文件说成未读</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline/runtime context 收束；我们新增显式只读优先级、repeated read_file guard 和 forced-final 已读文件证据摘要，触发后强制下一轮无工具最终回答。</t>
+          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline/runtime context 收束；我们新增显式只读优先级、repeated read_file guard、forced-final 已读文件证据摘要、原始请求摘要和已读一致性规则，触发后强制下一轮无工具最终回答。</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6657,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6712,12 +6756,12 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>当前 Codex 环境阻断代跑，已改本地扫描</t>
+          <t>已澄清并通过 full-access 代跑</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>用户已确认可外发给百炼；本次 Codex 执行环境策略拒绝代跑把企业私有代码/需求发送到三方 API。</t>
+          <t>用户已确认可外发给百炼；早期 Codex 受限环境拒绝代跑企业私有代码/需求到三方 API，full-access + network enabled 后已由 Agent 代跑 session `20260708T081827983347Z`。</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
@@ -6727,7 +6771,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>不绕过当前执行环境策略；改成本地只读扫描，记录结构、关键词和候选落点。用户在自己的允许环境中运行 LCA 时，可按 provider/permission 策略执行联网只读分析。</t>
+          <t>LCA 不内置“企业数据不能外发”禁令；是否可跑由用户授权、provider、permission 和当前宿主环境共同决定。</t>
         </is>
       </c>
     </row>
@@ -6968,7 +7012,7 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 修复，待用户复跑</t>
+          <t>已由 full-access 复跑验证进一步缓解</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -6983,7 +7027,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>已新增 duplicate-tool forced-final steering；下一步用户用 session `20260708T062614211387Z` 的同一命令复跑，验证是否能输出结构化分析。</t>
+          <t>session `20260708T081827983347Z` 未再因 `feePlan` 重复搜索硬停，并输出最终回答；后续问题转为 forced-final 证据一致性。</t>
         </is>
       </c>
     </row>
@@ -7000,7 +7044,7 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>已补第三版，待用户复跑验证</t>
+          <t>已由 full-access 复跑验证通过</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -7015,7 +7059,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已补 allowed-dir soft tool requirement：任务明确提到需求/文档且有 allowed dirs 时，满足前只暴露 `list_files` / `read_file`，要求先 `read_file` allowed-dir 下候选需求文档；下一次同命令应先读需求文档再搜索主代码库。</t>
+          <t>session `20260708T081827983347Z` 前两步即读取两份 allowed-dir 需求 md，说明 soft requirement 已稳定生效。</t>
         </is>
       </c>
     </row>
@@ -7064,7 +7108,7 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>已补 MVP 版，待用户复跑验证</t>
+          <t>已由 full-access 复跑验证通过收束</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -7079,7 +7123,7 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>已补同文件切片读取漂移 guard；下一次同命令应在证据足够后按 5 点要求输出，而不是继续读同一文件。</t>
+          <t>session `20260708T081827983347Z` 再次连续读取 `HandleCrclServiceApplication.java`，repeated read-file guard 触发并成功 forced-final，没有卡死。</t>
         </is>
       </c>
     </row>
@@ -7096,7 +7140,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>已补第二版，待用户复跑验证</t>
+          <t>已由 full-access 复跑验证部分通过</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -7111,7 +7155,39 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>已改为显式只读/不要修改文件/不要写文件优先于编辑词；重复工具 forced-final steering 会列出本轮已读文件，要求模型不要声称这些文件未读；新增回归测试覆盖该 prompt 形态。</t>
+          <t>session `20260708T081827983347Z` 证明显式只读优先生效，guard 触发成功；但仍暴露 PT-015：forced-final 后可能把已读文件称未读。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>PT-015</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>已补第三版，待复跑验证</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T081827983347Z` 已由 Agent 在 full-access 环境代跑；allowed-dir 前置读和 repeated read-file guard 均生效，但最终回答仍把已读 `QueryFeePlanInfoReq.java` 写成 not yet read，且未完全按用户 5 点结构输出。</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将当前任务、runtime state、tool evidence 和 steering 一起放回上下文，并用 tool-choice/forced-final 明确模型下一步必须回答什么，而不是只提醒“不要继续读”。</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>forced-final steering 已注入原始用户请求摘要；已读文件列表后追加“不得声称未读，如仍需实现级深读，应说明已读但缺少哪些细节”；测试覆盖该 steering 内容。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guard repeated empty search patterns
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 代跑企业压测 session `20260708T081827983347Z`，已验证 allowed-dir 需求文档前置读取和 repeated read-file guard 生效，但暴露 forced-final 后仍可能把已读文件说成未读，已补原始请求摘要和已读文件一致性规则。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 代跑企业压测，最新 session `20260708T083312934017` 已验证 allowed-dir 需求文档前置读取、repeated read-file guard、空搜索词跨路径 guard 和 forced-final 收束生效，最终按 5 点结构输出。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑企业项目联网压测 session `20260708T081827983347Z`：先读真实需求 md，读文件漂移 guard 成功触发并收束；但最终回答仍把已读 `QueryFeePlanInfoReq.java` 写成未读。已补 forced-final 原始请求摘要和已读文件一致性规则；下一步复跑同一命令，验证最终 5 点结构和证据一致性。</t>
+          <t>full-access 后 Agent 已代跑企业项目联网压测；session `20260708T082703005777Z` 暴露同一空搜索词跨路径扩散，已补搜索词级 guard；session `20260708T083312934017` 已先读需求、搜索代码、触发 guard 后按 5 点结构收束。下一步从“运行稳定性”转向回答准确性/项目覆盖评估。</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>当前 147 个测试通过</t>
+          <t>当前 148 个测试通过</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -2369,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J64"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已由 Agent 代跑，继续复测收尾质量</t>
+          <t>已由 Agent 代跑并复跑收束</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="H56" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T081827983347Z` 已跑通真实百炼链路；需求文档前置读取和 repeated read-file guard 通过，forced-final 后证据一致性仍需复测。目标仓库 runtime state 不应写入 `.local-agent`。</t>
+          <t>session `20260708T083312934017` 已验证真实需求文档前置读取、代码搜索、guard 收束和 5 点结构输出；目标仓库未写入 `.local-agent`。下一步转向回答准确性和跨项目覆盖评估。</t>
         </is>
       </c>
       <c r="I56" s="0"/>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已完成第三版，待复跑</t>
+          <t>已完成并复跑通过</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="H59" s="0" t="inlineStr">
         <is>
-          <t>system prompt/provider-bound context 增加 `[Workspace roots]`；`list_files {}` 根目录输出、path-not-found 和带 allowed-dir 的空搜索会提示 exact allowed dirs；需求/文档类任务创建 soft tool requirement，满足前只暴露 `list_files` / `read_file` 并要求读 allowed-dir 文档；测试覆盖不重复注入、工具观察提示和 soft requirement</t>
+          <t>system prompt/provider-bound context 增加 `[Workspace roots]`；`list_files {}` 根目录输出、path-not-found 和带 allowed-dir 的空搜索会提示 exact allowed dirs；需求/文档类任务创建 soft tool requirement；session `20260708T083312934017` 已先读两份 allowed-dir 需求 md</t>
         </is>
       </c>
       <c r="I59" s="0"/>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已完成第二版，待复跑</t>
+          <t>已完成并复跑通过</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="H61" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 病态子循环小上限：显式只读/不要修改文件/不要写文件优先于编辑词；只读/分析任务中近期同一路径 `read_file` 超阈值后返回 tool error，并注入 final-answer steering；下一轮 `tools=[]`</t>
+          <t>参考 OMP 病态子循环小上限：显式只读/不要修改文件/不要写文件优先于编辑词；只读/分析任务中近期同一路径 `read_file` 超阈值后返回 tool error 并 forced-final；session `20260708T083312934017` 已验证触发后按 5 点结构输出</t>
         </is>
       </c>
       <c r="I61" s="0"/>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已完成，待复跑</t>
+          <t>已完成并复跑收束</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="H62" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime context/steering：重复工具 forced-final 消息会列出本轮已成功 `read_file` 的路径，要求模型不要声称这些文件未读，并回到用户原始输出结构</t>
+          <t>参考 OMP runtime context/steering：重复工具 forced-final 消息会列出本轮已成功 `read_file` 的路径，要求模型不要声称这些文件未读，并回到用户原始输出结构；最终由 T-061 一起收束</t>
         </is>
       </c>
       <c r="I62" s="0"/>
@@ -5114,7 +5114,7 @@
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已完成，待复跑</t>
+          <t>已完成并复跑通过</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
@@ -5129,11 +5129,55 @@
       </c>
       <c r="H63" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime context/steering：forced-final 消息注入原始用户请求摘要，并明确已读文件不得称未读；如还需实现级深读，只能说明已读但缺少哪些细节</t>
+          <t>参考 OMP runtime context/steering：forced-final 消息注入原始用户请求摘要，并明确已读文件不得称未读；session `20260708T083312934017` 最终按 5 点结构输出，未再出现已读文件称未读</t>
         </is>
       </c>
       <c r="I63" s="0"/>
       <c r="J63" s="0"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t>T-062</t>
+        </is>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>search_code 空搜索词跨路径 guard</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>已完成并复跑通过</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T082703005777Z` 中同一无结果关键词 `exceptionCoreEnterprise` / `ExceptionCoreEnterprise` 在多级目录扩散搜索，绕过同参重复 guard</t>
+        </is>
+      </c>
+      <c r="H64" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP useless tool result / pruning / soft escalation：同一搜索词忽略大小写后多次无结果会跳过后续搜索并 forced-final；session `20260708T083312934017` 已按 5 点结构收束</t>
+        </is>
+      </c>
+      <c r="I64" s="0"/>
+      <c r="J64" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5144,7 +5188,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5931,7 +5975,7 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>已补第三版，待复跑</t>
+          <t>已复跑通过</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
@@ -5941,7 +5985,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>OMP 会显式提供 cwd/project context/rules，并通过 ToolChoiceQueue / soft tool requirement 做小上限纠偏；我们新增 `[Workspace roots]`、工具观察 roots 提示，并对需求/文档类任务前置 soft tool requirement。</t>
+          <t>OMP 会显式提供 cwd/project context/rules，并通过 ToolChoiceQueue / soft tool requirement 做小上限纠偏；我们新增 `[Workspace roots]`、工具观察 roots 提示，并对需求/文档类任务前置 soft tool requirement；session `20260708T083312934017` 已验证先读真实需求文档。</t>
         </is>
       </c>
     </row>
@@ -6005,54 +6049,54 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>已补第三版，待复跑</t>
+          <t>已复跑通过</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间；session `20260708T074609696125Z` 中显式只读任务因“下一步实现”措辞误关 guard；session `20260708T081827983347Z` 中 guard 成功收束，但最终仍把已读文件说成未读</t>
+          <t>session `20260708T073252231781Z` 中模型连续读取同一大文件多个相邻区间；session `20260708T074609696125Z` 中显式只读任务因“下一步实现”措辞误关 guard；session `20260708T081827983347Z` 中 guard 成功收束但证据一致性待补</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline/runtime context 收束；我们新增显式只读优先级、repeated read_file guard、forced-final 已读文件证据摘要、原始请求摘要和已读一致性规则，触发后强制下一轮无工具最终回答。</t>
+          <t>OMP 对病态子循环设置命名小上限，并通过 steering/pruning/deadline/runtime context 收束；我们新增显式只读优先级、repeated read_file guard、forced-final 已读文件证据摘要、原始请求摘要和已读一致性规则；session `20260708T083312934017` 已按 5 点结构输出。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-023</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>同一空搜索词跨路径扩散导致 token 浪费</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已补并复跑通过</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>session `20260708T082703005777Z` 中模型对同一无结果关键词反复切换 path 搜索，因参数不同绕过 exact duplicate guard</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 会把 no-op/useless tool result 降权、prune，并对 soft tool escalation 设置小上限；我们新增 search pattern 级 guard，按 pattern 而非完整参数统计无结果搜索，并在阈值后 forced-final。</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6108,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -6074,22 +6118,22 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6145,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -6111,7 +6155,7 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -6121,12 +6165,12 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6182,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -6148,22 +6192,22 @@
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6219,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -6185,7 +6229,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -6195,12 +6239,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6256,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -6222,7 +6266,7 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
@@ -6232,12 +6276,12 @@
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6293,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -6259,7 +6303,7 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
@@ -6269,12 +6313,12 @@
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6330,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6296,7 +6340,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -6306,12 +6350,12 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6367,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6333,7 +6377,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
@@ -6343,12 +6387,12 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6404,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6370,22 +6414,22 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6441,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6407,7 +6451,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -6417,12 +6461,12 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -6434,7 +6478,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6444,7 +6488,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -6454,12 +6498,12 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6515,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -6481,22 +6525,22 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -6508,32 +6552,32 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6589,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -6555,22 +6599,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6626,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -6592,7 +6636,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -6602,12 +6646,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -6619,30 +6663,67 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
           <t>ADR-017</t>
         </is>
       </c>
-      <c r="C41" s="0" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D41" s="0" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
-      <c r="E41" s="0" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F41" s="0" t="inlineStr">
+      <c r="F42" s="0" t="inlineStr">
         <is>
           <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
-      <c r="G41" s="0" t="inlineStr">
+      <c r="G42" s="0" t="inlineStr">
         <is>
           <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
@@ -6657,7 +6738,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7172,7 +7253,7 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>已补第三版，待复跑验证</t>
+          <t>已由复跑验证收束</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -7187,7 +7268,39 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>forced-final steering 已注入原始用户请求摘要；已读文件列表后追加“不得声称未读，如仍需实现级深读，应说明已读但缺少哪些细节”；测试覆盖该 steering 内容。</t>
+          <t>forced-final steering 已注入原始用户请求摘要和已读一致性规则；session `20260708T083312934017` 最终按 5 点结构输出，未再出现已读文件称未读。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>PT-016</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>已补并复跑通过</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T082703005777Z` 中模型反复搜索 `exceptionCoreEnterprise` / `ExceptionCoreEnterprise`，路径从全仓到多个子目录变化，绕过同参重复 guard。</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将 useless tool result 进入 pruning/steering，并对低价值工具循环设置小上限。</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>已新增 search_code 空搜索词级 guard；同一 pattern 忽略大小写多次无结果后跳过后续搜索并 forced-final。session `20260708T083312934017` 未再出现该循环。</t>
         </is>
       </c>
     </row>
@@ -7263,7 +7376,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 147 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 148 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten multi-project pressure-test steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 代跑企业压测，最新 session `20260708T083312934017` 已验证 allowed-dir 需求文档前置读取、repeated read-file guard、空搜索词跨路径 guard 和 forced-final 收束生效，最终按 5 点结构输出。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，最新 session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑企业项目联网压测；session `20260708T082703005777Z` 暴露同一空搜索词跨路径扩散，已补搜索词级 guard；session `20260708T083312934017` 已先读需求、搜索代码、触发 guard 后按 5 点结构收束。下一步从“运行稳定性”转向回答准确性/项目覆盖评估。</t>
+          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。下一步继续评估回答准确性和跨项目覆盖边界。</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>当前 148 个测试通过</t>
+          <t>当前 152 个测试通过</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -2369,12 +2369,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J68"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
@@ -5179,6 +5179,182 @@
       <c r="I64" s="0"/>
       <c r="J64" s="0"/>
     </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t>T-063</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="inlineStr">
+        <is>
+          <t>path escape roots hint</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
+          <t>已完成并复跑通过</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T084322924403Z` 中模型把主 `--cwd` 误写成父目录，工具错误没有给可行动纠偏，导致主项目未被检查</t>
+        </is>
+      </c>
+      <c r="H65" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime context/tool observation：公共 path resolver 越界错误返回 resolved path、primary workspace、allowed dirs，并提示父目录误用时使用 `.` 或精确 `--cwd`；session `20260708T085927874078` 已纠正回主项目</t>
+        </is>
+      </c>
+      <c r="I65" s="0"/>
+      <c r="J65" s="0"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t>T-064</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D66" s="0" t="inlineStr">
+        <is>
+          <t>LSP symbol 空 query guard</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
+          <t>已完成并复跑通过</t>
+        </is>
+      </c>
+      <c r="F66" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G66" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T084714338485Z` 中模型连续猜不存在的 `CoreEnterpriseBatchImport*` 符号，参数不同但全是低价值空 LSP 查询</t>
+        </is>
+      </c>
+      <c r="H66" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP useless result / pruning / soft escalation：连续一批 LSP symbol query 无结果后跳过并 forced-final；有命中则清空空探索计数</t>
+        </is>
+      </c>
+      <c r="I66" s="0"/>
+      <c r="J66" s="0"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t>T-065</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>Current task contract / evidence-backed path rule</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>已完成并复跑通过</t>
+        </is>
+      </c>
+      <c r="F67" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T085426840146Z` 最终只总结最后一份需求文档，没有按 6 点结构输出；回答也有把猜测路径当证据路径的风险</t>
+        </is>
+      </c>
+      <c r="H67" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime context/steering：每次 provider request 注入当前原始用户请求、最终输出结构和证据路径规则；session `20260708T085927874078` 已按 6 点结构输出</t>
+        </is>
+      </c>
+      <c r="I67" s="0"/>
+      <c r="J67" s="0"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t>T-066</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>多项目企业只读压测</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>已完成首轮</t>
+        </is>
+      </c>
+      <c r="F68" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>验证 `--cwd crcl-open` + `--allow-dir 需求目录` + `--allow-dir zqyl-user-center-service` 的跨项目链路</t>
+        </is>
+      </c>
+      <c r="H68" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T085927874078` 通过：定位主项目批量导入真实链路，并把辅助项目结算行/黑名单导入线索区分为支撑或相似模式；拓展服务费结算仍需补项目或确认新建</t>
+        </is>
+      </c>
+      <c r="I68" s="0"/>
+      <c r="J68" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5188,7 +5364,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6103,111 +6279,111 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-024</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>path escape 纠偏不足会让模型漏读主项目</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已补并复跑通过</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>session `20260708T084322924403Z` 中模型误用父目录后没有恢复，最终只分析辅助项目</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 会把 cwd/project context 和可行动工具观察持续放回上下文；我们把 roots hint 放进公共 path escape 错误，session `20260708T085927874078` 已验证可恢复。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-025</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>LSP 空 query 扩散导致 token 浪费</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已补并复跑通过</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>session `20260708T084714338485Z` 中模型猜测大量不存在符号名，参数不同绕过同参重复 guard</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 会把 useless result/pruning/soft escalation 结合使用；我们新增 LSP symbol 空 query 小上限并 forced-final。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>R-026</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>最终回答结构和证据路径可能漂移</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已补并复跑通过</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>session `20260708T085426840146Z` 最终只总结最后一个需求文档；此前也出现把未验证路径当下一步建议路径的倾向</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 将当前任务、runtime state 和 tool evidence 持续放进 provider context；我们新增 Current task contract 和 evidence-backed path rule。</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6395,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -6229,7 +6405,7 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -6239,12 +6415,12 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6432,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -6266,22 +6442,22 @@
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -6293,7 +6469,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -6303,22 +6479,22 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6506,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6340,7 +6516,7 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
@@ -6350,12 +6526,12 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6367,7 +6543,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6377,7 +6553,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
@@ -6387,12 +6563,12 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6580,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6414,7 +6590,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -6424,12 +6600,12 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6617,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6451,22 +6627,22 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6654,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6488,22 +6664,22 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6691,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -6525,22 +6701,22 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6728,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -6562,22 +6738,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -6589,32 +6765,32 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -6626,17 +6802,17 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -6646,12 +6822,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -6663,32 +6839,32 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -6700,30 +6876,141 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>ADR-015</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+        </is>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
           <t>ADR-017</t>
         </is>
       </c>
-      <c r="C42" s="0" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D42" s="0" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
-      <c r="E42" s="0" t="inlineStr">
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F42" s="0" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
-      <c r="G42" s="0" t="inlineStr">
+      <c r="G45" s="0" t="inlineStr">
         <is>
           <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
@@ -6738,7 +7025,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F21"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7301,6 +7588,102 @@
       <c r="F18" s="0" t="inlineStr">
         <is>
           <t>已新增 search_code 空搜索词级 guard；同一 pattern 忽略大小写多次无结果后跳过后续搜索并 forced-final。session `20260708T083312934017` 未再出现该循环。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>PT-017</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>已补并复跑通过</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T084322924403Z` 中模型误用父目录 `/Users/chengming/mycode/project/crcl-open`，工具错误未提示正确 primary workspace。</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>OMP 通过 cwd/project context 和工具观察提示模型可行动路径。</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>公共 path resolver 已在 path escape 错误中列出 primary workspace/allowed dirs；session `20260708T085927874078` 已恢复到 `.` 主项目。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>PT-018</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>已补并复跑通过</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T084714338485Z` 中模型连续猜不存在的 LSP symbol query。</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>OMP 对 useless result 和 soft tool escalation 设小上限。</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>已新增 LSP symbol 空 query guard；session `20260708T085927874078` 未再卡死。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>PT-019</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>已补并复跑通过</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>session `20260708T085426840146Z` 最终回答只总结最后一个需求文档，没有按 6 点结构输出。</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将当前任务和 runtime evidence 持续注入 provider context。</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>已新增 Current task contract 和 evidence-backed path rule；session `20260708T085927874078` 按 6 点结构输出。</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7699,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7376,7 +7759,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 148 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 152 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -7422,12 +7805,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>P7 综合真实压测与 token 预算评估</t>
+          <t>P7 轻量高级能力真实压测后续</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn 和 authored skills 是否足够日用。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir 和多项目只读压测主链路；下一步继续做回答准确性评估，尤其是跨项目缺失证据时的措辞和实现前二次验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add evidence ledger for grounded answers
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -100,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，最新 session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新小实现压测 session `20260708T092554037057Z` 已验证 Evidence Ledger 不破坏小改闭环，并暴露 `path#tag` 易误填和脏工作区 diff 归因问题。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -569,20 +569,38 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
+          <t>Evidence Ledger</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 会从 `read_file`、`search_code`、LSP、patch、run_tests、git 等工具结果提炼短证据账本，作为 provider-bound context 注入，并写入 session JSONL `evidence` 事件。</t>
+        </is>
+      </c>
+      <c r="D27" s="0"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B27" s="0" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C27" s="0" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D27" s="0"/>
+      <c r="D28" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -884,7 +902,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -899,7 +917,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。下一步继续评估回答准确性和跨项目覆盖边界。</t>
+          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。小实现压测 `20260708T092554037057Z` 已验证 Evidence Ledger 后小改闭环仍可跑通。下一步继续评估回答准确性、跨项目覆盖边界和工具参数可用性细节。</t>
         </is>
       </c>
     </row>
@@ -912,7 +930,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2333,32 +2351,62 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Evidence Ledger</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>当前 152 个测试通过</t>
+          <t>`src/local_agent/agent.py` / `tests/test_agent.py`</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>工具结果经 runtime 提炼成短证据账本；provider context 中提示模型区分证据事实与推断，session 中追加 `evidence` 事件</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>后续真实任务观察是否需要更结构化引用</t>
         </is>
       </c>
       <c r="F48" s="0"/>
       <c r="G48" s="0"/>
       <c r="H48" s="0"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>当前 153 个测试通过</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F49" s="0"/>
+      <c r="G49" s="0"/>
+      <c r="H49" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2369,7 +2417,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J71"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5355,6 +5403,138 @@
       <c r="I68" s="0"/>
       <c r="J68" s="0"/>
     </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t>T-067</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>Evidence Ledger MVP</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>已完成并小改压测通过</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>Current task contract 只约束“证据路径必须来自工具结果”，但长工具链后模型仍需要一份短证据账本来区分证据事实和推断</t>
+        </is>
+      </c>
+      <c r="H69" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime context / observation 思路：runtime 从工具结果中央提炼 evidence records，provider-bound 注入 `[Evidence ledger]`，session JSONL 追加 `evidence` 事件；测试覆盖 read_file 后账本注入，小实现压测 `20260708T092554037057Z` 通过</t>
+        </is>
+      </c>
+      <c r="I69" s="0"/>
+      <c r="J69" s="0"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t>T-068</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>apply_patch tag 参数易误填 `path#tag`</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>小实现压测中模型先把 `read_file` header `README.md#3988a904` 整串传给 `tag`，dry_run 连续失败后才自我修正为 `3988a904`</t>
+        </is>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t>可参考 OMP 更结构化的工具观察/编辑参数提示：短期可改 `read_file` 输出显式 `tag: 3988a904` 或让 `apply_patch` 兼容 `path#tag` 并给清晰警告；需保持 anchored patch 校验语义</t>
+        </is>
+      </c>
+      <c r="I70" s="0"/>
+      <c r="J70" s="0"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>T-069</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t>git_diff 归因区分已有工作区修改与本轮修改</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="F71" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
+        <is>
+          <t>小实现压测时工作区已有人工实现的 Evidence Ledger diff，模型的 `git_diff` 同时看到 README 小改和 agent.py 大改，虽能识别“非本轮改动”，但依赖推理</t>
+        </is>
+      </c>
+      <c r="H71" s="0" t="inlineStr">
+        <is>
+          <t>可参考 OMP task/worktree/session state 思路：后续可在 run start 记录 git status/diff baseline，最终 diff 摘要区分 pre-existing、this-run patch、untracked runtime files</t>
+        </is>
+      </c>
+      <c r="I71" s="0"/>
+      <c r="J71" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5364,7 +5544,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G48"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6390,74 +6570,74 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-027</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>模型可能把 `read_file` header 的 `path#tag` 整串误当成 patch tag</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已记录，待评估修复</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>小实现压测 session `20260708T092554037057Z` 中 dry_run 前三次因 `tag=README.md#3988a904` 失败，第四次改成纯 hash 后成功</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 的工具观察和编辑链路更强调结构化参数和 runtime 纠偏；LCA 可短期改 read_file 输出或 apply_patch 参数兼容来减少无效重试。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-028</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>脏工作区下最终 diff 摘要可能混入非本轮改动</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已记录，待评估修复</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>小实现压测 session `20260708T092554037057Z` 的 `git_diff` 同时包含 README 小改和正在开发的 Evidence Ledger 代码 diff；模型能分辨但依赖推理</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 更完整的 task/worktree/session state 能追踪任务边界；LCA 后续可在 run start 记录 baseline，并把本轮 patch records 与 git_diff 对照。</t>
         </is>
       </c>
     </row>
@@ -6469,7 +6649,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -6479,22 +6659,22 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6506,7 +6686,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6516,22 +6696,22 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6723,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6553,22 +6733,22 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6580,7 +6760,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6590,7 +6770,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -6600,12 +6780,12 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6617,7 +6797,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6627,7 +6807,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -6637,12 +6817,12 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6834,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6664,7 +6844,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -6674,12 +6854,12 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6871,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -6701,7 +6881,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -6711,12 +6891,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6728,7 +6908,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -6738,22 +6918,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6765,7 +6945,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -6775,22 +6955,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -6802,7 +6982,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -6812,7 +6992,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -6822,12 +7002,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -6839,7 +7019,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -6849,22 +7029,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -6876,32 +7056,32 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -6913,32 +7093,32 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -6950,7 +7130,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -6960,22 +7140,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -6987,32 +7167,143 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
+          <t>ADR-015</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+        </is>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>ADR-016</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F46" s="0" t="inlineStr">
+        <is>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+        </is>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
           <t>ADR-017</t>
         </is>
       </c>
-      <c r="C45" s="0" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D45" s="0" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
-      <c r="E45" s="0" t="inlineStr">
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F45" s="0" t="inlineStr">
+      <c r="F47" s="0" t="inlineStr">
         <is>
           <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
-      <c r="G45" s="0" t="inlineStr">
+      <c r="G47" s="0" t="inlineStr">
         <is>
           <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ADR-018</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+        </is>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -7025,7 +7316,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F24"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7684,6 +7975,102 @@
       <c r="F21" s="0" t="inlineStr">
         <is>
           <t>已新增 Current task contract 和 evidence-backed path rule；session `20260708T085927874078` 按 6 点结构输出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>PT-020</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>已补并小改压测通过</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Current task contract 能要求 evidence-backed path，但长工具链后模型仍需要一份短证据账本来避免最终回答把推断当事实。</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会把 runtime state、tool evidence 和 steering 持续放进模型上下文；证据不是长期 memory，而是本轮 provider context。</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>已新增 Evidence Ledger：runtime 中央观察 `read_file`、`search_code`、LSP、patch、run_tests、git 等工具结果，提炼短 evidence records，注入 `[Evidence ledger]` provider context，并写 session `evidence` 事件；小实现压测 `20260708T092554037057Z` 跑通。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>PT-021</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>已记录，待评估修复</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>小实现压测中模型把 `read_file` header `README.md#3988a904` 整串作为 `apply_patch.tag`，导致 dry_run 连续失败；随后改成纯 hash 才成功。</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>OMP 更倾向用结构化工具观察和编辑流程降低模型手工解析参数的机会；工具错误也要给可行动纠偏。</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>短期候选：read_file 输出显式 `tag: 3988a904`；或 apply_patch 接受 `path#tag` 并提取 hash，同时提示模型后续只传 hash。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>PT-022</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>已记录，待评估修复</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>小实现压测时 `git_diff` 包含 README 小改和正在开发的 Evidence Ledger 代码 diff；模型识别出 agent.py 是既有改动，但这种区分依赖推理。</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 task/worktree/session state 更能区分任务边界和已有 WIP；普通 CLI 也应清楚记录 run start baseline。</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>后续候选：run start 记录 git status/diff baseline，最终 diff 摘要按 pre-existing / this-run patch / runtime state 分组。</t>
         </is>
       </c>
     </row>
@@ -7759,7 +8146,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 152 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 153 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make patch tags easier to reuse
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>当前 153 个测试通过</t>
+          <t>当前 155 个测试通过</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="H70" s="0" t="inlineStr">
         <is>
-          <t>可参考 OMP 更结构化的工具观察/编辑参数提示：短期可改 `read_file` 输出显式 `tag: 3988a904` 或让 `apply_patch` 兼容 `path#tag` 并给清晰警告；需保持 anchored patch 校验语义</t>
+          <t>已参考 OMP 结构化工具观察/编辑参数提示：`read_file` 现在显式输出 `tag: &lt;hash&gt;`；`apply_patch` 兼容 `[path#hash]` / `path#hash` 并提示下次传纯 hash，anchored hash 校验不放宽；测试覆盖。</t>
         </is>
       </c>
       <c r="I70" s="0"/>
@@ -6590,7 +6590,7 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>OMP 的工具观察和编辑链路更强调结构化参数和 runtime 纠偏；LCA 可短期改 read_file 输出或 apply_patch 参数兼容来减少无效重试。</t>
+          <t>已加双保险：`read_file` 显式输出 pure tag；`apply_patch` 兼容误传的 `path#tag` / `[path#tag]`，但仍用 hash 校验当前文件。</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>短期候选：read_file 输出显式 `tag: 3988a904`；或 apply_patch 接受 `path#tag` 并提取 hash，同时提示模型后续只传 hash。</t>
+          <t>已实现：`read_file` 显式输出 `tag: &lt;hash&gt;`；`apply_patch` 接受 `path#tag` / `[path#tag]` 并提取 hash，同时提示模型后续只传纯 hash。</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 153 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 155 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Attribute git diff to current agent run
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新小实现压测 session `20260708T092554037057Z` 已验证 Evidence Ledger 不破坏小改闭环，并暴露 `path#tag` 易误填和脏工作区 diff 归因问题。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新小实现压测 session `20260708T092554037057Z` 已验证 Evidence Ledger 不破坏小改闭环，并暴露的 `path#tag` 易误填和脏工作区 diff 归因问题均已补 MVP 版防护。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>当前 155 个测试通过</t>
+          <t>当前 156 个测试通过</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="H71" s="0" t="inlineStr">
         <is>
-          <t>可参考 OMP task/worktree/session state 思路：后续可在 run start 记录 git status/diff baseline，最终 diff 摘要区分 pre-existing、this-run patch、untracked runtime files</t>
+          <t>已参考 OMP task/worktree/session state 思路：每轮 run start 捕获 git baseline 并写 session；`git_diff` 追加 attribution 小节，按 pre-existing dirty files、this-session apply_patch files、mixed files、new unattributed files 提示模型分开总结。</t>
         </is>
       </c>
       <c r="I71" s="0"/>
@@ -6627,7 +6627,7 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>OMP 更完整的 task/worktree/session state 能追踪任务边界；LCA 后续可在 run start 记录 baseline，并把本轮 patch records 与 git_diff 对照。</t>
+          <t>已参考 OMP task/worktree/session state：run start 记录 baseline，`git_diff` 对照本轮 patch records 输出归因提示；同一文件若运行前已 dirty 且本轮又修改，会标成 mixed。</t>
         </is>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>后续候选：run start 记录 git status/diff baseline，最终 diff 摘要按 pre-existing / this-run patch / runtime state 分组。</t>
+          <t>已实现：run start 记录 git status/diff baseline；`git_diff` 读取本 session patch records 并追加 attribution，区分 pre-existing、this-session、mixed、new unattributed。</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 155 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 156 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record T-069 attribution pressure test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新小实现压测 session `20260708T092554037057Z` 已验证 Evidence Ledger 不破坏小改闭环，并暴露的 `path#tag` 易误填和脏工作区 diff 归因问题均已补 MVP 版防护。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新 T-069 归因复测 session `20260708T094926471758Z` 验证 attribution 能正确区分 pre-existing 与 this-session，同时暴露最终 diff 细节概括仍需增强。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -2417,7 +2417,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J72"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5535,6 +5535,50 @@
       <c r="I71" s="0"/>
       <c r="J71" s="0"/>
     </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>T-070</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t>最终 diff 细节概括准确性</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t>已记录，待评估</t>
+        </is>
+      </c>
+      <c r="F72" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
+        <is>
+          <t>T-069 复测 session `20260708T094926471758Z` 中 attribution 分类正确，但模型把“重复标题 + smoke-test 标记”概括为 exactly one insertion，且选择的 README 改动低价值</t>
+        </is>
+      </c>
+      <c r="H72" s="0" t="inlineStr">
+        <is>
+          <t>可参考 OMP runtime observation/reviewer 思路：后续可让 `git_diff` 输出轻量 diff stats / hunk summary，或在 final steering 中要求引用实际 hunk 增删行；必要时增加 reviewer 风格自检。</t>
+        </is>
+      </c>
+      <c r="I72" s="0"/>
+      <c r="J72" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5544,7 +5588,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6644,37 +6688,37 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-029</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>最终 diff 细节可能被模型过度简化或说错</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已记录，待评估修复</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-069 复测 session `20260708T094926471758Z` 中 attribution 分类正确，但模型没有准确描述实际 diff hunk；低价值 README smoke-test 改动已撤回</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>OMP 通过更结构化 runtime state/tool observation 和 reviewer/verification 降低最终回答漂移；LCA 后续可给 `git_diff` 增加 diff stats/hunk summary，并在 final steering 中要求按实际 hunk 总结。</t>
         </is>
       </c>
     </row>
@@ -6686,7 +6730,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -6696,22 +6740,22 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6723,7 +6767,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6733,7 +6777,7 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
@@ -6743,12 +6787,12 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6804,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6770,22 +6814,22 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6797,7 +6841,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6807,7 +6851,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -6817,12 +6861,12 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6878,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6844,7 +6888,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -6854,12 +6898,12 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6915,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -6881,7 +6925,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -6891,12 +6935,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6908,7 +6952,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -6918,7 +6962,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -6928,12 +6972,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -6945,7 +6989,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -6955,7 +6999,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -6965,12 +7009,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -6982,7 +7026,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -6992,22 +7036,22 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7019,7 +7063,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7029,7 +7073,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7039,12 +7083,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7056,7 +7100,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7066,7 +7110,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7076,12 +7120,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7137,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7103,22 +7147,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7130,32 +7174,32 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7211,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7177,22 +7221,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7204,7 +7248,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7214,7 +7258,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -7224,12 +7268,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7285,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7251,22 +7295,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7278,30 +7322,67 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
+          <t>ADR-017</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+        </is>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
           <t>ADR-018</t>
         </is>
       </c>
-      <c r="C48" s="0" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D48" s="0" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
-      <c r="E48" s="0" t="inlineStr">
+      <c r="E49" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F48" s="0" t="inlineStr">
+      <c r="F49" s="0" t="inlineStr">
         <is>
           <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
-      <c r="G48" s="0" t="inlineStr">
+      <c r="G49" s="0" t="inlineStr">
         <is>
           <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
@@ -7316,7 +7397,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8071,6 +8152,38 @@
       <c r="F24" s="0" t="inlineStr">
         <is>
           <t>已实现：run start 记录 git status/diff baseline；`git_diff` 读取本 session patch records 并追加 attribution，区分 pre-existing、this-session、mixed、new unattributed。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>PT-023</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>已记录，待评估修复</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>T-069 归因复测中 `[diff attribution]` 正确区分 `review_by_myself.md` 和 `README.md`，但模型把实际 “重复标题 + smoke-test 标记” 概括成 exactly one insertion；临时 README 改动已撤回。</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>OMP 倾向把最终回答建立在结构化 runtime observation 上，并通过 reviewer/verification 约束结论。</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>后续候选：`git_diff` 输出 diff stats/hunk summary，final steering 要求引用实际 hunk 增删行，必要时增加 reviewer 自检。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add structured git diff summaries
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；最新 T-069 归因复测 session `20260708T094926471758Z` 验证 attribution 能正确区分 pre-existing 与 this-session，同时暴露最终 diff 细节概括仍需增强。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，减少脏工作区和 hunk 细节误读。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1269,12 +1269,12 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>untracked 时解释空 diff 原因</t>
+          <t>untracked 时解释空 diff 原因；git_diff 输出 diff summary 和 attribution</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>初始 commit 后 diff 更清晰</t>
+          <t>初始 commit 后 diff 更清晰；脏工作区下能区分运行前已有和本轮 patch</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>当前 156 个测试通过</t>
+          <t>当前 157 个测试通过</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="H72" s="0" t="inlineStr">
         <is>
-          <t>可参考 OMP runtime observation/reviewer 思路：后续可让 `git_diff` 输出轻量 diff stats / hunk summary，或在 final steering 中要求引用实际 hunk 增删行；必要时增加 reviewer 风格自检。</t>
+          <t>已参考 OMP runtime observation 思路：`git_diff` 追加 `[diff summary]`，按文件输出 `+N/-M`、hunk 数、hunk header 和少量 added/removed 片段；回归测试覆盖重复标题 + smoke-test 行实际为 `+3 -0`。</t>
         </is>
       </c>
       <c r="I72" s="0"/>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>OMP 通过更结构化 runtime state/tool observation 和 reviewer/verification 降低最终回答漂移；LCA 后续可给 `git_diff` 增加 diff stats/hunk summary，并在 final steering 中要求按实际 hunk 总结。</t>
+          <t>已参考 OMP runtime state/tool observation：`git_diff` 追加结构化 diff summary，直接提供文件级增删统计和 hunk snippets；后续再观察是否需要 reviewer 自检。</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>已记录，待评估修复</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>后续候选：`git_diff` 输出 diff stats/hunk summary，final steering 要求引用实际 hunk 增删行，必要时增加 reviewer 自检。</t>
+          <t>已实现：`git_diff` 输出 `[diff summary]`，包含总文件数、`+N/-M`、hunk 数和少量 added/removed 片段，降低模型粗读 unified diff 的机会。</t>
         </is>
       </c>
     </row>
@@ -8259,7 +8259,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 156 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 157 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record T-070 diff summary retest
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，减少脏工作区和 hunk 细节误读。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成并复测通过</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="H72" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP runtime observation 思路：`git_diff` 追加 `[diff summary]`，按文件输出 `+N/-M`、hunk 数、hunk header 和少量 added/removed 片段；回归测试覆盖重复标题 + smoke-test 行实际为 `+3 -0`。</t>
+          <t>已参考 OMP runtime observation 思路：`git_diff` 追加 `[diff summary]`，按文件输出 `+N/-M`、hunk 数、hunk header 和少量 added/removed 片段；回归测试覆盖重复标题 + smoke-test 行实际为 `+3 -0`；百炼复测 session `20260708T100128250335Z` 已正确总结 `1 file(s), +1 -1, 1 hunk(s)` 和 attribution。</t>
         </is>
       </c>
       <c r="I72" s="0"/>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭并复测通过</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP runtime state/tool observation：`git_diff` 追加结构化 diff summary，直接提供文件级增删统计和 hunk snippets；后续再观察是否需要 reviewer 自检。</t>
+          <t>已参考 OMP runtime state/tool observation：`git_diff` 追加结构化 diff summary，直接提供文件级增删统计和 hunk snippets；百炼复测 session `20260708T100128250335Z` 已正确引用 summary 和 attribution。</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭并复测通过</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>已实现：`git_diff` 输出 `[diff summary]`，包含总文件数、`+N/-M`、hunk 数和少量 added/removed 片段，降低模型粗读 unified diff 的机会。</t>
+          <t>已实现：`git_diff` 输出 `[diff summary]`，包含总文件数、`+N/-M`、hunk 数和少量 added/removed 片段；百炼复测 session `20260708T100128250335Z` 已正确总结 `+1/-1`、1 hunk、本轮 README 和运行前 `review_by_myself.md`。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record P7 stage review decision
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -7,9 +7,10 @@
     <sheet name="已完成功能" sheetId="3" r:id="rId3"/>
     <sheet name="下一步 Todo" sheetId="4" r:id="rId4"/>
     <sheet name="风险与决策" sheetId="5" r:id="rId5"/>
-    <sheet name="P7 综合压测问题" sheetId="6" r:id="rId6"/>
-    <sheet name="P5 收口结论" sheetId="7" r:id="rId7"/>
-    <sheet name="推荐工作流" sheetId="8" r:id="rId8"/>
+    <sheet name="P7 阶段回顾" sheetId="6" r:id="rId6"/>
+    <sheet name="P7 综合压测问题" sheetId="7" r:id="rId7"/>
+    <sheet name="P5 收口结论" sheetId="8" r:id="rId8"/>
+    <sheet name="推荐工作流" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -167,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution；2026-07-09 阶段回顾结论是先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 作为条件触发项后补。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -917,7 +918,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。小实现压测 `20260708T092554037057Z` 已验证 Evidence Ledger 后小改闭环仍可跑通。下一步继续评估回答准确性、跨项目覆盖边界和工具参数可用性细节。</t>
+          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。小实现压测 `20260708T092554037057Z` 已验证 Evidence Ledger 后小改闭环仍可跑通。T-071 阶段回顾已决定下一步进入真实需求实现压测；reviewer / 完整 ToolChoiceQueue 仅在压测暴露具体失败后定向补。</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2418,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5579,6 +5580,138 @@
       <c r="I72" s="0"/>
       <c r="J72" s="0"/>
     </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>T-071</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>P7 阶段回顾与 OMP 差距决策</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>T-070 后需要决定继续补 reviewer/ToolChoiceQueue，还是进入真实需求实现压测</t>
+        </is>
+      </c>
+      <c r="H73" s="0" t="inlineStr">
+        <is>
+          <t>新增 `docs/stage-review-2026-07-09.md`；结论是当前主链路已具备低风险实战条件，先做真实需求实现压测。</t>
+        </is>
+      </c>
+      <c r="I73" s="0"/>
+      <c r="J73" s="0"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t>T-072</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t>真实需求实现压测</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F74" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G74" s="0" t="inlineStr">
+        <is>
+          <t>只有真实需求实现才能检验默认工作流、multi-root、LSP、Evidence Ledger、patch、tests、diff attribution 是否形成完整闭环</t>
+        </is>
+      </c>
+      <c r="H74" s="0" t="inlineStr">
+        <is>
+          <t>选择一个低风险需求；压测前记录 git status；写入前 dry_run；写入后 run_tests + git_diff；压测问题回写文档和 Excel。</t>
+        </is>
+      </c>
+      <c r="I74" s="0"/>
+      <c r="J74" s="0"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t>T-073</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>P7/P8</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t>reviewer / 完整 ToolChoiceQueue 条件触发评估</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F75" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G75" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 reviewer 和 ToolChoiceQueue 很强，但应由真实失败样本驱动裁剪</t>
+        </is>
+      </c>
+      <c r="H75" s="0" t="inlineStr">
+        <is>
+          <t>若 T-072 暴露关键工具不用/乱用，补 ToolChoiceQueue；若暴露 patch 或总结质量问题，补轻量 reviewer。</t>
+        </is>
+      </c>
+      <c r="I75" s="0"/>
+      <c r="J75" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5588,7 +5721,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6725,37 +6858,37 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-030</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>过早补完整 reviewer / ToolChoiceQueue 会增加复杂度但未必命中当前痛点</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>开放并受控</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>OMP 的 reviewer、subagents、ToolChoiceQueue 很强，但 LCA 当前还缺真实实现压测的失败样本；提前完整搬入可能拖慢 MVP 验证</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>先进入 T-072 真实需求实现压测；若压测暴露工具选择失控，按 OMP 裁剪 ToolChoiceQueue；若暴露 patch/总结质量不稳，按 OMP 裁剪轻量 reviewer。</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6900,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -6777,22 +6910,22 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6937,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6814,7 +6947,7 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
@@ -6824,12 +6957,12 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -6841,7 +6974,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6851,22 +6984,22 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -6878,7 +7011,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -6888,7 +7021,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -6898,12 +7031,12 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -6915,7 +7048,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -6925,7 +7058,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -6935,12 +7068,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -6952,7 +7085,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -6962,7 +7095,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -6972,12 +7105,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -6989,7 +7122,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -6999,7 +7132,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -7009,12 +7142,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7159,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7036,7 +7169,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -7046,12 +7179,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7196,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7073,22 +7206,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7233,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7110,7 +7243,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7120,12 +7253,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7137,7 +7270,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7147,7 +7280,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7157,12 +7290,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7307,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7184,22 +7317,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7211,32 +7344,32 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7381,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7258,22 +7391,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7285,7 +7418,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7295,7 +7428,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -7305,12 +7438,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7322,7 +7455,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7332,22 +7465,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7359,32 +7492,106 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
+          <t>ADR-017</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="inlineStr">
+        <is>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+        </is>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
           <t>ADR-018</t>
         </is>
       </c>
-      <c r="C49" s="0" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D49" s="0" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
-      <c r="E49" s="0" t="inlineStr">
+      <c r="E50" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F49" s="0" t="inlineStr">
+      <c r="F50" s="0" t="inlineStr">
         <is>
           <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
-      <c r="G49" s="0" t="inlineStr">
+      <c r="G50" s="0" t="inlineStr">
         <is>
           <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ADR-019</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="inlineStr">
+        <is>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+        </is>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -7396,6 +7603,187 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D8"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>P7 阶段回顾</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>依据</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>后续</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>阶段判断</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>可以进入真实需求实现压测</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>读、搜、改、测、diff、approval、budget、compaction、memory、todo、ask_user、Evidence Ledger、diff attribution/summary 主链路已闭环</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>执行 T-072</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>与 OMP 的主要差距</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>差距集中在高级工程化，不阻塞低风险实战</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>完整 ToolChoiceQueue、reviewer/subagents、完整 LSP/DAP、browser/TUI、AST edit、managed skills 仍后置</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>由压测失败形态触发</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>已关闭风险</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>P0/P1 runtime 风险已基本收口</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Python 3.12 patch、非交互审批、orphan tool_calls、max_steps、allowed-dir、重复工具、证据漂移、diff 混淆等均已有修复或缓解</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>继续用真实任务验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>reviewer 决策</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>暂不先做完整 reviewer</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>当前还没有真实实现压测中的 patch 质量失败样本；过早实现会增加复杂度</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>若 T-072 暴露 patch/总结质量不稳，再做轻量 post-diff reviewer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>ToolChoiceQueue 决策</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>暂不先做完整 ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>已有 allowed-dir soft requirement、duplicate forced-final、todo steering、pruning；还缺“关键工具长期不用/乱用”的新失败样本</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>若 T-072 暴露工具选择失控，再按 OMP 裁剪 ToolChoiceQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>真实需求实现压测</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>阶段回顾文档见 `docs/stage-review-2026-07-09.md`</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>压测后更新压测文档、项目状态和 Excel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F25"/>
   <cols>
@@ -8194,7 +8582,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C7"/>
   <cols>
@@ -8321,7 +8709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F15"/>
   <cols>

</xml_diff>

<commit_message>
Record T-072 implementation pressure test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution；2026-07-09 阶段回顾结论是先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 作为条件触发项后补。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution；2026-07-09 阶段回顾后已执行 T-072 首轮真实需求实现压测，暴露无关 patch 和反事实 workspace 判断，T-073 升级为下一步：先做轻量 relevance gate / reviewer。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。小实现压测 `20260708T092554037057Z` 已验证 Evidence Ledger 后小改闭环仍可跑通。T-071 阶段回顾已决定下一步进入真实需求实现压测；reviewer / 完整 ToolChoiceQueue 仅在压测暴露具体失败后定向补。</t>
+          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。T-072 首轮真实需求实现压测 session `20260709T013441841983Z` 未通过：模型漂移到 `deployMessage/nacos` 并产生无关 patch。下一步 T-073 做 relevance gate / reviewer。</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5647,7 @@
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>首轮完成但未通过</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="H74" s="0" t="inlineStr">
         <is>
-          <t>选择一个低风险需求；压测前记录 git status；写入前 dry_run；写入后 run_tests + git_diff；压测问题回写文档和 Excel。</t>
+          <t>session `20260709T013441841983Z` 读取真实需求后漂移到 `deployMessage/nacos`，修改无关 Redis 配置并错误声称 worktree 无 `pom.xml/src`；问题已记录到 `docs/pressure-test-2026-07-09.md`。</t>
         </is>
       </c>
       <c r="I74" s="0"/>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -5686,12 +5686,12 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>reviewer / 完整 ToolChoiceQueue 条件触发评估</t>
+          <t>轻量 reviewer / pre-edit relevance gate</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>下一步</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
@@ -5701,12 +5701,12 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 reviewer 和 ToolChoiceQueue 很强，但应由真实失败样本驱动裁剪</t>
+          <t>T-072 已暴露无关 patch 和反事实 workspace 判断；需要把需求、证据、编辑目标和最终 diff 绑紧</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
         <is>
-          <t>若 T-072 暴露关键工具不用/乱用，补 ToolChoiceQueue；若暴露 patch 或总结质量问题，补轻量 reviewer。</t>
+          <t>写入前检查目标文件是否来自近期证据；workspace-root evidence 进入 Evidence Ledger；最终 diff reviewer 能指出变更与需求不相关并要求回滚/重定位。</t>
         </is>
       </c>
       <c r="I75" s="0"/>
@@ -5721,7 +5721,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6895,37 +6895,37 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-031</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>真实实现任务可能产生无关 patch</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-072 session `20260709T013441841983Z` 读取正确需求后漂移到 Nacos/Redis 配置，并把无关注释当成实现锚点；dry_run/hash 校验只能保证位置正确，不能保证业务相关</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>下一步 T-073 做 pre-edit relevance gate：`apply_patch` 真写入前检查目标文件是否来自近期需求/代码证据；同时做轻量 diff reviewer。</t>
         </is>
       </c>
     </row>
@@ -6937,7 +6937,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -6947,22 +6947,22 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
@@ -6994,12 +6994,12 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7011,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -7021,22 +7021,22 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -7068,12 +7068,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7085,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -7105,12 +7105,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -7132,7 +7132,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -7142,12 +7142,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -7179,12 +7179,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7216,12 +7216,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7243,22 +7243,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7290,12 +7290,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7307,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -7327,12 +7327,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7344,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7354,22 +7354,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7381,32 +7381,32 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7428,22 +7428,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7455,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7465,7 +7465,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -7475,12 +7475,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7492,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -7502,22 +7502,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -7539,22 +7539,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -7566,32 +7566,106 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
+          <t>ADR-018</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="inlineStr">
+        <is>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+        </is>
+      </c>
+      <c r="G51" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
           <t>ADR-019</t>
         </is>
       </c>
-      <c r="C51" s="0" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D51" s="0" t="inlineStr">
+      <c r="D52" s="0" t="inlineStr">
         <is>
           <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
-      <c r="E51" s="0" t="inlineStr">
+      <c r="E52" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F51" s="0" t="inlineStr">
+      <c r="F52" s="0" t="inlineStr">
         <is>
           <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
-      <c r="G51" s="0" t="inlineStr">
+      <c r="G52" s="0" t="inlineStr">
         <is>
           <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>ADR-020</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="inlineStr">
+        <is>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+        </is>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7681,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -7762,17 +7836,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>真实需求实现压测</t>
+          <t>轻量 relevance gate / reviewer</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾文档见 `docs/stage-review-2026-07-09.md`</t>
+          <t>T-072 首轮实现压测已证明真实实现任务可能写入无关文件</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>压测后更新压测文档、项目状态和 Excel</t>
+          <t>先做 T-073，再复跑 T-072</t>
         </is>
       </c>
     </row>
@@ -7785,7 +7859,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8572,6 +8646,102 @@
       <c r="F25" s="0" t="inlineStr">
         <is>
           <t>已实现：`git_diff` 输出 `[diff summary]`，包含总文件数、`+N/-M`、hunk 数和少量 added/removed 片段；百炼复测 session `20260708T100128250335Z` 已正确总结 `+1/-1`、1 hunk、本轮 README 和运行前 `review_by_myself.md`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>PT-024</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>新增，待修</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>T-072 真实实现压测 session `20260709T013441841983Z` 读取正确需求后漂移到 `deployMessage/nacos`，并把 Redis 配置注释当成需求实现锚点。</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会把任务目标、runtime state、工具证据和编辑/验证流程持续绑定；重要编辑可通过 reviewer 或 ToolChoiceQueue 纠偏。</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>下一步 T-073 增加 pre-edit relevance gate：`apply_patch` 真写入前检查目标文件是否来自近期 read/search/LSP/evidence，低相关路径要求模型重新定位或解释相关性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>PT-025</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>新增，待修</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>T-072 最终回答错误声称 worktree 无 `pom.xml` / `src`，但实际 worktree 根目录存在二者。</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会把 cwd/project context、workspace tree、active repo context 持续作为系统上下文和 runtime observation。</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>Evidence Ledger 增加 workspace-root evidence；最终回答中“无 pom/src/无法测试”类结论必须来自工具证据，否则标为未验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>PT-026</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>新增，待修</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>为无人值守压测设置 `apply_patch=allow` 后，无关 patch 被直接写入。</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 permission 和 reviewer/verification 共同降低副作用风险；权限放开不等于不做 runtime gate。</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>下一轮真实业务实现压测默认不使用 `yolo/apply_patch=allow`；若需要无人值守，必须先有 relevance gate/reviewer。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add patch relevance guard
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测，session `20260708T085927874078` 已验证 path escape roots hint、LSP 空 query guard、Current task contract 和证据路径规则，最终按 6 点结构输出；T-069/T-070 已补 `git_diff` attribution 与 diff summary，T-070 复测 session `20260708T100128250335Z` 已验证百炼模型能正确引用 summary + attribution；2026-07-09 阶段回顾后已执行 T-072 首轮真实需求实现压测，暴露无关 patch 和反事实 workspace 判断，T-073 升级为下一步：先做轻量 relevance gate / reviewer。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，下一步 T-074 处理 comment-only 低价值实现与受控新文件策略。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>full-access 后 Agent 已代跑单项目和多项目企业项目联网压测；session `20260708T085927874078` 已先读需求、纠正父目录 path escape、定位真实 `limitConstituteAllotImport` 证据，并按 6 点结构输出。T-072 首轮真实需求实现压测 session `20260709T013441841983Z` 未通过：模型漂移到 `deployMessage/nacos` 并产生无关 patch。下一步 T-073 做 relevance gate / reviewer。</t>
+          <t>T-073 已完成并复跑：session `20260709T021349259159Z` 未再触碰 `deployMessage/nacos`，也未再声称无 `pom.xml/src`；但模型退化为 JavaDoc 注释 patch，下一步 T-074 做真实实现质量 gate / safe new-file policy。</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2382,32 +2382,62 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Relevance gate / diff reviewer</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>当前 157 个测试通过</t>
+          <t>`src/local_agent/agent.py`、`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`src/local_agent/tools/relevance.py`</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>真实 apply_patch 写入前检查目标已读和低相关配置路径；workspace-root evidence 进入 Evidence Ledger；git_diff 对低相关本轮 patch 追加 reviewer 提示；patch log 归一 workspace 内绝对路径</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>T-074 做实现质量 gate</t>
         </is>
       </c>
       <c r="F49" s="0"/>
       <c r="G49" s="0"/>
       <c r="H49" s="0"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>当前 161 个测试通过</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F50" s="0"/>
+      <c r="G50" s="0"/>
+      <c r="H50" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2418,7 +2448,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J76"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5691,7 +5721,7 @@
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>已完成并复跑</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
@@ -5706,11 +5736,55 @@
       </c>
       <c r="H75" s="0" t="inlineStr">
         <is>
-          <t>写入前检查目标文件是否来自近期证据；workspace-root evidence 进入 Evidence Ledger；最终 diff reviewer 能指出变更与需求不相关并要求回滚/重定位。</t>
+          <t>已实现真实写入前 relevance gate、workspace-root evidence、diff reviewer 和 patch log 相对路径归一；复跑 session `20260709T021349259159Z` 未再触碰 `deployMessage/nacos`，也未再声称无 `pom.xml/src`。</t>
         </is>
       </c>
       <c r="I75" s="0"/>
       <c r="J75" s="0"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t>T-074</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>P7/P8</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>真实实现质量 gate / safe new-file policy</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F76" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G76" s="0" t="inlineStr">
+        <is>
+          <t>T-073 复跑证明能挡无关目录漂移，但模型在新文件权限被拒后退化为只加 JavaDoc 注释</t>
+        </is>
+      </c>
+      <c r="H76" s="0" t="inlineStr">
+        <is>
+          <t>防止 comment-only 伪实现；允许受控新文件/新目录或要求模型明确说明权限不足；复跑真实需求时应产生业务逻辑价值或诚实停止。</t>
+        </is>
+      </c>
+      <c r="I76" s="0"/>
+      <c r="J76" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5721,7 +5795,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6915,7 +6989,7 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解，继续观察</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
@@ -6925,44 +6999,44 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-073 做 pre-edit relevance gate：`apply_patch` 真写入前检查目标文件是否来自近期需求/代码证据；同时做轻量 diff reviewer。</t>
+          <t>已完成 T-073：真实写入前目标文件必须已读；代码实现任务写部署/配置类低相关路径会被拦截或要求用户确认；workspace-root evidence 和 diff reviewer 已落地；复跑未再触碰 `deployMessage/nacos`。</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>下一步 T-074 做实现质量 gate 和 safe new-file policy：comment-only patch 要被识别为文档改动，真实实现任务要么做有逻辑价值的小切片，要么诚实说明权限/依赖不足。</t>
         </is>
       </c>
     </row>
@@ -6974,7 +7048,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -6984,22 +7058,22 @@
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7085,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -7021,7 +7095,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -7031,12 +7105,12 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7122,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -7058,22 +7132,22 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7159,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -7095,7 +7169,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -7105,12 +7179,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7196,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -7132,7 +7206,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -7142,12 +7216,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7233,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7169,7 +7243,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -7179,12 +7253,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7270,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7206,7 +7280,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7216,12 +7290,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7307,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7243,7 +7317,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7253,12 +7327,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7344,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7280,22 +7354,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7381,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7317,7 +7391,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -7327,12 +7401,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7418,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7354,7 +7428,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -7364,12 +7438,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7381,7 +7455,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7391,22 +7465,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7418,32 +7492,32 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7529,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7465,22 +7539,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7566,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -7502,7 +7576,7 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -7512,12 +7586,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7603,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -7539,22 +7613,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7566,7 +7640,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -7576,22 +7650,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -7603,32 +7677,32 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -7640,32 +7714,106 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
+          <t>ADR-019</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="inlineStr">
+        <is>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+        </is>
+      </c>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
           <t>ADR-020</t>
         </is>
       </c>
-      <c r="C53" s="0" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D53" s="0" t="inlineStr">
+      <c r="D54" s="0" t="inlineStr">
         <is>
           <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
-      <c r="E53" s="0" t="inlineStr">
+      <c r="E54" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F53" s="0" t="inlineStr">
+      <c r="F54" s="0" t="inlineStr">
         <is>
           <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
-      <c r="G53" s="0" t="inlineStr">
+      <c r="G54" s="0" t="inlineStr">
         <is>
           <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>ADR-021</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t>下一步做 no-comment-only reviewer / safe new-file policy</t>
+        </is>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7829,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -7726,17 +7874,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>可以进入真实需求实现压测</t>
+          <t>真实需求压测进入“质量门”阶段</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>读、搜、改、测、diff、approval、budget、compaction、memory、todo、ask_user、Evidence Ledger、diff attribution/summary 主链路已闭环</t>
+          <t>T-073 已挡住无关配置 patch 和 workspace 反事实，但仍暴露 comment-only 伪实现</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072</t>
+          <t>执行 T-074</t>
         </is>
       </c>
     </row>
@@ -7792,17 +7940,17 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>暂不先做完整 reviewer</t>
+          <t>先做轻量实现质量 gate</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>当前还没有真实实现压测中的 patch 质量失败样本；过早实现会增加复杂度</t>
+          <t>T-073 复跑已出现 patch 质量失败样本：只加 JavaDoc 注释但声称完成实现切片</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>若 T-072 暴露 patch/总结质量不稳，再做轻量 post-diff reviewer</t>
+          <t>先做 no-comment-only reviewer，再决定是否需要完整 reviewer/subagent</t>
         </is>
       </c>
     </row>
@@ -7836,17 +7984,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>轻量 relevance gate / reviewer</t>
+          <t>实现质量 gate / safe new-file policy</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-072 首轮实现压测已证明真实实现任务可能写入无关文件</t>
+          <t>T-073 复跑证明 relevance 有效，但真实实现仍可能退化为低价值注释</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 T-073，再复跑 T-072</t>
+          <t>先做 T-074，再复跑同一需求</t>
         </is>
       </c>
     </row>
@@ -7859,7 +8007,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8662,12 +8810,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>新增，待修</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>T-072 真实实现压测 session `20260709T013441841983Z` 读取正确需求后漂移到 `deployMessage/nacos`，并把 Redis 配置注释当成需求实现锚点。</t>
+          <t>T-072 真实实现压测 session `20260709T013441841983Z` 读取正确需求后漂移到 `deployMessage/nacos`，并把 Redis 配置注释当成需求实现锚点。T-073 复跑 session `20260709T021349259159Z` 未再触碰该目录。</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -8677,7 +8825,7 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-073 增加 pre-edit relevance gate：`apply_patch` 真写入前检查目标文件是否来自近期 read/search/LSP/evidence，低相关路径要求模型重新定位或解释相关性。</t>
+          <t>已实现 pre-edit relevance gate：真实写入前目标必须已读；代码实现任务写低相关配置/部署路径会被拦或要求确认；`git_diff` 增加 reviewer 提示。</t>
         </is>
       </c>
     </row>
@@ -8694,12 +8842,12 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>新增，待修</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>T-072 最终回答错误声称 worktree 无 `pom.xml` / `src`，但实际 worktree 根目录存在二者。</t>
+          <t>T-072 最终回答错误声称 worktree 无 `pom.xml` / `src`，但实际 worktree 根目录存在二者。T-073 复跑未再出现该反事实。</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -8709,7 +8857,7 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 增加 workspace-root evidence；最终回答中“无 pom/src/无法测试”类结论必须来自工具证据，否则标为未验证。</t>
+          <t>Evidence Ledger 已增加 workspace-root evidence；最终回答中“无 pom/src/无法测试”类结论必须来自工具证据，否则标为未验证。</t>
         </is>
       </c>
     </row>
@@ -8726,22 +8874,86 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
+          <t>已缓解，继续观察</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>为无人值守压测设置 `apply_patch=allow` 后，无关 patch 被直接写入。T-073 后即使 `apply_patch=allow`，runtime relevance gate 仍会在真实写入前做目标相关性检查。</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 permission 和 reviewer/verification 共同降低副作用风险；权限放开不等于不做 runtime gate。</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>无人值守压测仍建议用临时 worktree；高风险路径需要 relevance gate/reviewer；真实业务提交前仍需人工 review。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>PT-027</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
           <t>新增，待修</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t>为无人值守压测设置 `apply_patch=allow` 后，无关 patch 被直接写入。</t>
-        </is>
-      </c>
-      <c r="E28" s="0" t="inlineStr">
-        <is>
-          <t>OMP 的 permission 和 reviewer/verification 共同降低副作用风险；权限放开不等于不做 runtime gate。</t>
-        </is>
-      </c>
-      <c r="F28" s="0" t="inlineStr">
-        <is>
-          <t>下一轮真实业务实现压测默认不使用 `yolo/apply_patch=allow`；若需要无人值守，必须先有 relevance gate/reviewer。</t>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>T-073 复跑中模型定位到相关 Java DTO，但 `write_file` 被 deny 后退化为只给字段补 JavaDoc，并把它包装成“健壮性/校验相关”实现。</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>OMP 可通过 reviewer、tool-choice queue、todo/plan consistency 和 verification 判断 patch 是否真正满足任务，而不是只看 patch 语法成功。</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>下一步 T-074 做 no-comment-only reviewer / implementation-quality gate；真实实现任务中 comment-only patch 要么标为文档改动，要么要求重新定位或停止说明权限不足。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>PT-028</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>新增，待修</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>T-073 复跑曾尝试新增 validator 注解和目录，但 `shell=deny` / `write_file=deny` 使新文件路径被拦，导致模型降级。</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 permission model 支持按工具和上下文请求权限；新文件写入应由审批/策略控制，而非一概 deny。</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>设计 safe new-file policy：已读父目录、路径在 workspace、任务需要且用户允许时，可 prompt/allow `write_file` 或专门的 create-file workflow；否则让模型明确无法安全实现。</t>
         </is>
       </c>
     </row>
@@ -8817,7 +9029,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 157 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 161 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add implementation quality guard
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,9 +101,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，下一步 T-074 处理 comment-only 低价值实现与受控新文件策略。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073/T-074 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，T-074 implementation-quality reviewer / safe new-file policy 缓解 comment-only 低价值实现与新文件权限降级。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -588,20 +588,38 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
+          <t>Implementation quality / safe new-file</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>`git_diff` 会对 comment-only 代码实现 patch 输出 reviewer warning；`write_file dry_run=true` 可预览新文件 diff，真实创建写 patch log，`rollback_patch` 可删除本 session 新建文件。</t>
+        </is>
+      </c>
+      <c r="D28" s="0"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B28" s="0" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D28" s="0"/>
+      <c r="D29" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -903,7 +921,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -918,7 +936,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>T-073 已完成并复跑：session `20260709T021349259159Z` 未再触碰 `deployMessage/nacos`，也未再声称无 `pom.xml/src`；但模型退化为 JavaDoc 注释 patch，下一步 T-074 做真实实现质量 gate / safe new-file policy。</t>
+          <t>T-074 已完成并复跑：session `20260709T025706579604Z` 未再产生 comment-only 伪实现，也未因新文件权限降级乱改；下一步补 no-edit final hygiene 或接入真实目标服务继续实现压测。</t>
         </is>
       </c>
     </row>
@@ -931,9 +949,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
@@ -2402,7 +2420,7 @@
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>T-074 做实现质量 gate</t>
+          <t>日用反馈补测</t>
         </is>
       </c>
       <c r="F49" s="0"/>
@@ -2412,32 +2430,62 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Implementation quality / safe new-file</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>当前 161 个测试通过</t>
+          <t>`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`tests/test_tools.py`</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>comment-only 代码实现 diff 会被 reviewer 标红；新文件创建支持 dry-run diff、patch log 和 rollback 删除</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>T-075 处理 no-edit final hygiene</t>
         </is>
       </c>
       <c r="F50" s="0"/>
       <c r="G50" s="0"/>
       <c r="H50" s="0"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>当前 164 个测试通过</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F51" s="0"/>
+      <c r="G51" s="0"/>
+      <c r="H51" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2448,7 +2496,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J77"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5765,7 +5813,7 @@
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>已完成并复跑</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
@@ -5780,11 +5828,55 @@
       </c>
       <c r="H76" s="0" t="inlineStr">
         <is>
-          <t>防止 comment-only 伪实现；允许受控新文件/新目录或要求模型明确说明权限不足；复跑真实需求时应产生业务逻辑价值或诚实停止。</t>
+          <t>已补 comment-only 代码实现 reviewer、`write_file dry_run=true` 新文件预览、创建文件 patch log 和 rollback 删除；复跑 session `20260709T025706579604Z` 未再产生伪实现，而是判断当前仓库不包含目标服务后诚实停止。</t>
         </is>
       </c>
       <c r="I76" s="0"/>
       <c r="J76" s="0"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t>T-075</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t>P7/P8</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t>no-edit final hygiene / 跨服务目标接入</t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F77" s="0" t="inlineStr">
+        <is>
+          <t>Agent + User</t>
+        </is>
+      </c>
+      <c r="G77" s="0" t="inlineStr">
+        <is>
+          <t>T-074 复跑说明“安全停止”有效，但 no-edit 路径没有维护 todo，也没有调用 git_diff 证明无改动；同时真实实现很可能需要 `zqyl-investment-plan` 服务源码</t>
+        </is>
+      </c>
+      <c r="H77" s="0" t="inlineStr">
+        <is>
+          <t>补停止路径收束规范；若用户提供目标服务路径，则作为 `--cwd` 或 `--allow-dir` 继续真实实现压测。</t>
+        </is>
+      </c>
+      <c r="I77" s="0"/>
+      <c r="J77" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5795,7 +5887,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7026,7 +7118,7 @@
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
@@ -7036,44 +7128,44 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-074 做实现质量 gate 和 safe new-file policy：comment-only patch 要被识别为文档改动，真实实现任务要么做有逻辑价值的小切片，要么诚实说明权限/依赖不足。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>下一步 T-075 参考 OMP current task / tool-choice steering 思路：即使选择 no-edit stop，也要输出 todo 状态、git status/diff 或明确说明无须验证。</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7177,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -7095,22 +7187,22 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7214,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -7132,7 +7224,7 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -7142,12 +7234,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7251,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -7169,22 +7261,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7288,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -7206,7 +7298,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -7216,12 +7308,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7325,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7243,7 +7335,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -7253,12 +7345,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7362,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7280,7 +7372,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7290,12 +7382,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7399,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7317,7 +7409,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7327,12 +7419,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7436,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7354,7 +7446,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7364,12 +7456,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7381,7 +7473,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7391,22 +7483,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7510,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7428,7 +7520,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -7438,12 +7530,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7547,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7465,7 +7557,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -7475,12 +7567,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7584,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7502,22 +7594,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7529,32 +7621,32 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7566,7 +7658,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -7576,22 +7668,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7603,7 +7695,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -7613,7 +7705,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -7623,12 +7715,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7732,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -7650,22 +7742,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7677,7 +7769,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -7687,22 +7779,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -7714,32 +7806,32 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7843,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -7761,7 +7853,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -7771,12 +7863,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -7788,32 +7880,106 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
+          <t>ADR-020</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+        </is>
+      </c>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
           <t>ADR-021</t>
         </is>
       </c>
-      <c r="C55" s="0" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D55" s="0" t="inlineStr">
+      <c r="D56" s="0" t="inlineStr">
         <is>
           <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
-      <c r="E55" s="0" t="inlineStr">
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="inlineStr">
+        <is>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+        </is>
+      </c>
+      <c r="G56" s="0" t="inlineStr">
+        <is>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>ADR-022</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F55" s="0" t="inlineStr">
-        <is>
-          <t>下一步做 no-comment-only reviewer / safe new-file policy</t>
-        </is>
-      </c>
-      <c r="G55" s="0" t="inlineStr">
-        <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；先补“什么算有效实现”和“何时允许新文件”。</t>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t>下一步做 T-075</t>
+        </is>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；但停止路径也需要 todo/git_diff/原因归档，不能只靠最终文字。</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7995,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -7874,17 +8040,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>真实需求压测进入“质量门”阶段</t>
+          <t>真实需求压测进入“质量门 + 收束规范”阶段</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-073 已挡住无关配置 patch 和 workspace 反事实，但仍暴露 comment-only 伪实现</t>
+          <t>T-073 已挡住无关配置 patch 和 workspace 反事实；T-074 已挡住 comment-only 伪实现，但 no-edit 停止路径仍需更可审计</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>执行 T-074</t>
+          <t>执行 T-075 或接入目标服务继续压测</t>
         </is>
       </c>
     </row>
@@ -7940,17 +8106,17 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>先做轻量实现质量 gate</t>
+          <t>先保留轻量实现质量 gate</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑已出现 patch 质量失败样本：只加 JavaDoc 注释但声称完成实现切片</t>
+          <t>T-074 已补 no-comment-only reviewer，复跑未再产生伪实现</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>先做 no-comment-only reviewer，再决定是否需要完整 reviewer/subagent</t>
+          <t>继续用真实任务验证；若后续出现更复杂 patch 质量问题，再补完整 reviewer/subagent</t>
         </is>
       </c>
     </row>
@@ -7984,17 +8150,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>实现质量 gate / safe new-file policy</t>
+          <t>no-edit final hygiene / 目标服务接入</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑证明 relevance 有效，但真实实现仍可能退化为低价值注释</t>
+          <t>T-074 复跑证明安全停止有效，但缺 todo/git_diff 收束；当前 `crcl-open` 不是需求目标服务</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 T-074，再复跑同一需求</t>
+          <t>补 T-075，或找到 `zqyl-investment-plan` 路径后继续实现压测</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8173,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8906,12 +9072,12 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>新增，待修</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑中模型定位到相关 Java DTO，但 `write_file` 被 deny 后退化为只给字段补 JavaDoc，并把它包装成“健壮性/校验相关”实现。</t>
+          <t>T-073 复跑中模型定位到相关 Java DTO，但 `write_file` 被 deny 后退化为只给字段补 JavaDoc，并把它包装成“健壮性/校验相关”实现。T-074 复跑未再产生 comment-only patch。</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
@@ -8921,7 +9087,7 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-074 做 no-comment-only reviewer / implementation-quality gate；真实实现任务中 comment-only patch 要么标为文档改动，要么要求重新定位或停止说明权限不足。</t>
+          <t>已新增 implementation-quality reviewer：本轮代码实现 diff 如果只有注释/文档，会提示不要声称行为/校验/解析/测试变化；复跑 session `20260709T025706579604Z` 选择停止而非伪实现。</t>
         </is>
       </c>
     </row>
@@ -8938,22 +9104,54 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
+          <t>已缓解并复跑</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>T-073 复跑曾尝试新增 validator 注解和目录，但 `shell=deny` / `write_file=deny` 使新文件路径被拦，导致模型降级。T-074 后新文件创建可先 dry-run，并能记录/回滚。</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的 permission model 支持按工具和上下文请求权限；新文件写入应由审批/策略控制，而非一概 deny。</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>`write_file` 支持 `dry_run=true` 新文件 diff 预览；真实创建会记录 patch log；`rollback_patch` 可删除本 session 创建的新文件。复跑中未因新文件权限降级改注释。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>PT-029</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
           <t>新增，待修</t>
         </is>
       </c>
-      <c r="D30" s="0" t="inlineStr">
-        <is>
-          <t>T-073 复跑曾尝试新增 validator 注解和目录，但 `shell=deny` / `write_file=deny` 使新文件路径被拦，导致模型降级。</t>
-        </is>
-      </c>
-      <c r="E30" s="0" t="inlineStr">
-        <is>
-          <t>OMP 的 permission model 支持按工具和上下文请求权限；新文件写入应由审批/策略控制，而非一概 deny。</t>
-        </is>
-      </c>
-      <c r="F30" s="0" t="inlineStr">
-        <is>
-          <t>设计 safe new-file policy：已读父目录、路径在 workspace、任务需要且用户允许时，可 prompt/allow `write_file` 或专门的 create-file workflow；否则让模型明确无法安全实现。</t>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>T-074 复跑中模型正确判断当前 `crcl-open` 只是 `zqyl-investment-plan` 调用方并停止，但没有维护 todo，也没有调用 `git_diff` 证明无改动。</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>OMP 会持续注入 current task / todo / tool evidence，并通过 tool-choice steering 约束最终回答前的必要收束步骤。</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>下一步 T-075：no-edit stop 也要输出 todo 状态和 git status/diff，或在最终回答中明确说明未改动且为何未运行测试。</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9227,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 161 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 164 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -9080,7 +9278,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir 和多项目只读压测主链路；下一步继续做回答准确性评估，尤其是跨项目缺失证据时的措辞和实现前二次验证。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate 和 implementation-quality gate；下一步补 no-edit final hygiene，并继续做目标服务接入后的真实实现压测。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add no-edit final hygiene
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073/T-074 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，T-074 implementation-quality reviewer / safe new-file policy 缓解 comment-only 低价值实现与新文件权限降级。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073/T-074/T-075 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，T-074 implementation-quality reviewer / safe new-file policy 缓解 comment-only 低价值实现与新文件权限降级，T-075 no-edit final hygiene 让安全停止路径也补 todo/git 收束证据。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -606,20 +606,38 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
+          <t>No-edit final hygiene</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>实现任务准备以“无法安全实现/目标服务缺失/无改动”停止时，runtime 会要求先做 todo/git 收束，并临时只开放 todo/git hygiene 工具。</t>
+        </is>
+      </c>
+      <c r="D29" s="0"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B29" s="0" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C29" s="0" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D29" s="0"/>
+      <c r="D30" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -921,7 +939,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy、no-edit final hygiene</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -936,7 +954,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>T-074 已完成并复跑：session `20260709T025706579604Z` 未再产生 comment-only 伪实现，也未因新文件权限降级乱改；下一步补 no-edit final hygiene 或接入真实目标服务继续实现压测。</t>
+          <t>T-075 已完成 MVP 版；下一步接入真实目标服务继续实现压测，或复跑 T-074 no-edit 场景验证收束表现。</t>
         </is>
       </c>
     </row>
@@ -949,7 +967,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2450,7 +2468,7 @@
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>T-075 处理 no-edit final hygiene</t>
+          <t>真实目标服务压测</t>
         </is>
       </c>
       <c r="F50" s="0"/>
@@ -2460,32 +2478,62 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>No-edit final hygiene</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>当前 164 个测试通过</t>
+          <t>`src/local_agent/agent.py`、`tests/test_agent.py`</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>Provider context 提前说明无改动停止要可审计；runtime 发现过早 no-edit final 时追加 steering，并限制下一轮工具到 todo/git 收束集合</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>真实目标服务压测</t>
         </is>
       </c>
       <c r="F51" s="0"/>
       <c r="G51" s="0"/>
       <c r="H51" s="0"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>当前 166 个测试通过</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F52" s="0"/>
+      <c r="G52" s="0"/>
+      <c r="H52" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5857,7 +5905,7 @@
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
@@ -5872,7 +5920,7 @@
       </c>
       <c r="H77" s="0" t="inlineStr">
         <is>
-          <t>补停止路径收束规范；若用户提供目标服务路径，则作为 `--cwd` 或 `--allow-dir` 继续真实实现压测。</t>
+          <t>已补 provider context 和 runtime steering：过早 no-edit final 会被要求先做 todo/git hygiene。下一步接入目标服务路径继续真实实现压测。</t>
         </is>
       </c>
       <c r="I77" s="0"/>
@@ -7155,7 +7203,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -7165,7 +7213,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-075 参考 OMP current task / tool-choice steering 思路：即使选择 no-edit stop，也要输出 todo 状态、git status/diff 或明确说明无须验证。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -7969,17 +8017,17 @@
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>下一步做 T-075</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；但停止路径也需要 todo/git_diff/原因归档，不能只靠最终文字。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -7995,7 +8043,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -8040,17 +8088,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>真实需求压测进入“质量门 + 收束规范”阶段</t>
+          <t>真实需求压测进入“目标服务验证”阶段</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-073 已挡住无关配置 patch 和 workspace 反事实；T-074 已挡住 comment-only 伪实现，但 no-edit 停止路径仍需更可审计</t>
+          <t>T-073 已挡住无关配置 patch 和 workspace 反事实；T-074 已挡住 comment-only 伪实现；T-075 已补 no-edit 停止收束</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>执行 T-075 或接入目标服务继续压测</t>
+          <t>接入目标服务继续压测</t>
         </is>
       </c>
     </row>
@@ -8150,17 +8198,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>no-edit final hygiene / 目标服务接入</t>
+          <t>目标服务接入</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑证明安全停止有效，但缺 todo/git_diff 收束；当前 `crcl-open` 不是需求目标服务</t>
+          <t>当前 `crcl-open` 不是需求目标服务；T-075 已补安全停止收束</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>补 T-075，或找到 `zqyl-investment-plan` 路径后继续实现压测</t>
+          <t>找到 `zqyl-investment-plan` 路径后继续实现压测</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9184,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>新增，待修</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -9151,7 +9199,7 @@
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>下一步 T-075：no-edit stop 也要输出 todo 状态和 git status/diff，或在最终回答中明确说明未改动且为何未运行测试。</t>
+          <t>T-075 已实现 no-edit final hygiene：实现任务准备无改动停止时，会先要求 todo/git 收束；测试覆盖过早 final 被 steering 到 `todo_add` + `git_status`。</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9275,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 164 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 166 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9326,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate 和 implementation-quality gate；下一步补 no-edit final hygiene，并继续做目标服务接入后的真实实现压测。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate 和 no-edit final hygiene；下一步继续做目标服务接入后的真实实现压测。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add event command protocol
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P7：轻量高级能力与真实压测</t>
+          <t>P8：前端协议与交互基础</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、authored skills discovery，并通过综合压测发现和修复重复工具调用循环，新增 OMP 风格 tool result pruning / todo steering；2026-07-08 已按 OMP 思路完成 runtime state 与 cwd 分层，自动 memory consolidation 默认写 state dir；full-access 后 Agent 已代跑单项目和多项目企业压测；T-069/T-070 已补 `git_diff` attribution 与 diff summary；2026-07-09 已完成 T-072/T-073/T-074/T-075 真实需求实现压测闭环：T-073 relevance gate / reviewer 缓解无关配置 patch 和反事实 workspace 判断，T-074 implementation-quality reviewer / safe new-file policy 缓解 comment-only 低价值实现与新文件权限降级，T-075 no-edit final hygiene 让安全停止路径也补 todo/git 收束证据。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1，Runtime 开始产出 typed events，CLI 的 session/tool 日志由 `StderrEventSink` 渲染，session JSONL 追加 `event_v1` 供后续 replay；下一步 T-077 做 terminal-native frontend。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -624,20 +624,38 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
+          <t>Event/Command Protocol</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>`src/local_agent/protocol/events.py` / `commands.py` 提供 dataclass event/command shape；Runtime 可注入 `EventSink`，CLI 使用 `StderrEventSink` 渲染，session JSONL 写入 `event_v1`。</t>
+        </is>
+      </c>
+      <c r="D30" s="0"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B30" s="0" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C30" s="0" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D30" s="0"/>
+      <c r="D31" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -648,7 +666,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -944,17 +962,49 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>高级轻量能力主线已收口，后续按真实压测失败形态补 path-scoped rules、完整 reviewer 或 ToolChoiceQueue。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>前端协议与交互基础</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Event/Command Protocol、event replay、terminal-native frontend</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
           <t>进行中</t>
         </is>
       </c>
-      <c r="E10" s="0" t="inlineStr">
-        <is>
-          <t>99%</t>
-        </is>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t>T-075 已完成 MVP 版；下一步接入真实目标服务继续实现压测，或复跑 T-074 no-edit 场景验证收束表现。</t>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>T-076 已完成协议层；下一步做 T-077 `prompt_toolkit + rich` Terminal Frontend MVP。</t>
         </is>
       </c>
     </row>
@@ -967,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H53"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2508,32 +2558,62 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Event/Command Protocol</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>当前 166 个测试通过</t>
+          <t>`src/local_agent/protocol/events.py`、`src/local_agent/protocol/commands.py`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>Runtime 产出 typed events，CLI 通过 stderr sink 渲染，session JSONL 写入 `event_v1`，命令协议 shape 已固化</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>T-077 接 Terminal Frontend</t>
         </is>
       </c>
       <c r="F52" s="0"/>
       <c r="G52" s="0"/>
       <c r="H52" s="0"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>当前 171 个测试通过</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F53" s="0"/>
+      <c r="G53" s="0"/>
+      <c r="H53" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2544,7 +2624,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J79"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -5926,6 +6006,94 @@
       <c r="I77" s="0"/>
       <c r="J77" s="0"/>
     </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t>T-076</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="D78" s="0" t="inlineStr">
+        <is>
+          <t>Event/Command Protocol v1</t>
+        </is>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F78" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G78" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime/TUI engine 分层，先让 Runtime 产出 replayable typed events，避免后续 terminal frontend 继续窥探 print/stderr</t>
+        </is>
+      </c>
+      <c r="H78" s="0" t="inlineStr">
+        <is>
+          <t>已新增 dataclass `AgentEvent` / `AgentCommand`、`EventEmitter` / `EventSink` / `StderrEventSink`；`AgentRuntime` 写 session `event_v1` 并通过事件渲染 session/tool 日志；测试覆盖协议 shape 和 runtime event stream。</t>
+        </is>
+      </c>
+      <c r="I78" s="0"/>
+      <c r="J78" s="0"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t>T-077</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Frontend MVP</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F79" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G79" s="0" t="inlineStr">
+        <is>
+          <t>用户希望更自然的一键交互；事件协议已就绪，可以做 terminal-native interactive frontend</t>
+        </is>
+      </c>
+      <c r="H79" s="0" t="inlineStr">
+        <is>
+          <t>使用 `prompt_toolkit` 负责输入、多行编辑、历史和快捷键，`rich` 负责 assistant/tool/diff/error/todo/approval 输出；保留原生 scrollback，不做 fullscreen TUI。</t>
+        </is>
+      </c>
+      <c r="I79" s="0"/>
+      <c r="J79" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5935,7 +6103,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G59"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7220,37 +7388,37 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7430,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -7272,22 +7440,22 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7467,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -7309,7 +7477,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -7319,12 +7487,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7336,7 +7504,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -7346,22 +7514,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7541,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7383,7 +7551,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -7393,12 +7561,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7578,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7420,7 +7588,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7430,12 +7598,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7615,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7457,7 +7625,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7467,12 +7635,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7652,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7494,7 +7662,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7504,12 +7672,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7521,7 +7689,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7531,7 +7699,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -7541,12 +7709,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7726,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7568,22 +7736,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7763,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7605,7 +7773,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -7615,12 +7783,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7800,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7642,7 +7810,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -7652,12 +7820,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7669,7 +7837,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7679,22 +7847,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7706,32 +7874,32 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7911,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -7753,22 +7921,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7948,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -7790,7 +7958,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -7800,12 +7968,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -7817,7 +7985,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -7827,22 +7995,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -7854,7 +8022,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -7864,22 +8032,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -7891,32 +8059,32 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -7928,7 +8096,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -7938,7 +8106,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -7948,12 +8116,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -7965,7 +8133,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -7975,22 +8143,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8002,32 +8170,106 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
+          <t>ADR-021</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+        </is>
+      </c>
+      <c r="G57" s="0" t="inlineStr">
+        <is>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
           <t>ADR-022</t>
         </is>
       </c>
-      <c r="C57" s="0" t="inlineStr">
+      <c r="C58" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D57" s="0" t="inlineStr">
+      <c r="D58" s="0" t="inlineStr">
         <is>
           <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
-      <c r="E57" s="0" t="inlineStr">
+      <c r="E58" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F57" s="0" t="inlineStr">
+      <c r="F58" s="0" t="inlineStr">
         <is>
           <t>已完成 T-075</t>
         </is>
       </c>
-      <c r="G57" s="0" t="inlineStr">
+      <c r="G58" s="0" t="inlineStr">
         <is>
           <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>ADR-024</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-076</t>
+        </is>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -8088,17 +8330,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>真实需求压测进入“目标服务验证”阶段</t>
+          <t>P8 前端协议基础已启动</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-073 已挡住无关配置 patch 和 workspace 反事实；T-074 已挡住 comment-only 伪实现；T-075 已补 no-edit 停止收束</t>
+          <t>T-076 已让 Runtime 产出 typed events，后续交互层可复用同一事件流</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>接入目标服务继续压测</t>
+          <t>先做 Terminal Frontend MVP，再按用户项目边界进入目标项目分析</t>
         </is>
       </c>
     </row>
@@ -8198,17 +8440,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>目标服务接入</t>
+          <t>Terminal Frontend MVP</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>当前 `crcl-open` 不是需求目标服务；T-075 已补安全停止收束</t>
+          <t>Event/Command Protocol 已完成，用户后续会给项目边界定义再做目标项目分析</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>找到 `zqyl-investment-plan` 路径后继续实现压测</t>
+          <t>做 T-077：`prompt_toolkit + rich` 的 terminal-native frontend</t>
         </is>
       </c>
     </row>
@@ -9215,7 +9457,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9275,7 +9517,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P7 当前代码已跑通 166 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P8 当前代码已跑通 171 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -9321,12 +9563,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>P7 轻量高级能力真实压测后续</t>
+          <t>P8 前端协议与交互基础</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate 和 no-edit final hygiene；下一步继续做目标服务接入后的真实实现压测。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene 和 Event/Command Protocol；下一步做 Terminal Frontend MVP。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add terminal frontend MVP
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P8：前端协议与交互基础</t>
+          <t>P8：前端协议与交互基础 MVP 已完成</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1，Runtime 开始产出 typed events，CLI 的 session/tool 日志由 `StderrEventSink` 渲染，session JSONL 追加 `event_v1` 供后续 replay；下一步 T-077 做 terminal-native frontend。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1 和 T-077 Terminal Frontend MVP，Runtime 产出 typed events，CLI/session/tool 日志和 terminal frontend 共用事件流，session JSONL 追加 `event_v1` 供后续 replay。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -642,20 +642,38 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
+          <t>Terminal Frontend</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>`./agent`、`./agent --chat`、`./agent chat` 进入 terminal-native 交互；可选 `prompt_toolkit` / `rich` 增强输入和输出，缺失时降级。</t>
+        </is>
+      </c>
+      <c r="D31" s="0"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B31" s="0" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C31" s="0" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D31" s="0"/>
+      <c r="D32" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -994,17 +1012,17 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>T-076 已完成协议层；下一步做 T-077 `prompt_toolkit + rich` Terminal Frontend MVP。</t>
+          <t>T-076/T-077 已完成；完整 async command bus 和更重 UI 后置，下一步按用户项目边界做项目清单分析压测。</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H54"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2588,32 +2606,62 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Terminal Frontend</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>当前 171 个测试通过</t>
+          <t>`src/local_agent/frontends/terminal/`、`src/local_agent/cli.py`</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>append-only 交互前端，`./agent` / `--chat` / `chat` 入口，可选 `prompt_toolkit` / `rich`，approval events 可见</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>真实交互压测</t>
         </is>
       </c>
       <c r="F53" s="0"/>
       <c r="G53" s="0"/>
       <c r="H53" s="0"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>当前 178 个测试通过</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F54" s="0"/>
+      <c r="G54" s="0"/>
+      <c r="H54" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2624,7 +2672,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J80"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6073,7 +6121,7 @@
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
@@ -6088,11 +6136,55 @@
       </c>
       <c r="H79" s="0" t="inlineStr">
         <is>
-          <t>使用 `prompt_toolkit` 负责输入、多行编辑、历史和快捷键，`rich` 负责 assistant/tool/diff/error/todo/approval 输出；保留原生 scrollback，不做 fullscreen TUI。</t>
+          <t>`./agent`、`./agent --chat`、`./agent chat` 可进入交互；可选 `prompt_toolkit` 提供多行输入/历史，`rich` 提供结构化输出；缺依赖时降级；保留原生 scrollback，不做 fullscreen TUI。</t>
         </is>
       </c>
       <c r="I79" s="0"/>
       <c r="J79" s="0"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>T-078</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t>P8/P9</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t>项目边界驱动的项目清单分析压测</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F80" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G80" s="0" t="inlineStr">
+        <is>
+          <t>用户后续会给项目边界定义；先让 LCA 分析某需求需要哪些项目/服务/目录，再接入具体目标项目做需求实现设计</t>
+        </is>
+      </c>
+      <c r="H80" s="0" t="inlineStr">
+        <is>
+          <t>用 LCA 在只读模式读取边界定义和现有项目结构，输出“需要接入项目清单、证据路径、缺口和下一步分析命令”。</t>
+        </is>
+      </c>
+      <c r="I80" s="0"/>
+      <c r="J80" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6103,7 +6195,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7425,37 +7517,37 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -7467,7 +7559,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -7477,22 +7569,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7596,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -7514,7 +7606,7 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -7524,12 +7616,12 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7633,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7551,22 +7643,22 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7578,7 +7670,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7588,7 +7680,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -7598,12 +7690,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7615,7 +7707,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7625,7 +7717,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -7635,12 +7727,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7652,7 +7744,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7662,7 +7754,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7672,12 +7764,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7689,7 +7781,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7699,7 +7791,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -7709,12 +7801,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7818,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7736,7 +7828,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -7746,12 +7838,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7763,7 +7855,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7773,22 +7865,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7800,7 +7892,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7810,7 +7902,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -7820,12 +7912,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7929,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7847,7 +7939,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -7857,12 +7949,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -7874,7 +7966,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -7884,22 +7976,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -7911,32 +8003,32 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -7948,7 +8040,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -7958,22 +8050,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -7985,7 +8077,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -7995,7 +8087,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -8005,12 +8097,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8022,7 +8114,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8032,22 +8124,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -8059,7 +8151,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8069,22 +8161,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -8096,32 +8188,32 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -8133,7 +8225,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -8143,7 +8235,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -8153,12 +8245,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -8170,7 +8262,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -8180,22 +8272,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8207,7 +8299,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -8217,7 +8309,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -8227,12 +8319,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -8244,32 +8336,106 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
+          <t>ADR-022</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-075</t>
+        </is>
+      </c>
+      <c r="G59" s="0" t="inlineStr">
+        <is>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
           <t>ADR-024</t>
         </is>
       </c>
-      <c r="C59" s="0" t="inlineStr">
+      <c r="C60" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D59" s="0" t="inlineStr">
+      <c r="D60" s="0" t="inlineStr">
         <is>
           <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
-      <c r="E59" s="0" t="inlineStr">
+      <c r="E60" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F59" s="0" t="inlineStr">
+      <c r="F60" s="0" t="inlineStr">
         <is>
           <t>已完成 T-076</t>
         </is>
       </c>
-      <c r="G59" s="0" t="inlineStr">
+      <c r="G60" s="0" t="inlineStr">
         <is>
           <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>ADR-025</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-077</t>
+        </is>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -8330,17 +8496,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>P8 前端协议基础已启动</t>
+          <t>P8 前端协议基础 MVP 已完成</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076 已让 Runtime 产出 typed events，后续交互层可复用同一事件流</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先做 Terminal Frontend MVP，再按用户项目边界进入目标项目分析</t>
+          <t>按用户项目边界进入目标项目分析</t>
         </is>
       </c>
     </row>
@@ -8440,17 +8606,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP</t>
+          <t>项目边界分析压测</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>Event/Command Protocol 已完成，用户后续会给项目边界定义再做目标项目分析</t>
+          <t>用户后续会给项目边界定义，再让 LCA 分析目标需求需要哪些项目</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>做 T-077：`prompt_toolkit + rich` 的 terminal-native frontend</t>
+          <t>做 T-078：只读分析项目边界，输出需要接入的项目/服务/目录清单</t>
         </is>
       </c>
     </row>
@@ -9457,7 +9623,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9517,7 +9683,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P8 当前代码已跑通 171 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P8 当前代码已跑通 178 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -9563,12 +9729,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>P8 前端协议与交互基础</t>
+          <t>项目边界分析与真实需求设计压测</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene 和 Event/Command Protocol；下一步做 Terminal Frontend MVP。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、Event/Command Protocol 和 Terminal Frontend MVP；下一步按用户提供的项目边界定义，让 LCA 先分析具体需要哪些项目。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve analysis skill steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -7,7 +7,7 @@
     <sheet name="已完成功能" sheetId="3" r:id="rId3"/>
     <sheet name="下一步 Todo" sheetId="4" r:id="rId4"/>
     <sheet name="风险与决策" sheetId="5" r:id="rId5"/>
-    <sheet name="P7 阶段回顾" sheetId="6" r:id="rId6"/>
+    <sheet name="阶段回顾" sheetId="6" r:id="rId6"/>
     <sheet name="P7 综合压测问题" sheetId="7" r:id="rId7"/>
     <sheet name="P5 收口结论" sheetId="8" r:id="rId8"/>
     <sheet name="推荐工作流" sheetId="9" r:id="rId9"/>
@@ -101,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P8：前端协议与交互基础 MVP 已完成</t>
+          <t>P9：真实需求使用准备</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1 和 T-077 Terminal Frontend MVP，Runtime 产出 typed events，CLI/session/tool 日志和 terminal frontend 共用事件流，session JSONL 追加 `event_v1` 供后续 replay。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077 Terminal Frontend MVP 和 T-078 项目边界分析 MVP。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -660,20 +660,38 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
+          <t>项目边界分析</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界和项目范围分析工作流放入本机 `.local-agent/memory` / `.local-agent/skills`；runtime 新增 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
+        </is>
+      </c>
+      <c r="D32" s="0"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B32" s="0" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D32" s="0"/>
+      <c r="D33" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -684,7 +702,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1026,6 +1044,38 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>真实需求使用准备</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>项目边界分析、用户确认项目范围、源码验证、实现设计</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>T-078 已完成项目边界分析 MVP；下一步跑真实需求“范围确认 → 源码验证”。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1035,7 +1085,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2636,32 +2686,62 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>项目边界分析</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>当前 178 个测试通过</t>
+          <t>`.local-agent/memory/enterprise-service-boundary.md`、`.local-agent/skills/project-scope-analysis/SKILL.md`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>只根据需求和服务边界圈项目范围；analysis-only 不走实现 hygiene；点名 skill 会先读正文；缺表格/段落会强制无工具重答</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>用真实需求继续压测</t>
         </is>
       </c>
       <c r="F54" s="0"/>
       <c r="G54" s="0"/>
       <c r="H54" s="0"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>当前 184 个测试通过</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F55" s="0"/>
+      <c r="G55" s="0"/>
+      <c r="H55" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2672,7 +2752,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J81"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6165,7 +6245,7 @@
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="F80" s="0" t="inlineStr">
@@ -6175,16 +6255,60 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>用户后续会给项目边界定义；先让 LCA 分析某需求需要哪些项目/服务/目录，再接入具体目标项目做需求实现设计</t>
+          <t>用户给出部门/业务线/负责服务边界，目标是先让 LCA 判断某需求需要关注哪些项目/服务，再接入源码</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
         <is>
-          <t>用 LCA 在只读模式读取边界定义和现有项目结构，输出“需要接入项目清单、证据路径、缺口和下一步分析命令”。</t>
+          <t>已按 OMP memory/skill 思路落地：边界表在本机 `.local-agent/memory`，工作流在 `.local-agent/skills`，不新增专用工具；runtime 补 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
         </is>
       </c>
       <c r="I80" s="0"/>
       <c r="J80" s="0"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t>T-079</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t>真实需求范围确认到源码验证压测</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+      <c r="F81" s="0" t="inlineStr">
+        <is>
+          <t>User + Agent</t>
+        </is>
+      </c>
+      <c r="G81" s="0" t="inlineStr">
+        <is>
+          <t>用户希望今天用起来；T-078 已能圈范围，下一步要验证它能从范围进入具体源码证据和实现设计</t>
+        </is>
+      </c>
+      <c r="H81" s="0" t="inlineStr">
+        <is>
+          <t>用户给一个真实需求，LCA 先输出项目范围表；用户确认后，用 `--cwd/--allow-dir` 接入候选项目源码，只读验证 API/controller/entity/test 证据。</t>
+        </is>
+      </c>
+      <c r="I81" s="0"/>
+      <c r="J81" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6195,7 +6319,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G64"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7554,74 +7678,74 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -7633,7 +7757,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -7643,22 +7767,22 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7670,7 +7794,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -7680,22 +7804,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7707,7 +7831,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7717,22 +7841,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7868,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7754,7 +7878,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -7764,12 +7888,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7905,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7791,7 +7915,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -7801,12 +7925,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -7818,7 +7942,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7828,7 +7952,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -7838,12 +7962,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -7855,7 +7979,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7865,7 +7989,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -7875,12 +7999,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -7892,7 +8016,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7902,22 +8026,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -7929,7 +8053,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -7939,22 +8063,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -7966,7 +8090,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -7976,7 +8100,7 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -7986,12 +8110,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -8003,7 +8127,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8013,22 +8137,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -8040,32 +8164,32 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -8077,32 +8201,32 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8238,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8124,22 +8248,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8275,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8161,22 +8285,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8312,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8198,7 +8322,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -8208,12 +8332,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -8225,17 +8349,17 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -8245,12 +8369,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -8262,32 +8386,32 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -8299,7 +8423,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -8309,22 +8433,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -8336,7 +8460,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -8346,22 +8470,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8497,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -8383,7 +8507,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -8393,12 +8517,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -8410,32 +8534,143 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
+          <t>ADR-022</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-075</t>
+        </is>
+      </c>
+      <c r="G61" s="0" t="inlineStr">
+        <is>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>ADR-024</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F62" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-076</t>
+        </is>
+      </c>
+      <c r="G62" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
           <t>ADR-025</t>
         </is>
       </c>
-      <c r="C61" s="0" t="inlineStr">
+      <c r="C63" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D61" s="0" t="inlineStr">
+      <c r="D63" s="0" t="inlineStr">
         <is>
           <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
-      <c r="E61" s="0" t="inlineStr">
+      <c r="E63" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F61" s="0" t="inlineStr">
+      <c r="F63" s="0" t="inlineStr">
         <is>
           <t>已完成 T-077</t>
         </is>
       </c>
-      <c r="G61" s="0" t="inlineStr">
+      <c r="G63" s="0" t="inlineStr">
         <is>
           <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>ADR-026</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-078</t>
+        </is>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -8459,7 +8694,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P7 阶段回顾</t>
+          <t>阶段回顾</t>
         </is>
       </c>
       <c r="B1" s="1"/>
@@ -8496,17 +8731,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>P8 前端协议基础 MVP 已完成</t>
+          <t>P9 真实需求使用准备进行中</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>按用户项目边界进入目标项目分析</t>
+          <t>进入真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -8606,17 +8841,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析压测</t>
+          <t>真实需求范围确认到源码验证压测</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>用户后续会给项目边界定义，再让 LCA 分析目标需求需要哪些项目</t>
+          <t>用户已给服务边界，T-078 已完成项目边界分析 MVP</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>做 T-078：只读分析项目边界，输出需要接入的项目/服务/目录清单</t>
+          <t>做 T-079：先用边界圈项目范围，用户确认后接入候选项目源码，只读验证 API/controller/entity/test 证据并形成实现设计</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9858,7 @@
   <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9683,7 +9918,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P8 当前代码已跑通 178 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 184 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -9729,12 +9964,12 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析与真实需求设计压测</t>
+          <t>真实需求设计与实现压测</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、Event/Command Protocol 和 Terminal Frontend MVP；下一步按用户提供的项目边界定义，让 LCA 先分析具体需要哪些项目。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve terminal frontend usability
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077 Terminal Frontend MVP 和 T-078 项目边界分析 MVP。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`./agent`、`./agent --chat`、`./agent chat` 进入 terminal-native 交互；可选 `prompt_toolkit` / `rich` 增强输入和输出，缺失时降级。</t>
+          <t>`./agent`、`./agent --chat`、`./agent chat` 进入 terminal-native 交互；可选 `prompt_toolkit` / `rich` 增强输入和输出，缺失时降级；支持 `/help`、`/status`、`/tools`、`/approval`。</t>
         </is>
       </c>
       <c r="D31" s="0"/>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>当前 184 个测试通过</t>
+          <t>当前 188 个测试通过</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
@@ -2752,7 +2752,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J83"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6310,6 +6310,94 @@
       <c r="I81" s="0"/>
       <c r="J81" s="0"/>
     </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t>T-080</t>
+        </is>
+      </c>
+      <c r="B82" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C82" s="0" t="inlineStr">
+        <is>
+          <t>P8/P9</t>
+        </is>
+      </c>
+      <c r="D82" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Frontend 命令可发现性</t>
+        </is>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="F82" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G82" s="0" t="inlineStr">
+        <is>
+          <t>用户询问 TUI 如何使用；设计文档要求 append-only terminal frontend，但现有命令入口不够自解释</t>
+        </is>
+      </c>
+      <c r="H82" s="0" t="inlineStr">
+        <is>
+          <t>已新增 `/help`、`/status`、`/tools`，启动横幅提示 `/help`；`/status` 输出 session/workspace/provider/model/budget/approval，`/tools` 列出工具名；不引入 fullscreen 或新依赖。</t>
+        </is>
+      </c>
+      <c r="I82" s="0"/>
+      <c r="J82" s="0"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t>T-081</t>
+        </is>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D83" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 行动计划</t>
+        </is>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F83" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G83" s="0" t="inlineStr">
+        <is>
+          <t>外部 review 指出 agent.py 过大、token budget、LSP、run collector 等架构差距；需要沉淀取舍，避免聊天结论丢失</t>
+        </is>
+      </c>
+      <c r="H83" s="0" t="inlineStr">
+        <is>
+          <t>新增 `docs/claude-review-action-plan-2026-07-09.md`；结论为先做日用/TUI/run summary，再按压测数据渐进拆模块，不先做大重构。</t>
+        </is>
+      </c>
+      <c r="I83" s="0"/>
+      <c r="J83" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -6319,7 +6407,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G67"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7752,74 +7840,74 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7919,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -7841,22 +7929,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7956,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7878,22 +7966,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7993,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -7915,22 +8003,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -7942,7 +8030,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -7952,7 +8040,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -7962,12 +8050,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -7979,7 +8067,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -7989,7 +8077,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -7999,12 +8087,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8016,7 +8104,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -8026,7 +8114,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -8036,12 +8124,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8141,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -8063,7 +8151,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -8073,12 +8161,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -8090,7 +8178,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -8100,22 +8188,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -8127,7 +8215,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8137,22 +8225,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -8164,7 +8252,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8174,7 +8262,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -8184,12 +8272,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -8201,7 +8289,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8211,22 +8299,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -8238,32 +8326,32 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -8275,32 +8363,32 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8400,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8322,22 +8410,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -8349,7 +8437,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -8359,22 +8447,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8386,7 +8474,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -8396,7 +8484,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -8406,12 +8494,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -8423,17 +8511,17 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -8443,12 +8531,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -8460,32 +8548,32 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -8497,7 +8585,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -8507,22 +8595,22 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -8534,7 +8622,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -8544,22 +8632,22 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8659,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -8581,7 +8669,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -8591,12 +8679,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -8608,7 +8696,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -8618,7 +8706,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -8628,12 +8716,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -8645,32 +8733,143 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
+          <t>ADR-024</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-076</t>
+        </is>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>ADR-025</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-077</t>
+        </is>
+      </c>
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
           <t>ADR-026</t>
         </is>
       </c>
-      <c r="C64" s="0" t="inlineStr">
+      <c r="C66" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D64" s="0" t="inlineStr">
+      <c r="D66" s="0" t="inlineStr">
         <is>
           <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
-      <c r="E64" s="0" t="inlineStr">
+      <c r="E66" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F64" s="0" t="inlineStr">
+      <c r="F66" s="0" t="inlineStr">
         <is>
           <t>已完成 T-078</t>
         </is>
       </c>
-      <c r="G64" s="0" t="inlineStr">
+      <c r="G66" s="0" t="inlineStr">
         <is>
           <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>ADR-027</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F67" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-081</t>
+        </is>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -9918,7 +10117,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 184 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 188 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add run summary coverage
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -101,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -660,7 +660,7 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析</t>
+          <t>Run summary / coverage</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界和项目范围分析工作流放入本机 `.local-agent/memory` / `.local-agent/skills`；runtime 新增 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
+          <t>每轮结束写 `run_summary` session 事件和 `RunSummary` typed event；`/status` 可看最近一轮终止原因、LLM/工具次数、guard/steering/compaction 统计。</t>
         </is>
       </c>
       <c r="D32" s="0"/>
@@ -678,20 +678,38 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
+          <t>项目边界分析</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界和项目范围分析工作流放入本机 `.local-agent/memory` / `.local-agent/skills`；runtime 新增 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
+        </is>
+      </c>
+      <c r="D33" s="0"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B33" s="0" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C33" s="0" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D33" s="0"/>
+      <c r="D34" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2752,7 +2770,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6398,6 +6416,50 @@
       <c r="I83" s="0"/>
       <c r="J83" s="0"/>
     </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t>T-082</t>
+        </is>
+      </c>
+      <c r="B84" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C84" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D84" s="0" t="inlineStr">
+        <is>
+          <t>Run summary / coverage MVP</t>
+        </is>
+      </c>
+      <c r="E84" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F84" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G84" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 和 OMP run-collector 思路都要求每轮可观测，压测复盘不能只靠最终文字</t>
+        </is>
+      </c>
+      <c r="H84" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 已记录 `run_summary` 和 `RunSummary` event，包含终止原因、耗时、LLM 请求数、工具调用/错误/无效结果、synthetic result、compaction、tool counts、guard hits 和 steering counts；`/status` 展示最近一轮摘要。</t>
+        </is>
+      </c>
+      <c r="I84" s="0"/>
+      <c r="J84" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -6407,7 +6469,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G69"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7914,37 +7976,37 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -7956,7 +8018,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -7966,22 +8028,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -7993,7 +8055,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -8003,7 +8065,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -8013,12 +8075,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8092,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -8040,22 +8102,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -8067,7 +8129,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -8077,7 +8139,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -8087,12 +8149,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8166,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -8114,7 +8176,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -8124,12 +8186,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8203,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -8151,7 +8213,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -8161,12 +8223,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -8178,7 +8240,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -8188,7 +8250,7 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -8198,12 +8260,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8277,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8225,7 +8287,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -8235,12 +8297,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -8252,7 +8314,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8262,22 +8324,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -8289,7 +8351,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8299,7 +8361,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -8309,12 +8371,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -8326,7 +8388,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8336,7 +8398,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -8346,12 +8408,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -8363,7 +8425,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8373,22 +8435,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -8400,32 +8462,32 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -8437,7 +8499,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -8447,22 +8509,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8536,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -8484,7 +8546,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -8494,12 +8556,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8573,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -8521,22 +8583,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -8548,7 +8610,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -8558,22 +8620,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -8585,32 +8647,32 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8684,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -8632,7 +8694,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -8642,12 +8704,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -8659,7 +8721,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -8669,22 +8731,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8758,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -8706,7 +8768,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -8716,12 +8778,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -8733,7 +8795,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -8743,7 +8805,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -8753,12 +8815,12 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -8770,7 +8832,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -8780,7 +8842,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -8790,12 +8852,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -8807,7 +8869,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -8817,7 +8879,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -8827,12 +8889,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -8844,32 +8906,106 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
+          <t>ADR-026</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F67" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-078</t>
+        </is>
+      </c>
+      <c r="G67" s="0" t="inlineStr">
+        <is>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
           <t>ADR-027</t>
         </is>
       </c>
-      <c r="C67" s="0" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D67" s="0" t="inlineStr">
+      <c r="D68" s="0" t="inlineStr">
         <is>
           <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
-      <c r="E67" s="0" t="inlineStr">
+      <c r="E68" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F67" s="0" t="inlineStr">
+      <c r="F68" s="0" t="inlineStr">
         <is>
           <t>已完成 T-081</t>
         </is>
       </c>
-      <c r="G67" s="0" t="inlineStr">
+      <c r="G68" s="0" t="inlineStr">
         <is>
           <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>ADR-028</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-082</t>
+        </is>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record qwen coder pressure test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板和 T-084 qwen3-coder-next 企业项目只读源码验证压测。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -1085,12 +1085,12 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>T-078 已完成项目边界分析 MVP；下一步跑真实需求“范围确认 → 源码验证”。</t>
+          <t>T-078 已完成项目边界分析 MVP；T-083 已固化压测模板；T-084 已完成 qwen3-coder-next 只读源码验证压测并记录新问题。</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J89"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6307,7 +6307,7 @@
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
-          <t>下一步</t>
+          <t>进行中</t>
         </is>
       </c>
       <c r="F81" s="0" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="H81" s="0" t="inlineStr">
         <is>
-          <t>用户给一个真实需求，LCA 先输出项目范围表；用户确认后，用 `--cwd/--allow-dir` 接入候选项目源码，只读验证 API/controller/entity/test 证据。</t>
+          <t>T-084 已完成一轮上线目录 SQL → 源码证据的只读验证；下一步补 T-085~T-087 后继续真实需求链路。</t>
         </is>
       </c>
       <c r="I81" s="0"/>
@@ -6459,6 +6459,226 @@
       </c>
       <c r="I84" s="0"/>
       <c r="J84" s="0"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t>T-083</t>
+        </is>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C85" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D85" s="0" t="inlineStr">
+        <is>
+          <t>真实需求压测模板</t>
+        </is>
+      </c>
+      <c r="E85" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F85" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G85" s="0" t="inlineStr">
+        <is>
+          <t>真实需求链路需要可复用步骤，否则每次压测都靠聊天记忆</t>
+        </is>
+      </c>
+      <c r="H85" s="0" t="inlineStr">
+        <is>
+          <t>新增 `docs/real-requirement-pressure-test-template.md`，覆盖范围判断、用户确认、源码只读验证、实现设计、小改压测、run summary 和问题记录。</t>
+        </is>
+      </c>
+      <c r="I85" s="0"/>
+      <c r="J85" s="0"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t>T-084</t>
+        </is>
+      </c>
+      <c r="B86" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C86" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D86" s="0" t="inlineStr">
+        <is>
+          <t>qwen3-coder-next 只读源码验证压测</t>
+        </is>
+      </c>
+      <c r="E86" s="0" t="inlineStr">
+        <is>
+          <t>已完成并记录问题</t>
+        </is>
+      </c>
+      <c r="F86" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G86" s="0" t="inlineStr">
+        <is>
+          <t>切换编码模型后，需要验证真实企业项目只读链路是否仍能收束</t>
+        </is>
+      </c>
+      <c r="H86" s="0" t="inlineStr">
+        <is>
+          <t>session `20260709T071219747931Z` 正常 final：153 秒、35 次 LLM 请求、78 次工具调用、33 次 compaction、18 次 LLM summary；读 YXK-397 SQL 并定位 `IntentionConfig*` 证据链；新增 PT-030~PT-032。</t>
+        </is>
+      </c>
+      <c r="I86" s="0"/>
+      <c r="J86" s="0"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t>T-085</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C87" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D87" s="0" t="inlineStr">
+        <is>
+          <t>todo 工具误参纠偏</t>
+        </is>
+      </c>
+      <c r="E87" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F87" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G87" s="0" t="inlineStr">
+        <is>
+          <t>T-084 中模型用 `key/content` 调 `todo_add`、用错误 id 调 `todo_update`</t>
+        </is>
+      </c>
+      <c r="H87" s="0" t="inlineStr">
+        <is>
+          <t>工具错误返回正确参数示例；可选兼容 `key -&gt; id`、`content -&gt; task`，但继续提示规范 schema。</t>
+        </is>
+      </c>
+      <c r="I87" s="0"/>
+      <c r="J87" s="0"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t>T-086</t>
+        </is>
+      </c>
+      <c r="B88" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D88" s="0" t="inlineStr">
+        <is>
+          <t>evidence-aware read repetition guard</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F88" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G88" s="0" t="inlineStr">
+        <is>
+          <t>T-084 中 `read_file` 54 次，同一路径重复读但 `guard_hits=0`</t>
+        </is>
+      </c>
+      <c r="H88" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP pruning / soft escalation：同路径同范围已读多次后返回 evidence 摘要并触发 final-answer steering。</t>
+        </is>
+      </c>
+      <c r="I88" s="0"/>
+      <c r="J88" s="0"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t>T-087</t>
+        </is>
+      </c>
+      <c r="B89" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C89" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D89" s="0" t="inlineStr">
+        <is>
+          <t>final structure / evidence hygiene 增强</t>
+        </is>
+      </c>
+      <c r="E89" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F89" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G89" s="0" t="inlineStr">
+        <is>
+          <t>T-084 最终把“项目表”退化成“表名表”，并对类作用有过度断言</t>
+        </is>
+      </c>
+      <c r="H89" s="0" t="inlineStr">
+        <is>
+          <t>增强 Current task contract / final gate，检查用户显式输出结构；类作用类结论必须标 verified 或 inferred。</t>
+        </is>
+      </c>
+      <c r="I89" s="0"/>
+      <c r="J89" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6469,7 +6689,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G73"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8013,74 +8233,74 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到证据足够时触发 final-answer steering。</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>增强 Current task contract 的 final structure gate 和 final evidence hygiene，要求输出结构匹配用户字段，类作用类结论必须标 verified 或 inferred。</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8312,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -8102,22 +8322,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -8129,7 +8349,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -8139,22 +8359,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8166,7 +8386,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -8176,22 +8396,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -8203,7 +8423,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -8213,7 +8433,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -8223,12 +8443,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -8240,7 +8460,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -8250,7 +8470,7 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -8260,12 +8480,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8277,7 +8497,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8287,7 +8507,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -8297,12 +8517,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -8314,7 +8534,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8324,7 +8544,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -8334,12 +8554,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8571,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8361,22 +8581,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8608,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8398,22 +8618,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8645,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8435,7 +8655,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -8445,12 +8665,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -8462,7 +8682,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8472,22 +8692,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -8499,32 +8719,32 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -8536,32 +8756,32 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -8573,7 +8793,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -8583,22 +8803,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -8610,7 +8830,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -8620,22 +8840,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8867,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -8657,7 +8877,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -8667,12 +8887,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -8684,17 +8904,17 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -8704,12 +8924,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -8721,32 +8941,32 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -8758,7 +8978,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -8768,22 +8988,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -8795,7 +9015,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -8805,22 +9025,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -8832,7 +9052,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -8842,7 +9062,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -8852,12 +9072,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -8869,7 +9089,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -8879,7 +9099,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -8889,12 +9109,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -8906,7 +9126,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -8916,7 +9136,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
@@ -8926,12 +9146,12 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -8943,7 +9163,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -8953,22 +9173,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -8980,32 +9200,180 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
+          <t>ADR-026</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-078</t>
+        </is>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>ADR-027</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-081</t>
+        </is>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
           <t>ADR-028</t>
         </is>
       </c>
-      <c r="C69" s="0" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D69" s="0" t="inlineStr">
+      <c r="D71" s="0" t="inlineStr">
         <is>
           <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
-      <c r="E69" s="0" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F69" s="0" t="inlineStr">
+      <c r="F71" s="0" t="inlineStr">
         <is>
           <t>已完成 T-082</t>
         </is>
       </c>
-      <c r="G69" s="0" t="inlineStr">
+      <c r="G71" s="0" t="inlineStr">
         <is>
           <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>ADR-029</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F72" s="0" t="inlineStr">
+        <is>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+        </is>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
+        <is>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>ADR-030</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>先做 T-085~T-087</t>
+        </is>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -9021,7 +9389,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -9071,12 +9439,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>进入真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>先补 T-085~T-087，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9176,17 +9544,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>真实需求范围确认到源码验证压测</t>
+          <t>补齐 T-085~T-087 后继续真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>用户已给服务边界，T-078 已完成项目边界分析 MVP</t>
+          <t>T-084 已证明新模型能跑通只读链路，但暴露重复读、todo 参数和最终结构/证据卫生问题</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>做 T-079：先用边界圈项目范围，用户确认后接入候选项目源码，只读验证 API/controller/entity/test 证据并形成实现设计</t>
+          <t>先做小修小补，再进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>
@@ -9199,7 +9567,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F34"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -10178,6 +10546,102 @@
       <c r="F31" s="0" t="inlineStr">
         <is>
           <t>T-075 已实现 no-edit final hygiene：实现任务准备无改动停止时，会先要求 todo/git 收束；测试覆盖过早 final 被 steering 到 `todo_add` + `git_status`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>PT-030</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>T-084 中模型首次用 `key/content/status` 调 `todo_add`，后续又用错误 id 调 `todo_update`；任务最终完成，但 todo 台账不可靠。</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>OMP 的高频状态工具需要强 schema 提示、UI 可见性和可行动错误。</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>T-085 候选：工具错误返回正确调用示例；可选兼容 `key -&gt; id`、`content -&gt; task`，同时继续提示规范参数名。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>PT-031</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>T-084 中 153 秒内调用 78 次工具，其中 `read_file` 54 次，同一批 SQL/Java/XML 文件多次重复读取，但 `guard_hits=0`、`steering_counts=0`。</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>OMP 将 tool result pruning、soft escalation、task state 和 evidence sufficiency 组合，用小上限把低价值重复探索切回回答。</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>T-086 候选：evidence-aware read repetition guard；同路径同范围成功读取多次后返回已读 evidence 摘要并触发 final-answer steering。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>PT-032</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>T-084 要求输出“必须关注/可能关注/暂不关注项目表”，最终变成“表名表”；对 `IntentionConfigApplication` 的作用也有过度断言。</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>OMP 持续注入 current task contract 和 runtime evidence；成熟 reviewer/final check 会要求 verified fact 与 inference 分开。</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>T-087 候选：增强 final structure gate 和 final evidence hygiene，检查显式输出结构，要求类作用类结论标 verified/inferred。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add evidence-aware read repetition guard
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -6615,7 +6615,7 @@
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F88" s="0" t="inlineStr">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="H88" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP pruning / soft escalation：同路径同范围已读多次后返回 evidence 摘要并触发 final-answer steering。</t>
+          <t>已参考 OMP pruning / soft escalation：只读/分析任务中，同路径同范围成功读取超过阈值后返回 evidence 摘要并触发 final-answer steering；编辑任务不启用该 guard。</t>
         </is>
       </c>
       <c r="I88" s="0"/>
@@ -8253,7 +8253,7 @@
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
@@ -8263,7 +8263,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到证据足够时触发 final-answer steering。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -10594,7 +10594,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>T-086 候选：evidence-aware read repetition guard；同路径同范围成功读取多次后返回已读 evidence 摘要并触发 final-answer steering。</t>
+          <t>T-086 已完成：同路径同范围成功读取多次后返回已读 evidence 摘要并触发 final-answer steering；只读/分析任务启用，编辑任务不启用。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve todo tool argument recovery
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -6571,7 +6571,7 @@
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
@@ -6586,7 +6586,7 @@
       </c>
       <c r="H87" s="0" t="inlineStr">
         <is>
-          <t>工具错误返回正确参数示例；可选兼容 `key -&gt; id`、`content -&gt; task`，但继续提示规范 schema。</t>
+          <t>已兼容 `key -&gt; id`、`content -&gt; task`，成功结果提示下次使用规范参数；缺参、未知 id、无更新字段错误会返回正确示例和已知 todo id。</t>
         </is>
       </c>
       <c r="I87" s="0"/>
@@ -9389,7 +9389,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -9439,12 +9439,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086 已补 todo 参数纠偏和重复读收束</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先补 T-085~T-087，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>先补 T-087，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9544,17 +9544,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>补齐 T-085~T-087 后继续真实需求链路</t>
+          <t>补齐 T-087 后继续真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路，但暴露重复读、todo 参数和最终结构/证据卫生问题</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读和 todo 参数问题已补，剩余重点是最终结构/证据卫生</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做小修小补，再进入用户真实需求的项目范围确认和源码验证</t>
+          <t>先做 final gate 小修，再进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>
@@ -10562,7 +10562,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>T-085 候选：工具错误返回正确调用示例；可选兼容 `key -&gt; id`、`content -&gt; task`，同时继续提示规范参数名。</t>
+          <t>T-085 已完成：兼容 `key -&gt; id`、`content -&gt; task`，同时继续提示规范参数名；未知 id 错误会列出已知 todo id 和正确调用示例。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record review follow-up backlog
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -2770,7 +2770,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J92"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6680,6 +6680,138 @@
       <c r="I89" s="0"/>
       <c r="J89" s="0"/>
     </row>
+    <row r="90">
+      <c r="A90" s="0" t="inlineStr">
+        <is>
+          <t>T-088</t>
+        </is>
+      </c>
+      <c r="B90" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C90" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D90" s="0" t="inlineStr">
+        <is>
+          <t>read-only evidence gate</t>
+        </is>
+      </c>
+      <c r="E90" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F90" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G90" s="0" t="inlineStr">
+        <is>
+          <t>密码加密问答压测中，模型未读关键登录/密码文件前先给推测型答案</t>
+        </is>
+      </c>
+      <c r="H90" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP current task / evidence context：用户要求“代码证据/不推测/找到实现”时，必须先读关键命中文件或明确缺证据，禁止先行业惯例推断。</t>
+        </is>
+      </c>
+      <c r="I90" s="0"/>
+      <c r="J90" s="0"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t>T-089</t>
+        </is>
+      </c>
+      <c r="B91" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C91" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D91" s="0" t="inlineStr">
+        <is>
+          <t>semantic exploration guard</t>
+        </is>
+      </c>
+      <c r="E91" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F91" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G91" s="0" t="inlineStr">
+        <is>
+          <t>密码加密问答压测中，用户纠正后出现同模块/父子目录/Path not found 扩散，exact duplicate guard 太晚</t>
+        </is>
+      </c>
+      <c r="H91" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP soft escalation / pruning：按模块、父目录、Path-not-found pattern 计数，超过阈值后要求改用 search_code 命中文件或收束回答。</t>
+        </is>
+      </c>
+      <c r="I91" s="0"/>
+      <c r="J91" s="0"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="inlineStr">
+        <is>
+          <t>T-090</t>
+        </is>
+      </c>
+      <c r="B92" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C92" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D92" s="0" t="inlineStr">
+        <is>
+          <t>terminal input/output isolation</t>
+        </is>
+      </c>
+      <c r="E92" s="0" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="F92" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G92" s="0" t="inlineStr">
+        <is>
+          <t>压测日志出现用户键盘输入混入工具日志，如 `33333333333[tool:start]`</t>
+        </is>
+      </c>
+      <c r="H92" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Frontend 继续强化 centralized renderer 和运行中输入管理；一次性 CLI 提示运行中不要直接敲字，推荐 `./agent --chat`。</t>
+        </is>
+      </c>
+      <c r="I92" s="0"/>
+      <c r="J92" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -6689,7 +6821,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G76"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8307,111 +8439,111 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-088：read-only evidence gate；最终回答必须绑定具体 read_file/search_code/lsp 证据，否则继续查或明确未找到。</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-089：semantic exploration guard；按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code 命中文件。</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>T-090：强化 Terminal Frontend renderer/输入管理；一次性 CLI 增加提示，推荐长交互用 `./agent --chat`。</t>
         </is>
       </c>
     </row>
@@ -8423,7 +8555,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -8433,7 +8565,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -8443,12 +8575,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8592,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -8470,22 +8602,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8497,7 +8629,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8507,22 +8639,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -8534,7 +8666,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8544,7 +8676,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -8554,12 +8686,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8703,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8581,7 +8713,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -8591,12 +8723,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8608,7 +8740,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8618,7 +8750,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -8628,12 +8760,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -8645,7 +8777,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8655,22 +8787,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8814,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8692,22 +8824,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -8719,7 +8851,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -8729,22 +8861,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -8756,7 +8888,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -8766,22 +8898,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -8793,32 +8925,32 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -8830,17 +8962,17 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -8850,12 +8982,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -8867,32 +8999,32 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -8904,7 +9036,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -8914,7 +9046,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -8924,12 +9056,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -8941,7 +9073,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -8951,7 +9083,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -8961,12 +9093,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -8978,32 +9110,32 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9015,17 +9147,17 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -9035,12 +9167,12 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9052,17 +9184,17 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -9072,12 +9204,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9089,7 +9221,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -9099,22 +9231,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -9126,7 +9258,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -9136,22 +9268,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -9163,7 +9295,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -9173,7 +9305,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
@@ -9183,12 +9315,12 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -9200,7 +9332,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -9210,7 +9342,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -9220,12 +9352,12 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -9237,7 +9369,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -9247,22 +9379,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -9274,7 +9406,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -9284,7 +9416,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -9294,12 +9426,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9443,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -9321,22 +9453,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -9348,30 +9480,141 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
+          <t>ADR-027</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-081</t>
+        </is>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>ADR-028</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F74" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-082</t>
+        </is>
+      </c>
+      <c r="G74" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t>ADR-029</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F75" s="0" t="inlineStr">
+        <is>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+        </is>
+      </c>
+      <c r="G75" s="0" t="inlineStr">
+        <is>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
           <t>ADR-030</t>
         </is>
       </c>
-      <c r="C73" s="0" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D73" s="0" t="inlineStr">
+      <c r="D76" s="0" t="inlineStr">
         <is>
           <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
-      <c r="E73" s="0" t="inlineStr">
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F73" s="0" t="inlineStr">
+      <c r="F76" s="0" t="inlineStr">
         <is>
           <t>先做 T-085~T-087</t>
         </is>
       </c>
-      <c r="G73" s="0" t="inlineStr">
+      <c r="G76" s="0" t="inlineStr">
         <is>
           <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
@@ -9389,7 +9632,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -9439,12 +9682,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086 已补 todo 参数纠偏和重复读收束</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086 已补 todo 参数纠偏和重复读收束；新 review 暴露 evidence-first 与语义探索 guard 缺口</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先补 T-087，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>先补 T-087/T-088，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9544,17 +9787,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>补齐 T-087 后继续真实需求链路</t>
+          <t>补齐 T-087/T-088 后继续真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读和 todo 参数问题已补，剩余重点是最终结构/证据卫生</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读和 todo 参数问题已补；密码加密问答 review 证明 evidence-first 仍需加强</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 final gate 小修，再进入用户真实需求的项目范围确认和源码验证</t>
+          <t>先做 final gate 和 evidence gate 小修，再进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strengthen final structure evidence hygiene
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -6659,7 +6659,7 @@
       </c>
       <c r="E89" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F89" s="0" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="H89" s="0" t="inlineStr">
         <is>
-          <t>增强 Current task contract / final gate，检查用户显式输出结构；类作用类结论必须标 verified 或 inferred。</t>
+          <t>已增强 Current task contract / final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
       <c r="I89" s="0"/>
@@ -8422,7 +8422,7 @@
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
@@ -8432,7 +8432,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>增强 Current task contract 的 final structure gate 和 final evidence hygiene，要求输出结构匹配用户字段，类作用类结论必须标 verified 或 inferred。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -9632,7 +9632,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -9682,12 +9682,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086 已补 todo 参数纠偏和重复读收束；新 review 暴露 evidence-first 与语义探索 guard 缺口</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087 已补 todo 参数纠偏、重复读收束和最终结构/证据卫生；新 review 暴露 evidence-first 与语义探索 guard 缺口</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先补 T-087/T-088，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>先补 T-088，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9787,17 +9787,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>补齐 T-087/T-088 后继续真实需求链路</t>
+          <t>补齐 T-088 后继续真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读和 todo 参数问题已补；密码加密问答 review 证明 evidence-first 仍需加强</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数和最终结构/证据卫生问题已补；密码加密问答 review 证明 evidence-first 仍需加强</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 final gate 和 evidence gate 小修，再进入用户真实需求的项目范围确认和源码验证</t>
+          <t>先做 read-only evidence gate，再进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>
@@ -10869,7 +10869,7 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
@@ -10884,7 +10884,7 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>T-087 候选：增强 final structure gate 和 final evidence hygiene，检查显式输出结构，要求类作用类结论标 verified/inferred。</t>
+          <t>T-087 已完成：项目范围表必须含项目/服务列；用户要求证据状态或回答含推断性表达时，final gate 要求已验证/推断标签。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add read-only evidence gate
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F90" s="0" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="H90" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP current task / evidence context：用户要求“代码证据/不推测/找到实现”时，必须先读关键命中文件或明确缺证据，禁止先行业惯例推断。</t>
+          <t>已参考 OMP current task / evidence context：代码证据/源码/不推测/怎么处理类问题若无成功 `read_file` 就准备回答，会被要求先查证据；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
       <c r="I90" s="0"/>
@@ -8459,7 +8459,7 @@
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
@@ -8469,7 +8469,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>T-088：read-only evidence gate；最终回答必须绑定具体 read_file/search_code/lsp 证据，否则继续查或明确未找到。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -9682,12 +9682,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087 已补 todo 参数纠偏、重复读收束和最终结构/证据卫生；新 review 暴露 evidence-first 与语义探索 guard 缺口</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生和 evidence-first gate；新 review 仍暴露语义探索 guard 缺口</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先补 T-088，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>先补 T-089，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9787,17 +9787,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>补齐 T-088 后继续真实需求链路</t>
+          <t>补齐 T-089 后继续真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数和最终结构/证据卫生问题已补；密码加密问答 review 证明 evidence-first 仍需加强</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生和 evidence-first 问题已补；密码加密问答 review 仍证明语义路径探索会扩散</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 read-only evidence gate，再进入用户真实需求的项目范围确认和源码验证</t>
+          <t>先做 semantic exploration guard，再进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add semantic exploration guard
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板和 T-084 qwen3-coder-next 企业项目只读源码验证压测。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测和 T-089 semantic exploration guard。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2464,7 +2464,7 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t>Tool result pruning</t>
+          <t>Semantic exploration guard</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
@@ -2474,17 +2474,17 @@
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>`ToolResult.useless` + provider-bound context pruning</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `_steer_after_semantic_exploration()`</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
+          <t>`list_files` 按模块/父目录归一语义探索 key；同一模块或同一 Path-not-found 父路径探索超过小上限后跳过目录猜测，并临时只开放 evidence tools</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>继续真实长任务观察</t>
+          <t>继续真实只读问答压测</t>
         </is>
       </c>
       <c r="F46" s="0"/>
@@ -2494,7 +2494,7 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t>Todo steering</t>
+          <t>Tool result pruning</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
@@ -2504,17 +2504,17 @@
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>provider-bound runtime todo reminder</t>
+          <t>`ToolResult.useless` + provider-bound context pruning</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
+          <t>`search_code` / LSP 空结果标记 useless；重复等价 read/search/LSP 旧结果在发给模型的上下文中替换为 notice，session 原文保留</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
+          <t>继续真实长任务观察</t>
         </is>
       </c>
       <c r="F47" s="0"/>
@@ -2524,7 +2524,7 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger</t>
+          <t>Todo steering</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
@@ -2534,17 +2534,17 @@
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/agent.py` / `tests/test_agent.py`</t>
+          <t>provider-bound runtime todo reminder</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>工具结果经 runtime 提炼成短证据账本；provider context 中提示模型区分证据事实与推断，session 中追加 `evidence` 事件</t>
+          <t>未完成 todo 会注入发送给模型的 system context，即使未触发 compaction 也能提醒模型保持任务方向</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>后续真实任务观察是否需要更结构化引用</t>
+          <t>后续评估 OMP 风格 eager todo / mid-run nudge</t>
         </is>
       </c>
       <c r="F48" s="0"/>
@@ -2554,7 +2554,7 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t>Relevance gate / diff reviewer</t>
+          <t>Evidence Ledger</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
@@ -2564,17 +2564,17 @@
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/agent.py`、`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`src/local_agent/tools/relevance.py`</t>
+          <t>`src/local_agent/agent.py` / `tests/test_agent.py`</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>真实 apply_patch 写入前检查目标已读和低相关配置路径；workspace-root evidence 进入 Evidence Ledger；git_diff 对低相关本轮 patch 追加 reviewer 提示；patch log 归一 workspace 内绝对路径</t>
+          <t>工具结果经 runtime 提炼成短证据账本；provider context 中提示模型区分证据事实与推断，session 中追加 `evidence` 事件</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>后续真实任务观察是否需要更结构化引用</t>
         </is>
       </c>
       <c r="F49" s="0"/>
@@ -2584,7 +2584,7 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t>Implementation quality / safe new-file</t>
+          <t>Relevance gate / diff reviewer</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`tests/test_tools.py`</t>
+          <t>`src/local_agent/agent.py`、`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`src/local_agent/tools/relevance.py`</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>comment-only 代码实现 diff 会被 reviewer 标红；新文件创建支持 dry-run diff、patch log 和 rollback 删除</t>
+          <t>真实 apply_patch 写入前检查目标已读和低相关配置路径；workspace-root evidence 进入 Evidence Ledger；git_diff 对低相关本轮 patch 追加 reviewer 提示；patch log 归一 workspace 内绝对路径</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>真实目标服务压测</t>
+          <t>日用反馈补测</t>
         </is>
       </c>
       <c r="F50" s="0"/>
@@ -2614,7 +2614,7 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t>No-edit final hygiene</t>
+          <t>Implementation quality / safe new-file</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
@@ -2624,12 +2624,12 @@
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/agent.py`、`tests/test_agent.py`</t>
+          <t>`src/local_agent/tools/files.py`、`src/local_agent/tools/git.py`、`tests/test_tools.py`</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>Provider context 提前说明无改动停止要可审计；runtime 发现过早 no-edit final 时追加 steering，并限制下一轮工具到 todo/git 收束集合</t>
+          <t>comment-only 代码实现 diff 会被 reviewer 标红；新文件创建支持 dry-run diff、patch log 和 rollback 删除</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -2644,7 +2644,7 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t>Event/Command Protocol</t>
+          <t>No-edit final hygiene</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
@@ -2654,17 +2654,17 @@
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/protocol/events.py`、`src/local_agent/protocol/commands.py`、`src/local_agent/agent.py`</t>
+          <t>`src/local_agent/agent.py`、`tests/test_agent.py`</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Runtime 产出 typed events，CLI 通过 stderr sink 渲染，session JSONL 写入 `event_v1`，命令协议 shape 已固化</t>
+          <t>Provider context 提前说明无改动停止要可审计；runtime 发现过早 no-edit final 时追加 steering，并限制下一轮工具到 todo/git 收束集合</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>T-077 接 Terminal Frontend</t>
+          <t>真实目标服务压测</t>
         </is>
       </c>
       <c r="F52" s="0"/>
@@ -2674,7 +2674,7 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend</t>
+          <t>Event/Command Protocol</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
@@ -2684,17 +2684,17 @@
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/frontends/terminal/`、`src/local_agent/cli.py`</t>
+          <t>`src/local_agent/protocol/events.py`、`src/local_agent/protocol/commands.py`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>append-only 交互前端，`./agent` / `--chat` / `chat` 入口，可选 `prompt_toolkit` / `rich`，approval events 可见</t>
+          <t>Runtime 产出 typed events，CLI 通过 stderr sink 渲染，session JSONL 写入 `event_v1`，命令协议 shape 已固化</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>真实交互压测</t>
+          <t>T-077 接 Terminal Frontend</t>
         </is>
       </c>
       <c r="F53" s="0"/>
@@ -2704,7 +2704,7 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析</t>
+          <t>Terminal Frontend</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
@@ -2714,17 +2714,17 @@
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/memory/enterprise-service-boundary.md`、`.local-agent/skills/project-scope-analysis/SKILL.md`、`src/local_agent/agent.py`</t>
+          <t>`src/local_agent/frontends/terminal/`、`src/local_agent/cli.py`</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>只根据需求和服务边界圈项目范围；analysis-only 不走实现 hygiene；点名 skill 会先读正文；缺表格/段落会强制无工具重答</t>
+          <t>append-only 交互前端，`./agent` / `--chat` / `chat` 入口，可选 `prompt_toolkit` / `rich`，approval events 可见</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>用真实需求继续压测</t>
+          <t>真实交互压测</t>
         </is>
       </c>
       <c r="F54" s="0"/>
@@ -2734,32 +2734,62 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>项目边界分析</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>当前 188 个测试通过</t>
+          <t>`.local-agent/memory/enterprise-service-boundary.md`、`.local-agent/skills/project-scope-analysis/SKILL.md`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>只根据需求和服务边界圈项目范围；analysis-only 不走实现 hygiene；点名 skill 会先读正文；缺表格/段落会强制无工具重答</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>用真实需求继续压测</t>
         </is>
       </c>
       <c r="F55" s="0"/>
       <c r="G55" s="0"/>
       <c r="H55" s="0"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>当前 198 个测试通过</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F56" s="0"/>
+      <c r="G56" s="0"/>
+      <c r="H56" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6747,7 +6777,7 @@
       </c>
       <c r="E91" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F91" s="0" t="inlineStr">
@@ -6762,7 +6792,7 @@
       </c>
       <c r="H91" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP soft escalation / pruning：按模块、父目录、Path-not-found pattern 计数，超过阈值后要求改用 search_code 命中文件或收束回答。</t>
+          <t>已参考 OMP soft escalation / pruning：按模块/父目录归一 `list_files` 语义探索 key，超过小上限后跳过目录猜测，并临时只开放 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
       <c r="I91" s="0"/>
@@ -8496,7 +8526,7 @@
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
@@ -8506,7 +8536,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>T-089：semantic exploration guard；按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code 命中文件。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -9682,12 +9712,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生和 evidence-first gate；新 review 仍暴露语义探索 guard 缺口</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate 和语义探索收束</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先补 T-089，再继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>下一步补 T-090 或继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9787,17 +9817,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>补齐 T-089 后继续真实需求链路</t>
+          <t>T-090 或真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生和 evidence-first 问题已补；密码加密问答 review 仍证明语义路径探索会扩散</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生、evidence-first 和语义探索扩散问题已补；剩余明显体验问题是终端输入输出隔离</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 semantic exploration guard，再进入用户真实需求的项目范围确认和源码验证</t>
+          <t>先做 terminal input/output isolation，或直接进入用户真实需求的项目范围确认和源码验证</t>
         </is>
       </c>
     </row>
@@ -10960,7 +10990,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 188 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 198 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -11011,7 +11041,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add terminal input isolation
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测和 T-089 semantic exploration guard。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard 和 T-090 terminal input/output isolation。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2734,7 +2734,7 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析</t>
+          <t>Terminal input isolation</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>`.local-agent/memory/enterprise-service-boundary.md`、`.local-agent/skills/project-scope-analysis/SKILL.md`、`src/local_agent/agent.py`</t>
+          <t>`src/local_agent/terminal_io.py`、`src/local_agent/cli.py`、`src/local_agent/frontends/terminal/app.py`</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>只根据需求和服务边界圈项目范围；analysis-only 不走实现 hygiene；点名 skill 会先读正文；缺表格/段落会强制无工具重答</t>
+          <t>一次性 CLI / REPL / terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>用真实需求继续压测</t>
+          <t>继续真实交互压测</t>
         </is>
       </c>
       <c r="F55" s="0"/>
@@ -2764,32 +2764,62 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>项目边界分析</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>当前 198 个测试通过</t>
+          <t>`.local-agent/memory/enterprise-service-boundary.md`、`.local-agent/skills/project-scope-analysis/SKILL.md`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>只根据需求和服务边界圈项目范围；analysis-only 不走实现 hygiene；点名 skill 会先读正文；缺表格/段落会强制无工具重答</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>用真实需求继续压测</t>
         </is>
       </c>
       <c r="F56" s="0"/>
       <c r="G56" s="0"/>
       <c r="H56" s="0"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>当前 202 个测试通过</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F57" s="0"/>
+      <c r="G57" s="0"/>
+      <c r="H57" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6821,7 +6851,7 @@
       </c>
       <c r="E92" s="0" t="inlineStr">
         <is>
-          <t>候选</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F92" s="0" t="inlineStr">
@@ -6836,7 +6866,7 @@
       </c>
       <c r="H92" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend 继续强化 centralized renderer 和运行中输入管理；一次性 CLI 提示运行中不要直接敲字，推荐 `./agent --chat`。</t>
+          <t>已新增 TTY echo 静默与 prompt 期恢复/flush，覆盖一次性 CLI、REPL 和 terminal chat。</t>
         </is>
       </c>
       <c r="I92" s="0"/>
@@ -8563,7 +8593,7 @@
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
@@ -8573,7 +8603,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>T-090：强化 Terminal Frontend renderer/输入管理；一次性 CLI 增加提示，推荐长交互用 `./agent --chat`。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -9712,12 +9742,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate 和语义探索收束</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步补 T-090 或继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>下一步继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
         </is>
       </c>
     </row>
@@ -9817,17 +9847,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>T-090 或真实需求链路</t>
+          <t>真实需求链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生、evidence-first 和语义探索扩散问题已补；剩余明显体验问题是终端输入输出隔离</t>
+          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生、evidence-first、语义探索扩散和终端输入污染问题已补</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 terminal input/output isolation，或直接进入用户真实需求的项目范围确认和源码验证</t>
+          <t>进入用户真实需求的项目范围确认和源码验证；必要时复跑密码加密问答样本</t>
         </is>
       </c>
     </row>
@@ -10990,7 +11020,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 198 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 202 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -11041,7 +11071,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
+          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Address review issues and split compaction
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard 和 T-090 terminal input/output isolation。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复和 T-092 compaction 渐进模块化 / LSP 置信度提示。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy、no-edit final hygiene</t>
+          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、LSP best-effort 置信度提示、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy、no-edit final hygiene</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>高级轻量能力主线已收口，后续按真实压测失败形态补 path-scoped rules、完整 reviewer 或 ToolChoiceQueue。</t>
+          <t>高级轻量能力主线已收口，后续按真实压测失败形态补 path-scoped rules、完整 reviewer 或 ToolChoiceQueue；架构债按 OMP 原则渐进拆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 202 个测试通过</t>
+          <t>当前 203 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J94"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6872,6 +6872,94 @@
       <c r="I92" s="0"/>
       <c r="J92" s="0"/>
     </row>
+    <row r="93">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t>T-091</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D93" s="0" t="inlineStr">
+        <is>
+          <t>Vue diff reviewer comment-only 误报修复</t>
+        </is>
+      </c>
+      <c r="E93" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F93" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G93" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 指出 `.vue` 模板标签可能被 implementation-quality reviewer 当成注释-only，导致真实 Vue 模板改动被误报</t>
+        </is>
+      </c>
+      <c r="H93" s="0" t="inlineStr">
+        <is>
+          <t>已把 comment-only 判断改为按文件类型处理：JavaDoc `&lt;p&gt;/&lt;li&gt;` 仅在 Java 中作为注释标记，Vue 模板 markup 不再算 comment-only；新增回归测试覆盖 Vue `&lt;p&gt;` 模板替换。</t>
+        </is>
+      </c>
+      <c r="I93" s="0"/>
+      <c r="J93" s="0"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>T-092</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D94" s="0" t="inlineStr">
+        <is>
+          <t>compaction 渐进模块化与 LSP 置信度提示</t>
+        </is>
+      </c>
+      <c r="E94" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F94" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G94" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 指出 `agent.py` 继续膨胀、compaction/token/context 应拆模块，且 Java/Vue LSP 正则回退与 Python AST 输出无区分</t>
+        </is>
+      </c>
+      <c r="H94" s="0" t="inlineStr">
+        <is>
+          <t>已新增 `src/local_agent/compaction.py`，迁出压缩阈值、provider-safe 清理、tool output pruning、summary transcript/cache helpers；Java/JS/TS/Vue LSP 输出新增 `[lsp confidence]` best-effort 提示，避免模型把轻量正则当完整 LSP。</t>
+        </is>
+      </c>
+      <c r="I94" s="0"/>
+      <c r="J94" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -6881,7 +6969,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G79"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8610,74 +8698,74 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8777,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -8699,22 +8787,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -8726,7 +8814,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8736,22 +8824,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8763,7 +8851,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8773,22 +8861,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8888,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8810,7 +8898,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -8820,12 +8908,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8925,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8847,7 +8935,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -8857,12 +8945,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8962,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8884,7 +8972,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -8894,12 +8982,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -8911,7 +8999,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -8921,7 +9009,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -8931,12 +9019,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -8948,7 +9036,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -8958,22 +9046,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -8985,7 +9073,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -8995,22 +9083,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9022,7 +9110,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9032,7 +9120,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -9042,12 +9130,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9059,7 +9147,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9069,22 +9157,22 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9096,32 +9184,32 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>不启动外部 language server</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
         </is>
       </c>
     </row>
@@ -9133,32 +9221,32 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9258,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9180,22 +9268,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9295,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9217,22 +9305,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -9244,7 +9332,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -9254,7 +9342,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -9264,12 +9352,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9281,17 +9369,17 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -9301,12 +9389,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9318,32 +9406,32 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9355,7 +9443,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -9365,22 +9453,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9480,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -9402,22 +9490,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -9429,7 +9517,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -9439,7 +9527,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
@@ -9449,12 +9537,12 @@
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9554,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -9476,7 +9564,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -9486,12 +9574,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -9503,7 +9591,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -9513,7 +9601,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
@@ -9523,12 +9611,12 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -9540,7 +9628,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -9550,22 +9638,22 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -9577,7 +9665,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -9587,7 +9675,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -9597,12 +9685,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -9614,7 +9702,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -9624,7 +9712,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
@@ -9634,12 +9722,12 @@
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -9651,32 +9739,143 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
+          <t>ADR-028</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F76" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-082</t>
+        </is>
+      </c>
+      <c r="G76" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>ADR-029</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F77" s="0" t="inlineStr">
+        <is>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+        </is>
+      </c>
+      <c r="G77" s="0" t="inlineStr">
+        <is>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
           <t>ADR-030</t>
         </is>
       </c>
-      <c r="C76" s="0" t="inlineStr">
+      <c r="C78" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D76" s="0" t="inlineStr">
+      <c r="D78" s="0" t="inlineStr">
         <is>
           <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
-      <c r="E76" s="0" t="inlineStr">
+      <c r="E78" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F76" s="0" t="inlineStr">
+      <c r="F78" s="0" t="inlineStr">
         <is>
           <t>先做 T-085~T-087</t>
         </is>
       </c>
-      <c r="G76" s="0" t="inlineStr">
+      <c r="G78" s="0" t="inlineStr">
         <is>
           <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t>ADR-031</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F79" s="0" t="inlineStr">
+        <is>
+          <t>已从 `compaction.py` 开始</t>
+        </is>
+      </c>
+      <c r="G79" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -9742,12 +9941,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步继续真实需求“范围确认 → 源码验证 → 实现设计/小改”</t>
+          <t>下一步继续真实需求“范围确认 → 源码验证 → 实现设计/小改”，并按 review 顺序继续拆 `agent.py` 小模块</t>
         </is>
       </c>
     </row>
@@ -11020,7 +11219,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 202 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 203 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add optional external LSP adapter
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言轻量 LSP、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复和 T-092 compaction 渐进模块化 / LSP 置信度提示。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示和 T-093 可选外部 LSP adapter。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -422,7 +422,7 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>轻量 LSP</t>
+          <t>LSP / Light fallback</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -432,7 +432,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`，覆盖 Python、Java、JavaScript、TypeScript、Vue。</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics` / `lsp_status`，覆盖 Python、Java、JavaScript、TypeScript、Vue；默认可用则外部 LSP，不可用则 light fallback。</t>
         </is>
       </c>
       <c r="D19" s="0"/>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>OMP 风格 auto summary、轻量 LSP、LSP 兼容别名、LSP best-effort 置信度提示、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy、no-edit final hygiene</t>
+          <t>OMP 风格 auto summary、多语言 LSP/light fallback、LSP 兼容别名、LSP best-effort 置信度提示、multi-root workspace roots、allowed-dir soft tool requirement、startup context/rules、startup memory、learn、memory consolidation、authored skills discovery、重复工具调用熔断、duplicate-tool forced-final steering、同文件切片读取漂移 guard、空搜索词跨路径 guard、path escape roots hint、LSP 空 query guard、Current task contract、Evidence Ledger、tool result pruning、todo steering、跨项目 env-file、runtime state dir、真实项目压测记录、relevance gate / diff reviewer、implementation-quality reviewer、safe new-file policy、no-edit final hygiene</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -2062,7 +2062,7 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>轻量 LSP 工具</t>
+          <t>LSP / Light fallback 工具</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2072,17 +2072,17 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics`</t>
+          <t>`lsp_symbols` / `lsp_workspace_symbols` / `lsp_document_symbols` / `lsp_definition` / `lsp_references` / `lsp_diagnostics` / `lsp_status`</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>Python、Java、JavaScript、TypeScript、Vue 静态导航，不启动外部 server；workspace/document symbols 是兼容别名</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 只读导航；可选外部 server，不可用则 light fallback；workspace/document symbols 是兼容别名</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>后续看是否升级完整 LSP</t>
+          <t>后续看是否补 rename/code action</t>
         </is>
       </c>
       <c r="F33" s="0"/>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 203 个测试通过</t>
+          <t>当前 206 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4643,7 +4643,7 @@
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已完成 MVP 版</t>
+          <t>已完成并被 T-093 增强</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
-          <t>Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics 已可用</t>
+          <t>Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics 已可用；T-093 已补可选外部 LSP adapter</t>
         </is>
       </c>
       <c r="I42" s="0"/>
@@ -6959,6 +6959,58 @@
       </c>
       <c r="I94" s="0"/>
       <c r="J94" s="0"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t>T-093</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D95" s="0" t="inlineStr">
+        <is>
+          <t>可选外部 LSP adapter</t>
+        </is>
+      </c>
+      <c r="E95" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F95" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G95" s="0" t="inlineStr">
+        <is>
+          <t>用户希望 Java、JS、Vue 等主流语言尽量完整；仅靠 regex fallback 与 OMP 的 LSP 子系统差距明显</t>
+        </is>
+      </c>
+      <c r="H95" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/lsp/`：stdio JSON-RPC client、Java `jdtls`、TypeScript `typescript-language-server --stdio`、Vue `vue-language-server --stdio`、嵌套项目 root marker、`lsp_status`、`AGENT_LSP_MODE=auto</t>
+        </is>
+      </c>
+      <c r="I95" s="0" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="J95" s="0" t="inlineStr">
+        <is>
+          <t>external` 和 `AGENT_LSP_*_COMMAND`；不自动下载依赖，不可用时回退 light fallback。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6969,7 +7021,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7280,12 +7332,12 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>已只引入多语言轻量 LSP、auto summary、multi-root、startup memory 和 learn，完整 DAP/TUI/subagents 继续后置</t>
+          <t>已引入 auto summary、multi-root、startup memory、learn 和可选外部 LSP adapter；完整 DAP/subagents/重 UI 继续后置</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们先做无外部依赖的本地 MVP。</t>
+          <t>OMP 将 LSP、subagents、AST edit、TUI 等做成可组合高级能力；我们只把 LSP 做成可选增强，不作为默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -8772,37 +8824,37 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -8814,7 +8866,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -8824,22 +8876,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8903,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8861,7 +8913,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -8871,12 +8923,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8888,7 +8940,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8898,22 +8950,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -8925,7 +8977,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8935,7 +8987,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -8945,12 +8997,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -8962,7 +9014,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -8972,7 +9024,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -8982,12 +9034,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -8999,7 +9051,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -9009,7 +9061,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -9019,12 +9071,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9036,7 +9088,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -9046,7 +9098,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -9056,12 +9108,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9125,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9083,7 +9135,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -9093,12 +9145,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -9110,7 +9162,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9120,22 +9172,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9147,7 +9199,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9157,7 +9209,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -9167,12 +9219,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9236,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9194,7 +9246,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -9204,12 +9256,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>不启动外部 language server</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics，不引入 npm/pip 依赖或后台进程；完整 LSP/DAP 后置。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9273,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9231,22 +9283,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -9258,32 +9310,32 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9347,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9305,22 +9357,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -9332,7 +9384,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -9342,7 +9394,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -9352,12 +9404,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9421,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -9379,22 +9431,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9406,7 +9458,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -9416,22 +9468,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9443,32 +9495,32 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9532,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -9490,7 +9542,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -9500,12 +9552,12 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -9517,7 +9569,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -9527,22 +9579,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9606,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -9564,7 +9616,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -9574,12 +9626,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9643,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -9601,7 +9653,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
@@ -9611,12 +9663,12 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -9628,7 +9680,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -9638,7 +9690,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
@@ -9648,12 +9700,12 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9717,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -9675,7 +9727,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -9685,12 +9737,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -9702,7 +9754,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -9712,22 +9764,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9791,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -9749,22 +9801,22 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -9776,7 +9828,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -9786,22 +9838,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -9813,7 +9865,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -9823,7 +9875,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
@@ -9833,12 +9885,12 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -9850,32 +9902,106 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
+          <t>ADR-030</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F79" s="0" t="inlineStr">
+        <is>
+          <t>先做 T-085~T-087</t>
+        </is>
+      </c>
+      <c r="G79" s="0" t="inlineStr">
+        <is>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
           <t>ADR-031</t>
         </is>
       </c>
-      <c r="C79" s="0" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D79" s="0" t="inlineStr">
+      <c r="D80" s="0" t="inlineStr">
         <is>
           <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
-      <c r="E79" s="0" t="inlineStr">
+      <c r="E80" s="0" t="inlineStr">
         <is>
           <t>已接受</t>
         </is>
       </c>
-      <c r="F79" s="0" t="inlineStr">
+      <c r="F80" s="0" t="inlineStr">
         <is>
           <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
-      <c r="G79" s="0" t="inlineStr">
+      <c r="G80" s="0" t="inlineStr">
         <is>
           <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t>ADR-032</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F81" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-093</t>
+        </is>
+      </c>
+      <c r="G81" s="0" t="inlineStr">
+        <is>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
       </c>
     </row>
@@ -9941,7 +10067,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -11219,7 +11345,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 203 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 206 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -11270,7 +11396,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言轻量 LSP、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record real project LSP availability test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示和 T-093 可选外部 LSP adapter。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter 和 T-094 真实项目 LSP 可用性压测。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J96"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7012,6 +7012,50 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t>T-094</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>真实项目 LSP 可用性压测</t>
+        </is>
+      </c>
+      <c r="E96" s="0" t="inlineStr">
+        <is>
+          <t>已完成并记录问题</t>
+        </is>
+      </c>
+      <c r="F96" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G96" s="0" t="inlineStr">
+        <is>
+          <t>T-093 需要在真实企业项目里验证 `lsp_status`、root marker、light fallback 和模型是否会正确使用 LSP 工具</t>
+        </is>
+      </c>
+      <c r="H96" s="0" t="inlineStr">
+        <is>
+          <t>`crcl-open` session `20260709T082448561892Z`、`zqyl-user-center-service` sessions `20260709T082459082275Z` / `20260709T082540210824Z` 通过；当前机器未安装 `jdtls` / TS / Vue server，LCA 正确回退 light fallback；Java 样本符号定位成功；记录一次模型路径字符误写。</t>
+        </is>
+      </c>
+      <c r="I96" s="0"/>
+      <c r="J96" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -7021,7 +7065,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8861,37 +8905,37 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>新增，待配置</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>下一步可做 T-095：预置/配置 jdtls，或在 VM 镜像中离线安装 language servers；LCA 继续不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8947,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -8913,22 +8957,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -8940,7 +8984,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8950,7 +8994,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -8960,12 +9004,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -8977,7 +9021,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -8987,22 +9031,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -9014,7 +9058,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -9024,7 +9068,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -9034,12 +9078,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -9051,7 +9095,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -9061,7 +9105,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -9071,12 +9115,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -9088,7 +9132,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -9098,7 +9142,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -9108,12 +9152,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9169,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9135,7 +9179,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -9145,12 +9189,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -9162,7 +9206,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9172,7 +9216,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -9182,12 +9226,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -9199,7 +9243,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9209,22 +9253,22 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9236,7 +9280,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9246,7 +9290,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -9256,12 +9300,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9273,7 +9317,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9283,22 +9327,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9310,7 +9354,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9320,22 +9364,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -9347,32 +9391,32 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -9384,7 +9428,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -9394,22 +9438,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9465,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -9431,7 +9475,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -9441,12 +9485,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -9458,7 +9502,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -9468,22 +9512,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9539,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -9505,22 +9549,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9532,32 +9576,32 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9613,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -9579,7 +9623,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
@@ -9589,12 +9633,12 @@
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -9606,7 +9650,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -9616,22 +9660,22 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -9643,7 +9687,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -9653,7 +9697,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
@@ -9663,12 +9707,12 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -9680,7 +9724,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -9690,7 +9734,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
@@ -9700,12 +9744,12 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -9717,7 +9761,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -9727,7 +9771,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -9737,12 +9781,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -9754,7 +9798,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -9764,7 +9808,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
@@ -9774,12 +9818,12 @@
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9835,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -9801,22 +9845,22 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -9828,7 +9872,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -9838,22 +9882,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -9865,7 +9909,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -9875,22 +9919,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -9902,7 +9946,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -9912,7 +9956,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
@@ -9922,12 +9966,12 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -9939,7 +9983,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -9949,7 +9993,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -9959,12 +10003,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -9976,30 +10020,67 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
+          <t>ADR-031</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F81" s="0" t="inlineStr">
+        <is>
+          <t>已从 `compaction.py` 开始</t>
+        </is>
+      </c>
+      <c r="G81" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B82" s="0" t="inlineStr">
+        <is>
           <t>ADR-032</t>
         </is>
       </c>
-      <c r="C81" s="0" t="inlineStr">
+      <c r="C82" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D81" s="0" t="inlineStr">
+      <c r="D82" s="0" t="inlineStr">
         <is>
           <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
-      <c r="E81" s="0" t="inlineStr">
+      <c r="E82" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F81" s="0" t="inlineStr">
+      <c r="F82" s="0" t="inlineStr">
         <is>
           <t>已完成 T-093</t>
         </is>
       </c>
-      <c r="G81" s="0" t="inlineStr">
+      <c r="G82" s="0" t="inlineStr">
         <is>
           <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
@@ -10067,12 +10148,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094 已完成真实项目 LSP 可用性压测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步继续真实需求“范围确认 → 源码验证 → 实现设计/小改”，并按 review 顺序继续拆 `agent.py` 小模块</t>
+          <t>下一步可选：预置 jdtls 做 external Java LSP 压测，或继续进入真实需求“范围确认 → 源码验证 → 实现设计/小改”。</t>
         </is>
       </c>
     </row>
@@ -11396,7 +11477,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；下一步用真实需求跑范围确认到源码验证。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-094 证明 external LSP 需要额外预置 server。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Java LSP resilience
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter 和 T-094 真实项目 LSP 可用性压测。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测和 T-096 Java LSP 韧性对齐 OMP。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 206 个测试通过</t>
+          <t>当前 209 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J98"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7056,6 +7056,94 @@
       <c r="I96" s="0"/>
       <c r="J96" s="0"/>
     </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>T-095</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D97" s="0" t="inlineStr">
+        <is>
+          <t>jdtls 预置、协议修复与 strict external 复测</t>
+        </is>
+      </c>
+      <c r="E97" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F97" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G97" s="0" t="inlineStr">
+        <is>
+          <t>T-094 证明当前环境未预置 jdtls，需要验证 external Java LSP 真链路</t>
+        </is>
+      </c>
+      <c r="H97" s="0" t="inlineStr">
+        <is>
+          <t>已通过 Homebrew 安装 `jdtls 1.60.0`；极小 Maven 项目 external symbols/definition/diagnostics 全通；真实企业项目 diagnostics 走 jdtls 且 OK，但缺公司内部 parent POM 导致 Maven project 未导入、external symbols/definition 为空；已补 LSP `rootPath` / `workspaceFolders` / server request 响应，并在 external 空结果时合并 light fallback；session `20260709T084323683100Z` 验证 Agent 可正确说明 external/fallback。</t>
+        </is>
+      </c>
+      <c r="I97" s="0"/>
+      <c r="J97" s="0"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="inlineStr">
+        <is>
+          <t>T-096</t>
+        </is>
+      </c>
+      <c r="B98" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t>Java LSP 韧性对齐 OMP</t>
+        </is>
+      </c>
+      <c r="E98" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F98" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G98" s="0" t="inlineStr">
+        <is>
+          <t>用户要求 Java 是主战场，LSP 韧性要和 OMP 一样；仅有启动/诊断不够</t>
+        </is>
+      </c>
+      <c r="H98" s="0" t="inlineStr">
+        <is>
+          <t>已补 `$/progress` project load 跟踪、project load 等待窗口、Java `workspace/configuration` 响应、`workspace/workspaceFolders` / `window/workDoneProgress/create` / dynamic registration server request 响应；真实企业项目缺 parent POM 时继续 external 边界说明 + fallback evidence。</t>
+        </is>
+      </c>
+      <c r="I98" s="0"/>
+      <c r="J98" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -7065,7 +7153,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8925,7 +9013,7 @@
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>新增，待配置</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
@@ -8935,44 +9023,44 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>下一步可做 T-095：预置/配置 jdtls，或在 VM 镜像中离线安装 language servers；LCA 继续不自动下载依赖。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
@@ -8984,7 +9072,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -8994,22 +9082,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -9021,7 +9109,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -9031,7 +9119,7 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -9041,12 +9129,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9146,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -9068,22 +9156,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -9095,7 +9183,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -9105,7 +9193,7 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -9115,12 +9203,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -9132,7 +9220,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -9142,7 +9230,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -9152,12 +9240,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9257,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9179,7 +9267,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -9189,12 +9277,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9206,7 +9294,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9216,7 +9304,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -9226,12 +9314,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -9243,7 +9331,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9253,7 +9341,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -9263,12 +9351,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -9280,7 +9368,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9290,22 +9378,22 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9317,7 +9405,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9327,7 +9415,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -9337,12 +9425,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9354,7 +9442,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9364,22 +9452,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9391,7 +9479,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9401,22 +9489,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -9428,32 +9516,32 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -9465,7 +9553,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -9475,22 +9563,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -9502,7 +9590,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -9512,7 +9600,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
@@ -9522,12 +9610,12 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -9539,7 +9627,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -9549,22 +9637,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9664,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -9586,22 +9674,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9613,32 +9701,32 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9650,7 +9738,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -9660,7 +9748,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -9670,12 +9758,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9775,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -9697,22 +9785,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -9724,7 +9812,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -9734,7 +9822,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
@@ -9744,12 +9832,12 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -9761,7 +9849,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -9771,7 +9859,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -9781,12 +9869,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -9798,7 +9886,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -9808,7 +9896,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
@@ -9818,12 +9906,12 @@
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9923,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -9845,7 +9933,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
@@ -9855,12 +9943,12 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -9872,7 +9960,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -9882,22 +9970,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -9909,7 +9997,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -9919,22 +10007,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -9946,7 +10034,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -9956,22 +10044,22 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -9983,7 +10071,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -9993,7 +10081,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -10003,12 +10091,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -10020,7 +10108,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -10030,7 +10118,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -10040,12 +10128,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -10057,30 +10145,67 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
+          <t>ADR-031</t>
+        </is>
+      </c>
+      <c r="C82" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D82" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+        </is>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F82" s="0" t="inlineStr">
+        <is>
+          <t>已从 `compaction.py` 开始</t>
+        </is>
+      </c>
+      <c r="G82" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
           <t>ADR-032</t>
         </is>
       </c>
-      <c r="C82" s="0" t="inlineStr">
+      <c r="C83" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D82" s="0" t="inlineStr">
+      <c r="D83" s="0" t="inlineStr">
         <is>
           <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
-      <c r="E82" s="0" t="inlineStr">
+      <c r="E83" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F82" s="0" t="inlineStr">
+      <c r="F83" s="0" t="inlineStr">
         <is>
           <t>已完成 T-093</t>
         </is>
       </c>
-      <c r="G82" s="0" t="inlineStr">
+      <c r="G83" s="0" t="inlineStr">
         <is>
           <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
@@ -10148,12 +10273,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094 已完成真实项目 LSP 可用性压测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096 已完成 jdtls 预置、协议修复、project load/configuration 韧性、真实项目 external/fallback 复测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步可选：预置 jdtls 做 external Java LSP 压测，或继续进入真实需求“范围确认 → 源码验证 → 实现设计/小改”。</t>
+          <t>下一步可选：补齐 Maven 私服/parent POM 后复测真正 type-aware Java navigation，或先进入真实需求“范围确认 → 源码验证 → 实现设计/小改”。</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11551,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 206 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 209 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>
@@ -11477,7 +11602,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-094 证明 external LSP 需要额外预置 server。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-095 已让 Java LSP 在 external 不完整时稳定回退并暴露 Maven parent POM 根因。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Java LSP project health probe
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测和 T-096 Java LSP 韧性对齐 OMP。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP 和 T-097 Java project health 探针。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 209 个测试通过</t>
+          <t>当前 210 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J99"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7143,6 +7143,50 @@
       </c>
       <c r="I98" s="0"/>
       <c r="J98" s="0"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t>T-097</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D99" s="0" t="inlineStr">
+        <is>
+          <t>Java project health 探针</t>
+        </is>
+      </c>
+      <c r="E99" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F99" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G99" s="0" t="inlineStr">
+        <is>
+          <t>Java 主战场需要一眼区分“jdtls 已安装”和“项目真的被导入”</t>
+        </is>
+      </c>
+      <c r="H99" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_status` 新增 `probe=true` / `path`，会启动匹配 external server 并调用 jdtls `java.project.getAll` / `java.project.listSourcePaths`；真实企业项目已验证输出 project/source path 为空和 Maven parent/私服/缓存修复提示。</t>
+        </is>
+      </c>
+      <c r="I99" s="0"/>
+      <c r="J99" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9060,7 +9104,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097 已让 `lsp_status probe=true` 可报告 project/source path 健康度；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10317,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096 已完成 jdtls 预置、协议修复、project load/configuration 韧性、真实项目 external/fallback 复测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、真实项目 external/fallback 复测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -11551,7 +11595,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 209 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 210 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Maven parent probe to Java LSP status
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP 和 T-097 Java project health 探针。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针和 T-098 Maven parent probe。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 210 个测试通过</t>
+          <t>当前 211 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J99"/>
+  <dimension ref="A1:J100"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7187,6 +7187,50 @@
       </c>
       <c r="I99" s="0"/>
       <c r="J99" s="0"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t>T-098</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C100" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D100" s="0" t="inlineStr">
+        <is>
+          <t>Maven parent probe</t>
+        </is>
+      </c>
+      <c r="E100" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F100" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G100" s="0" t="inlineStr">
+        <is>
+          <t>Java project health 需要进一步指出 Maven 导入失败的可行动根因</t>
+        </is>
+      </c>
+      <c r="H100" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_status probe=true` 会静态解析最近 `pom.xml` parent 链，检查 `relativePath` 和 `~/.m2/repository` parent POM；真实企业项目已直接定位缺失的 `com.yljr:parent` 版本。</t>
+        </is>
+      </c>
+      <c r="I100" s="0"/>
+      <c r="J100" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9104,7 +9148,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097 已让 `lsp_status probe=true` 可报告 project/source path 健康度；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098 已让 `lsp_status probe=true` 可报告 project/source path 健康度和缺失 Maven parent GAV；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10361,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、真实项目 external/fallback 复测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent probe、真实项目 external/fallback 复测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -11595,7 +11639,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 210 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 211 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Maven environment probe to Java LSP status
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针和 T-098 Maven parent probe。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe 和 T-099 Maven environment probe。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 211 个测试通过</t>
+          <t>当前 212 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7231,6 +7231,50 @@
       </c>
       <c r="I100" s="0"/>
       <c r="J100" s="0"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t>T-099</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C101" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D101" s="0" t="inlineStr">
+        <is>
+          <t>Maven environment probe</t>
+        </is>
+      </c>
+      <c r="E101" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F101" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G101" s="0" t="inlineStr">
+        <is>
+          <t>缺 parent POM 后还需要判断本机 Maven 私服/settings/local repo 是否准备好</t>
+        </is>
+      </c>
+      <c r="H101" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_status probe=true` 会报告 `mvn`、Maven settings、本地仓库和 mirror/server/profile/repository/activeProfile 数量；不输出私服 URL、账号或密码。</t>
+        </is>
+      </c>
+      <c r="I101" s="0"/>
+      <c r="J101" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9148,7 +9192,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098 已让 `lsp_status probe=true` 可报告 project/source path 健康度和缺失 Maven parent GAV；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
@@ -10361,7 +10405,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent probe、真实项目 external/fallback 复测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -11639,7 +11683,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 211 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 212 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Java LSP fallback for large projects
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe 和 T-099 Maven environment probe。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测和 T-101 query-aware LSP fallback。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 212 个测试通过</t>
+          <t>当前 213 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J103"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7275,6 +7275,94 @@
       </c>
       <c r="I101" s="0"/>
       <c r="J101" s="0"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t>T-100</t>
+        </is>
+      </c>
+      <c r="B102" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C102" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D102" s="0" t="inlineStr">
+        <is>
+          <t>Java LSP fallback 真实复测</t>
+        </is>
+      </c>
+      <c r="E102" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F102" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G102" s="0" t="inlineStr">
+        <is>
+          <t>验证 parent POM 缺失时，LCA 是否能解释 external LSP 边界并继续用 fallback/search/read_file 证据回答</t>
+        </is>
+      </c>
+      <c r="H102" s="0" t="inlineStr">
+        <is>
+          <t>`crcl-open` sessions `20260709T090514754843Z` / `20260709T090748481226Z` 已验证；第二轮 `lsp_symbols` / `lsp_definition` 直接返回 fallback 类/方法证据，最终回答正确说明 jdtls incomplete。</t>
+        </is>
+      </c>
+      <c r="I102" s="0"/>
+      <c r="J102" s="0"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t>T-101</t>
+        </is>
+      </c>
+      <c r="B103" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C103" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D103" s="0" t="inlineStr">
+        <is>
+          <t>query-aware LSP fallback</t>
+        </is>
+      </c>
+      <c r="E103" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F103" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G103" s="0" t="inlineStr">
+        <is>
+          <t>第一轮复测暴露大仓库根路径 fallback 受 300 文件窗口限制，可能漏掉明确类名</t>
+        </is>
+      </c>
+      <c r="H103" s="0" t="inlineStr">
+        <is>
+          <t>`lsp_symbols` / `lsp_definition` 带 query/symbol 时优先扫描文件名/路径匹配候选；新增 320 dummy Java 文件回归测试。</t>
+        </is>
+      </c>
+      <c r="I103" s="0"/>
+      <c r="J103" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9192,7 +9280,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；external 空结果时合并 light fallback 并标注 provider/confidence，避免 Agent 失明。真正 type-aware navigation 需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
@@ -10405,7 +10493,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -11683,7 +11771,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 212 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 213 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record T102 pressure test and sanitize invalid tool calls
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测和 T-101 query-aware LSP fallback。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware LSP fallback、T-102 拓展服务费结算真实需求链路压测和 T-103 provider-safe invalid tool_call normalization。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 213 个测试通过</t>
+          <t>当前 214 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J105"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7364,6 +7364,94 @@
       <c r="I103" s="0"/>
       <c r="J103" s="0"/>
     </row>
+    <row r="104">
+      <c r="A104" s="0" t="inlineStr">
+        <is>
+          <t>T-102</t>
+        </is>
+      </c>
+      <c r="B104" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C104" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D104" s="0" t="inlineStr">
+        <is>
+          <t>拓展服务费结算真实需求链路压测</t>
+        </is>
+      </c>
+      <c r="E104" s="0" t="inlineStr">
+        <is>
+          <t>已完成阶段 1-3</t>
+        </is>
+      </c>
+      <c r="F104" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G104" s="0" t="inlineStr">
+        <is>
+          <t>验证 LCA 能否从真实需求做范围判断、源码可用性核对、源码只读验证</t>
+        </is>
+      </c>
+      <c r="H104" s="0" t="inlineStr">
+        <is>
+          <t>范围判断通过；源码验证表明当前本机缺主候选 `zqyl-manager`、`zqyl-loan-application`、`ysd-provider`，仅有弱相关证据，暂不能进入实现设计。</t>
+        </is>
+      </c>
+      <c r="I104" s="0"/>
+      <c r="J104" s="0"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t>T-103</t>
+        </is>
+      </c>
+      <c r="B105" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C105" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D105" s="0" t="inlineStr">
+        <is>
+          <t>provider-safe invalid tool_call normalization</t>
+        </is>
+      </c>
+      <c r="E105" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F105" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G105" s="0" t="inlineStr">
+        <is>
+          <t>T-102 暴露模型空工具名会污染历史并导致百炼 400</t>
+        </is>
+      </c>
+      <c r="H105" s="0" t="inlineStr">
+        <is>
+          <t>assistant message 入历史前规范化 tool_call id/name/arguments；空工具名替换为 `__invalid_tool_call`，保持 tool_result 配对；新增回归测试。</t>
+        </is>
+      </c>
+      <c r="I105" s="0"/>
+      <c r="J105" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -7373,7 +7461,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -9287,37 +9375,37 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9417,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -9339,22 +9427,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -9366,7 +9454,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -9376,7 +9464,7 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -9386,12 +9474,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9491,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -9413,22 +9501,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9528,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -9450,7 +9538,7 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -9460,12 +9548,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9565,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9487,7 +9575,7 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -9497,12 +9585,12 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -9514,7 +9602,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9524,7 +9612,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -9534,12 +9622,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9639,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9561,7 +9649,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -9571,12 +9659,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9676,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9598,7 +9686,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -9608,12 +9696,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9713,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9635,22 +9723,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9750,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9672,7 +9760,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -9682,12 +9770,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9699,7 +9787,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9709,22 +9797,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9824,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -9746,22 +9834,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -9773,32 +9861,32 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9898,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -9820,22 +9908,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9935,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -9857,7 +9945,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
@@ -9867,12 +9955,12 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9972,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -9894,22 +9982,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -9921,7 +10009,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -9931,22 +10019,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -9958,32 +10046,32 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -9995,7 +10083,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -10005,7 +10093,7 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
@@ -10015,12 +10103,12 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -10032,7 +10120,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -10042,22 +10130,22 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -10069,7 +10157,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -10079,7 +10167,7 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -10089,12 +10177,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10194,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -10116,7 +10204,7 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
@@ -10126,12 +10214,12 @@
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -10143,7 +10231,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -10153,7 +10241,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
@@ -10163,12 +10251,12 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -10180,7 +10268,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -10190,7 +10278,7 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
@@ -10200,12 +10288,12 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -10217,7 +10305,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -10227,22 +10315,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10342,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -10264,22 +10352,22 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -10291,7 +10379,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -10301,22 +10389,22 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -10328,7 +10416,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -10338,7 +10426,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -10348,12 +10436,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -10365,7 +10453,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -10375,7 +10463,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
@@ -10385,12 +10473,12 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -10402,30 +10490,67 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
+          <t>ADR-031</t>
+        </is>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D83" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+        </is>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F83" s="0" t="inlineStr">
+        <is>
+          <t>已从 `compaction.py` 开始</t>
+        </is>
+      </c>
+      <c r="G83" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B84" s="0" t="inlineStr">
+        <is>
           <t>ADR-032</t>
         </is>
       </c>
-      <c r="C83" s="0" t="inlineStr">
+      <c r="C84" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D83" s="0" t="inlineStr">
+      <c r="D84" s="0" t="inlineStr">
         <is>
           <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
-      <c r="E83" s="0" t="inlineStr">
+      <c r="E84" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F83" s="0" t="inlineStr">
+      <c r="F84" s="0" t="inlineStr">
         <is>
           <t>已完成 T-093</t>
         </is>
       </c>
-      <c r="G83" s="0" t="inlineStr">
+      <c r="G84" s="0" t="inlineStr">
         <is>
           <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
@@ -10493,12 +10618,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步可选：补齐 Maven 私服/parent POM 后复测真正 type-aware Java navigation，或先进入真实需求“范围确认 → 源码验证 → 实现设计/小改”。</t>
+          <t>下一步需要补充拓展服务费结算的主候选源码，或换一个当前源码覆盖充分的真实需求进入实现设计/小改。</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11896,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 213 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 214 个 unittest、compileall 和 diff check。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record T104 payment service source validation
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware LSP fallback、T-102 拓展服务费结算真实需求链路压测和 T-103 provider-safe invalid tool_call normalization。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware LSP fallback、T-102 拓展服务费结算真实需求链路压测、T-103 provider-safe invalid tool_call normalization 和 T-104 msp-pay / zqylpayment 用户确认范围源码复核。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J106"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7451,6 +7451,50 @@
       </c>
       <c r="I105" s="0"/>
       <c r="J105" s="0"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="inlineStr">
+        <is>
+          <t>T-104</t>
+        </is>
+      </c>
+      <c r="B106" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C106" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D106" s="0" t="inlineStr">
+        <is>
+          <t>msp-pay / zqylpayment 用户确认范围源码复核</t>
+        </is>
+      </c>
+      <c r="E106" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F106" s="0" t="inlineStr">
+        <is>
+          <t>Agent + User</t>
+        </is>
+      </c>
+      <c r="G106" s="0" t="inlineStr">
+        <is>
+          <t>用户确认服务费结算前端应为 `msp-pay`、后端应为 `zqylpayment`，需要复核此前“缺主候选源码”的判断</t>
+        </is>
+      </c>
+      <c r="H106" s="0" t="inlineStr">
+        <is>
+          <t>session `20260709T092317272887Z` 以 `zqylpaymentmaster9d423763` 为 cwd、`mpspaymasterce6ca65` 和需求目录为 allow-dir；结论是两者是合理候选但只部分支持，仍缺结算单实体、状态 60、制单/回退/下载中心等证据。</t>
+        </is>
+      </c>
+      <c r="I106" s="0"/>
+      <c r="J106" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8290,12 +8334,12 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>用户确认当前测试项目可能不覆盖完整需求；`拓展服务费结算` 可能在 incentive/settlement 等其他项目</t>
+          <t>用户确认 `拓展服务费结算` 前端大概率是 `msp-pay`、后端大概率是 `zqylpayment`；T-104 复核显示这两个项目是合理候选但仍只部分覆盖，核心结算实体/流程证据未闭环</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>OMP 依赖用户提供完整 workspace/context；我们记录为压测边界，后续用多个 `--allow-dir` 接入相关项目，或者要求 Agent 明确输出“还需要哪个项目”。</t>
+          <t>OMP 依赖用户提供完整 workspace/context；我们记录为压测边界，后续用多个 `--allow-dir` 接入相关项目，并要求 Agent 区分“候选范围被用户确认”和“源码证据已闭环”。</t>
         </is>
       </c>
     </row>
@@ -10618,12 +10662,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复；T-104 已按用户确认的 `msp-pay` / `zqylpayment` 做源码复核</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步需要补充拓展服务费结算的主候选源码，或换一个当前源码覆盖充分的真实需求进入实现设计/小改。</t>
+          <t>下一步在这两个候选项目内做更窄的证据补全，确认现有能力复用点和必须新建能力，再进入实现设计/小改。</t>
         </is>
       </c>
     </row>
@@ -11947,7 +11991,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-095 已让 Java LSP 在 external 不完整时稳定回退并暴露 Maven parent POM 根因。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-104 已将用户确认的 `msp-pay` / `zqylpayment` 作为合理候选复核，下一步补齐服务费结算核心证据后再进入实现设计。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add final answer steering and token budget
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware LSP fallback、T-102 拓展服务费结算真实需求链路压测、T-103 provider-safe invalid tool_call normalization 和 T-104 msp-pay / zqylpayment 用户确认范围源码复核。</t>
+          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware fallback、T-102 拓展服务费结算真实需求链路压测、T-103 provider-safe invalid tool_call normalization、T-104 msp-pay / zqylpayment 用户确认范围源码复核、T-105 窄范围证据补全、T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>`context_char_budget` / `context_recent_messages`</t>
+          <t>`context_char_budget` / `context_token_budget` / `context_recent_messages`</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>下一步补 token 预算、输出 reserve；字符阈值保留兜底</t>
+          <t>token budget + reserve 已完成 MVP；provider/model 专用 tokenizer 和输出 reserve 后置</t>
         </is>
       </c>
       <c r="F30" s="0"/>
@@ -2830,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J109"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>已实现字符阈值 deterministic compaction；LLM summary 已补，下一步升级 token budget / reserve</t>
+          <t>已实现字符阈值 deterministic compaction、LLM summary、本地 token budget + 15% reserve；后续再评估 provider/model 专用 tokenizer 和输出 reserve</t>
         </is>
       </c>
       <c r="I12" s="0"/>
@@ -7495,6 +7495,138 @@
       </c>
       <c r="I106" s="0"/>
       <c r="J106" s="0"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t>T-105</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C107" s="0" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="D107" s="0" t="inlineStr">
+        <is>
+          <t>msp-pay / zqylpayment 窄范围证据补全压测</t>
+        </is>
+      </c>
+      <c r="E107" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F107" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G107" s="0" t="inlineStr">
+        <is>
+          <t>沿 T-104 继续只读补齐状态枚举、费用明细、制单/回退、下载中心和前端页面证据</t>
+        </is>
+      </c>
+      <c r="H107" s="0" t="inlineStr">
+        <is>
+          <t>session `20260709T092951071920Z` 找到 `PreOrderStatusEnum`、`PlatOrderStatusEnum`、`OrderStatusEnum`、`FeeDetailEntity`、`PlatformOrderController`、`preOrderManagement/list.vue` 等证据；结论是现有平台缴费/预制单框架可复用，但未找到拓展服务费结算专属实体/状态 60 闭环。</t>
+        </is>
+      </c>
+      <c r="I107" s="0"/>
+      <c r="J107" s="0"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t>T-106</t>
+        </is>
+      </c>
+      <c r="B108" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C108" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D108" s="0" t="inlineStr">
+        <is>
+          <t>FinalAnswer Steerer 第一块抽象 + source-grounded numeric guard</t>
+        </is>
+      </c>
+      <c r="E108" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F108" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G108" s="0" t="inlineStr">
+        <is>
+          <t>T-105 暴露最终回答把源码枚举 `2/3` 误报成 `50/60`；同时 review 指出 final-answer guard 继续堆在 `agent.py`</t>
+        </is>
+      </c>
+      <c r="H108" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/steering/final_answer.py`，把 read-only evidence、no-edit hygiene、final structure、source-grounded numeric 等最终回答纠偏移出 `agent.py`；数字/状态码类结论若与已读源码不一致，会强制无工具重写。</t>
+        </is>
+      </c>
+      <c r="I108" s="0"/>
+      <c r="J108" s="0"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t>T-107</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C109" s="0" t="inlineStr">
+        <is>
+          <t>P9/P10</t>
+        </is>
+      </c>
+      <c r="D109" s="0" t="inlineStr">
+        <is>
+          <t>Context token budget + reserve MVP</t>
+        </is>
+      </c>
+      <c r="E109" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F109" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G109" s="0" t="inlineStr">
+        <is>
+          <t>review 指出上下文治理仍是字符预算，不符合 OMP token + reserve 原则</t>
+        </is>
+      </c>
+      <c r="H109" s="0" t="inlineStr">
+        <is>
+          <t>新增本地 token 估算、`context_token_budget` / `AGENT_CONTEXT_TOKEN_BUDGET` / `--context-token-budget`，按 token 或 char 任一超阈值触发 compaction，并至少预留 15% 下一轮预算；char budget 继续作为兜底。</t>
+        </is>
+      </c>
+      <c r="I109" s="0"/>
+      <c r="J109" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7505,7 +7637,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G88"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7594,12 +7726,12 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>已做 OMP 风格 reserve 阈值、auto LLM summary、当前用户请求保留、超大 tool 输出截断和单 system 摘要合并；后续再评估精确 token 预算、输出 reserve、recent 保留</t>
+          <t>已做 OMP 风格 reserve 阈值、auto LLM summary、当前用户请求保留、超大 tool 输出截断、单 system 摘要合并和 token budget MVP；后续再评估 provider/model 专用 tokenizer、输出 reserve 和 recent 保留策略</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>OMP 按上下文 token 预算触发压缩，给下一轮 prompt/输出预留 reserve，并把早期历史压成 summary；我们当前用字符窗口近似，下一步可升级为 token 估算。</t>
+          <t>OMP 按上下文 token 预算触发压缩，给下一轮 prompt/输出预留 reserve，并把早期历史压成 summary；我们先用本地轻量 token 估算 + 15% reserve，字符预算保留为无 tokenizer fallback。</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8853,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-053</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -8731,22 +8863,22 @@
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>源码证据型最终回答可能误报数字/状态码</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>已关闭 MVP 版，继续压测</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>T-105 session `20260709T092951071920Z` 读到 `PreOrderStatusEnum.MAKING(2)` / `MADE(3)`，最终却误报为 `50/60`</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>参考 OMP runtime evidence/steering 边界：新增 source-grounded numeric final steerer，记录本轮 `read_file` 源码证据；最终回答涉及枚举、状态码、接口、字段等数字事实时，若与已读源码片段不一致，会强制无工具重写并要求标注未确认。</t>
         </is>
       </c>
     </row>
@@ -8758,32 +8890,32 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-054</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>`agent.py` steering/guard 继续膨胀</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已开始缓解，继续拆</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>review 指出 compaction 已拆出，但 semantic/read-only/final guard 又继续进入 `agent.py`，不符合 OMP 一职责一文件原则</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>已完成 FinalAnswer Steerer 第一块抽象：最终回答相关 steering 移到 `src/local_agent/steering/final_answer.py`；后续继续按低风险边界拆 evidence ledger、run collector、startup context、memory consolidation 和 semantic exploration steerer。</t>
         </is>
       </c>
     </row>
@@ -8795,32 +8927,32 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8964,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -8842,22 +8974,22 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -8869,7 +9001,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -8879,7 +9011,7 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -8889,12 +9021,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -8906,7 +9038,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -8916,22 +9048,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -8943,7 +9075,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -8953,7 +9085,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -8963,12 +9095,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -8980,7 +9112,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -8990,22 +9122,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -9017,7 +9149,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -9027,7 +9159,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -9037,12 +9169,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -9054,7 +9186,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -9064,22 +9196,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -9091,7 +9223,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -9101,22 +9233,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -9128,17 +9260,17 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -9148,12 +9280,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -9165,17 +9297,17 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -9185,12 +9317,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -9202,17 +9334,17 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -9222,12 +9354,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -9239,32 +9371,32 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -9276,7 +9408,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -9286,22 +9418,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9445,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -9323,22 +9455,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9482,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -9360,22 +9492,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -9387,32 +9519,32 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -9424,106 +9556,106 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -9535,7 +9667,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -9545,22 +9677,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -9572,7 +9704,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -9582,22 +9714,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9741,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9619,22 +9751,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9778,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9656,7 +9788,7 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -9666,12 +9798,12 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -9683,7 +9815,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9693,7 +9825,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -9703,12 +9835,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -9720,7 +9852,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9730,7 +9862,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -9740,12 +9872,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9757,7 +9889,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9767,7 +9899,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -9777,12 +9909,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9926,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9804,22 +9936,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -9831,7 +9963,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9841,22 +9973,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -9868,7 +10000,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -9878,22 +10010,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -9905,7 +10037,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -9915,22 +10047,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -9942,32 +10074,32 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -9979,32 +10111,32 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10148,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -10026,22 +10158,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -10053,7 +10185,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -10063,22 +10195,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10222,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -10100,7 +10232,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -10110,12 +10242,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -10127,17 +10259,17 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
@@ -10147,12 +10279,12 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -10164,32 +10296,32 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10333,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -10211,22 +10343,22 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10370,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -10248,22 +10380,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10407,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -10285,7 +10417,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
@@ -10295,12 +10427,12 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -10312,7 +10444,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -10322,7 +10454,7 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
@@ -10332,12 +10464,12 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -10349,7 +10481,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -10359,7 +10491,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
@@ -10369,12 +10501,12 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10518,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -10396,22 +10528,22 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -10423,7 +10555,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -10433,7 +10565,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -10443,12 +10575,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10592,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -10470,7 +10602,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -10480,12 +10612,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -10497,7 +10629,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -10507,22 +10639,22 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -10534,7 +10666,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -10544,7 +10676,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
@@ -10554,12 +10686,12 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -10571,32 +10703,180 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
+          <t>ADR-030</t>
+        </is>
+      </c>
+      <c r="C84" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D84" s="0" t="inlineStr">
+        <is>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+        </is>
+      </c>
+      <c r="E84" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F84" s="0" t="inlineStr">
+        <is>
+          <t>先做 T-085~T-087</t>
+        </is>
+      </c>
+      <c r="G84" s="0" t="inlineStr">
+        <is>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t>ADR-031</t>
+        </is>
+      </c>
+      <c r="C85" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D85" s="0" t="inlineStr">
+        <is>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+        </is>
+      </c>
+      <c r="E85" s="0" t="inlineStr">
+        <is>
+          <t>已接受</t>
+        </is>
+      </c>
+      <c r="F85" s="0" t="inlineStr">
+        <is>
+          <t>已从 `compaction.py` 开始</t>
+        </is>
+      </c>
+      <c r="G85" s="0" t="inlineStr">
+        <is>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B86" s="0" t="inlineStr">
+        <is>
           <t>ADR-032</t>
         </is>
       </c>
-      <c r="C84" s="0" t="inlineStr">
+      <c r="C86" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D84" s="0" t="inlineStr">
+      <c r="D86" s="0" t="inlineStr">
         <is>
           <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
-      <c r="E84" s="0" t="inlineStr">
+      <c r="E86" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F84" s="0" t="inlineStr">
+      <c r="F86" s="0" t="inlineStr">
         <is>
           <t>已完成 T-093</t>
         </is>
       </c>
-      <c r="G84" s="0" t="inlineStr">
+      <c r="G86" s="0" t="inlineStr">
         <is>
           <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t>ADR-033</t>
+        </is>
+      </c>
+      <c r="C87" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D87" s="0" t="inlineStr">
+        <is>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+        </is>
+      </c>
+      <c r="E87" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F87" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-106</t>
+        </is>
+      </c>
+      <c r="G87" s="0" t="inlineStr">
+        <is>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B88" s="0" t="inlineStr">
+        <is>
+          <t>ADR-034</t>
+        </is>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D88" s="0" t="inlineStr">
+        <is>
+          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F88" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-107</t>
+        </is>
+      </c>
+      <c r="G88" s="0" t="inlineStr">
+        <is>
+          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
         </is>
       </c>
     </row>
@@ -10662,12 +10942,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复；T-104 已按用户确认的 `msp-pay` / `zqylpayment` 做源码复核</t>
+          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复；T-104/T-105 已按用户确认的 `msp-pay` / `zqylpayment` 做源码复核和窄范围证据补全；T-106/T-107 已补 FinalAnswer Steerer 第一块抽象、source-grounded numeric guard 和 token budget MVP</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步在这两个候选项目内做更窄的证据补全，确认现有能力复用点和必须新建能力，再进入实现设计/小改。</t>
+          <t>下一步复测 T-105 同类证据任务，观察枚举/状态码是否仍会误报；并继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11974,7 +12254,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；token budget / output reserve / managed skills 继续后置评估。</t>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；provider/model 专用 tokenizer、输出 reserve、managed skills 和完整 ToolChoiceQueue 继续后置评估。</t>
         </is>
       </c>
     </row>
@@ -11991,7 +12271,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP 和项目边界分析 MVP；T-104 已将用户确认的 `msp-pay` / `zqylpayment` 作为合理候选复核，下一步补齐服务费结算核心证据后再进入实现设计。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP、项目边界分析 MVP、source-grounded numeric guard 和 token budget MVP；下一步复测服务费结算证据链，确认现有能力复用点和必须新建能力后再进入实现设计。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add requirement contract and tool choice queue
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P9：真实需求使用准备</t>
+          <t>P10：Intelligence Runtime 骨架</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P6 默认工作流 MVP 已落地；P7 已补 OMP 风格 auto summary、多语言 LSP/light fallback、multi-root、startup context/rules、startup memory、learn、可选 memory consolidation、runtime state dir、Evidence Ledger、relevance gate、implementation-quality gate 和 no-edit final hygiene；2026-07-09 已完成 T-076 Event/Command Protocol v1、T-077/T-080 Terminal Frontend MVP 与命令可发现性、T-078 项目边界分析 MVP、T-081 Claude review 行动计划、T-082 run summary / coverage MVP、T-083 真实需求压测模板、T-084 qwen3-coder-next 企业项目只读源码验证压测、T-089 semantic exploration guard、T-090 terminal input/output isolation、T-091 Vue diff reviewer 误报修复、T-092 compaction 渐进模块化 / LSP 置信度提示、T-093 可选外部 LSP adapter、T-094 真实项目 LSP 可用性压测、T-095 jdtls 预置/strict external 复测、T-096 Java LSP 韧性对齐 OMP、T-097 Java project health 探针、T-098 Maven parent probe、T-099 Maven environment probe、T-100 Java LSP fallback 真实复测、T-101 query-aware fallback、T-102 拓展服务费结算真实需求链路压测、T-103 provider-safe invalid tool_call normalization、T-104 msp-pay / zqylpayment 用户确认范围源码复核、T-105 窄范围证据补全、T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP。</t>
+          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-111 MiniToolChoiceQueue。下一步是 T-110 CompletionAudit、Planner/Explore 和二阶段 reviewer。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,11 +216,11 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>完整 unittest、compileall、diff check、xlsx 检查通过。</t>
+          <t>完整 unittest 通过；xlsx 同步后继续检查。</t>
         </is>
       </c>
       <c r="D7" s="0"/>
@@ -720,10 +720,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -1091,6 +1091,38 @@
       <c r="F12" s="0" t="inlineStr">
         <is>
           <t>T-078 已完成项目边界分析 MVP；T-083 已固化压测模板；T-084 已完成 qwen3-coder-next 只读源码验证压测并记录新问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Intelligence Runtime 骨架</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、Reviewer</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>已完成 RequirementContract 和 MiniToolChoiceQueue MVP；下一步 CompletionAudit。</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2836,12 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 214 个测试通过</t>
+          <t>当前 232 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>unittest、compileall、diff check、xlsx 检查通过</t>
+          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -2830,7 +2862,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J113"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7628,6 +7660,182 @@
       <c r="I109" s="0"/>
       <c r="J109" s="0"/>
     </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t>T-108</t>
+        </is>
+      </c>
+      <c r="B110" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C110" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D110" s="0" t="inlineStr">
+        <is>
+          <t>source-grounded numeric / token budget 复测</t>
+        </is>
+      </c>
+      <c r="E110" s="0" t="inlineStr">
+        <is>
+          <t>已完成并记录问题</t>
+        </is>
+      </c>
+      <c r="F110" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G110" s="0" t="inlineStr">
+        <is>
+          <t>验证 T-106/T-107 是否能避免状态码误报和 provider 崩溃</t>
+        </is>
+      </c>
+      <c r="H110" s="0" t="inlineStr">
+        <is>
+          <t>session `20260709T095626110047Z` 枚举数字回答正确，且 provider-safe 修复后百炼不再 400；但模型在 `msp-pay` 大搜索结果后未继续读关键文件就下结论，触发 T-109/T-111。</t>
+        </is>
+      </c>
+      <c r="I110" s="0"/>
+      <c r="J110" s="0"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t>T-109</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C111" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D111" s="0" t="inlineStr">
+        <is>
+          <t>RequirementContract MVP</t>
+        </is>
+      </c>
+      <c r="E111" s="0" t="inlineStr">
+        <is>
+          <t>已完成并集成</t>
+        </is>
+      </c>
+      <c r="F111" s="0" t="inlineStr">
+        <is>
+          <t>小红 + Agent</t>
+        </is>
+      </c>
+      <c r="G111" s="0" t="inlineStr">
+        <is>
+          <t>让每轮任务先有目标、范围、验收项、证据要求和验证要求，避免任务漂移</t>
+        </is>
+      </c>
+      <c r="H111" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/task_contract.py` 和测试；runtime 每轮 provider request 注入 `[Requirement contract]`。</t>
+        </is>
+      </c>
+      <c r="I111" s="0"/>
+      <c r="J111" s="0"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t>T-110</t>
+        </is>
+      </c>
+      <c r="B112" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C112" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D112" s="0" t="inlineStr">
+        <is>
+          <t>CompletionAudit MVP</t>
+        </is>
+      </c>
+      <c r="E112" s="0" t="inlineStr">
+        <is>
+          <t>已完成最小切片，继续增强</t>
+        </is>
+      </c>
+      <c r="F112" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G112" s="0" t="inlineStr">
+        <is>
+          <t>最终回答前逐项核对 contract，解决“缺证据却说完成”</t>
+        </is>
+      </c>
+      <c r="H112" s="0" t="inlineStr">
+        <is>
+          <t>已补 source evidence false-negative gate：最终回答说“未找到/读取不完整”，但 read_file evidence 中包含用户请求符号时强制无工具重答；数字比对会剥离 read_file 行号。完整逐项验收审计后续继续。</t>
+        </is>
+      </c>
+      <c r="I112" s="0"/>
+      <c r="J112" s="0"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t>T-111</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C113" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D113" s="0" t="inlineStr">
+        <is>
+          <t>MiniToolChoiceQueue MVP</t>
+        </is>
+      </c>
+      <c r="E113" s="0" t="inlineStr">
+        <is>
+          <t>已完成并集成</t>
+        </is>
+      </c>
+      <c r="F113" s="0" t="inlineStr">
+        <is>
+          <t>Zeno + Agent</t>
+        </is>
+      </c>
+      <c r="G113" s="0" t="inlineStr">
+        <is>
+          <t>解决只读证据任务过早回答、需求文档未读、写后缺测试/diff 的工具选择问题</t>
+        </is>
+      </c>
+      <c r="H113" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/tool_choice_queue.py` 和测试；runtime 根据 contract/task kind、工具摘要和可用工具集合，阶段性收窄 tool schemas 并追加 runtime steering。</t>
+        </is>
+      </c>
+      <c r="I113" s="0"/>
+      <c r="J113" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -7637,7 +7845,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G91"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8794,17 +9002,17 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>开放并受控</t>
+          <t>已触发裁剪版 MVP，继续受控</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 reviewer、subagents、ToolChoiceQueue 很强，但 LCA 当前还缺真实实现压测的失败样本；提前完整搬入可能拖慢 MVP 验证</t>
+          <t>T-108/T-105 类压测证明仅靠 prompt 和 final steering 仍会出现关键证据没读够就下结论；但完整 OMP ToolChoiceQueue/reviewer/subagents 仍过重</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>先进入 T-072 真实需求实现压测；若压测暴露工具选择失控，按 OMP 裁剪 ToolChoiceQueue；若暴露 patch/总结质量不稳，按 OMP 裁剪轻量 reviewer。</t>
+          <t>已按 OMP 工具调度原则裁剪出 MiniToolChoiceQueue，只覆盖只读证据、需求文档前置读取、写后测试/diff hygiene；完整 reviewer、Planner/Explore、subagents 继续等真实失败样本触发。</t>
         </is>
       </c>
     </row>
@@ -8927,7 +9135,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-055</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -8937,22 +9145,22 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>无效 tool_call 参数会污染下一轮 provider 请求</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>T-108 首轮复测中百炼拒绝历史消息：无效工具调用的 `function.arguments` 为空或畸形 JSON，导致下一轮 HTTP 400</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>已在 assistant message 入历史前把工具名、id、arguments 统一归一为 provider-safe JSON object 字符串；空/畸形参数写入 `_invalid_arguments`，并补回归测试。</t>
         </is>
       </c>
     </row>
@@ -8964,17 +9172,17 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-056</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>read_file 行号会干扰源码数字事实比对</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -8984,12 +9192,12 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>T-108 窄复测中，模型把枚举状态误报成 1/3/5；numeric guard 因 read_file 内容含 `1:`、`3:`、`5:` 行号而误以为这些数字有源码证据</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>source numeric guard 比对前会剥离 read_file 行号前缀，再判断状态码/枚举值是否出现在源码内容中；新增回归测试覆盖错误数字刚好等于行号的情况。</t>
         </is>
       </c>
     </row>
@@ -9001,32 +9209,32 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9246,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -9048,22 +9256,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9283,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -9085,7 +9293,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -9095,12 +9303,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -9112,7 +9320,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -9122,22 +9330,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9357,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -9159,7 +9367,7 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -9169,12 +9377,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9394,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -9196,22 +9404,22 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -9223,7 +9431,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -9233,7 +9441,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -9243,12 +9451,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -9260,7 +9468,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -9270,22 +9478,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9505,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -9307,22 +9515,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -9334,17 +9542,17 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -9354,12 +9562,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -9371,17 +9579,17 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -9391,12 +9599,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -9408,17 +9616,17 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -9428,12 +9636,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -9445,32 +9653,32 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9690,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -9492,22 +9700,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9727,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -9529,22 +9737,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -9556,7 +9764,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -9566,22 +9774,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -9593,32 +9801,32 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -9630,106 +9838,106 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9949,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -9751,22 +9959,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -9778,7 +9986,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -9788,22 +9996,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -9815,7 +10023,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -9825,22 +10033,22 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -9852,7 +10060,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -9862,7 +10070,7 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -9872,12 +10080,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -9889,7 +10097,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -9899,7 +10107,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -9909,12 +10117,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -9926,7 +10134,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -9936,7 +10144,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -9946,12 +10154,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -9963,7 +10171,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -9973,7 +10181,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -9983,12 +10191,12 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -10000,7 +10208,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -10010,22 +10218,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10245,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -10047,22 +10255,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -10074,7 +10282,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -10084,22 +10292,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -10111,7 +10319,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -10121,22 +10329,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -10148,32 +10356,32 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -10185,32 +10393,32 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10430,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -10232,22 +10440,22 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -10259,7 +10467,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -10269,22 +10477,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -10296,7 +10504,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -10306,7 +10514,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
@@ -10316,12 +10524,12 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -10333,17 +10541,17 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
@@ -10353,12 +10561,12 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -10370,32 +10578,32 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -10407,7 +10615,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -10417,22 +10625,22 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -10444,7 +10652,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -10454,22 +10662,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10689,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -10491,7 +10699,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
@@ -10501,12 +10709,12 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -10518,7 +10726,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -10528,7 +10736,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
@@ -10538,12 +10746,12 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -10555,7 +10763,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -10565,7 +10773,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -10575,12 +10783,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -10592,7 +10800,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -10602,22 +10810,22 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10837,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -10639,7 +10847,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
@@ -10649,12 +10857,12 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -10666,7 +10874,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -10676,7 +10884,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
@@ -10686,12 +10894,12 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -10703,7 +10911,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -10713,22 +10921,22 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -10740,7 +10948,7 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -10750,7 +10958,7 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
@@ -10760,12 +10968,12 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -10777,7 +10985,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-032</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -10787,22 +10995,22 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-093</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -10814,7 +11022,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-033</t>
+          <t>ADR-031</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -10824,22 +11032,22 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-106</t>
+          <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -10851,32 +11059,143 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
+          <t>ADR-032</t>
+        </is>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D88" s="0" t="inlineStr">
+        <is>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F88" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-093</t>
+        </is>
+      </c>
+      <c r="G88" s="0" t="inlineStr">
+        <is>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B89" s="0" t="inlineStr">
+        <is>
+          <t>ADR-033</t>
+        </is>
+      </c>
+      <c r="C89" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D89" s="0" t="inlineStr">
+        <is>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+        </is>
+      </c>
+      <c r="E89" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F89" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-106</t>
+        </is>
+      </c>
+      <c r="G89" s="0" t="inlineStr">
+        <is>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B90" s="0" t="inlineStr">
+        <is>
           <t>ADR-034</t>
         </is>
       </c>
-      <c r="C88" s="0" t="inlineStr">
+      <c r="C90" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D88" s="0" t="inlineStr">
+      <c r="D90" s="0" t="inlineStr">
         <is>
           <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
         </is>
       </c>
-      <c r="E88" s="0" t="inlineStr">
+      <c r="E90" s="0" t="inlineStr">
         <is>
           <t>已接受并落地</t>
         </is>
       </c>
-      <c r="F88" s="0" t="inlineStr">
+      <c r="F90" s="0" t="inlineStr">
         <is>
           <t>已完成 T-107</t>
         </is>
       </c>
-      <c r="G88" s="0" t="inlineStr">
+      <c r="G90" s="0" t="inlineStr">
         <is>
           <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B91" s="0" t="inlineStr">
+        <is>
+          <t>ADR-035</t>
+        </is>
+      </c>
+      <c r="C91" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D91" s="0" t="inlineStr">
+        <is>
+          <t>P10 采用裁剪版 Intelligence Runtime，不一次性复制 OMP 大系统</t>
+        </is>
+      </c>
+      <c r="E91" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地部分</t>
+        </is>
+      </c>
+      <c r="F91" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-109/T-111，T-110 待做</t>
+        </is>
+      </c>
+      <c r="G91" s="0" t="inlineStr">
+        <is>
+          <t>T-108 证明需要比 prompt 更硬的目标契约和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + MiniToolChoiceQueue，后续再补 CompletionAudit、Planner/Explore 和 reviewer。</t>
         </is>
       </c>
     </row>
@@ -10892,7 +11211,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -10937,17 +11256,17 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>P9 真实需求使用准备进行中</t>
+          <t>P10 Intelligence Runtime 骨架进行中</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-077 已让 Runtime 产出 typed events，并提供 terminal-native 交互入口；T-078 已把项目边界分析沉淀为本机 memory/skill 和通用 runtime gate；T-084 已完成新模型只读源码验证压测；T-085/T-086/T-087/T-088/T-089/T-090 已补 todo 参数纠偏、重复读收束、最终结构/证据卫生、evidence-first gate、语义探索收束和终端输入隔离；T-091/T-092 已修 Vue reviewer 误报并启动 OMP 风格渐进模块化；T-093 已补可选外部 LSP adapter；T-094/T-095/T-096/T-097/T-098/T-099/T-100/T-101 已完成 jdtls 预置、协议修复、project load/configuration 韧性、project health 探针、Maven parent/environment probe、真实项目 external/fallback 复测和 query-aware fallback；T-102/T-103 已完成真实需求链路压测和非法 tool_call 修复；T-104/T-105 已按用户确认的 `msp-pay` / `zqylpayment` 做源码复核和窄范围证据补全；T-106/T-107 已补 FinalAnswer Steerer 第一块抽象、source-grounded numeric guard 和 token budget MVP</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-111 已补 RequirementContract 和 MiniToolChoiceQueue</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步复测 T-105 同类证据任务，观察枚举/状态码是否仍会误报；并继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>下一步做 T-110 CompletionAudit，并继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -10964,7 +11283,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>完整 ToolChoiceQueue、reviewer/subagents、完整 LSP/DAP、browser/TUI、AST edit、managed skills 仍后置</t>
+          <t>完整 reviewer/subagents、完整 LSP/DAP、browser/TUI、AST edit、managed skills 仍后置；ToolChoiceQueue 已有裁剪版 MVP</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
@@ -11025,17 +11344,17 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>暂不先做完整 ToolChoiceQueue</t>
+          <t>已做裁剪版 MiniToolChoiceQueue</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已有 allowed-dir soft requirement、duplicate forced-final、todo steering、pruning；还缺“关键工具长期不用/乱用”的新失败样本</t>
+          <t>当前覆盖只读证据、需求文档前置读取、写后测试/diff hygiene；不做完整多队列/并发/子任务调度</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>若 T-072 暴露工具选择失控，再按 OMP 裁剪 ToolChoiceQueue</t>
+          <t>后续若仍出现关键工具不用/乱用，再扩展 queue 规则；若出现 patch/总结质量不稳，补 reviewer。</t>
         </is>
       </c>
     </row>
@@ -11047,17 +11366,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>真实需求链路</t>
+          <t>CompletionAudit + 真实需求设计链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-084 已证明新模型能跑通只读链路；重复读、todo 参数、最终结构/证据卫生、evidence-first、语义探索扩散和终端输入污染问题已补</t>
+          <t>T-108 已证明 source-grounded numeric guard 生效，但暴露搜索结果过大后未继续读关键证据；T-109/T-111 已补 contract/queue</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>进入用户真实需求的项目范围确认和源码验证；必要时复跑密码加密问答样本</t>
+          <t>先做 T-110 CompletionAudit，再继续服务费结算实现设计压测。</t>
         </is>
       </c>
     </row>
@@ -12220,7 +12539,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P9 当前代码已跑通 214 个 unittest、compileall 和 diff check。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 232 个 unittest。</t>
         </is>
       </c>
     </row>
@@ -12254,7 +12573,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；provider/model 专用 tokenizer、输出 reserve、managed skills 和完整 ToolChoiceQueue 继续后置评估。</t>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；provider/model 专用 tokenizer、输出 reserve、managed skills、完整 reviewer 和完整 OMP ToolChoiceQueue 继续后置评估。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add completion audit steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-111 MiniToolChoiceQueue。下一步是 T-110 CompletionAudit、Planner/Explore 和二阶段 reviewer。</t>
+          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue。下一步是 Planner/Explore 和二阶段 reviewer。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract 和 MiniToolChoiceQueue MVP；下一步 CompletionAudit。</t>
+          <t>已完成 RequirementContract、CompletionAudit 和 MiniToolChoiceQueue MVP；下一步 Planner/Explore。</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 232 个测试通过</t>
+          <t>当前 237 个测试通过</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -7766,12 +7766,12 @@
       </c>
       <c r="D112" s="0" t="inlineStr">
         <is>
-          <t>CompletionAudit MVP</t>
+          <t>CompletionAudit 完整版</t>
         </is>
       </c>
       <c r="E112" s="0" t="inlineStr">
         <is>
-          <t>已完成最小切片，继续增强</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F112" s="0" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="H112" s="0" t="inlineStr">
         <is>
-          <t>已补 source evidence false-negative gate：最终回答说“未找到/读取不完整”，但 read_file evidence 中包含用户请求符号时强制无工具重答；数字比对会剥离 read_file 行号。完整逐项验收审计后续继续。</t>
+          <t>新增 `src/local_agent/completion_audit.py`，按 RequirementContract 核对验收项、证据项和验证项；证据型只读回答缺源码路径/证据状态会强制无工具重写，实现任务写后缺 `run_tests` / `git_diff` 会只开放缺失验证工具；session payload 记录 missing audit items。</t>
         </is>
       </c>
       <c r="I112" s="0"/>
@@ -11190,12 +11190,12 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-109/T-111，T-110 待做</t>
+          <t>已完成 T-109/T-110/T-111</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>T-108 证明需要比 prompt 更硬的目标契约和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + MiniToolChoiceQueue，后续再补 CompletionAudit、Planner/Explore 和 reviewer。</t>
+          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue，后续再补 Planner/Explore 和 reviewer。</t>
         </is>
       </c>
     </row>
@@ -11261,12 +11261,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-111 已补 RequirementContract 和 MiniToolChoiceQueue</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111 已补 RequirementContract、CompletionAudit 和 MiniToolChoiceQueue</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步做 T-110 CompletionAudit，并继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>下一步进入 Planner/Explore 两阶段或继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11366,17 +11366,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>CompletionAudit + 真实需求设计链路</t>
+          <t>Planner/Explore + 真实需求设计链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-108 已证明 source-grounded numeric guard 生效，但暴露搜索结果过大后未继续读关键证据；T-109/T-111 已补 contract/queue</t>
+          <t>T-109/T-110/T-111 已补 contract/audit/queue，最终回答和工具选择主骨架已具备</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 T-110 CompletionAudit，再继续服务费结算实现设计压测。</t>
+          <t>先做 Planner/Explore 两阶段计划，或用服务费结算需求继续压测实现设计链路。</t>
         </is>
       </c>
     </row>
@@ -12539,7 +12539,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 232 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 237 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add planner explore phase gating
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue。下一步是 Planner/Explore 和二阶段 reviewer。</t>
+          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue、T-112 Planner/Explore。下一步是二阶段 reviewer。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit 和 MiniToolChoiceQueue MVP；下一步 Planner/Explore。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue 和 Planner/Explore MVP；下一步 Reviewer。</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H58"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2826,32 +2826,62 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>Planner/Explore</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>当前 237 个测试通过</t>
+          <t>`src/local_agent/planner.py`、`src/local_agent/tool_choice_queue.py`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+          <t>实现任务在 explore 阶段只开放 list/read/search/LSP/todo/ask/git 状态检查；读到本地证据后进入 ready_to_implement，写后进入 verify</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>真实实现压测</t>
         </is>
       </c>
       <c r="F57" s="0"/>
       <c r="G57" s="0"/>
       <c r="H57" s="0"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>当前 244 个测试通过</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F58" s="0"/>
+      <c r="G58" s="0"/>
+      <c r="H58" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2862,7 +2892,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J114"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7835,6 +7865,50 @@
       </c>
       <c r="I113" s="0"/>
       <c r="J113" s="0"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t>T-112</t>
+        </is>
+      </c>
+      <c r="B114" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C114" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D114" s="0" t="inlineStr">
+        <is>
+          <t>Planner/Explore 两阶段 MVP</t>
+        </is>
+      </c>
+      <c r="E114" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F114" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G114" s="0" t="inlineStr">
+        <is>
+          <t>复杂实现任务先只读侦察和形成计划，再进入写入，减少上来乱改</t>
+        </is>
+      </c>
+      <c r="H114" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/planner.py` 和测试；runtime 注入 `[Planner / Explore]` 阶段上下文；MiniToolChoiceQueue 在 explore 阶段隐藏写入/执行工具，读到本地证据后释放写入工具。</t>
+        </is>
+      </c>
+      <c r="I114" s="0"/>
+      <c r="J114" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11190,12 +11264,12 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-109/T-110/T-111</t>
+          <t>已完成 T-109/T-110/T-111/T-112</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue，后续再补 Planner/Explore 和 reviewer。</t>
+          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue + Planner/Explore，后续再补 reviewer。</t>
         </is>
       </c>
     </row>
@@ -11261,12 +11335,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111 已补 RequirementContract、CompletionAudit 和 MiniToolChoiceQueue</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111/T-112 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue 和 Planner/Explore</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步进入 Planner/Explore 两阶段或继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>下一步进入二阶段 Reviewer，或继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11366,17 +11440,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Planner/Explore + 真实需求设计链路</t>
+          <t>二阶段 Reviewer + 真实需求设计链路</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-109/T-110/T-111 已补 contract/audit/queue，最终回答和工具选择主骨架已具备</t>
+          <t>T-109/T-110/T-111/T-112 已补 contract/audit/queue/planner，最终回答和工具选择主骨架已具备</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做 Planner/Explore 两阶段计划，或用服务费结算需求继续压测实现设计链路。</t>
+          <t>先做写后 reviewer，或用服务费结算需求继续压测实现设计链路。</t>
         </is>
       </c>
     </row>
@@ -12539,7 +12613,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 237 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 244 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add patch reviewer steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-09 继续完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue、T-112 Planner/Explore。下一步是二阶段 reviewer。</t>
+          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-10 已完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue、T-112 Planner/Explore、T-113 二阶段 Patch Reviewer。下一步用真实小改压测验证 reviewer 是否能驱动模型补测试、查调用方或诚实停止。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue 和 Planner/Explore MVP；下一步 Reviewer。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore 和二阶段 Patch Reviewer MVP；下一步真实小改复测。</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2856,32 +2856,62 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>二阶段 Patch Reviewer</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>当前 244 个测试通过</t>
+          <t>`src/local_agent/patch_reviewer.py`、`src/local_agent/steering/final_answer.py`</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+          <t>写后读取 `git_diff` 的结构化 diff/reviewer 信号，检查显式要求的测试是否进入 diff、公开 API 是否在写后检索调用方、低相关/注释型 patch 是否被处理；发现问题时只开放修复/验证/回滚工具，随后再走 CompletionAudit</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>真实小改压测</t>
         </is>
       </c>
       <c r="F58" s="0"/>
       <c r="G58" s="0"/>
       <c r="H58" s="0"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>当前 253 个测试通过</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F59" s="0"/>
+      <c r="G59" s="0"/>
+      <c r="H59" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2892,7 +2922,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J114"/>
+  <dimension ref="A1:J115"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7909,6 +7939,50 @@
       </c>
       <c r="I114" s="0"/>
       <c r="J114" s="0"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t>T-113</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C115" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D115" s="0" t="inlineStr">
+        <is>
+          <t>二阶段 Patch Reviewer MVP</t>
+        </is>
+      </c>
+      <c r="E115" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F115" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G115" s="0" t="inlineStr">
+        <is>
+          <t>仅有 `git_diff` 警告不足以阻止模型把无关/注释型 patch 说成完成；写后需要独立检查“是否满足契约、是否漏测试/调用方”。</t>
+        </is>
+      </c>
+      <c r="H115" s="0" t="inlineStr">
+        <is>
+          <t>新增 `src/local_agent/patch_reviewer.py`：读取已收集的 write / `git_diff` / search/LSP 结果，阻断缺显式测试 diff、公开 API 无写后调用方检索、低相关或 comment-only diff；`PatchReviewSteerer` 在 CompletionAudit 前收束到修复、验证、回滚工具。ToolChoiceQueue 在已有 diff 但待验证时保留受控修复工具，避免 reviewer 与 queue 互相卡死。</t>
+        </is>
+      </c>
+      <c r="I115" s="0"/>
+      <c r="J115" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9076,17 +9150,17 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>已触发裁剪版 MVP，继续受控</t>
+          <t>已缓解，继续受控</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>T-108/T-105 类压测证明仅靠 prompt 和 final steering 仍会出现关键证据没读够就下结论；但完整 OMP ToolChoiceQueue/reviewer/subagents 仍过重</t>
+          <t>T-108/T-105 类压测证明仅靠 prompt 和 final steering 仍会出现关键证据没读够就下结论；完整 OMP ToolChoiceQueue/reviewer/subagents 仍过重。</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>已按 OMP 工具调度原则裁剪出 MiniToolChoiceQueue，只覆盖只读证据、需求文档前置读取、写后测试/diff hygiene；完整 reviewer、Planner/Explore、subagents 继续等真实失败样本触发。</t>
+          <t>已按 OMP 工具调度原则裁剪出 MiniToolChoiceQueue、Planner/Explore 和二阶段 Patch Reviewer；Reviewer 仅消费已有 diff/工具证据，不引入第二个 Agent。完整多队列调度和 subagents 继续等真实失败样本触发。</t>
         </is>
       </c>
     </row>
@@ -11264,12 +11338,12 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-109/T-110/T-111/T-112</t>
+          <t>已完成 T-109/T-110/T-111/T-112/T-113</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前先落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue + Planner/Explore，后续再补 reviewer。</t>
+          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue + Planner/Explore + Patch Reviewer；不引入第二个 Agent。</t>
         </is>
       </c>
     </row>
@@ -11335,12 +11409,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111/T-112 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue 和 Planner/Explore</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111/T-112/T-113 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore 和 Patch Reviewer。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步进入二阶段 Reviewer，或继续按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>下一步用真实小改压测验证 reviewer，然后按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11440,17 +11514,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>二阶段 Reviewer + 真实需求设计链路</t>
+          <t>Patch Reviewer 真实小改复测</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-109/T-110/T-111/T-112 已补 contract/audit/queue/planner，最终回答和工具选择主骨架已具备</t>
+          <t>T-109/T-110/T-111/T-112/T-113 已补 contract/audit/queue/planner/reviewer，最终回答、工具选择和写后审查主骨架已具备</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先做写后 reviewer，或用服务费结算需求继续压测实现设计链路。</t>
+          <t>用一个显式要求“改代码并补测试”的小任务，验证模型会补测试/检索调用方/复查 diff，而不是绕过 reviewer。</t>
         </is>
       </c>
     </row>
@@ -12613,7 +12687,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 244 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 253 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden patch review pressure controls
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P9 已完成真实需求使用准备的阶段性 MVP：项目边界分析、真实需求模板、企业项目只读源码验证、Java LSP 韧性、拓展服务费结算链路压测和服务范围复核；2026-07-10 已完成 T-106 source-grounded numeric guard / FinalAnswer Steerer 第一块抽象、T-107 token budget + reserve MVP、T-108 source-grounded numeric/token budget 复测、T-109 RequirementContract、T-110 CompletionAudit、T-111 MiniToolChoiceQueue、T-112 Planner/Explore、T-113 二阶段 Patch Reviewer。下一步用真实小改压测验证 reviewer 是否能驱动模型补测试、查调用方或诚实停止。</t>
+          <t>T-113/T-114 真实百炼压测已关闭“Reviewer 只在最终回答运行”和“无证据 blocked/no-edit 放行”两个 runtime 漏口；完整端到端 reviewer 复测尚未通过，因为模型频繁错传 `apply_patch` / `todo_*` 参数。下一步 T-115 在 ToolRegistry 边界做受限兼容归一，再复测。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore 和二阶段 Patch Reviewer MVP；下一步真实小改复测。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate；下一步 ToolRegistry 参数归一与真实复测。</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2866,17 +2866,17 @@
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/patch_reviewer.py`、`src/local_agent/steering/final_answer.py`</t>
+          <t>`src/local_agent/patch_reviewer.py`、`src/local_agent/steering/final_answer.py`、`src/local_agent/agent.py`</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>写后读取 `git_diff` 的结构化 diff/reviewer 信号，检查显式要求的测试是否进入 diff、公开 API 是否在写后检索调用方、低相关/注释型 patch 是否被处理；发现问题时只开放修复/验证/回滚工具，随后再走 CompletionAudit</t>
+          <t>成功 `git_diff` 后立即检查显式测试 diff、公开 API 调用方和已有 diff reviewer finding；若有风险，停止同批后续工具并只开放修复/验证/回滚，最终回答仍有兜底审查</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>真实小改压测</t>
+          <t>完成 T-115 后重跑真实小改</t>
         </is>
       </c>
       <c r="F58" s="0"/>
@@ -2886,32 +2886,62 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t>测试覆盖</t>
+          <t>No-edit evidence gate</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成 MVP 版</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>当前 253 个测试通过</t>
+          <t>`src/local_agent/completion_audit.py`</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+          <t>实现任务的 blocked/no-edit 必须由 search/LSP 未命中、路径缺失、runtime relevance/approval 拒绝等工具事实支撑；模型文本不足以放行</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>日用反馈补测</t>
+          <t>继续真实任务观察</t>
         </is>
       </c>
       <c r="F59" s="0"/>
       <c r="G59" s="0"/>
       <c r="H59" s="0"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t>测试覆盖</t>
+        </is>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>当前 257 个测试通过</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>日用反馈补测</t>
+        </is>
+      </c>
+      <c r="F60" s="0"/>
+      <c r="G60" s="0"/>
+      <c r="H60" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2922,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J117"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7963,7 +7993,7 @@
       </c>
       <c r="E115" s="0" t="inlineStr">
         <is>
-          <t>已完成</t>
+          <t>已完成并压测修正</t>
         </is>
       </c>
       <c r="F115" s="0" t="inlineStr">
@@ -7978,11 +8008,99 @@
       </c>
       <c r="H115" s="0" t="inlineStr">
         <is>
-          <t>新增 `src/local_agent/patch_reviewer.py`：读取已收集的 write / `git_diff` / search/LSP 结果，阻断缺显式测试 diff、公开 API 无写后调用方检索、低相关或 comment-only diff；`PatchReviewSteerer` 在 CompletionAudit 前收束到修复、验证、回滚工具。ToolChoiceQueue 在已有 diff 但待验证时保留受控修复工具，避免 reviewer 与 queue 互相卡死。</t>
+          <t>新增 `patch_reviewer.py`；成功 `git_diff` 后立即运行 reviewer，若 finding 存在则跳过同批后续 tool call、写 runtime steering 并仅开放修复/验证/回滚；最终回答仍有兜底。覆盖缺显式测试 diff、公开 API 无写后调用方检索、低相关/comment-only diff。</t>
         </is>
       </c>
       <c r="I115" s="0"/>
       <c r="J115" s="0"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t>T-114</t>
+        </is>
+      </c>
+      <c r="B116" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C116" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D116" s="0" t="inlineStr">
+        <is>
+          <t>no-edit evidence gate</t>
+        </is>
+      </c>
+      <c r="E116" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F116" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G116" s="0" t="inlineStr">
+        <is>
+          <t>T-113 压测显示模型可在未写入时仅凭“blocked/unexecuted”自述逃过 CompletionAudit。</t>
+        </is>
+      </c>
+      <c r="H116" s="0" t="inlineStr">
+        <is>
+          <t>CompletionAudit 现在要求工具观察到具体阻断条件；没有 search/LSP 未命中、路径缺失、relevance/approval 拒绝等证据时，会开放 read/search/apply_patch 继续任务。</t>
+        </is>
+      </c>
+      <c r="I116" s="0"/>
+      <c r="J116" s="0"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t>T-115</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C117" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D117" s="0" t="inlineStr">
+        <is>
+          <t>Tool argument compatibility normalization</t>
+        </is>
+      </c>
+      <c r="E117" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F117" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G117" s="0" t="inlineStr">
+        <is>
+          <t>百炼压测多次出现旧式 `apply_patch` 字段、字符串行号和 todo status 方言，造成大量无效调用与 token 浪费。</t>
+        </is>
+      </c>
+      <c r="H117" s="0" t="inlineStr">
+        <is>
+          <t>在 ToolRegistry 单一边界受限归一已知别名/数值，不放宽任意 schema；补回归后重跑 Reviewer 压测。</t>
+        </is>
+      </c>
+      <c r="I117" s="0"/>
+      <c r="J117" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7993,7 +8111,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -9357,7 +9475,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-057</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -9367,22 +9485,22 @@
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>provider 的工具参数方言导致有效任务无法进入写入/验证闭环</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>开放，T-115</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>2026-07-10 三轮百炼压测中出现 `file_hash`/`old_str`/`new_str`、`mode=edit`、字符串行号、`todo_add status=pending` 和原始 `&lt;tool_call&gt;` 文本；73 次工具调用中有 16 次错误。</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>按 OMP 的 tool-call 归一边界设计 T-115：只在 ToolRegistry 接收明确列出的兼容别名，原始 schema 和 anchored 安全校验仍生效。</t>
         </is>
       </c>
     </row>
@@ -9394,32 +9512,32 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9549,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -9441,7 +9559,7 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -9451,12 +9569,12 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -9468,7 +9586,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -9478,22 +9596,22 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9623,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -9515,22 +9633,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -9542,7 +9660,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -9552,7 +9670,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -9562,12 +9680,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9697,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -9589,7 +9707,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -9599,12 +9717,12 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -9616,7 +9734,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -9626,22 +9744,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -9653,7 +9771,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -9663,22 +9781,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -9690,7 +9808,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -9700,22 +9818,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9845,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -9737,7 +9855,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -9747,12 +9865,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -9764,17 +9882,17 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -9784,12 +9902,12 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9919,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -9811,7 +9929,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -9821,12 +9939,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -9838,17 +9956,17 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -9858,12 +9976,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9993,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -9885,22 +10003,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -9912,7 +10030,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -9922,22 +10040,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -9949,7 +10067,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -9959,22 +10077,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -9986,7 +10104,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -9996,22 +10114,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -10023,32 +10141,32 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10178,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -10070,59 +10188,59 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10252,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -10144,22 +10262,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -10171,7 +10289,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -10181,7 +10299,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -10191,12 +10309,12 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -10208,7 +10326,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -10218,22 +10336,22 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10363,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -10255,7 +10373,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -10265,12 +10383,12 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -10282,7 +10400,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -10292,7 +10410,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -10302,12 +10420,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -10319,7 +10437,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -10329,7 +10447,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -10339,12 +10457,12 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -10356,7 +10474,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -10366,7 +10484,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -10376,12 +10494,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -10393,7 +10511,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -10403,7 +10521,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -10413,12 +10531,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -10430,7 +10548,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -10440,22 +10558,22 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -10467,7 +10585,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -10477,7 +10595,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
@@ -10487,12 +10605,12 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10622,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -10514,22 +10632,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10659,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -10551,22 +10669,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -10578,32 +10696,32 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -10615,7 +10733,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -10625,22 +10743,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -10652,7 +10770,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -10662,7 +10780,7 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
@@ -10672,12 +10790,12 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -10689,7 +10807,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -10699,22 +10817,22 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -10726,7 +10844,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -10736,22 +10854,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -10763,32 +10881,32 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -10800,7 +10918,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -10810,7 +10928,7 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
@@ -10820,12 +10938,12 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -10837,7 +10955,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -10847,22 +10965,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -10874,7 +10992,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -10884,7 +11002,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
@@ -10894,12 +11012,12 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -10911,7 +11029,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -10921,7 +11039,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -10931,12 +11049,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -10948,7 +11066,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -10958,7 +11076,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -10968,12 +11086,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -10985,7 +11103,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -10995,7 +11113,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
@@ -11005,12 +11123,12 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -11022,7 +11140,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -11032,22 +11150,22 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -11059,7 +11177,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -11069,22 +11187,22 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -11096,7 +11214,7 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -11106,22 +11224,22 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -11133,7 +11251,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -11143,7 +11261,7 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
@@ -11153,12 +11271,12 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -11170,7 +11288,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -11180,7 +11298,7 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
@@ -11190,12 +11308,12 @@
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -11207,7 +11325,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>ADR-032</t>
+          <t>ADR-031</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -11217,22 +11335,22 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-093</t>
+          <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -11244,7 +11362,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>ADR-033</t>
+          <t>ADR-032</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -11254,7 +11372,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr">
@@ -11264,12 +11382,12 @@
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-106</t>
+          <t>已完成 T-093</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
       </c>
     </row>
@@ -11281,7 +11399,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>ADR-034</t>
+          <t>ADR-033</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -11291,7 +11409,7 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr">
@@ -11301,12 +11419,12 @@
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-107</t>
+          <t>已完成 T-106</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
         </is>
       </c>
     </row>
@@ -11318,32 +11436,69 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
+          <t>ADR-034</t>
+        </is>
+      </c>
+      <c r="C91" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D91" s="0" t="inlineStr">
+        <is>
+          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+        </is>
+      </c>
+      <c r="E91" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F91" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-107</t>
+        </is>
+      </c>
+      <c r="G91" s="0" t="inlineStr">
+        <is>
+          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B92" s="0" t="inlineStr">
+        <is>
           <t>ADR-035</t>
         </is>
       </c>
-      <c r="C91" s="0" t="inlineStr">
+      <c r="C92" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D91" s="0" t="inlineStr">
+      <c r="D92" s="0" t="inlineStr">
         <is>
           <t>P10 采用裁剪版 Intelligence Runtime，不一次性复制 OMP 大系统</t>
         </is>
       </c>
-      <c r="E91" s="0" t="inlineStr">
+      <c r="E92" s="0" t="inlineStr">
         <is>
           <t>已接受并落地部分</t>
         </is>
       </c>
-      <c r="F91" s="0" t="inlineStr">
-        <is>
-          <t>已完成 T-109/T-110/T-111/T-112/T-113</t>
-        </is>
-      </c>
-      <c r="G91" s="0" t="inlineStr">
-        <is>
-          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract + CompletionAudit + MiniToolChoiceQueue + Planner/Explore + Patch Reviewer；不引入第二个 Agent。</t>
+      <c r="F92" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-109/T-110/T-111/T-112/T-113/T-114</t>
+        </is>
+      </c>
+      <c r="G92" s="0" t="inlineStr">
+        <is>
+          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate；不引入第二个 Agent。</t>
         </is>
       </c>
     </row>
@@ -11409,12 +11564,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-108 复测证明 provider-safe/numeric guard 有效但暴露证据未读够就下结论；T-109/T-110/T-111/T-112/T-113 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore 和 Patch Reviewer。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-114 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate。T-113 真实压测同时暴露 provider 参数方言问题。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>下一步用真实小改压测验证 reviewer，然后按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>先做 T-115 的 ToolRegistry 受限参数归一，再重跑 reviewer；随后按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11514,17 +11669,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Patch Reviewer 真实小改复测</t>
+          <t>ToolRegistry 参数归一后重跑 Reviewer</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-109/T-110/T-111/T-112/T-113 已补 contract/audit/queue/planner/reviewer，最终回答、工具选择和写后审查主骨架已具备</t>
+          <t>T-113/T-114 已关闭 reviewer 时点和无证据 no-edit 漏口；但百炼常错传 edit/todo 参数，当前压测无法稳定进入写入/验证闭环。</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>用一个显式要求“改代码并补测试”的小任务，验证模型会补测试/检索调用方/复查 diff，而不是绕过 reviewer。</t>
+          <t>T-115 只兼容已观测参数别名和数值类型，不降低 schema、hash 或权限边界；完成后再用显式“改代码并补测试”任务复测 reviewer。</t>
         </is>
       </c>
     </row>
@@ -11537,7 +11692,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -12612,6 +12767,38 @@
       <c r="F34" s="0" t="inlineStr">
         <is>
           <t>T-087 已完成：项目范围表必须含项目/服务列；用户要求证据状态或回答含推断性表达时，final gate 要求已验证/推断标签。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>PT-033</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>已修复，端到端待重跑</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>20260710 百炼压测显示 Reviewer 原本只在 final 时才生效，且模型可用无证据 `blocked/unexecuted` 自述结束；同轮暴露大量 `apply_patch` / `todo_*` 参数方言。</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>OMP 在 active loop 中观察工具结果，并在 protocol boundary 归一工具调用。</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>T-113 前移 post-diff reviewer；T-114 要求 no-edit 工具证据；T-115 待在 ToolRegistry 归一已知 provider aliases。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
     </row>
@@ -12687,7 +12874,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 253 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 257 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize provider tool arguments safely
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-113/T-114 真实百炼压测已关闭“Reviewer 只在最终回答运行”和“无证据 blocked/no-edit 放行”两个 runtime 漏口；完整端到端 reviewer 复测尚未通过，因为模型频繁错传 `apply_patch` / `todo_*` 参数。下一步 T-115 在 ToolRegistry 边界做受限兼容归一，再复测。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-115 已在 ToolRegistry 单一边界完成已观测标量参数归一，并以真实临时 worktree 跑通源码修改、测试修改、定向测试和 diff；但 57 次调用中仍有 25 次无效尝试，主要是 raw unified diff、批量 todo 与 preview 缺失。下一步 T-116/T-117 收紧 preview contract 和 numeric guard 作用域。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate；下一步 ToolRegistry 参数归一与真实复测。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一和真实小改复测；下一步 preview contract 与 numeric guard 作用域。</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>完成 T-115 后重跑真实小改</t>
+          <t>T-115 真实小改已复测；下一步 T-116 preview contract</t>
         </is>
       </c>
       <c r="F58" s="0"/>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>当前 257 个测试通过</t>
+          <t>当前 261 个测试通过</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J119"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="E117" s="0" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成并压测</t>
         </is>
       </c>
       <c r="F117" s="0" t="inlineStr">
@@ -8091,16 +8091,104 @@
       </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
-          <t>百炼压测多次出现旧式 `apply_patch` 字段、字符串行号和 todo status 方言，造成大量无效调用与 token 浪费。</t>
+          <t>百炼压测多次出现旧式 `apply_patch` 字段、字符串行号、字符串布尔值、`run_tests.cmd` 和 todo status 方言。</t>
         </is>
       </c>
       <c r="H117" s="0" t="inlineStr">
         <is>
-          <t>在 ToolRegistry 单一边界受限归一已知别名/数值，不放宽任意 schema；补回归后重跑 Reviewer 压测。</t>
+          <t>`ToolRegistry` 在 schema 校验前仅归一已观测 scalar alias：`file_hash`/`file_hash_tag`/`source_hash_tag`/`hash_tag -&gt; tag`、`old_str/new_str`、`mode=edit`、整数/布尔字符串、`cmd -&gt; command`、todo `key/content/pending`；冲突直接拒绝。真实 session `20260710T020730075094Z` 改 2 文件、定向 6 测试 OK、diff +8/-0。</t>
         </is>
       </c>
       <c r="I117" s="0"/>
       <c r="J117" s="0"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t>T-116</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C118" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D118" s="0" t="inlineStr">
+        <is>
+          <t>Preview contract / unsafe structured-call gate</t>
+        </is>
+      </c>
+      <c r="E118" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F118" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G118" s="0" t="inlineStr">
+        <is>
+          <t>T-115 复测仍出现 `patch_content` raw diff、todo array 和没有成功 preview 就 real patch；这些不能由参数别名安全解释。</t>
+        </is>
+      </c>
+      <c r="H118" s="0" t="inlineStr">
+        <is>
+          <t>参考 OMP tool requirement/active-loop steering：对要求 preview 的任务，在首个 real patch 前只开放 `apply_patch dry_run=true` 与必要 read；raw diff / bulk todo 保持明确失败并给 canonical 示例。</t>
+        </is>
+      </c>
+      <c r="I118" s="0"/>
+      <c r="J118" s="0"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t>T-117</t>
+        </is>
+      </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C119" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D119" s="0" t="inlineStr">
+        <is>
+          <t>Source numeric guard scope correction</t>
+        </is>
+      </c>
+      <c r="E119" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F119" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G119" s="0" t="inlineStr">
+        <is>
+          <t>T-115 复测中 diff hunk、+/- 统计和测试数量被误判为源码状态码数字，触发两次无工具重写。</t>
+        </is>
+      </c>
+      <c r="H119" s="0" t="inlineStr">
+        <is>
+          <t>区分 source code facts 与 git/test observation；枚举/状态码/接口常量继续 source-grounded，比对 diff/test 数字时使用对应 tool evidence。</t>
+        </is>
+      </c>
+      <c r="I119" s="0"/>
+      <c r="J119" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8111,7 +8199,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G94"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -9490,17 +9578,17 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>开放，T-115</t>
+          <t>已缓解，继续观察</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>2026-07-10 三轮百炼压测中出现 `file_hash`/`old_str`/`new_str`、`mode=edit`、字符串行号、`todo_add status=pending` 和原始 `&lt;tool_call&gt;` 文本；73 次工具调用中有 16 次错误。</t>
+          <t>T-115 已收敛 `file_hash*` / `source_hash_tag` / `hash_tag`、`old_str/new_str`、`mode=edit`、整数/布尔字符串、`run_tests.cmd` 和 todo scalar 方言；真实小改已完成源码/测试/定向测试/diff。</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>按 OMP 的 tool-call 归一边界设计 T-115：只在 ToolRegistry 接收明确列出的兼容别名，原始 schema 和 anchored 安全校验仍生效。</t>
+          <t>按 OMP 的 tool-call 归一边界，只在 ToolRegistry 接收明确已观测的 scalar alias；schema、hash、approval 和 anchored patch 校验不变。raw diff / bulk todo 不隐式执行，交由 T-116。</t>
         </is>
       </c>
     </row>
@@ -9512,7 +9600,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-058</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -9522,22 +9610,22 @@
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>raw diff / bulk todo 形式无法安全映射到细粒度工具</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>开放，T-116</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>T-115 复测 57 次调用中 25 次错误，包含 `patch_content` unified diff、`todo` / `todo_items` 数组和不完整 patch 参数。</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>参考 OMP 工具协议边界：不把不等价结构自动拆成带副作用的多次调用；以 preview contract 和可行动 schema error 引导模型回到 anchored patch / 单条 todo。</t>
         </is>
       </c>
     </row>
@@ -9549,7 +9637,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-059</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -9559,22 +9647,22 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>source numeric guard 会误拦 diff/test 观测数字</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>开放，T-117</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>T-115 复测将 hunk 坐标、`+8/-0` 和测试计数送入源码数字比对，触发 2 次无工具 final 重写。</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>保持对枚举/状态码/接口常量的源码校验，排除 git/test 工具事实或让其匹配各自 tool evidence。</t>
         </is>
       </c>
     </row>
@@ -9586,32 +9674,32 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9711,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -9633,22 +9721,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9748,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -9670,7 +9758,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -9680,12 +9768,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -9697,7 +9785,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -9707,22 +9795,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -9734,7 +9822,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -9744,7 +9832,7 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -9754,12 +9842,12 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -9771,7 +9859,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -9781,22 +9869,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -9808,7 +9896,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -9818,7 +9906,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -9828,12 +9916,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -9845,7 +9933,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -9855,22 +9943,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -9882,7 +9970,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -9892,22 +9980,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -9919,17 +10007,17 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -9939,12 +10027,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -9956,17 +10044,17 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -9976,12 +10064,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -9993,17 +10081,17 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -10013,12 +10101,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -10030,32 +10118,32 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -10067,7 +10155,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -10077,22 +10165,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10192,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -10114,22 +10202,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -10141,7 +10229,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -10151,22 +10239,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -10178,32 +10266,32 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -10215,106 +10303,106 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -10326,7 +10414,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -10336,22 +10424,22 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -10363,7 +10451,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -10373,22 +10461,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -10400,7 +10488,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -10410,22 +10498,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -10437,7 +10525,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -10447,7 +10535,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -10457,12 +10545,12 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -10474,7 +10562,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -10484,7 +10572,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -10494,12 +10582,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10599,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -10521,7 +10609,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -10531,12 +10619,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -10548,7 +10636,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -10558,7 +10646,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
@@ -10568,12 +10656,12 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10673,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -10595,22 +10683,22 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -10622,7 +10710,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -10632,22 +10720,22 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -10659,7 +10747,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -10669,22 +10757,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -10696,7 +10784,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -10706,22 +10794,22 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -10733,32 +10821,32 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -10770,32 +10858,32 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -10807,7 +10895,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -10817,22 +10905,22 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -10844,7 +10932,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -10854,22 +10942,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -10881,7 +10969,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -10891,7 +10979,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
@@ -10901,12 +10989,12 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -10918,17 +11006,17 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
@@ -10938,12 +11026,12 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -10955,32 +11043,32 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -10992,7 +11080,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -11002,22 +11090,22 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11117,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -11039,22 +11127,22 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11154,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -11076,7 +11164,7 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -11086,12 +11174,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11191,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -11113,7 +11201,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
@@ -11123,12 +11211,12 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -11140,7 +11228,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -11150,7 +11238,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
@@ -11160,12 +11248,12 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -11177,7 +11265,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -11187,22 +11275,22 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -11214,7 +11302,7 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -11224,7 +11312,7 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
@@ -11234,12 +11322,12 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -11251,7 +11339,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -11261,7 +11349,7 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
@@ -11271,12 +11359,12 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -11288,7 +11376,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -11298,22 +11386,22 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11413,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -11335,7 +11423,7 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr">
@@ -11345,12 +11433,12 @@
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -11362,7 +11450,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>ADR-032</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -11372,22 +11460,22 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-093</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -11399,7 +11487,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>ADR-033</t>
+          <t>ADR-031</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -11409,22 +11497,22 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-106</t>
+          <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -11436,7 +11524,7 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>ADR-034</t>
+          <t>ADR-032</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -11446,7 +11534,7 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
       <c r="E91" s="0" t="inlineStr">
@@ -11456,12 +11544,12 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-107</t>
+          <t>已完成 T-093</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
       </c>
     </row>
@@ -11473,32 +11561,106 @@
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
+          <t>ADR-033</t>
+        </is>
+      </c>
+      <c r="C92" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D92" s="0" t="inlineStr">
+        <is>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+        </is>
+      </c>
+      <c r="E92" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F92" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-106</t>
+        </is>
+      </c>
+      <c r="G92" s="0" t="inlineStr">
+        <is>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t>ADR-034</t>
+        </is>
+      </c>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D93" s="0" t="inlineStr">
+        <is>
+          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+        </is>
+      </c>
+      <c r="E93" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F93" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-107</t>
+        </is>
+      </c>
+      <c r="G93" s="0" t="inlineStr">
+        <is>
+          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
           <t>ADR-035</t>
         </is>
       </c>
-      <c r="C92" s="0" t="inlineStr">
+      <c r="C94" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D92" s="0" t="inlineStr">
+      <c r="D94" s="0" t="inlineStr">
         <is>
           <t>P10 采用裁剪版 Intelligence Runtime，不一次性复制 OMP 大系统</t>
         </is>
       </c>
-      <c r="E92" s="0" t="inlineStr">
+      <c r="E94" s="0" t="inlineStr">
         <is>
           <t>已接受并落地部分</t>
         </is>
       </c>
-      <c r="F92" s="0" t="inlineStr">
-        <is>
-          <t>已完成 T-109/T-110/T-111/T-112/T-113/T-114</t>
-        </is>
-      </c>
-      <c r="G92" s="0" t="inlineStr">
-        <is>
-          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate；不引入第二个 Agent。</t>
+      <c r="F94" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-109/T-110/T-111/T-112/T-113/T-114/T-115</t>
+        </is>
+      </c>
+      <c r="G94" s="0" t="inlineStr">
+        <is>
+          <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate 和受限 ToolRegistry 归一；不引入第二个 Agent。</t>
         </is>
       </c>
     </row>
@@ -11514,7 +11676,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -11564,12 +11726,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-114 已补 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer 和 no-edit evidence gate。T-113 真实压测同时暴露 provider 参数方言问题。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-115 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一。真实小改交付链路已跑通，但工具调用效率仍不合格。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先做 T-115 的 ToolRegistry 受限参数归一，再重跑 reviewer；随后按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>先做 T-116 preview contract 与 T-117 numeric guard scope，再按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
         </is>
       </c>
     </row>
@@ -11669,17 +11831,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>ToolRegistry 参数归一后重跑 Reviewer</t>
+          <t>Preview contract 与 numeric guard scope</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-113/T-114 已关闭 reviewer 时点和无证据 no-edit 漏口；但百炼常错传 edit/todo 参数，当前压测无法稳定进入写入/验证闭环。</t>
+          <t>T-115 真实复测已完成源码、测试、定向 run_tests、git_diff 和最终结构，但 57 次工具调用中仍有 25 次错误。</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>T-115 只兼容已观测参数别名和数值类型，不降低 schema、hash 或权限边界；完成后再用显式“改代码并补测试”任务复测 reviewer。</t>
+          <t>T-116 不执行 raw diff/bulk todo，只引导/限制首个 real patch 前先有有效 dry-run；T-117 让 diff/test 数字不再被当作源码枚举事实。</t>
         </is>
       </c>
     </row>
@@ -11692,7 +11854,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -12783,7 +12945,7 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>已修复，端到端待重跑</t>
+          <t>已修复，持续验证</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
@@ -12798,7 +12960,39 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>T-113 前移 post-diff reviewer；T-114 要求 no-edit 工具证据；T-115 待在 ToolRegistry 归一已知 provider aliases。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-113 前移 post-diff reviewer；T-114 要求 no-edit 工具证据；T-115 已归一安全 scalar aliases 并重跑真实小改。详见 `docs/pressure-test-2026-07-10.md`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>PT-036</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>已缓解，继续优化</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>T-115 真实小改成功交付 2 文件、定向 6 测试和 diff，但共 57 tool calls / 25 errors；安全的 scalar 参数方言已可归一，raw diff/bulk todo 仍被拒绝。</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>OMP 在协议边界归一可确定的输入，active loop 以 tool requirement 防止无效路径扩散。</t>
+        </is>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>T-115 已完成 scalar normalization；T-116/T-117 待处理 preview contract 和 numeric guard 误拦。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
     </row>
@@ -12874,7 +13068,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 257 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 261 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden preview and final steering
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-115 已在 ToolRegistry 单一边界完成已观测标量参数归一，并以真实临时 worktree 跑通源码修改、测试修改、定向测试和 diff；但 57 次调用中仍有 25 次无效尝试，主要是 raw unified diff、批量 todo 与 preview 缺失。下一步 T-116/T-117 收紧 preview contract 和 numeric guard 作用域。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-116 已用 hard pre-tool gate 阻止未预览的真实 patch；T-117 已消除 diff/test 数字触发源码数字 guard；T-118 已修复“待写入 read-only 字面量”误分成只读任务。当前开放问题是模型在 preview error 后的纠错，以及 source-evidence false-negative 与 CompletionAudit 的优先级。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一和真实小改复测；下一步 preview contract 与 numeric guard 作用域。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope 和 quoted literal 分类修复；下一步 source-evidence false-negative 收束。</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>当前 261 个测试通过</t>
+          <t>当前 267 个测试通过</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J121"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8125,7 +8125,7 @@
       </c>
       <c r="E118" s="0" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成 MVP，继续压测</t>
         </is>
       </c>
       <c r="F118" s="0" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="H118" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP tool requirement/active-loop steering：对要求 preview 的任务，在首个 real patch 前只开放 `apply_patch dry_run=true` 与必要 read；raw diff / bulk todo 保持明确失败并给 canonical 示例。</t>
+          <t>`apply_patch` real write 前会对明确要求 preview 的任务检查同路径/同 tag/同 range/同 old/new/mode 的成功 dry-run；raw diff / bulk todo 仍明确失败。真实复测证明 direct write 被拦，preview 后同锚点 write 可放行。</t>
         </is>
       </c>
       <c r="I118" s="0"/>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="E119" s="0" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成 MVP</t>
         </is>
       </c>
       <c r="F119" s="0" t="inlineStr">
@@ -8184,11 +8184,99 @@
       </c>
       <c r="H119" s="0" t="inlineStr">
         <is>
-          <t>区分 source code facts 与 git/test observation；枚举/状态码/接口常量继续 source-grounded，比对 diff/test 数字时使用对应 tool evidence。</t>
+          <t>仅在请求/最终回答含真正的枚举、状态码、接口、字段或独立 `code` 数字事实时启用；跳过 apply_patch/tag/diff/test observation。后续压测 run summary 不再触发该 guard。</t>
         </is>
       </c>
       <c r="I119" s="0"/>
       <c r="J119" s="0"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t>T-118</t>
+        </is>
+      </c>
+      <c r="B120" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C120" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D120" s="0" t="inlineStr">
+        <is>
+          <t>quoted read-only literal task classification</t>
+        </is>
+      </c>
+      <c r="E120" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F120" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G120" s="0" t="inlineStr">
+        <is>
+          <t>实现任务要写入 `只读`/`read-only` 文本或测试断言时，deterministic classifier 把数据误当作禁止修改指令。</t>
+        </is>
+      </c>
+      <c r="H120" s="0" t="inlineStr">
+        <is>
+          <t>明确实现意图优先；仅 `不要修改` / `do not edit` / `no changes` 等真正禁止修改的指令覆盖。新增回归测试。</t>
+        </is>
+      </c>
+      <c r="I120" s="0"/>
+      <c r="J120" s="0"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
+          <t>T-119</t>
+        </is>
+      </c>
+      <c r="B121" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C121" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D121" s="0" t="inlineStr">
+        <is>
+          <t>实现任务 final-guard scope / CompletionAudit priority</t>
+        </is>
+      </c>
+      <c r="E121" s="0" t="inlineStr">
+        <is>
+          <t>已完成并压测</t>
+        </is>
+      </c>
+      <c r="F121" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G121" s="0" t="inlineStr">
+        <is>
+          <t>源码数字/证据类 final guard 不能抢占实现任务的锚点修复、补测试和验证。</t>
+        </is>
+      </c>
+      <c r="H121" s="0" t="inlineStr">
+        <is>
+          <t>T-119 将这类 final guard 限定为 `read-only` contract；真实 session `20260710T022516812575Z` 在两处初始 patch 失败后仍完成两份文件 preview、写入、定向 6 测试和 diff。</t>
+        </is>
+      </c>
+      <c r="I121" s="0"/>
+      <c r="J121" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8199,7 +8287,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G95"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -9615,17 +9703,17 @@
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>开放，T-116</t>
+          <t>已缓解，继续观察</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>T-115 复测 57 次调用中 25 次错误，包含 `patch_content` unified diff、`todo` / `todo_items` 数组和不完整 patch 参数。</t>
+          <t>T-116 真实复测确认这类输入保持明确失败；未发生未经 anchored/hash/preview 验证的写入。</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 工具协议边界：不把不等价结构自动拆成带副作用的多次调用；以 preview contract 和可行动 schema error 引导模型回到 anchored patch / 单条 todo。</t>
+          <t>参考 OMP 工具协议边界：不把不等价结构自动拆成带副作用的多次调用；preview contract 拦真实写入，后续只改善可行动反馈。</t>
         </is>
       </c>
     </row>
@@ -9652,17 +9740,17 @@
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>开放，T-117</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>T-115 复测将 hunk 坐标、`+8/-0` 和测试计数送入源码数字比对，触发 2 次无工具 final 重写。</t>
+          <t>T-115 将 hunk 坐标、`+8/-0` 和测试计数送入源码数字比对；T-117 后续复测未再触发该 guard。</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>保持对枚举/状态码/接口常量的源码校验，排除 git/test 工具事实或让其匹配各自 tool evidence。</t>
+          <t>保持枚举/状态码/接口常量的源码校验，排除 apply_patch/tag/diff/test 工具观测数字。</t>
         </is>
       </c>
     </row>
@@ -9674,32 +9762,32 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-060</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>source-backed final guard 抢占未完成实现任务的修复空间</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>T-119 真实写入会话在初始 patch 失败后继续完成 preview、写入、测试和 diff，run summary 未记录 final steering。</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>源码数字/证据类 final guard 仅用于 `read-only` contract；实现任务继续由 CompletionAudit、Patch Reviewer 和 ToolChoiceQueue 驱动受控修复。</t>
         </is>
       </c>
     </row>
@@ -9711,32 +9799,32 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -9748,7 +9836,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -9758,7 +9846,7 @@
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -9768,12 +9856,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9873,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -9795,22 +9883,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -9822,7 +9910,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -9832,22 +9920,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -9859,7 +9947,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -9869,7 +9957,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -9879,12 +9967,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -9896,7 +9984,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -9906,7 +9994,7 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -9916,12 +10004,12 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -9933,7 +10021,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -9943,22 +10031,22 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -9970,7 +10058,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -9980,22 +10068,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -10007,7 +10095,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -10017,22 +10105,22 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -10044,7 +10132,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -10054,7 +10142,7 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -10064,12 +10152,12 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -10081,17 +10169,17 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -10101,12 +10189,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10206,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -10128,7 +10216,7 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -10138,12 +10226,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -10155,17 +10243,17 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -10175,12 +10263,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10280,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -10202,22 +10290,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10317,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -10239,22 +10327,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -10266,7 +10354,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -10276,22 +10364,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -10303,7 +10391,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -10313,22 +10401,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -10340,32 +10428,32 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
@@ -10377,7 +10465,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -10387,59 +10475,59 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -10451,7 +10539,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -10461,22 +10549,22 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -10488,7 +10576,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -10498,7 +10586,7 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -10508,12 +10596,12 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10613,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -10535,22 +10623,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -10562,7 +10650,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -10572,7 +10660,7 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
@@ -10582,12 +10670,12 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -10599,7 +10687,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -10609,7 +10697,7 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
@@ -10619,12 +10707,12 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10724,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -10646,7 +10734,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
@@ -10656,12 +10744,12 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -10673,7 +10761,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -10683,7 +10771,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
@@ -10693,12 +10781,12 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -10710,7 +10798,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -10720,7 +10808,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -10730,12 +10818,12 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10835,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -10757,22 +10845,22 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -10784,7 +10872,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -10794,7 +10882,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -10804,12 +10892,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10909,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -10831,22 +10919,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -10858,7 +10946,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -10868,22 +10956,22 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -10895,32 +10983,32 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -10932,7 +11020,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -10942,22 +11030,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -10969,7 +11057,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -10979,7 +11067,7 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
@@ -10989,12 +11077,12 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -11006,7 +11094,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -11016,22 +11104,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -11043,7 +11131,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -11053,22 +11141,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -11080,32 +11168,32 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -11117,7 +11205,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -11127,7 +11215,7 @@
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -11137,12 +11225,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -11154,7 +11242,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -11164,22 +11252,22 @@
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -11191,7 +11279,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -11201,7 +11289,7 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
@@ -11211,12 +11299,12 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -11228,7 +11316,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -11238,7 +11326,7 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
@@ -11248,12 +11336,12 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -11265,7 +11353,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -11275,7 +11363,7 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
@@ -11285,12 +11373,12 @@
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -11302,7 +11390,7 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -11312,7 +11400,7 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
@@ -11322,12 +11410,12 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -11339,7 +11427,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -11349,22 +11437,22 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -11376,7 +11464,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -11386,22 +11474,22 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -11413,7 +11501,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -11423,22 +11511,22 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -11450,7 +11538,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -11460,7 +11548,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr">
@@ -11470,12 +11558,12 @@
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -11487,7 +11575,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -11497,7 +11585,7 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr">
@@ -11507,12 +11595,12 @@
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -11524,7 +11612,7 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>ADR-032</t>
+          <t>ADR-031</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -11534,22 +11622,22 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
       <c r="E91" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-093</t>
+          <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -11561,7 +11649,7 @@
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>ADR-033</t>
+          <t>ADR-032</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -11571,7 +11659,7 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
       <c r="E92" s="0" t="inlineStr">
@@ -11581,12 +11669,12 @@
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-106</t>
+          <t>已完成 T-093</t>
         </is>
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
       </c>
     </row>
@@ -11598,7 +11686,7 @@
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>ADR-034</t>
+          <t>ADR-033</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -11608,7 +11696,7 @@
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
         </is>
       </c>
       <c r="E93" s="0" t="inlineStr">
@@ -11618,12 +11706,12 @@
       </c>
       <c r="F93" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-107</t>
+          <t>已完成 T-106</t>
         </is>
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
         </is>
       </c>
     </row>
@@ -11635,30 +11723,67 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
+          <t>ADR-034</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D94" s="0" t="inlineStr">
+        <is>
+          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+        </is>
+      </c>
+      <c r="E94" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F94" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-107</t>
+        </is>
+      </c>
+      <c r="G94" s="0" t="inlineStr">
+        <is>
+          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
           <t>ADR-035</t>
         </is>
       </c>
-      <c r="C94" s="0" t="inlineStr">
+      <c r="C95" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D94" s="0" t="inlineStr">
+      <c r="D95" s="0" t="inlineStr">
         <is>
           <t>P10 采用裁剪版 Intelligence Runtime，不一次性复制 OMP 大系统</t>
         </is>
       </c>
-      <c r="E94" s="0" t="inlineStr">
+      <c r="E95" s="0" t="inlineStr">
         <is>
           <t>已接受并落地部分</t>
         </is>
       </c>
-      <c r="F94" s="0" t="inlineStr">
+      <c r="F95" s="0" t="inlineStr">
         <is>
           <t>已完成 T-109/T-110/T-111/T-112/T-113/T-114/T-115</t>
         </is>
       </c>
-      <c r="G94" s="0" t="inlineStr">
+      <c r="G95" s="0" t="inlineStr">
         <is>
           <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate 和受限 ToolRegistry 归一；不引入第二个 Agent。</t>
         </is>
@@ -11676,7 +11801,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -11726,12 +11851,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-115 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一。真实小改交付链路已跑通，但工具调用效率仍不合格。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-119 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract 与 final-guard scope。真实小改交付链路已跑通，但工具调用效率仍不合格。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>先做 T-116 preview contract 与 T-117 numeric guard scope，再按 OMP 边界拆 evidence/run collector/startup/memory，而不是继续堆 `agent.py`。</t>
+          <t>保持 OMP 的“协议边界 + active loop observer + 小上限”原则，下一步基于 PT-042 降低 anchored patch 试错；结构拆分仍按独立边界推进，不再往 `agent.py` 堆新 guard。</t>
         </is>
       </c>
     </row>
@@ -11831,17 +11956,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Preview contract 与 numeric guard scope</t>
+          <t>Anchored patch 参数效率 / 真实需求回归</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-115 真实复测已完成源码、测试、定向 run_tests、git_diff 和最终结构，但 57 次工具调用中仍有 25 次错误。</t>
+          <t>T-119 已证明初始 patch 失败后仍能继续完成受控修复；剩余主要问题是 provider 首次命中 anchored patch schema 的效率。</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>T-116 不执行 raw diff/bulk todo，只引导/限制首个 real patch 前先有有效 dry-run；T-117 让 diff/test 数字不再被当作源码枚举事实。</t>
+          <t>维持 hard preview/hash 边界，不自动执行 raw diff；用真实需求观察并仅归一安全等价的新参数方言。</t>
         </is>
       </c>
     </row>
@@ -12982,7 +13107,7 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>T-115 真实小改成功交付 2 文件、定向 6 测试和 diff，但共 57 tool calls / 25 errors；安全的 scalar 参数方言已可归一，raw diff/bulk todo 仍被拒绝。</t>
+          <t>T-115 真实小改成功交付 2 文件、定向 6 测试和 diff，但共 57 tool calls / 25 errors；T-119 虽完成同类两文件任务，仍有 14 次调用 / 6 次错误。安全的 scalar 参数方言已可归一，raw diff/bulk todo 仍被拒绝。</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -12992,7 +13117,7 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>T-115 已完成 scalar normalization；T-116/T-117 待处理 preview contract 和 numeric guard 误拦。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-115/T-116/T-117/T-119 已完成 scalar normalization、preview contract、numeric guard scope 和实现任务 final-guard scope；后续只按安全等价样本降低 anchored patch 试错。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
     </row>
@@ -13068,7 +13193,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 261 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 267 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pin requirement evidence through compaction
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>当前 267 个测试通过</t>
+          <t>当前 273 个测试通过</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J123"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8278,6 +8278,94 @@
       <c r="I121" s="0"/>
       <c r="J121" s="0"/>
     </row>
+    <row r="122">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
+          <t>T-120</t>
+        </is>
+      </c>
+      <c r="B122" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t>Pinned requirement evidence / compaction authority</t>
+        </is>
+      </c>
+      <c r="E122" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 并复测</t>
+        </is>
+      </c>
+      <c r="F122" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G122" s="0" t="inlineStr">
+        <is>
+          <t>真实服务费结算设计 session `20260710T024503106586Z` 经 12 次 LLM summary 后将后期规划误写为当前双审/支付流程。</t>
+        </is>
+      </c>
+      <c r="H122" s="0" t="inlineStr">
+        <is>
+          <t>成功 `read_file` 的 requirement/spec Markdown 以高优先级 pinned context 注入每次 provider request；最终需求事实要求真实 requirement path:line。session `20260710T025606504484Z` 已不再编造双审/支付当前范围。</t>
+        </is>
+      </c>
+      <c r="I122" s="0"/>
+      <c r="J122" s="0"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="inlineStr">
+        <is>
+          <t>T-121</t>
+        </is>
+      </c>
+      <c r="B123" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C123" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D123" s="0" t="inlineStr">
+        <is>
+          <t>真实设计 evidence matrix / cross-root ToolChoiceQueue</t>
+        </is>
+      </c>
+      <c r="E123" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F123" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G123" s="0" t="inlineStr">
+        <is>
+          <t>T-120 复测仍在后端候选目录进行 57 次调用，未读取用户声明前端，造成复用结论过弱。</t>
+        </is>
+      </c>
+      <c r="H123" s="0" t="inlineStr">
+        <is>
+          <t>对齐 OMP ToolChoiceQueue：需求已读后，对用户声明的前后端 roots 建立最小 `read_file` evidence requirement；未覆盖 root 先 soft/hard escalate，覆盖后限制低价值路径探索并收束。</t>
+        </is>
+      </c>
+      <c r="I123" s="0"/>
+      <c r="J123" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -8287,7 +8375,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G97"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -9799,7 +9887,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-061</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -9809,22 +9897,22 @@
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>requirement source 被 LLM compaction 改写，真实设计范围漂移</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>已缓解，继续观察</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>session `20260710T024503106586Z` 将后期规划编造成当前双审/支付；T-120 复测已修正当前期事实。</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>按 OMP current context 优先级：需求正文独立 pinned，普通 compaction summary 只能辅助导航；最终需求事实要求 path:line。</t>
         </is>
       </c>
     </row>
@@ -9836,32 +9924,32 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-062</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>跨前后端设计未覆盖最小源码证据集就持续探索</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>开放，T-121</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>session `20260710T025606504484Z` 57 次调用却未读取前端候选源码，最终复用结论不足。</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>按 OMP ToolChoiceQueue / soft escalation，为 user-declared roots 建立 evidence matrix 和小上限。</t>
         </is>
       </c>
     </row>
@@ -9873,32 +9961,32 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -9910,7 +9998,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -9920,22 +10008,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -9947,7 +10035,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -9957,7 +10045,7 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -9967,12 +10055,12 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -9984,7 +10072,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -9994,22 +10082,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -10021,7 +10109,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -10031,7 +10119,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -10041,12 +10129,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10146,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -10068,22 +10156,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -10095,7 +10183,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -10105,7 +10193,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -10115,12 +10203,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -10132,7 +10220,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -10142,22 +10230,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -10169,7 +10257,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -10179,22 +10267,22 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -10206,17 +10294,17 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -10226,12 +10314,12 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -10243,17 +10331,17 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -10263,12 +10351,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -10280,17 +10368,17 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -10300,12 +10388,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -10317,32 +10405,32 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10442,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -10364,22 +10452,22 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -10391,7 +10479,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -10401,22 +10489,22 @@
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -10428,7 +10516,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -10438,22 +10526,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
@@ -10465,32 +10553,32 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
@@ -10502,106 +10590,106 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
@@ -10613,7 +10701,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -10623,22 +10711,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -10650,7 +10738,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -10660,22 +10748,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -10687,7 +10775,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -10697,22 +10785,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -10724,7 +10812,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -10734,7 +10822,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
@@ -10744,12 +10832,12 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -10761,7 +10849,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -10771,7 +10859,7 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
@@ -10781,12 +10869,12 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -10798,7 +10886,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -10808,7 +10896,7 @@
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -10818,12 +10906,12 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10923,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -10845,7 +10933,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
@@ -10855,12 +10943,12 @@
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -10872,7 +10960,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -10882,22 +10970,22 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -10909,7 +10997,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -10919,22 +11007,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -10946,7 +11034,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -10956,22 +11044,22 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -10983,7 +11071,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -10993,22 +11081,22 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -11020,32 +11108,32 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -11057,32 +11145,32 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11182,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -11104,22 +11192,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -11131,7 +11219,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -11141,22 +11229,22 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -11168,7 +11256,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -11178,7 +11266,7 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
@@ -11188,12 +11276,12 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -11205,17 +11293,17 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
@@ -11225,12 +11313,12 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
         </is>
       </c>
     </row>
@@ -11242,32 +11330,32 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-018</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
         </is>
       </c>
     </row>
@@ -11279,7 +11367,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-019</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -11289,22 +11377,22 @@
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
         </is>
       </c>
     </row>
@@ -11316,7 +11404,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -11326,22 +11414,22 @@
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
         </is>
       </c>
     </row>
@@ -11353,7 +11441,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-021</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -11363,7 +11451,7 @@
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
@@ -11373,12 +11461,12 @@
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
         </is>
       </c>
     </row>
@@ -11390,7 +11478,7 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-022</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -11400,7 +11488,7 @@
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
@@ -11410,12 +11498,12 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-077</t>
+          <t>已完成 T-075</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
+          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11515,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-026</t>
+          <t>ADR-024</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -11437,7 +11525,7 @@
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
+          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
@@ -11447,12 +11535,12 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-078</t>
+          <t>已完成 T-076</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
+          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
         </is>
       </c>
     </row>
@@ -11464,7 +11552,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-027</t>
+          <t>ADR-025</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -11474,22 +11562,22 @@
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
+          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-081</t>
+          <t>已完成 T-077</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
+          <t>`./agent` / `--chat` / `chat` 共用事件 sink，approval 仍走同步 stdin 但发 approval events；可选 `prompt_toolkit` / `rich` 增强体验，缺依赖时降级，符合封闭 VM 可预置依赖原则。</t>
         </is>
       </c>
     </row>
@@ -11501,7 +11589,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>ADR-028</t>
+          <t>ADR-026</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -11511,7 +11599,7 @@
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
+          <t>企业服务边界用 memory/skill 承载，不新增专用工具</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr">
@@ -11521,12 +11609,12 @@
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-082</t>
+          <t>已完成 T-078</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
+          <t>组织边界是用户个人长期上下文，不是通用 Agent tool；参考 OMP authored skills / project memory，把边界和工作流沉淀为本机上下文，代码只补通用 runtime 能力，包括 analysis-only、named skill soft requirement、custom memory read 和 final-structure gate。</t>
         </is>
       </c>
     </row>
@@ -11538,7 +11626,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>ADR-029</t>
+          <t>ADR-027</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -11548,7 +11636,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
+          <t>Claude review 先转为行动计划，不立即做 P0 大拆分</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr">
@@ -11558,12 +11646,12 @@
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
+          <t>已完成 T-081</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
+          <t>OMP 架构原则继续作为方向；但 LCA 当前以真实日用闭环为先。先补 TUI 可发现性和 run summary/coverage，再用压测数据驱动模块拆分、token budget 和 LSP provider 增强。</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11663,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>ADR-030</t>
+          <t>ADR-028</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -11585,22 +11673,22 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
+          <t>Run summary 先做 runtime 内轻量 collector，暂不拆大模块</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>先做 T-085~T-087</t>
+          <t>已完成 T-082</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
+          <t>参考 OMP run-collector 的可观测性原则，但当前先把计数和终止原因汇总到 `RunSummary` / `run_summary`，服务压测和 `/status`；等数据稳定后再抽 `run_collector.py` 或 Steerer 协议。</t>
         </is>
       </c>
     </row>
@@ -11612,7 +11700,7 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>ADR-031</t>
+          <t>ADR-029</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -11622,7 +11710,7 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
+          <t>默认编码模型切到 `qwen3-coder-next` 做日用压测</t>
         </is>
       </c>
       <c r="E91" s="0" t="inlineStr">
@@ -11632,12 +11720,12 @@
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>已从 `compaction.py` 开始</t>
+          <t>本地 `.env` 已切换，连通性返回 OK；`.env` 不提交 token</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
+          <t>阿里云百炼 Qwen-Coder 文档把 `qwen3-coder-next` 用作代码任务/tool interaction 示例模型；本地真实压测 T-084 已能正常收束。</t>
         </is>
       </c>
     </row>
@@ -11649,7 +11737,7 @@
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>ADR-032</t>
+          <t>ADR-030</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -11659,22 +11747,22 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
+          <t>P9 压测问题优先补 runtime steering，不先做大重构</t>
         </is>
       </c>
       <c r="E92" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-093</t>
+          <t>先做 T-085~T-087</t>
         </is>
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
+          <t>T-084 暴露的是重复读、todo 参数纠偏、最终结构/证据卫生；这些适合在工具错误、evidence-aware guard、final gate 层小步修复，不需要立刻大拆 `agent.py` 或上完整 ToolChoiceQueue。</t>
         </is>
       </c>
     </row>
@@ -11686,7 +11774,7 @@
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>ADR-033</t>
+          <t>ADR-031</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -11696,22 +11784,22 @@
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+          <t>OMP 架构差距用渐进模块化关闭，不做一次性大搬家</t>
         </is>
       </c>
       <c r="E93" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F93" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-106</t>
+          <t>已从 `compaction.py` 开始</t>
         </is>
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+          <t>Claude review 对 `agent.py` 过大的判断成立；但一次性 Steerer/ToolChoiceQueue 大改回归面太大。先把纯函数和边界清楚的子系统抽出，保持行为不变、测试先行。</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11811,7 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>ADR-034</t>
+          <t>ADR-032</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -11733,7 +11821,7 @@
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+          <t>LSP 按 OMP client 思路做可选外部 adapter，保留 light fallback</t>
         </is>
       </c>
       <c r="E94" s="0" t="inlineStr">
@@ -11743,12 +11831,12 @@
       </c>
       <c r="F94" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-107</t>
+          <t>已完成 T-093</t>
         </is>
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+          <t>Java/TypeScript/Vue 的完整代码导航应优先交给成熟 language server；但 LCA 仍不在运行时自动下载依赖，也不把外部 server 作为默认强依赖。封闭 VM 可预置 jdtls/npm 包，或用 `AGENT_LSP_*_COMMAND` 指向离线安装路径。</t>
         </is>
       </c>
     </row>
@@ -11760,30 +11848,104 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
+          <t>ADR-033</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D95" s="0" t="inlineStr">
+        <is>
+          <t>Final-answer steering 先抽统一 Steerer 协议的一块，不再把最终回答 guard 塞进 `agent.py`</t>
+        </is>
+      </c>
+      <c r="E95" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F95" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-106</t>
+        </is>
+      </c>
+      <c r="G95" s="0" t="inlineStr">
+        <is>
+          <t>对标 OMP“主循环调度，guard/observer/reviewer 分离”的原则；本轮先抽 final-answer steering，降低回归面并直接修 T-105 枚举误报，后续再拆 semantic/evidence/run collector。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t>ADR-034</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>Token budget 采用本地估算 + reserve，字符预算保留兜底</t>
+        </is>
+      </c>
+      <c r="E96" s="0" t="inlineStr">
+        <is>
+          <t>已接受并落地</t>
+        </is>
+      </c>
+      <c r="F96" s="0" t="inlineStr">
+        <is>
+          <t>已完成 T-107</t>
+        </is>
+      </c>
+      <c r="G96" s="0" t="inlineStr">
+        <is>
+          <t>OMP 按 token/context window 管理 compaction 并预留下一轮预算；LCA 当前不引入重 tokenizer 依赖，先用 CJK/ASCII 轻量估算触发压缩，`context_char_budget` 继续作为 fallback。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
           <t>ADR-035</t>
         </is>
       </c>
-      <c r="C95" s="0" t="inlineStr">
+      <c r="C97" s="0" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D95" s="0" t="inlineStr">
+      <c r="D97" s="0" t="inlineStr">
         <is>
           <t>P10 采用裁剪版 Intelligence Runtime，不一次性复制 OMP 大系统</t>
         </is>
       </c>
-      <c r="E95" s="0" t="inlineStr">
+      <c r="E97" s="0" t="inlineStr">
         <is>
           <t>已接受并落地部分</t>
         </is>
       </c>
-      <c r="F95" s="0" t="inlineStr">
+      <c r="F97" s="0" t="inlineStr">
         <is>
           <t>已完成 T-109/T-110/T-111/T-112/T-113/T-114/T-115</t>
         </is>
       </c>
-      <c r="G95" s="0" t="inlineStr">
+      <c r="G97" s="0" t="inlineStr">
         <is>
           <t>T-108 证明需要比 prompt 更硬的目标契约、完成审计和工具调度；但 LCA 仍是单用户、单 Agent、本地 MVP。当前已落地 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate 和受限 ToolRegistry 归一；不引入第二个 Agent。</t>
         </is>
@@ -11801,7 +11963,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -11851,12 +12013,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-119 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract 与 final-guard scope。真实小改交付链路已跑通，但工具调用效率仍不合格。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-120 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope与 pinned requirement evidence。真实小改交付链路已跑通，但跨项目设计的工具调用效率和 evidence coverage 仍不合格。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>保持 OMP 的“协议边界 + active loop observer + 小上限”原则，下一步基于 PT-042 降低 anchored patch 试错；结构拆分仍按独立边界推进，不再往 `agent.py` 堆新 guard。</t>
+          <t>按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则，先做 T-121 evidence matrix；结构拆分仍按独立边界推进，不再往 `agent.py` 堆新 guard。</t>
         </is>
       </c>
     </row>
@@ -11956,17 +12118,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Anchored patch 参数效率 / 真实需求回归</t>
+          <t>真实设计 evidence matrix / ToolChoiceQueue</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-119 已证明初始 patch 失败后仍能继续完成受控修复；剩余主要问题是 provider 首次命中 anchored patch schema 的效率。</t>
+          <t>T-120 已修正需求正文被摘要改写，但复测暴露前后端证据覆盖不足和探索扩散。</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>维持 hard preview/hash 边界，不自动执行 raw diff；用真实需求观察并仅归一安全等价的新参数方言。</t>
+          <t>先实现 T-121，再重跑服务费结算只读设计；anchored patch 参数效率继续作为后续独立风险观察。</t>
         </is>
       </c>
     </row>
@@ -13193,7 +13355,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 267 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 273 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Require cross-root design evidence
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-116 已用 hard pre-tool gate 阻止未预览的真实 patch；T-117 已消除 diff/test 数字触发源码数字 guard；T-118 已修复“待写入 read-only 字面量”误分成只读任务。当前开放问题是模型在 preview error 后的纠错，以及 source-evidence false-negative 与 CompletionAudit 的优先级。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-121 已让跨前后端只读设计任务先覆盖需求、主后端和用户指定前端源码，再撤回工具并收束回答。当前继续观察 anchored patch 参数纠错与跨项目设计的工具调用成本。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,11 +216,11 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>完整 unittest 通过；xlsx 同步后继续检查。</t>
+          <t>完整 unittest、compileall、xlsx 同步和 diff check 已通过。</t>
         </is>
       </c>
       <c r="D7" s="0"/>
@@ -2926,12 +2926,12 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>当前 273 个测试通过</t>
+          <t>当前 280 个测试通过</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>unittest 通过；同步 Excel 后检查 xlsx</t>
+          <t>unittest、compileall、xlsx 和 diff check 通过</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -8345,7 +8345,7 @@
       </c>
       <c r="E123" s="0" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成并真实复测</t>
         </is>
       </c>
       <c r="F123" s="0" t="inlineStr">
@@ -8360,7 +8360,7 @@
       </c>
       <c r="H123" s="0" t="inlineStr">
         <is>
-          <t>对齐 OMP ToolChoiceQueue：需求已读后，对用户声明的前后端 roots 建立最小 `read_file` evidence requirement；未覆盖 root 先 soft/hard escalate，覆盖后限制低价值路径探索并收束。</t>
+          <t>跨 root 只读设计任务要求主 workspace 和每个用户指定代码目录各成功读取至少一份源码；覆盖后只保留有限补读，或接近 deadline 时预留最终回答时间。session `20260710T032336652934Z` 读取需求、`zqylpayment` Java 与 `msp-pay` JS/Vue 后以 final 收束（127 秒、19 次只读工具、0 错误）。</t>
         </is>
       </c>
       <c r="I123" s="0"/>
@@ -9939,7 +9939,7 @@
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>开放，T-121</t>
+          <t>已关闭 MVP，继续观察</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
@@ -9949,7 +9949,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>按 OMP ToolChoiceQueue / soft escalation，为 user-declared roots 建立 evidence matrix 和小上限。</t>
+          <t>T-121 按 OMP ToolChoiceQueue / soft escalation，为 user-declared roots 建立 evidence matrix；session `20260710T032336652934Z` 已读需求、后端 Java 与前端 JS/Vue 后收束。后续继续观察探索成本。</t>
         </is>
       </c>
     </row>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 273 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 280 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh project roadmap after T-121
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope 和 quoted literal 分类修复；下一步 source-evidence false-negative 收束。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal 分类、pinned requirement evidence 与 cross-root evidence matrix；下一步以真实需求设计/小改验证这些护栏的协同效果。</t>
         </is>
       </c>
     </row>
@@ -11963,7 +11963,7 @@
   <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -12013,12 +12013,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-120 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope与 pinned requirement evidence。真实小改交付链路已跑通，但跨项目设计的工具调用效率和 evidence coverage 仍不合格。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-121 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope、pinned requirement evidence 与 cross-root evidence matrix。真实小改交付链路已跑通，跨项目设计的最小 evidence coverage 也已验证。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则，先做 T-121 evidence matrix；结构拆分仍按独立边界推进，不再往 `agent.py` 堆新 guard。</t>
+          <t>继续按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则，用真实需求设计和小改压测检验协同效果；结构拆分仍按独立边界推进。</t>
         </is>
       </c>
     </row>
@@ -12118,17 +12118,17 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>真实设计 evidence matrix / ToolChoiceQueue</t>
+          <t>真实需求设计与小改压测</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>T-120 已修正需求正文被摘要改写，但复测暴露前后端证据覆盖不足和探索扩散。</t>
+          <t>T-121 已在服务费结算任务中验证需求、后端与前端最小 evidence coverage，并以 final 收束。</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>先实现 T-121，再重跑服务费结算只读设计；anchored patch 参数效率继续作为后续独立风险观察。</t>
+          <t>选择一个范围和验收边界明确的真实切片：先产出 evidence-backed 设计，再实施小改、运行测试和 diff reviewer；anchored patch 参数效率继续作为独立风险观察。</t>
         </is>
       </c>
     </row>
@@ -13406,7 +13406,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP、项目边界分析 MVP、source-grounded numeric guard 和 token budget MVP；下一步复测服务费结算证据链，确认现有能力复用点和必须新建能力后再进入实现设计。</t>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP、项目边界分析 MVP、source-grounded numeric guard、token budget、pinned requirement evidence 和 cross-root evidence matrix；下一步进入一项边界明确的真实需求设计和小改验证。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Extract tool loop steering registry
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -104,7 +104,7 @@
   <dimension ref="A1:D34"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P10：Intelligence Runtime 骨架</t>
+          <t>P10：Intelligence Runtime 骨架 + P0a 架构还债</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-121 已让跨前后端只读设计任务先覆盖需求、主后端和用户指定前端源码，再撤回工具并收束回答。当前继续观察 anchored patch 参数纠错与跨项目设计的工具调用成本。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-123 已把五类病态工具循环的软纠偏、硬停止与跨 root 设计证据收束迁入独立 steering 模块，`agent.py` 从 3875 行降至 3607 行；下一步是 P0b `RunContext`，再回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal 分类、pinned requirement evidence 与 cross-root evidence matrix；下一步以真实需求设计/小改验证这些护栏的协同效果。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry。下一步完成 P0b `RunContext` / `RunStats` 状态收拢，再以真实小改验证协同效果。</t>
         </is>
       </c>
     </row>
@@ -2476,12 +2476,12 @@
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `_steer_after_duplicate_tool_call()`</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `steering/tool_loop.py`</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error；重复命中后注入 runtime steering，下一轮不给工具 schema，强制模型从已有证据输出最终回答；连续命中仍有硬停兜底</t>
+          <t>最近窗口内同名同参工具调用超过阈值会返回 tool error；ToolLoop registry 按优先级注入 runtime steering，下一轮不给工具 schema，强制模型从已有证据输出最终回答；连续命中仍有硬停兜底</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `_steer_after_semantic_exploration()`</t>
+          <t>`AgentRuntime._execute_tool_with_repeat_guard()` / `steering/tool_loop.py`</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J124"/>
+  <dimension ref="A1:J125"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8409,6 +8409,50 @@
       </c>
       <c r="I124" s="0"/>
       <c r="J124" s="0"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t>T-123</t>
+        </is>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C125" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t>P0a ToolLoop steering registry</t>
+        </is>
+      </c>
+      <c r="E125" s="0" t="inlineStr">
+        <is>
+          <t>已完成并回归</t>
+        </is>
+      </c>
+      <c r="F125" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G125" s="0" t="inlineStr">
+        <is>
+          <t>review 指出 `agent.py` 同时存在 inline `steer_after` / hard-stop / final steerer 三条轨，新增 guard 持续膨胀主文件。</t>
+        </is>
+      </c>
+      <c r="H125" s="0" t="inlineStr">
+        <is>
+          <t>新增 `steering/tool_loop.py` 与 `steering/termination.py`：五类病态工具循环（重复调用、空 search/LSP、重复 read、语义路径探索）以显式优先级统一 soft steering 与 hard stop；跨 root 设计证据覆盖/收束迁入 `design_evidence.py`。`agent.py` 由 3875 降至 3607 行；291 个 unittest 回归通过。</t>
+        </is>
+      </c>
+      <c r="I125" s="0"/>
+      <c r="J125" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9687,7 +9731,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解，继续拆</t>
+          <t>已完成 P0a，P0b 进行中</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -9697,7 +9741,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>已完成 FinalAnswer Steerer 第一块抽象：最终回答相关 steering 移到 `src/local_agent/steering/final_answer.py`；后续继续按低风险边界拆 evidence ledger、run collector、startup context、memory consolidation 和 semantic exploration steerer。</t>
+          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination 与 design-evidence coverage，主文件从 3875 降至 3607 行。下一步将 run 级可变状态收拢至 `RunContext`，并迁出 `RunStats`；在此之前不在 `agent.py` 新增 feature guard。</t>
         </is>
       </c>
     </row>
@@ -12057,12 +12101,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-121 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope、pinned requirement evidence 与 cross-root evidence matrix。真实小改交付链路已跑通，跨项目设计的最小 evidence coverage 也已验证。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-122 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成第一批 ToolLoop steering 模块化。真实小改交付链路已跑通，跨项目设计的最小 evidence coverage 也已验证。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>继续按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则，用真实需求设计和小改压测检验协同效果；结构拆分仍按独立边界推进。</t>
+          <t>继续按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则完成 P0b `RunContext` / `RunStats` 收拢，再用真实需求设计和小改压测检验协同效果。</t>
         </is>
       </c>
     </row>
@@ -13399,7 +13443,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 287 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 291 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Extract run collector and isolate run evidence
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P10：Intelligence Runtime 骨架 + P0a 架构还债</t>
+          <t>P10：Intelligence Runtime 骨架 + P0b 架构还债</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-123 已把五类病态工具循环的软纠偏、硬停止与跨 root 设计证据收束迁入独立 steering 模块，`agent.py` 从 3875 行降至 3607 行；下一步是 P0b `RunContext`，再回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-123 已完成 ToolLoop steering 拆分；T-124 已迁出 RunCollector，并修复连续任务之间的证据/范围状态泄漏，`agent.py` 现为 3538 行。下一步是完整 `RunContext`，再回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry。下一步完成 P0b `RunContext` / `RunStats` 状态收拢，再以真实小改验证协同效果。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry，T-124 已迁出 RunCollector 并隔离跨 run 证据。下一步完成 P0b `RunContext` 状态收拢，再以真实小改验证协同效果。</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J126"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8453,6 +8453,50 @@
       </c>
       <c r="I125" s="0"/>
       <c r="J125" s="0"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t>T-124</t>
+        </is>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C126" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t>P0b RunCollector 与跨 run evidence reset</t>
+        </is>
+      </c>
+      <c r="E126" s="0" t="inlineStr">
+        <is>
+          <t>已完成并回归</t>
+        </is>
+      </c>
+      <c r="F126" s="0" t="inlineStr">
+        <is>
+          <t>Agent + 小红</t>
+        </is>
+      </c>
+      <c r="G126" s="0" t="inlineStr">
+        <is>
+          <t>review 发现连续终端任务会保留上一轮 `read_file` 证据、relevance、evidence ledger 与“本轮范围读取次数”，可能让下一任务误判证据已满足。</t>
+        </is>
+      </c>
+      <c r="H126" s="0" t="inlineStr">
+        <is>
+          <t>新增 `run_collector.py` 承接 RunStats、compaction/tool 计数和 summary 计算；每轮开始清空本轮 evidence、preview、relevance 和 read range 状态，保留明确属于 session 的审批与重复调用历史。新增跨 run 泄漏和 collector 单测；`agent.py` 降至 3538 行，294 个 unittest 通过。</t>
+        </is>
+      </c>
+      <c r="I126" s="0"/>
+      <c r="J126" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9731,7 +9775,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已完成 P0a，P0b 进行中</t>
+          <t>P0b 进行中</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -9741,7 +9785,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination 与 design-evidence coverage，主文件从 3875 降至 3607 行。下一步将 run 级可变状态收拢至 `RunContext`，并迁出 `RunStats`；在此之前不在 `agent.py` 新增 feature guard。</t>
+          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination 与 design-evidence coverage；T-124 已抽 RunCollector 并修复跨 run evidence leak，主文件降至 3538 行。下一步收拢剩余 run state 到 `RunContext`；在此之前不在 `agent.py` 新增 feature guard。</t>
         </is>
       </c>
     </row>
@@ -13443,7 +13487,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 291 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 294 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consolidate run state in RunContext
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -168,7 +168,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-123 已完成 ToolLoop steering 拆分；T-124 已迁出 RunCollector，并修复连续任务之间的证据/范围状态泄漏，`agent.py` 现为 3538 行。下一步是完整 `RunContext`，再回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-123 已完成 ToolLoop steering 拆分；T-124/T-125 已迁出 RunCollector，并将任务合同、队列、证据、preview、steering 和本轮 metadata 收拢为 `RunContext`，`agent.py` 现为 3445 行。下一步回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry，T-124 已迁出 RunCollector 并隔离跨 run 证据。下一步完成 P0b `RunContext` 状态收拢，再以真实小改验证协同效果。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry，T-124/T-125 已完成 P0b RunCollector / RunContext 收拢。下一步以真实小改验证协同效果。</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J127"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8497,6 +8497,50 @@
       </c>
       <c r="I126" s="0"/>
       <c r="J126" s="0"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t>T-125</t>
+        </is>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C127" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t>P0b RunContext 状态收拢</t>
+        </is>
+      </c>
+      <c r="E127" s="0" t="inlineStr">
+        <is>
+          <t>已完成并回归</t>
+        </is>
+      </c>
+      <c r="F127" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G127" s="0" t="inlineStr">
+        <is>
+          <t>`AgentRuntime` 仍持有任务合同、工具队列、证据、preview、final steering 和 run metadata，P0b 尚未完成单一任务状态边界。</t>
+        </is>
+      </c>
+      <c r="H127" s="0" t="inlineStr">
+        <is>
+          <t>新增 `run_context.py`，统一当前 run 的 deadline/baseline、contract、queue、设计证据、Evidence Ledger、preview、final steering、ToolLoop registry 和 Collector；session 消息、审批与 recent guard 保留 Runtime。新增 RunContext reset 回归；`agent.py` 降至 3445 行，295 个 unittest 通过。</t>
+        </is>
+      </c>
+      <c r="I127" s="0"/>
+      <c r="J127" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9775,7 +9819,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>P0b 进行中</t>
+          <t>已完成 P0b 基线，继续观察</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -9785,7 +9829,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination 与 design-evidence coverage；T-124 已抽 RunCollector 并修复跨 run evidence leak，主文件降至 3538 行。下一步收拢剩余 run state 到 `RunContext`；在此之前不在 `agent.py` 新增 feature guard。</t>
+          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination；T-124/T-125 已抽 RunCollector / RunContext，主文件降至 3445 行。后续新 guard 继续只进独立 steering 模块；真实压测后再决定是否拆 SessionGuardState。</t>
         </is>
       </c>
     </row>
@@ -13487,7 +13531,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 294 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 295 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record P0b patch pressure test
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J127"/>
+  <dimension ref="A1:J128"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8541,6 +8541,50 @@
       </c>
       <c r="I127" s="0"/>
       <c r="J127" s="0"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t>T-126</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C128" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
+        <is>
+          <t>P0b 后真实小改压测</t>
+        </is>
+      </c>
+      <c r="E128" s="0" t="inlineStr">
+        <is>
+          <t>首轮未通过，待复跑</t>
+        </is>
+      </c>
+      <c r="F128" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G128" s="0" t="inlineStr">
+        <is>
+          <t>隔离 worktree session `20260710T154146640779Z` 在多轮读 `test_patch.py` / `anchored.py` 后未进入 preview、写入、测试、diff 或 final；worktree 无 diff。</t>
+        </is>
+      </c>
+      <c r="H128" s="0" t="inlineStr">
+        <is>
+          <t>先用重定向输出的独立 worktree 复跑，排除外部终端截断；若复现，优先增强已有 Planner/ToolChoiceQueue/ToolLoop registry 的阶段转换，不在 `agent.py` 新增控制分支。</t>
+        </is>
+      </c>
+      <c r="I128" s="0"/>
+      <c r="J128" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Update P0b patch pressure results
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -8565,7 +8565,7 @@
       </c>
       <c r="E128" s="0" t="inlineStr">
         <is>
-          <t>首轮未通过，待复跑</t>
+          <t>部分通过，继续观察自主选点</t>
         </is>
       </c>
       <c r="F128" s="0" t="inlineStr">
@@ -8575,12 +8575,12 @@
       </c>
       <c r="G128" s="0" t="inlineStr">
         <is>
-          <t>隔离 worktree session `20260710T154146640779Z` 在多轮读 `test_patch.py` / `anchored.py` 后未进入 preview、写入、测试、diff 或 final；worktree 无 diff。</t>
+          <t>自主选点 session `20260710T154146640779Z` 多轮读 `test_patch.py` / `anchored.py` 后未进入交付；精确目标复跑 `20260710T154432520729Z` 则完成 todo、read、dry_run、真实 patch、定向 3 测试和 diff，仅改一份测试文件。</t>
         </is>
       </c>
       <c r="H128" s="0" t="inlineStr">
         <is>
-          <t>先用重定向输出的独立 worktree 复跑，排除外部终端截断；若复现，优先增强已有 Planner/ToolChoiceQueue/ToolLoop registry 的阶段转换，不在 `agent.py` 新增控制分支。</t>
+          <t>P0b 未破坏受控小改闭环；下一次真实失败若仍是探索过宽，优先收紧已有 Planner/ToolChoiceQueue/ToolLoop registry 的阶段转换，不在 `agent.py` 新增控制分支。</t>
         </is>
       </c>
       <c r="I128" s="0"/>

</xml_diff>

<commit_message>
Thin runtime orchestration and constrain small edits
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -163,12 +163,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P10：Intelligence Runtime 骨架 + P0b 架构还债</t>
+          <t>P10：Intelligence Runtime 骨架 + P0c 架构还债</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-123 已完成 ToolLoop steering 拆分；T-124/T-125 已迁出 RunCollector，并将任务合同、队列、证据、preview、steering 和本轮 metadata 收拢为 `RunContext`，`agent.py` 现为 3445 行。下一步回到真实小改压测。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-123~T-127 已抽 ToolLoop、RunCollector/RunContext、StartupContext、EvidenceLedger、SoftToolRequirement 与 SessionGuardState；`agent.py` 现为 2494 行。下一步在隔离 worktree 复跑自主小改的 `candidate_committed → preview → write → test → diff` 链路。详见 `docs/pressure-test-2026-07-10.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、numeric guard scope、quoted literal分类、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成 P0a ToolLoop steering registry，T-124/T-125 已完成 P0b RunCollector / RunContext 收拢。下一步以真实小改验证协同效果。</t>
+          <t>已完成 RequirementContract、CompletionAudit、MiniToolChoiceQueue、Planner/Explore、post-diff Patch Reviewer、no-edit evidence gate、ToolRegistry 参数归一、preview contract、pinned requirement evidence 与 cross-root evidence matrix；T-123~T-127 已完成 ToolLoop、RunCollector/RunContext、StartupContext、EvidenceLedger 与 SessionGuardState 模块化，并为自主小改加入 `candidate_committed` 收束。下一步以隔离 worktree 真实复跑验证协同效果。</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J129"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -8585,6 +8585,50 @@
       </c>
       <c r="I128" s="0"/>
       <c r="J128" s="0"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="inlineStr">
+        <is>
+          <t>T-127</t>
+        </is>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C129" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D129" s="0" t="inlineStr">
+        <is>
+          <t>P0c 状态边界迁移与自主小改候选收束</t>
+        </is>
+      </c>
+      <c r="E129" s="0" t="inlineStr">
+        <is>
+          <t>已完成单元回归，待真实复跑</t>
+        </is>
+      </c>
+      <c r="F129" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G129" s="0" t="inlineStr">
+        <is>
+          <t>T-126 暴露自主选点会在已读 source/test 后继续宽泛探索；review 也要求迁出 Evidence、Startup、session guard state。</t>
+        </is>
+      </c>
+      <c r="H129" s="0" t="inlineStr">
+        <is>
+          <t>新增 `startup_context.py`、`soft_tool_requirement.py`、`evidence.py`、`session_guard_state.py`；Queue 在明确自主小改且 source+test 已读后进入 `candidate_committed`，只开放 preview/write/test/diff，preview 锚点失败才允许精确重读。`agent.py` 3445 -&gt; 2494，303 tests 通过。</t>
+        </is>
+      </c>
+      <c r="I129" s="0"/>
+      <c r="J129" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9863,7 +9907,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>已完成 P0b 基线，继续观察</t>
+          <t>P0c 已缓解，继续观察</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -9873,7 +9917,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination；T-124/T-125 已抽 RunCollector / RunContext，主文件降至 3445 行。后续新 guard 继续只进独立 steering 模块；真实压测后再决定是否拆 SessionGuardState。</t>
+          <t>T-106 已抽 FinalAnswer Steerer；T-123 已抽 ToolLoop steering/termination；T-124/T-125 已抽 RunCollector / RunContext；T-127 已抽 StartupContext、EvidenceLedger、SoftToolRequirement 与 SessionGuardState，主文件降至 2494 行。后续新 guard 继续只进独立 steering/阶段模块。</t>
         </is>
       </c>
     </row>
@@ -12233,12 +12277,12 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-122 已补 contract/audit/queue/planner/reviewer/no-edit evidence/ToolRegistry 归一、preview contract、final-guard scope、pinned requirement evidence 与 cross-root evidence matrix；T-123 已完成第一批 ToolLoop steering 模块化。真实小改交付链路已跑通，跨项目设计的最小 evidence coverage 也已验证。</t>
+          <t>T-076/T-107 已完成 typed events、terminal frontend、项目边界分析、run summary、真实需求压测、Java LSP 韧性、source-grounded numeric guard 和 token budget；T-109~T-127 已补 contract/audit/queue/planner/reviewer、ToolLoop registry、RunCollector/RunContext、StartupContext、EvidenceLedger、SessionGuardState 和自主小改候选收束。真实小改交付链路已跑通，跨项目设计的最小 evidence coverage 也已验证。</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>继续按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则完成 P0b `RunContext` / `RunStats` 收拢，再用真实需求设计和小改压测检验协同效果。</t>
+          <t>继续按 OMP 的“协议边界 + active loop observer + ToolChoiceQueue 小上限”原则在隔离 worktree 复跑自主小改；不通过则只在现有 Planner/Queue 中修正。</t>
         </is>
       </c>
     </row>
@@ -13575,7 +13619,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 295 个 unittest。</t>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；P10 当前代码已跑通 303 个 unittest。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document T-141 finalization reliability rollout
</commit_message>
<xml_diff>
--- a/docs/local-coding-agent-project-management.xlsx
+++ b/docs/local-coding-agent-project-management.xlsx
@@ -6,11 +6,13 @@
     <sheet name="阶段路线图" sheetId="2" r:id="rId2"/>
     <sheet name="已完成功能" sheetId="3" r:id="rId3"/>
     <sheet name="下一步 Todo" sheetId="4" r:id="rId4"/>
-    <sheet name="风险与决策" sheetId="5" r:id="rId5"/>
-    <sheet name="阶段回顾" sheetId="6" r:id="rId6"/>
-    <sheet name="P7 综合压测问题" sheetId="7" r:id="rId7"/>
-    <sheet name="P5 收口结论" sheetId="8" r:id="rId8"/>
-    <sheet name="推荐工作流" sheetId="9" r:id="rId9"/>
+    <sheet name="下一步 Todo" sheetId="5" r:id="rId5"/>
+    <sheet name="风险与决策" sheetId="6" r:id="rId6"/>
+    <sheet name="风险与决策" sheetId="7" r:id="rId7"/>
+    <sheet name="阶段回顾" sheetId="8" r:id="rId8"/>
+    <sheet name="P7 综合压测问题" sheetId="9" r:id="rId9"/>
+    <sheet name="P5 收口结论" sheetId="10" r:id="rId10"/>
+    <sheet name="推荐工作流" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -101,10 +103,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D37"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
@@ -163,12 +165,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>P10：Intelligence Runtime 骨架 + P0c 架构还债</t>
+          <t>P11：真实跨项目任务收束与日用稳定</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>T-123~T-127 已抽 ToolLoop、RunCollector/RunContext、StartupContext、EvidenceLedger、SoftToolRequirement 与 SessionGuardState；`agent.py` 现为 2494 行。下一步在隔离 worktree 复跑自主小改的 `candidate_committed → preview → write → test → diff` 链路。详见 `docs/pressure-test-2026-07-10.md`。</t>
+          <t>T-128~T-140 已完成 dynamic workspace roots、`/move`、跨 root 只读设计、有界 inventory、path-scoped rules、stable/dev 通道与 benchmark；T-141 已补 bounded finalization coordinator、provider schema violation telemetry 和 multi-root evidence provenance。下一步仍是补结算 DDL、模板/下载中心或正确业务 owner 的源码证据，再走明确小改链路。详见 `docs/pressure-test-2026-07-11.md`。</t>
         </is>
       </c>
       <c r="D4" s="0"/>
@@ -204,7 +206,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>`./agent` 会自动加载安装目录 `.env`，也可显式传 `--env-file`；真实环境变量优先。</t>
+          <t>优先级为真实环境变量、显式 env-file、用户级 `${AGENT_CONFIG_DIR:-~/.config/local-coding-agent}/.env`、workspace `.env`；stable snapshot 不携带密钥。</t>
         </is>
       </c>
       <c r="D6" s="0"/>
@@ -216,11 +218,11 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <v>303</v>
+        <v>441</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>完整 unittest、compileall、xlsx 同步和 diff check 已通过。</t>
+          <t>完整 unittest、compileall、diff check、Excel ZIP integrity 和 deterministic benchmark 已在本轮最终收尾统一通过。</t>
         </is>
       </c>
       <c r="D7" s="0"/>
@@ -458,7 +460,7 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>Startup context / sticky rules</t>
+          <t>Stable / Dev release channels</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -468,7 +470,7 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>用户级和项目级 `AGENTS.md` 启动注入；用户级和项目级 `RULES.md` 每次 provider request 前注入。</t>
+          <t>`lca` 指向已验证的不可变 source snapshot，`lca-dev` 指向当前源码；`lca-release publish` 先跑离线 gate 再原子 promote，失败保留旧 stable snapshot。</t>
         </is>
       </c>
       <c r="D21" s="0"/>
@@ -476,7 +478,7 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>Startup memory</t>
+          <t>Path-scoped rules</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -486,7 +488,7 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>新 session 自动注入项目 `.local-agent/memory/{project,decisions,conventions,learned}.md` 和 state dir `memory/*.md`，作为 advisory context。</t>
+          <t>每个 canonical workspace root 可定义 `.local-agent/rules/*.md`；每轮只注入轻量 metadata，用户或工具路径命中时才注入对应规则正文，规则不改变工具权限。</t>
         </is>
       </c>
       <c r="D22" s="0"/>
@@ -494,7 +496,7 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>Learn 工具</t>
+          <t>Offline benchmark / eval</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -504,7 +506,7 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
+          <t>`benchmarks/tasks` 的隔离 fixture 默认使用 deterministic fake provider 跑真实 Runtime，并输出 JSON/Markdown 结果；`--live` 才显式使用外部 provider。</t>
         </is>
       </c>
       <c r="D23" s="0"/>
@@ -512,7 +514,7 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>Memory consolidation</t>
+          <t>Startup context / sticky rules</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -522,19 +524,15 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>默认 `off`；显式 `--memory-consolidation auto</t>
-        </is>
-      </c>
-      <c r="D24" s="0" t="inlineStr">
-        <is>
-          <t>llm` 后从 session 抽取长期经验；默认写 state dir，`--memory-scope project` 才写 `.local-agent/memory/*.md`。</t>
-        </is>
-      </c>
+          <t>用户级和项目级 `AGENTS.md` 启动注入；用户级和项目级 `RULES.md` 每次 provider request 前注入。</t>
+        </is>
+      </c>
+      <c r="D24" s="0"/>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>Authored skills discovery</t>
+          <t>Startup memory</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -544,7 +542,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
+          <t>新 session 自动注入项目 `.local-agent/memory/{project,decisions,conventions,learned}.md` 和 state dir `memory/*.md`，作为 advisory context。</t>
         </is>
       </c>
       <c r="D25" s="0"/>
@@ -552,7 +550,7 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>Runtime state dir</t>
+          <t>Learn 工具</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -562,7 +560,7 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
+          <t>`learn` 写入 `.local-agent/memory/learned.md`，用于显式沉淀可复用经验。</t>
         </is>
       </c>
       <c r="D26" s="0"/>
@@ -570,7 +568,7 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger</t>
+          <t>Memory consolidation</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -580,15 +578,19 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>Runtime 会从 `read_file`、`search_code`、LSP、patch、run_tests、git 等工具结果提炼短证据账本，作为 provider-bound context 注入，并写入 session JSONL `evidence` 事件。</t>
-        </is>
-      </c>
-      <c r="D27" s="0"/>
+          <t>默认 `off`；显式 `--memory-consolidation auto</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>llm` 后从 session 抽取长期经验；默认写 state dir，`--memory-scope project` 才写 `.local-agent/memory/*.md`。</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>Implementation quality / safe new-file</t>
+          <t>Authored skills discovery</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -598,7 +600,7 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>`git_diff` 会对 comment-only 代码实现 patch 输出 reviewer warning；`write_file dry_run=true` 可预览新文件 diff，真实创建写 patch log，`rollback_patch` 可删除本 session 新建文件。</t>
+          <t>新 session 扫描 `.local-agent/skills/&lt;name&gt;/SKILL.md`，只注入 name、description、source path，正文按需读取。</t>
         </is>
       </c>
       <c r="D28" s="0"/>
@@ -606,7 +608,7 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>No-edit final hygiene</t>
+          <t>Runtime state dir</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -616,7 +618,7 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>实现任务准备以“无法安全实现/目标服务缺失/无改动”停止时，runtime 会要求先做 todo/git 收束，并临时只开放 todo/git hygiene 工具。</t>
+          <t>`--state-dir` / `AGENT_STATE_DIR`；sessions/todos/patch logs 默认写入用户级 state root 下的 workspace-specific 目录。</t>
         </is>
       </c>
       <c r="D29" s="0"/>
@@ -624,7 +626,7 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>Event/Command Protocol</t>
+          <t>Evidence Ledger</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -634,7 +636,7 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>`src/local_agent/protocol/events.py` / `commands.py` 提供 dataclass event/command shape；Runtime 可注入 `EventSink`，CLI 使用 `StderrEventSink` 渲染，session JSONL 写入 `event_v1`。</t>
+          <t>Runtime 会从 `read_file`、`search_code`、LSP、patch、run_tests、git 等工具结果提炼短证据账本，作为 provider-bound context 注入，并写入 session JSONL `evidence` 事件。</t>
         </is>
       </c>
       <c r="D30" s="0"/>
@@ -642,7 +644,7 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend</t>
+          <t>Implementation quality / safe new-file</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -652,7 +654,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>`./agent`、`./agent --chat`、`./agent chat` 进入 terminal-native 交互；可选 `prompt_toolkit` / `rich` 增强输入和输出，缺失时降级；支持 `/help`、`/status`、`/tools`、`/approval`。</t>
+          <t>`git_diff` 会对 comment-only 代码实现 patch 输出 reviewer warning；`write_file dry_run=true` 可预览新文件 diff，真实创建写 patch log，`rollback_patch` 可删除本 session 新建文件。</t>
         </is>
       </c>
       <c r="D31" s="0"/>
@@ -660,7 +662,7 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>Run summary / coverage</t>
+          <t>No-edit final hygiene</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -670,7 +672,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>每轮结束写 `run_summary` session 事件和 `RunSummary` typed event；`/status` 可看最近一轮终止原因、LLM/工具次数、guard/steering/compaction 统计。</t>
+          <t>实现任务准备以“无法安全实现/目标服务缺失/无改动”停止时，runtime 会要求先做 todo/git 收束，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
       <c r="D32" s="0"/>
@@ -678,7 +680,7 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>项目边界分析</t>
+          <t>Event/Command Protocol</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -688,7 +690,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>企业服务边界和项目范围分析工作流放入本机 `.local-agent/memory` / `.local-agent/skills`；runtime 新增 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
+          <t>`src/local_agent/protocol/events.py` / `commands.py` 提供 dataclass event/command shape；Runtime 可注入 `EventSink`，CLI 使用 `StderrEventSink` 渲染，session JSONL 写入 `event_v1`。</t>
         </is>
       </c>
       <c r="D33" s="0"/>
@@ -696,24 +698,658 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
+          <t>Terminal Frontend</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>`./agent`、`./agent --chat`、`./agent chat` 进入 terminal-native 交互；可选 `prompt_toolkit` / `rich` 增强输入和输出，缺失时降级；支持 `/help`、`/status`、`/tools`、`/approval`，并对 `/`、`/workspace`、`/approval` 提供带说明的 Tab 补全。</t>
+        </is>
+      </c>
+      <c r="D34" s="0"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>Run summary / coverage</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>每轮结束写 `run_summary` session 事件和 `RunSummary` typed event；`/status` 可看最近一轮终止原因、LLM/工具次数、guard/steering/compaction 统计。</t>
+        </is>
+      </c>
+      <c r="D35" s="0"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>项目边界分析</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>已完成 MVP 版</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>企业服务边界和项目范围分析工作流放入本机 `.local-agent/memory` / `.local-agent/skills`；runtime 新增 analysis-only 任务识别、named skill soft requirement、自定义 memory_read 安全读取和 final structure gate。</t>
+        </is>
+      </c>
+      <c r="D36" s="0"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
           <t>Memory / Skills 设计</t>
         </is>
       </c>
-      <c r="B34" s="0" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C34" s="0" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>见 `docs/memory-skills-implementation-plan.md`；Markdown memory 注入、`learn`、memory consolidation 和 authored skills discovery 已完成，path-scoped rules / managed skills 后置。</t>
         </is>
       </c>
-      <c r="D34" s="0"/>
+      <c r="D37" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C7"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>P5 收口结论</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>主链路</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>百炼真实小改复测已跑通 todo、dry_run、apply_patch、session allow、rollback、run_tests、git_diff。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>测试</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>P5 收口时 90 个 unittest、compileall、xlsx 检查、diff check 均通过；当前代码已跑通 441 个 unittest。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>日用入口</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>README 已补只读分析和小改任务命令模板。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>开放风险</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>可接受</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>shell 仍非沙箱、prompt injection 仍需靠审批和封闭 VM；provider/model 专用 tokenizer、输出 reserve、managed skills、完整 reviewer 和完整 OMP ToolChoiceQueue 继续后置评估。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>下一阶段</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>真实需求设计与实现压测</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>已验证默认工作流、auto summary、多语言 LSP/light fallback、multi-root、startup memory、learn、authored skills、runtime state dir、多项目只读压测主链路、relevance gate、implementation-quality gate、no-edit final hygiene、semantic exploration guard、terminal input isolation、Event/Command Protocol、Terminal Frontend MVP、项目边界分析 MVP、source-grounded numeric guard、token budget、pinned requirement evidence 和 cross-root evidence matrix；下一步进入一项边界明确的真实需求设计和小改验证。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F15"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>推荐工作流</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>步骤</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>操作</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>建议命令/做法</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>原因</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>适用阶段</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>1</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>确认需求</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>需求复杂时先写到 `docs/requirements/*.md`</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>避免长 prompt 挤占上下文</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>P2+</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>让 Agent 分段 `read_file`</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>启动 Agent</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>`./agent "描述当前项目"`；跨项目用 `./agent --cwd /path/to/project ...`</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>一键启动，默认当前目录为 workspace；跨项目时安装目录 `.env` 会自动作为 `--env-file` 加载</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>P3+</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>token 可来自环境变量、显式 `--env-file` 或 `.env`</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>3</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>权限模式</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>默认 always-ask；写操作可用 write；可信重复工具可 tool-approval allow；信任仓库才 yolo</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>平衡安全和效率</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>P5+</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>`--tool-approval run_tests=allow,shell=prompt,write_file=deny` 可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>4</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>修改前</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Agent 默认会按需 `list_files/read_file/search_code/lsp_*`</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>减少凭空猜测</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>P6+</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>用户不必手写工具顺序</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>5</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>修改时</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>修改已有文件使用 `apply_patch`，写入前优先 `dry_run=true`</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>保留 hash/old_text 校验</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>P1+</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>已写入默认 prompt 和工具描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>6</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>修改后</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>默认应 `run_tests + git_diff`</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>形成可验证闭环</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>P6+</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>自然语言任务默认走验证闭环</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>长任务</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>默认维护 todo，再做实现，再验证；默认 `--summary-mode auto` 按阈值触发 LLM summary</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>防止漏任务并治理长上下文</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>Auto summary 需真实 provider 压测</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>8</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>多目录任务</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>`./agent --cwd /path/to/code --allow-dir /path/to/requirements "读取需求并修改代码"`</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>支持需求文档目录 + 代码项目目录</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>allowed dir 只扩展文件/search/LSP/patch 工具</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>常驻上下文</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>用户级 `AGENTS.md` 放个人偏好，项目 `.local-agent/AGENTS.md` 放项目背景；短规则放对应 `RULES.md`</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>减少重复提示，并让短规则跨长会话可见</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>可用 `AGENT_CONFIG_DIR` 改用户级目录；都是 advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>10</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>项目记忆</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>把长期约定写入 `.local-agent/memory/*.md`，或让 Agent 在明确要求时调用 `learn`；需要自动整理时开启 `--memory-consolidation auto`，默认写 state memory，团队共享才加 `--memory-scope project`</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>减少重复交代项目约定</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>memory 是 advisory，当前用户指令优先；默认不隐式写项目文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>本地 skills</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>将可复用工作流写到 `.local-agent/skills/&lt;name&gt;/SKILL.md`，带 `name` / `description` frontmatter</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>降低重复提示成本</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>P7+</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>启动只注入 metadata，正文按需 read_file</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>有歧义</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>使用 `ask_user` 中途问用户</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>避免模型瞎猜</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>P3+</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>非交互会返回明确错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>同步 Excel</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>`python3 scripts/sync_project_excel.py`</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Excel 是开发展示产物，Markdown 是开发事实源</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>P2+</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>无第三方依赖</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -2926,7 +3562,7 @@
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>当前 287 个测试通过</t>
+          <t>当前 441 个测试通过</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -2952,13 +3588,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:J139"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="48" customWidth="1"/>
@@ -6548,7 +7184,7 @@
       </c>
       <c r="H82" s="0" t="inlineStr">
         <is>
-          <t>已新增 `/help`、`/status`、`/tools`，启动横幅提示 `/help`；`/status` 输出 session/workspace/provider/model/budget/approval，`/tools` 列出工具名；不引入 fullscreen 或新依赖。</t>
+          <t>已新增 `/help`、`/status`、`/tools`，启动横幅提示 `/help`；安装可选 `prompt_toolkit` 后，`/`、`/workspace` 和 `/approval` 支持带说明的 Tab 补全；`/status` 输出 session/workspace/provider/model/budget/approval，`/tools` 列出工具名；不引入 fullscreen 或新依赖。</t>
         </is>
       </c>
       <c r="I82" s="0"/>
@@ -8609,7 +9245,7 @@
       </c>
       <c r="E129" s="0" t="inlineStr">
         <is>
-          <t>已完成单元回归，待真实复跑</t>
+          <t>结构完成；真实压测转入 T-129 闭环</t>
         </is>
       </c>
       <c r="F129" s="0" t="inlineStr">
@@ -8624,11 +9260,451 @@
       </c>
       <c r="H129" s="0" t="inlineStr">
         <is>
-          <t>新增 `startup_context.py`、`soft_tool_requirement.py`、`evidence.py`、`session_guard_state.py`；Queue 在明确自主小改且 source+test 已读后进入 `candidate_committed`，只开放 preview/write/test/diff，preview 锚点失败才允许精确重读。`agent.py` 3445 -&gt; 2494，303 tests 通过。</t>
+          <t>新增 `startup_context.py`、`soft_tool_requirement.py`、`evidence.py`、`session_guard_state.py`；Queue 在明确自主小改且 source+test 已读后进入 `candidate_committed`，`agent.py` 3445 -&gt; 2494。T-129 针对真实压测补齐执行边界、候选路径范围与病态重试上限。</t>
         </is>
       </c>
       <c r="I129" s="0"/>
       <c r="J129" s="0"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="inlineStr">
+        <is>
+          <t>T-128</t>
+        </is>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C130" s="0" t="inlineStr">
+        <is>
+          <t>P10/P11</t>
+        </is>
+      </c>
+      <c r="D130" s="0" t="inlineStr">
+        <is>
+          <t>Dynamic Workspace Roots + OMP 风格 `/move`</t>
+        </is>
+      </c>
+      <c r="E130" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实复测</t>
+        </is>
+      </c>
+      <c r="F130" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G130" s="0" t="inlineStr">
+        <is>
+          <t>跨项目任务过去需退出并以另一 `--cwd` 重启；现在 chat 可追加 roots 或原子移动同一 session 的 primary。</t>
+        </is>
+      </c>
+      <c r="H130" s="0" t="inlineStr">
+        <is>
+          <t>T-128A roots 与 T-128B `/move` 都已落地：只迁移当前 session 的 JSONL/todo/patch artifacts，失败回滚；新 primary 重载 startup context/memory/skills、切换 Git/shell/LSP root，旧 primary 保留为 session root。已补 Runtime post-commit 失败补偿：`relocate`、session append 或 context reload 失败时还原内存、artifact 和 JSONL。真实 session `20260711T005836257738Z` 覆盖 move、双 root 读取、Git primary 与重开恢复。详见 `docs/dynamic-workspace-roots-design.md`、`docs/pressure-test-2026-07-11.md`。</t>
+        </is>
+      </c>
+      <c r="I130" s="0"/>
+      <c r="J130" s="0"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="inlineStr">
+        <is>
+          <t>T-129</t>
+        </is>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C131" s="0" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D131" s="0" t="inlineStr">
+        <is>
+          <t>自主小改候选的执行边界与病态循环收束</t>
+        </is>
+      </c>
+      <c r="E131" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实复测</t>
+        </is>
+      </c>
+      <c r="F131" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G131" s="0" t="inlineStr">
+        <is>
+          <t>T-127 首次复测暴露局部只读误分类、provider 可调用未暴露工具、候选重读扩散与无效 anchored patch 循环。</t>
+        </is>
+      </c>
+      <c r="H131" s="0" t="inlineStr">
+        <is>
+          <t>TaskContract/Queue 统一任务语义；Registry 强制 runtime allowlist；candidate 仅回读已选路径且最多 4 次；连续 3 次失败 preview 以 `tool_choice_queue` 明确停止。最终 session `20260710T232919852951Z` 无 workspace diff，311 tests 通过。详见 `docs/pressure-test-2026-07-11.md`。</t>
+        </is>
+      </c>
+      <c r="I131" s="0"/>
+      <c r="J131" s="0"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="inlineStr">
+        <is>
+          <t>T-130</t>
+        </is>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t>真实跨项目需求只读压测</t>
+        </is>
+      </c>
+      <c r="E132" s="0" t="inlineStr">
+        <is>
+          <t>部分通过，未进入业务写入</t>
+        </is>
+      </c>
+      <c r="F132" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G132" s="0" t="inlineStr">
+        <is>
+          <t>用“拓展服务费结算”需求、`zqylpayment` 后端和 `mpspay` 前端验证 LCA 是否已能自动形成可实施范围。</t>
+        </is>
+      </c>
+      <c r="H132" s="0" t="inlineStr">
+        <is>
+          <t>首轮 session `20260711T013052126987Z` 成功读取三 root 证据，但 323 秒内发生 68 次工具调用、9 次错误、11 次无效结果；deny-capability 已在 session `20260711T014124870469Z` 复测为仅三次指定 read、0 error。订单费用/制单状态、结算单 DDL、模板/下载中心契约未定位，不允许开始业务 patch。T-131 收束跨 root evidence budget/候选事实边界。详见 `docs/pressure-test-2026-07-11.md`。</t>
+        </is>
+      </c>
+      <c r="I132" s="0"/>
+      <c r="J132" s="0"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="inlineStr">
+        <is>
+          <t>T-131</t>
+        </is>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C133" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D133" s="0" t="inlineStr">
+        <is>
+          <t>跨 root 只读设计收束与最终答复韧性</t>
+        </is>
+      </c>
+      <c r="E133" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实复测</t>
+        </is>
+      </c>
+      <c r="F133" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G133" s="0" t="inlineStr">
+        <is>
+          <t>T-130 首轮被误分类和无界 final hygiene 拖至 timeout；需要按 OMP continuation/deadline 原则收束，而不是加主循环总步数。</t>
+        </is>
+      </c>
+      <c r="H133" s="0" t="inlineStr">
+        <is>
+          <t>TaskContract 识别全局禁写；RunContext 对无工具 final resample 上限 8 次且工具后重置；deadline reserve 跳过可选改写。最终答复将纯展示重写与硬性证据/验收门槛分级：仅展示问题可在超时退回草稿，硬门槛在 deadline、continuation 或 timeout 下明确返回未完成/未验证，绝不复用被打回的草稿。真实 session `20260711T115451962229Z` 为 3 reads、0 error、22.3 秒、无 steering hit。详见 `docs/pressure-test-2026-07-11.md`。</t>
+        </is>
+      </c>
+      <c r="I133" s="0"/>
+      <c r="J133" s="0"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="inlineStr">
+        <is>
+          <t>T-132</t>
+        </is>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C134" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D134" s="0" t="inlineStr">
+        <is>
+          <t>文件发现与负向证据可靠性</t>
+        </is>
+      </c>
+      <c r="E134" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实复测</t>
+        </is>
+      </c>
+      <c r="F134" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G134" s="0" t="inlineStr">
+        <is>
+          <t>`/add-dir` inventory 曾把 `search_code` 内容 no-match、截断 `list_files` 和 primary Git 失败错误外推为“added root 可能没有源码”。</t>
+        </is>
+      </c>
+      <c r="H134" s="0" t="inlineStr">
+        <is>
+          <t>A/B：唯一模型可见的 `glob_files` 负责授权 multi-root 的 filename/path discovery；类型匹配负向证据进入 EvidenceLedger、CompletionAudit、FinalAnswerSteerer。C：ToolChoiceQueue 要求每个 authorized root 有成功 glob，限制为 glob/list/read，按 root 两次且总计八次 discovery 后强制收束。20260711T160120792100Z 暴露“盘点”未识别为 inventory，20260711T160317681068 暴露 inventory 错接 candidate read budget；均已修复。最终 live `20260711T160446291065Z` 为 6 LLM/7 tools/0 error，双 root 均覆盖且无 shell/Git/测试/写入。</t>
+        </is>
+      </c>
+      <c r="I134" s="0"/>
+      <c r="J134" s="0"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="inlineStr">
+        <is>
+          <t>T-133</t>
+        </is>
+      </c>
+      <c r="B135" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C135" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D135" s="0" t="inlineStr">
+        <is>
+          <t>Terminal Command Routing / Nested Interaction + shared Command handler</t>
+        </is>
+      </c>
+      <c r="E135" s="0" t="inlineStr">
+        <is>
+          <t>已完成最小实现</t>
+        </is>
+      </c>
+      <c r="F135" s="0" t="inlineStr">
+        <is>
+          <t>Agent + 小红</t>
+        </is>
+      </c>
+      <c r="G135" s="0" t="inlineStr">
+        <is>
+          <t>`/workspace` / `/move` 已有 command dataclass，但 terminal frontend 仍直接调用 Runtime；真实样本还证明 ask/approval 与主 prompt 共用 stdin 时，`/help` / `/workspace list` 会被误回传模型。</t>
+        </is>
+      </c>
+      <c r="H135" s="0" t="inlineStr">
+        <is>
+          <t>严格按 OMP：无 `/` 的文本仍是普通 prompt；shared `TerminalCommandRegistry` 已统一 help/completion/dispatch；`InteractionRequest/Result` + `CHAT/ASK/APPROVAL` focus ownership 已隔离嵌套输入。`/cancel` 回传 cancelled tool result，ASK/APPROVAL slash text 不进入主 dispatcher 或模型；完整 async Command Bus 后置。详见 `docs/terminal-command-routing-and-nested-interaction-design.md`。</t>
+        </is>
+      </c>
+      <c r="I135" s="0"/>
+      <c r="J135" s="0"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="inlineStr">
+        <is>
+          <t>T-134</t>
+        </is>
+      </c>
+      <c r="B136" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C136" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D136" s="0" t="inlineStr">
+        <is>
+          <t>`/move` 后 terminal history 分区重绑定</t>
+        </is>
+      </c>
+      <c r="E136" s="0" t="inlineStr">
+        <is>
+          <t>待开始</t>
+        </is>
+      </c>
+      <c r="F136" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G136" s="0" t="inlineStr">
+        <is>
+          <t>PromptSession/FileHistory 在 chat 启动时绑定旧 state partition，迁移后重启 history 可能断裂。</t>
+        </is>
+      </c>
+      <c r="H136" s="0" t="inlineStr">
+        <is>
+          <t>将 prompt/history 创建与当前 Runtime state dir 解耦；`/move` 成功后安全切换 history path，并覆盖重启回放。</t>
+        </is>
+      </c>
+      <c r="I136" s="0"/>
+      <c r="J136" s="0"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="inlineStr">
+        <is>
+          <t>T-135</t>
+        </is>
+      </c>
+      <c r="B137" s="0" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C137" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D137" s="0" t="inlineStr">
+        <is>
+          <t>项目状态与 Excel 同步</t>
+        </is>
+      </c>
+      <c r="E137" s="0" t="inlineStr">
+        <is>
+          <t>已完成并持续同步</t>
+        </is>
+      </c>
+      <c r="F137" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G137" s="0" t="inlineStr">
+        <is>
+          <t>文档一度仍显示 303/287 tests，无法反映当前运行基线。</t>
+        </is>
+      </c>
+      <c r="H137" s="0" t="inlineStr">
+        <is>
+          <t>当前已统一为 441 个 unittest；每次状态变更后由 `scripts/sync_project_excel.py` 从本 Markdown 重新生成 Excel。</t>
+        </is>
+      </c>
+      <c r="I137" s="0"/>
+      <c r="J137" s="0"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="inlineStr">
+        <is>
+          <t>T-136</t>
+        </is>
+      </c>
+      <c r="B138" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C138" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D138" s="0" t="inlineStr">
+        <is>
+          <t>真实服务费结算 owner 定位与 evidence 收束</t>
+        </is>
+      </c>
+      <c r="E138" s="0" t="inlineStr">
+        <is>
+          <t>已完成第一轮，业务 owner 仍部分缺证据</t>
+        </is>
+      </c>
+      <c r="F138" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G138" s="0" t="inlineStr">
+        <is>
+          <t>requirement primary + 两个 code roots 的真实百炼压测暴露 soft requirement 错绑、owner 任务未触发 cross-root bounded follow-up、final evidence false positive。</t>
+        </is>
+      </c>
+      <c r="H138" s="0" t="inlineStr">
+        <is>
+          <t>仅在 ToolRegistry、soft requirement、evidence/final steerer 中修真实失败；OMP `glob` 方言 `path+pattern` / `maxResults` 在 registry 单点归一。最终 session `20260711T141702815603Z`：134,077 ms、27 tools、0 error、四段式 final；结算 DDL、模板/下载中心契约仍不可当作已定位。</t>
+        </is>
+      </c>
+      <c r="I138" s="0"/>
+      <c r="J138" s="0"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="inlineStr">
+        <is>
+          <t>T-137</t>
+        </is>
+      </c>
+      <c r="B139" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C139" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D139" s="0" t="inlineStr">
+        <is>
+          <t>Terminal chat Enter 提交与多行换行</t>
+        </is>
+      </c>
+      <c r="E139" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实 TTY 复测</t>
+        </is>
+      </c>
+      <c r="F139" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G139" s="0" t="inlineStr">
+        <is>
+          <t>启用 `prompt_toolkit` 时 chat 使用多行编辑器，普通 Enter 插入换行，`/help` 和普通聊天文本都看似无响应。</t>
+        </is>
+      </c>
+      <c r="H139" s="0" t="inlineStr">
+        <is>
+          <t>所有 CHAT 输入改用 Enter 提交；`Esc` + `Enter` 插入多行换行。真实 TTY 已验证 `/help` 和普通文本的 Enter 行为。</t>
+        </is>
+      </c>
+      <c r="I139" s="0"/>
+      <c r="J139" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8639,13 +9715,216 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>下一步 Todo</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>T-138</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Stable / Dev release channels</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>已完成并加固</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>日常 `lca` 不应受工作树未提交变更影响，同时开发仍需立即验证当前源码。</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>新增离线 `lca-release install/publish/promote/status/rollback`：stable 使用原子切换的不可变 source snapshot，`lca-dev` 指向 recorded checkout；publish 前运行 unittest、compileall、diff check 并校验 source digest，失败保持旧 stable。token 从用户级 `${AGENT_CONFIG_DIR:-~/.config/local-coding-agent}/.env` 加载，显式 env-file/真实环境优先，snapshot 不含 `.env`；安装后用 `type -a lca` 检查旧 alias，不自动改 shell 配置。提交 `ee42e2a`、`36573f7`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>T-139</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Path-scoped rules MVP</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>已完成并加固</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>多 root 项目需要局部约定，不能把 A 项目规则污染 B 项目或把自然语言规则当权限。</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>每个 root 的 `.local-agent/rules/*.md` 以 root-relative glob/priority 生效；metadata 每轮可见，正文仅命中路径加载，add/remove/move 后重建索引，坏配置降级。规则目录/文件 strict-resolve 后必须仍在 canonical root；外部或断裂 symlink 不读、不注入，只留 diagnostic。提交 `2a64a59`、`075503f`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>T-140</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Offline reproducible benchmark / eval harness</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实 provider 复测</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Runtime 升级需要不依赖网络、可比较且不污染真实仓库的验收基线。</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>新增 6 个隔离 fixture：单 root、multi-root、scoped negative evidence、小改测 diff、denied schema、budget stop；默认 fake provider，`--live` 显式压测临时 fixture，输出 JSON/Markdown。live 使用 semantic answer/regex + root coverage，报告含 session/run、bounded redacted error、compaction gain；phantom tool evidence 与 active schema 有回归。提交 `4069836`、`9588db9`、`03f7039`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Xiaoya black-box multi-root finalization reliability</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>已完成并真实复测</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>stable `f155a8a` 的黑盒 fixture 曾暴露 finalization ping-pong、无 `run_summary` 悬挂 session、provider 越界工具调用缺少单独遥测，以及 primary 文档证据误导 sibling root。</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>引入独立 `FinalizationCoordinator` 与外层 chat timeout，把 terminal owner、aggregate finalization budget 和 unresolved gate 从主循环里收束出来；`ToolRegistry` / `RunSummary` 单列 `provider_schema_violations`；Evidence / ToolChoiceResult 保留 `root` + `scope` provenance。全量 441 tests、offline benchmark 6/6 通过；百炼 live 两轮四个 session 全部 final、0 error、无悬挂。提交 `e0aeb75`、`d295c5b`、`8527915`。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G107"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
@@ -9944,17 +11223,17 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭 HTTP 400，兼容性继续观察</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>T-108 首轮复测中百炼拒绝历史消息：无效工具调用的 `function.arguments` 为空或畸形 JSON，导致下一轮 HTTP 400</t>
+          <t>T-108 首轮复测中百炼拒绝历史消息：无效工具调用的 `function.arguments` 为空或畸形 JSON，导致下一轮 HTTP 400；T-132C session `20260711T131716175598Z` 仍有 provider-invalid name/arguments。</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>已在 assistant message 入历史前把工具名、id、arguments 统一归一为 provider-safe JSON object 字符串；空/畸形参数写入 `_invalid_arguments`，并补回归测试。</t>
+          <t>assistant message 入历史前把工具名、id、arguments 统一归一为 provider-safe JSON object 字符串；空/畸形参数写入 `_invalid_arguments` 并作为可审计 tool error，而非新增 schema alias 或污染下一轮请求。</t>
         </is>
       </c>
     </row>
@@ -10225,7 +11504,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>R-032</t>
+          <t>R-063</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -10235,22 +11514,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>真实实现可能退化成低价值注释 patch</t>
+          <t>文件发现工具缺位导致错误负向结论</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>已缓解并复跑</t>
+          <t>已关闭 MVP，持续压测</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
+          <t>原样本把内容 no-match、截断目录和 primary Git 失败外推为“没有源码”；首轮 T-132A/B 又暴露百炼会传 `glob_files.path` 与超大结果。</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
+          <t>OMP `glob`/`grep` 分工已落地为 `glob_files`/`search_code`；结构化 complete/truncated/missing metadata 已进入 EvidenceLedger、CompletionAudit 和 FinalAnswerSteerer。T-132C 要求逐 authorized root glob 覆盖、inventory 有界且记录 discovery/misuse；session `20260711T131716175598Z` 没有错误外推。</t>
         </is>
       </c>
     </row>
@@ -10262,32 +11541,32 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>R-033</t>
+          <t>R-069</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>no-edit 停止路径可能跳过收束工具</t>
+          <t>finalization ping-pong 或 root-local 证据漂移导致黑盒 session 不终止</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已关闭 MVP，继续观察 provider 收敛效率</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
+          <t>小牙黑盒 multi-root fixture 在 stable `f155a8a` 上曾出现 `requirement_evidence` / `negative_existence` / `completion_audit` / `tool_usage_evidence` / `forced_final` 交替触发，且有样本没有 `run_summary` 挂住；同时 primary 文档的 “No source code lives here” 会被误导到 sibling service。</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
+          <t>对齐 OMP queue/turn owner：`FinalizationCoordinator` 独立收束 terminal owner、aggregate budget 与 timeout；provider 越界调用单列 telemetry；evidence 记录 `root/scope` provenance。两轮百炼 live fixture 已全部稳定终止。</t>
         </is>
       </c>
     </row>
@@ -10299,32 +11578,32 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>R-035</t>
+          <t>R-032</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
+          <t>真实实现可能退化成低价值注释 patch</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>已缓解并复跑</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
+          <t>T-073 复跑 session `20260709T021349259159Z` 中模型定位到相关 Java 文件，但因 `write_file` 被 deny，最终只给 DTO 字段补 JavaDoc；这不能算真实业务实现</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
+          <t>T-074 已补 implementation-quality reviewer：本轮代码 diff 若只有注释/文档改动，`git_diff` 会提示不能声称行为、校验、解析或测试覆盖变化；复跑 session `20260709T025706579604Z` 没有再做 comment-only patch。</t>
         </is>
       </c>
     </row>
@@ -10336,7 +11615,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>R-036</t>
+          <t>R-033</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -10346,22 +11625,22 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>完整 async command bus 过早引入会扩大复杂度</t>
+          <t>no-edit 停止路径可能跳过收束工具</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
+          <t>T-074 复跑中模型正确停止并说明目标实现属于 `zqyl-investment-plan`，但没有维护 todo，也没有调用 git_diff 证明无改动</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
+          <t>T-075 已参考 OMP current task / tool-choice steering 思路：no-edit stop 缺 todo/git 收束时会触发 runtime steering，并临时只开放 todo/git hygiene 工具。</t>
         </is>
       </c>
     </row>
@@ -10373,7 +11652,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>R-037</t>
+          <t>R-035</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -10383,7 +11662,7 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>纯分析任务被实现任务 hygiene 带偏</t>
+          <t>Runtime 与前端输出耦合会阻碍后续终端体验</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -10393,12 +11672,12 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
+          <t>工具日志、审批显示、最终输出如果继续散落在 Runtime/CLI print，后续 `prompt_toolkit + rich` 前端难以复用和 replay</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
+          <t>T-076 已参考 OMP runtime/TUI 分层思路：Runtime 产出 typed events，CLI 只是第一消费者，session 写 `event_v1`。</t>
         </is>
       </c>
     </row>
@@ -10410,7 +11689,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>R-038</t>
+          <t>R-036</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -10420,22 +11699,22 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>点名 authored skill 但模型不读正文</t>
+          <t>完整 async command bus 过早引入会扩大复杂度</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>已关闭 MVP 版</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
+          <t>T-077 已满足本地 terminal 交互，但 approval/cancel/interrupt 仍是同步路径；如果立刻搬完整异步 command bus，会影响当前稳定的单 Agent runtime</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
+          <t>参考 OMP 分层但按 LCA 裁剪：MVP 先保留同步 `AgentRuntime.run()`，把 event/replay/terminal 输入输出打通；等真实交互压测需要取消、远程 UI 或并发审批时，再升级 Command Bus。</t>
         </is>
       </c>
     </row>
@@ -10447,7 +11726,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>R-039</t>
+          <t>R-037</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -10457,7 +11736,7 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>TUI 命令不可发现会降低日用体验</t>
+          <t>纯分析任务被实现任务 hygiene 带偏</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -10467,12 +11746,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
+          <t>“根据需求和服务边界圈项目范围”曾被 `需求/项目` 等关键词误判为实现任务，导致 git/todo/no-edit 审计干扰或最终只说 ready</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
+          <t>已补 analysis-only 任务识别；此类任务不加 coding workflow nudge、不触发 no-edit final hygiene；纯只读分析默认跳过 todo；final structure gate 会在缺表格/缺指定段落/ready-to-output 时强制无工具重答。</t>
         </is>
       </c>
     </row>
@@ -10484,7 +11763,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>R-040</t>
+          <t>R-038</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -10494,22 +11773,22 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
+          <t>点名 authored skill 但模型不读正文</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>新增，受控</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
+          <t>T-078 压测中模型只看 skill metadata 时，范围分析规则无法充分生效</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
+          <t>已参考 OMP soft tool requirement 思路：prompt 点名已发现的 project skill 时，runtime 会软性要求先 `read_file` 对应 `SKILL.md`。</t>
         </is>
       </c>
     </row>
@@ -10521,7 +11800,7 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>R-041</t>
+          <t>R-039</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -10531,7 +11810,7 @@
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>压测复盘缺少结构化 run coverage</t>
+          <t>TUI 命令不可发现会降低日用体验</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -10541,12 +11820,12 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
+          <t>交互入口已有，但用户需要记 `/approval` 等命令，且缺少当前 runtime 状态视图</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
+          <t>已参考 terminal frontend 设计文档，在 append-only 前端内新增 `/help`、`/status`、`/tools`，不做 fullscreen。</t>
         </is>
       </c>
     </row>
@@ -10558,7 +11837,7 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>R-042</t>
+          <t>R-040</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -10568,22 +11847,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>只读源码验证中重复读取过多</t>
+          <t>过早大拆 `agent.py` 可能打断真实使用验证</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>新增，受控</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
+          <t>Claude review 指出 `agent.py` 已大，但 P0 大拆分会扩大回归面，影响今天可用目标</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
+          <t>接受架构方向但调整顺序：先做 run summary/coverage 和真实压测，再按 startup_context/evidence/compaction/memory_consolidation/steering 分批抽模块。</t>
         </is>
       </c>
     </row>
@@ -10595,7 +11874,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>R-043</t>
+          <t>R-041</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -10605,22 +11884,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>最终回答轻微结构漂移和过度断言</t>
+          <t>压测复盘缺少结构化 run coverage</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP 版</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
+          <t>只有 session 原文和最终回答时，很难判断模型卡在哪个 guard、用了多少工具、是否触发 compaction 或为什么结束</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
+          <t>已参考 OMP run-collector 思路，新增每轮 `run_summary`：工具次数、guard/steering、compaction、termination reason 统一落 session 和事件流。</t>
         </is>
       </c>
     </row>
@@ -10632,17 +11911,17 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>R-044</t>
+          <t>R-042</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>证据型只读问题先输出推测</t>
+          <t>只读源码验证中重复读取过多</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -10652,12 +11931,12 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
+          <t>T-084 中 `read_file` 54 次、`list_files` 10 次，重复读取同一批证据文件但没有 guard/steering 命中</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
+          <t>已参考 OMP pruning / soft escalation / evidence sufficiency：对已读同范围做 evidence-aware repetition guard，达到阈值后返回已有 evidence 摘要并触发 final-answer steering。</t>
         </is>
       </c>
     </row>
@@ -10669,17 +11948,17 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>R-045</t>
+          <t>R-043</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>语义级路径探索扩散</t>
+          <t>最终回答轻微结构漂移和过度断言</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -10689,12 +11968,12 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
+          <t>T-084 要求项目表，但最终输出表名表；还把 `IntentionConfigApplication` 表述为 Spring Boot 启动/配置类，证据不足</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
+          <t>已增强 Current task contract 和 final gate：项目范围表必须含项目/服务列；证据状态要求会触发已验证/推断标签检查。</t>
         </is>
       </c>
     </row>
@@ -10706,17 +11985,17 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>R-046</t>
+          <t>R-044</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>终端输出被用户输入污染</t>
+          <t>证据型只读问题先输出推测</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -10726,12 +12005,12 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
+          <t>“前端密码加密/后端怎么处理”问题中，模型未读关键登录/密码文件就先给“可能 HTTPS 明文 + 后端哈希”的推测</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
+          <t>T-088 已完成：无成功 `read_file` 的证据型回答会被 runtime steering 拦住并临时只开放证据工具；search/LSP no-match 负向证据可明确收束。</t>
         </is>
       </c>
     </row>
@@ -10743,32 +12022,32 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>R-047</t>
+          <t>R-045</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
+          <t>语义级路径探索扩散</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
+          <t>用户纠正后出现大量相似目录 list_files、父子目录扩散、Path not found 和大目录读取；exact duplicate guard 太晚命中</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
+          <t>T-089 已完成：semantic exploration guard 按模块/父目录/Path-not-found pattern 小上限收束，并引导回 search_code/read_file/LSP 证据工具。</t>
         </is>
       </c>
     </row>
@@ -10780,7 +12059,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>R-048</t>
+          <t>R-046</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -10790,22 +12069,22 @@
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>`agent.py` 继续膨胀影响后续维护</t>
+          <t>终端输出被用户输入污染</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>已开始缓解</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
+          <t>日志出现 `33333333333[tool:start]`，说明一次性 CLI 运行中键盘输入被终端 echo 到 transcript</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
+          <t>T-090 已完成：一次性 CLI、REPL 和 terminal chat 在 agent run 期间关闭 TTY echo；approval / ask_user 会恢复输入并 flush 误敲缓冲。</t>
         </is>
       </c>
     </row>
@@ -10817,7 +12096,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>R-049</t>
+          <t>R-064</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -10827,22 +12106,22 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
+          <t>主 command 与嵌套 ask/approval 输入归属混淆</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>已缓解</t>
+          <t>已关闭 MVP，继续观察 async 场景</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
+          <t>用户在 ask 内输入 `/help`、`/workspace list` 会被当作模型答案；漏写 `/` 的 add-dir 样本也容易让用户误以为命令已执行。</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
+          <t>T-133 参考 OMP InputController/Extension UI focus ownership：只有 `/` 开头的 CHAT 文本进 command registry；ASK/APPROVAL 使用 frontend-focused controller，slash text 本地消费，`/cancel` 回传 cancelled tool result。完整 streaming queue 后置。</t>
         </is>
       </c>
     </row>
@@ -10854,7 +12133,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>R-050</t>
+          <t>R-065</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -10864,22 +12143,22 @@
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>真实环境未预置外部 LSP server</t>
+          <t>prompt 中声明“禁止 LSP”等工具限制不是权限边界</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>已部分关闭，转为 R-051</t>
+          <t>开放，使用显式 policy</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
+          <t>T-136 prompt 写了“禁止 LSP”，但未通过 tool policy deny，provider 仍调用 `lsp_workspace_symbols`。</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
+          <t>对齐 OMP active-tool / mode 模型：权限必须由 active tool set/approval policy 实施；需要禁用 LSP 时显式 deny 各 LSP 工具，不解析自然语言关键词作为安全策略。</t>
         </is>
       </c>
     </row>
@@ -10891,32 +12170,32 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>R-051</t>
+          <t>R-047</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
+          <t>Vue 模板改动可能被 comment-only reviewer 误报</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>已缓解，根因待环境补齐</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
+          <t>implementation-quality reviewer 原本使用全局注释行判断，JavaDoc 标签规则可能误伤 Vue/JSX 模板 markup</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
+          <t>T-091 已完成：comment-only 判断按文件后缀区分，JavaDoc markup 只在 Java 中生效，Vue `&lt;p&gt;` 模板替换不会触发实现质量误报。</t>
         </is>
       </c>
     </row>
@@ -10928,291 +12207,291 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>R-052</t>
+          <t>R-048</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>非法 tool_call 污染历史导致 provider 400</t>
+          <t>`agent.py` 继续膨胀影响后续维护</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>已关闭</t>
+          <t>已开始缓解</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
+          <t>Claude review 指出 OMP 的主循环、compaction、telemetry、LSP 等关注点分离，而 LCA 的 `agent.py` 已承担过多职责</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
+          <t>T-092 已先抽出 `compaction.py`，后续继续按低风险顺序拆 `evidence.py` / `run_collector.py` / `startup_context.py` / `memory_consolidation.py`，暂不一次性重写主循环。</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>ADR-001</t>
+          <t>R-049</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
+          <t>Java/JS/Vue 仅靠轻量 LSP 会漏报或误报</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已缓解</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>好设计可直接采用，复杂度按需收敛</t>
+          <t>企业项目以 Java/Vue/JS 为主，regex fallback 难以提供完整 definition/reference/diagnostic 证据</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
+          <t>T-093 已参考 OMP 的 LSP client 子系统，接入可选外部 language server；无依赖时仍回退 light fallback 并标注 confidence，避免封闭 VM 默认强依赖。</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>ADR-002</t>
+          <t>R-050</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>max_steps 只作为防失控保险丝</t>
+          <t>真实环境未预置外部 LSP server</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已部分关闭，转为 R-051</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>默认值已改为 0，不限步</t>
+          <t>T-094 证明当前机器只有 `mvn` / `npm`，没有 `jdtls`、`typescript-language-server`、`vue-language-server`，因此 Java 企业项目仍只能走 light fallback</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
+          <t>T-095 已安装 `jdtls 1.60.0`；TS/Vue server 仍未预置，后续按真实前端项目再处理。</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>ADR-003</t>
+          <t>R-051</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>todo、ask_user、per-tool approval 是主功能</t>
+          <t>JDTLS 在企业项目上 diagnostics 可用但 symbols/definition 未达标</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>已落地</t>
+          <t>已缓解，根因待环境补齐</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>P3 已实现</t>
+          <t>T-095 证明极小 Maven 项目 external code navigation 全通，但 `crcl-open` / `zqyl-user-center-service` 因缺公司内部 parent POM 无法被 Maven/jdtls 导入为完整 Java project</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
+          <t>T-095/T-096 已补 OMP 风格 LSP 初始化、server request 响应、project load 等待和 Java configuration；T-097/T-098/T-099 已让 `lsp_status probe=true` 可报告 project/source path 健康度、缺失 Maven parent GAV 和 Maven settings/localRepository/mirror/profile 环境状态；T-100/T-101 已验证并增强 external 不完整时的 fallback 类/方法定位。真正 type-aware navigation 仍需要补齐本地 Maven 私服/parent POM/依赖缓存。</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>ADR-004</t>
+          <t>R-052</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>高</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>第一阶段 memory 用 Markdown</t>
+          <t>非法 tool_call 污染历史导致 provider 400</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>后续看需求升级</t>
+          <t>T-102 session `20260709T091405931143Z` 中模型生成空工具名，下一轮百炼拒绝历史消息</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
+          <t>T-103 已按 OMP provider-safe / synthetic result 思路，在 runtime 边界规范化 assistant tool_call，保证后续请求合法，同时向模型回传未知/无效工具错误。</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>ADR-005</t>
+          <t>R-066</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Patch 先用 anchored patch，不上 AST edit</t>
+          <t>开发工作树未提交变更影响日用入口</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP，继续观察发布纪律</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>P5 再评估 preview/rollback</t>
+          <t>Stable snapshot 与 dev checkout 已分离；publish 是显式离线 gate + 原子 promote，失败保留旧 stable。</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
+          <t>对齐 OMP 已安装 CLI 与开发 checkout 分离原则。</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>ADR-006</t>
+          <t>R-067</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>长需求建议放文件让 Agent read_file</t>
+          <t>多 root 规则相互污染或被误当作权限</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP，继续观察 prompt 成本</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>README 已写推荐工作流</t>
+          <t>Path rule index 以 canonical root 隔离；规则 advisory，不扩大 shell/Git/patch 权限。</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
+          <t>对齐 OMP project context/discovery；自然语言规则不是 policy。</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t>ADR</t>
+          <t>风险</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>ADR-007</t>
+          <t>R-068</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>中</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>封闭 VM 下不做公网搜索/自动下载</t>
+          <t>Runtime 改动缺少可重复离线验收基线</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已关闭 MVP，持续扩充任务</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>依赖提前准备</t>
+          <t>临时 fixture + deterministic provider 跑完整 Runtime，live provider 仅显式执行。</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
+          <t>对齐 OMP run/coverage 可观测性。</t>
         </is>
       </c>
     </row>
@@ -11224,7 +12503,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>ADR-008</t>
+          <t>ADR-001</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -11234,7 +12513,7 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
+          <t>优先采纳 OMP 成熟设计，按本地目标裁剪</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -11244,12 +12523,12 @@
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>持续同步本文件和 `project-status.md`</t>
+          <t>好设计可直接采用，复杂度按需收敛</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
+          <t>OMP 是重要参考实现；我们不为了“避免复制”而绕开好设计。采用标准是收益是否大于复杂度，并且不破坏个人本地使用、封闭 VM、无公网依赖和第一阶段 MVP 边界。</t>
         </is>
       </c>
     </row>
@@ -11261,7 +12540,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-002</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -11271,22 +12550,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>OMP 核心架构笔记单独固化</t>
+          <t>max_steps 只作为防失控保险丝</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>见 `docs/omp-core-architecture-notes.md`</t>
+          <t>默认值已改为 0，不限步</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
+          <t>OMP 的 stepCounter 主要用于 telemetry，终止靠无 tool_calls、deadline、abort；我们把 `max_steps` 仅作为显式保险丝。</t>
         </is>
       </c>
     </row>
@@ -11298,7 +12577,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>ADR-010</t>
+          <t>ADR-003</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -11308,22 +12587,22 @@
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
+          <t>todo、ask_user、per-tool approval 是主功能</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已落地</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
+          <t>P3 已实现</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
+          <t>OMP 将 todo、approval、elicitation 做成可观测会话能力；我们 P3 先做终端轻量版，后续再补 UI 化。</t>
         </is>
       </c>
     </row>
@@ -11335,7 +12614,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>ADR-011</t>
+          <t>ADR-004</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -11345,22 +12624,22 @@
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>默认采用 OMP 风格 auto summary</t>
+          <t>第一阶段 memory 用 Markdown</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
+          <t>后续看需求升级</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
+          <t>OMP 有本地 memory 后台抽取，并在启动时注入 Memory Guidance；我们先用项目 Markdown，后续再做自动整理。</t>
         </is>
       </c>
     </row>
@@ -11372,7 +12651,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>ADR-012</t>
+          <t>ADR-005</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -11382,22 +12661,22 @@
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>LSP 第一版做轻量多语言静态工具</t>
+          <t>Patch 先用 anchored patch，不上 AST edit</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>已接受并被 ADR-032 增强</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
+          <t>P5 再评估 preview/rollback</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
+          <t>OMP 的 edit/apply_patch 结合审批、渲染和更丰富编辑链路；我们先做 anchored patch 与 dry_run，AST edit 后置。</t>
         </is>
       </c>
     </row>
@@ -11409,7 +12688,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>ADR-013</t>
+          <t>ADR-006</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -11419,22 +12698,22 @@
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
+          <t>长需求建议放文件让 Agent read_file</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>已接受并部分落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
+          <t>README 已写推荐工作流</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
+          <t>OMP 会自动发现 context files，也支持按需读取 Markdown；我们让复杂需求落 md，再用 `read_file` 分段注入。</t>
         </is>
       </c>
     </row>
@@ -11446,17 +12725,17 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>ADR-014</t>
+          <t>ADR-007</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>Runtime 问题优先采用 OMP 已验证设计</t>
+          <t>封闭 VM 下不做公网搜索/自动下载</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
@@ -11466,12 +12745,12 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
+          <t>依赖提前准备</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
+          <t>OMP 可接 web、MCP、插件等外部能力，并由配置和 approval 管控；我们封闭 VM 默认离线，依赖提前准备。</t>
         </is>
       </c>
     </row>
@@ -11483,32 +12762,32 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>ADR-015</t>
+          <t>ADR-008</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>人工上下文按 AGENTS/RULES 分层</t>
+          <t>Excel 给人看，Markdown 给开发协作 Agent 读</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
+          <t>持续同步本文件和 `project-status.md`</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
+          <t>这套项目管理文档服务于开发 LCA 的过程，不是 LCA 运行时 memory。我们以 Markdown 作为开发项目事实源，Excel 只生成展示视图。</t>
         </is>
       </c>
     </row>
@@ -11520,32 +12799,32 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>ADR-016</t>
+          <t>ADR-009</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
+          <t>OMP 核心架构笔记单独固化</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
+          <t>见 `docs/omp-core-architecture-notes.md`</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
+          <t>OMP 的关键判断来自源码和 docs，需要沉淀成项目 context；我们单独维护笔记，避免每次重复扫源码。</t>
         </is>
       </c>
     </row>
@@ -11557,32 +12836,32 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>ADR-017</t>
+          <t>ADR-010</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
+          <t>P6 优先实现 OMP 默认工作流的本地 MVP 版</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并落地</t>
         </is>
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>先找 OMP 已验证设计，再按 LCA 本地个人 Agent、封闭 VM、单 Agent 和无自动下载边界裁剪</t>
+          <t>已做 system prompt、tool descriptions、轻量 runtime nudge</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>用户明确要求后续解决问题都参考 OMP；allowed-dir 问题按 OMP 显式提供 cwd/project context 的思路，落地为 `[Workspace roots]` 注入。</t>
+          <t>OMP 的体验来自系统上下文、工具规范和 runtime 纠偏共同作用；我们直接采纳分层设计，但暂不搬入完整 ToolChoiceQueue、subagents 等复杂能力。</t>
         </is>
       </c>
     </row>
@@ -11594,17 +12873,17 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>ADR-018</t>
+          <t>ADR-011</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>Evidence Ledger 作为 provider-bound runtime context，而不是长期 memory</t>
+          <t>默认采用 OMP 风格 auto summary</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
@@ -11614,12 +12893,12 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>工具证据是本轮会话事实，应帮助最终回答区分证据与推断，但不应写入项目长期 memory 或替代 session 原文</t>
+          <t>`summary_mode=auto` 默认，`local` / `llm` 可选</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP 将 runtime state / tool evidence / steering 持续放进模型上下文的做法；LCA 中 Evidence Ledger 由 runtime 中央观察工具结果生成，短窗口注入 provider context，并写 session `evidence` 事件用于审计。</t>
+          <t>小历史不摘要；超过 reserve 阈值才调用已配置 AI API 做 LLM summary；失败回退 local summary。</t>
         </is>
       </c>
     </row>
@@ -11631,32 +12910,32 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>ADR-019</t>
+          <t>ADR-012</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>P7 后续先进入真实需求实现压测，reviewer / 完整 ToolChoiceQueue 条件触发</t>
+          <t>LSP 第一版做轻量多语言静态工具</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并被 ADR-032 增强</t>
         </is>
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>执行 T-072；T-073 按压测失败形态选择实现</t>
+          <t>第一版不启动外部 language server；T-093 后支持可选外部 adapter</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>阶段回顾显示当前主链路已具备低风险实战条件；完整 reviewer / ToolChoiceQueue 应根据真实实现压测暴露的问题裁剪，而不是在缺少失败样本时提前做重。</t>
+          <t>第一版满足 Python、Java、JavaScript、TypeScript、Vue 的 symbols/definition/references/diagnostics；后续按 ADR-032 接入可选外部 LSP，不自动下载依赖。</t>
         </is>
       </c>
     </row>
@@ -11668,32 +12947,32 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>ADR-013</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>T-073 优先做轻量 relevance gate / reviewer，不先做完整 ToolChoiceQueue</t>
+          <t>Memory / skills 按 OMP 思路分阶段本地化</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
-          <t>已接受</t>
+          <t>已接受并部分落地</t>
         </is>
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>先做写入前目标相关性检查、workspace-root evidence 和最终 diff reviewer</t>
+          <t>Markdown memory 启动注入、显式 `learn` 和 authored skills discovery 已完成</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>T-072 失败点是无关 patch 和反事实 workspace 判断；完整 ToolChoiceQueue 继续作为工具选择失控时的后补。</t>
+          <t>后续最后才评估 managed skills/autolearn；不引入 Hindsight、Mnemopi、向量库或插件市场。</t>
         </is>
       </c>
     </row>
@@ -11705,32 +12984,32 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>ADR-021</t>
+          <t>ADR-014</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>T-074 先补实现质量 gate 和受控新文件策略，再决定是否上完整 ToolChoiceQueue</t>
+          <t>Runtime 问题优先采用 OMP 已验证设计</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+          <t>已接受</t>
         </is>
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>已完成 no-comment-only reviewer / safe new-file policy</t>
+          <t>直接采纳 OMP 的成熟机制，再按本地/封闭 VM/MVP 边界裁剪</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>T-073 证明 relevance gate 有效，但仍不能保证 patch 有业务实现价值；T-074 已先补“什么算有效实现”和“何时允许新文件”。</t>
+          <t>对 deadline、compaction、permission、synthetic tool result、todo/tool-choice steering、pruning 这类 OMP 已覆盖的问题，不再为了“自己造一套”而绕开；LCA 不内置“企业数据不能外发”禁令，但必须尊重当前执行宿主或企业环境的策略拦截。</t>
         </is>
       </c>
     </row>
@@ -11742,17 +13021,17 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>ADR-022</t>
+          <t>ADR-015</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>实现任务允许诚实停止，但 no-edit final 也要可审计</t>
+          <t>人工上下文按 AGENTS/RULES 分层</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
@@ -11762,12 +13041,12 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-075</t>
+          <t>`AGENTS.md` 适合启动背景，`RULES.md` 适合短 sticky rules；二者不同于长期 memory、skills 和 session summary</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>T-074 证明“证据不足时停止”比强行注释 patch 更好；T-075 用 provider context + runtime steering 保证停止路径也补 todo/git 证据。</t>
+          <t>参照 Claude Code 的 CLAUDE.md/rules 与 OMP 的 AGENTS.md/RULES.md 思路；LCA 使用用户级配置目录和项目 `.local-agent` 目录做本地 MVP。</t>
         </is>
       </c>
     </row>
@@ -11779,17 +13058,17 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>ADR-024</t>
+          <t>ADR-016</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>Runtime 先产出 replayable typed events，再做 Terminal Frontend</t>
+          <t>Session memory consolidation 默认关闭，开启后默认写 state memory</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
@@ -11799,12 +13078,12 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>已完成 T-076</t>
+          <t>这一步不同于只发给模型的 context compaction；默认 off 保护只读分析，开启后默认写用户级 state dir；只有显式 `memory_scope=project` 才写项目 `.local-agent/memory`</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>参考 OMP runtime/TUI engine 分层，但本地化为 Python dataclass、`EventEmitter`、`EventSink` 和 session `event_v1`；暂不引入 Pydantic、异步队列或重 UI。</t>
+          <t>显式 `auto/llm` 后才用当前 provider 抽取长期记忆；memory 仍是 advisory，当前用户指令和源码证据优先。</t>
         </is>
       </c>
     </row>
@@ -11816,32 +13095,32 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>ADR-025</t>
+          <t>ADR-017</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>Terminal Frontend MVP 保持同步 runtime，先不引入完整 async command bus</t>
+          <t>解决 runtime/工具/上下文问题时先查 OMP 做法</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>已接受并落地</t>
+         